<commit_message>
Record Stage 6.2 CI and acceptance progress
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbcc6ef6dd7244740"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R56af74fc9480497f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R6942fa7d3d094c43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R86a466bdba814c62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R320ca74f24944b28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Ra60c38c0f75045a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R1c516358d9f8461d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rfd9626648cc64d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rd484d1c0a10f4c27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rea01f118d0ac4593"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R9e05219a75484dfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R3dad5851471c4e9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R537b13b82f414621"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rdc41449dc64c4131"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1c37802400834376"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R333281003a734f29"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1316,7 +1316,7 @@
       </x:c>
       <x:c r="B8" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>26</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C8" s="88"/>
       <x:c r="D8" s="97" t="str">
@@ -1332,7 +1332,7 @@
         <x:v>Next functionality</x:v>
       </x:c>
       <x:c r="H8" s="98" t="str">
-        <x:v>Stage 6.2 CI, testing and staging</x:v>
+        <x:v>Persistent staging, required CI check and monitoring</x:v>
       </x:c>
       <x:c r="I8" s="98"/>
       <x:c r="J8" s="99"/>
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="B10" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>24</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C10" s="88"/>
       <x:c r="D10" s="97" t="str">
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.837810945273632</x:v>
+        <x:v>0.8504975124378114</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1504,7 +1504,7 @@
       </x:c>
       <x:c r="B17" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>26</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C17" s="110" t="str">
         <x:v>Foundation exists; end-to-end feature incomplete</x:v>
@@ -1542,7 +1542,7 @@
       </x:c>
       <x:c r="B19" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>24</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C19" s="110" t="str">
         <x:v>Not implemented</x:v>
@@ -1617,10 +1617,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B24" s="115" t="str">
-        <x:v>Homepage branch review and merge</x:v>
+        <x:v>Homepage review and merge — completed</x:v>
       </x:c>
       <x:c r="C24" s="107" t="str">
-        <x:v>Owner approved visuals; commit 936baee is pushed. Review branch and merge only after approval.</x:v>
+        <x:v>PR #5 reviewed and merged into main on 30 Sep 2026 (merge c1ef18d).</x:v>
       </x:c>
       <x:c r="D24" s="88"/>
       <x:c r="E24" s="88"/>
@@ -1635,10 +1635,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B25" s="117" t="str">
-        <x:v>Stage 6.2 quality system</x:v>
+        <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>Add CI, integration/E2E foundation and staging; retain live map acceptance as an explicit blocker.</x:v>
+        <x:v>PR #6: CI passed; isolated DB tests 3/3, sweep 99 URLs/0 issues, desktop/mobile Chromium 11 passed. Persistent online staging remains open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1653,10 +1653,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B26" s="117" t="str">
-        <x:v>Database and browser acceptance</x:v>
+        <x:v>Persistent staging and monitoring</x:v>
       </x:c>
       <x:c r="C26" s="110" t="str">
-        <x:v>Complete populated seller, dealer and admin journeys and record defects before launch.</x:v>
+        <x:v>Configure hosted preview with separate DB/media, require passing PR check, and enable external alerts.</x:v>
       </x:c>
       <x:c r="D26" s="88"/>
       <x:c r="E26" s="88"/>
@@ -1671,10 +1671,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B27" s="117" t="str">
-        <x:v>Stage 6.2 quality system</x:v>
+        <x:v>Complete remaining launch acceptance</x:v>
       </x:c>
       <x:c r="C27" s="110" t="str">
-        <x:v>Add CI, automated integration/E2E foundation and staging when functionality is complete.</x:v>
+        <x:v>Automate registration, listing submission/contact, dealer registration, moderation mutations and Safari mobile; verify live provider integrations.</x:v>
       </x:c>
       <x:c r="D27" s="88"/>
       <x:c r="E27" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5abc97d90bb643a6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44369242059c4d35"/>
 </x:worksheet>
 </file>
 
@@ -1856,7 +1856,7 @@
         <x:v>Active package</x:v>
       </x:c>
       <x:c r="B7" s="127" t="str">
-        <x:v>Homepage visual package pushed; Stage 6.2 next</x:v>
+        <x:v>Stage 6.2 CI and isolated DB/browser acceptance in PR #6; persistent online staging remains open</x:v>
       </x:c>
       <x:c r="C7" s="127"/>
       <x:c r="D7" s="127"/>
@@ -1868,7 +1868,7 @@
         <x:v>Current branch</x:v>
       </x:c>
       <x:c r="B8" s="127" t="str">
-        <x:v>codex/homepage-visuals (pushed)</x:v>
+        <x:v>codex/launch-quality-system (pushed; PR #6 open)</x:v>
       </x:c>
       <x:c r="C8" s="127"/>
       <x:c r="D8" s="127"/>
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Owner approved homepage visuals on 30 Sep 2026. Commit 936baee is pushed to origin/codex/homepage-visuals. Full checks, lint and build pass; final cross-route browser/DB and live Google Maps acceptance remain open.</x:v>
+        <x:v>Homepage PR #5 merged into main on 30 Sep 2026. Stage 6.2 PR #6 GitHub Actions run #36631593477 passed: seeded test DB, 3 database checks, 99-route sweep and desktop/mobile Chromium suite. Online staging, required branch check, external monitoring and deeper transaction/browser journeys remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2694,10 +2694,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F12" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G12" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.85</x:v>
       </x:c>
       <x:c r="H12" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2718,10 +2718,10 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>No CI/CD workflow exists.</x:v>
+        <x:v>PR #6 GitHub Actions run #36631593477 passed migrations, seeds, DB tests, checks, lint, build, sweep and Chromium.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
-        <x:v>Create GitHub Actions workflow and required checks.</x:v>
+        <x:v>Mark check required in branch protection and demonstrate deliberate failure blocks merge.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2765,10 +2765,10 @@
         <x:v>Deployment smoke; robots noindex; data isolation</x:v>
       </x:c>
       <x:c r="N13" s="136" t="str">
-        <x:v>Only local preview is currently established.</x:v>
+        <x:v>CI creates an isolated ephemeral test environment; persistent hosted preview is not configured.</x:v>
       </x:c>
       <x:c r="O13" s="136" t="str">
-        <x:v>Choose hosting and configure staging.</x:v>
+        <x:v>Select hosting, separate staging DB and durable media; then verify noindex and deployment smoke.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2882,10 +2882,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F16" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G16" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.45</x:v>
       </x:c>
       <x:c r="H16" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2906,10 +2906,10 @@
         <x:v>Unit; integration; transaction tests</x:v>
       </x:c>
       <x:c r="N16" s="136" t="str">
-        <x:v>Only SEO policy assertions currently exist.</x:v>
+        <x:v>Node test runner validates seeded reference data, all three inventory verticals and taxonomy facet integrity on isolated PostgreSQL.</x:v>
       </x:c>
       <x:c r="O16" s="136" t="str">
-        <x:v>Add test runner and seeded test database.</x:v>
+        <x:v>Add transactional success/validation/authorization/rollback tests for critical actions.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2929,10 +2929,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F17" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G17" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.55</x:v>
       </x:c>
       <x:c r="H17" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2953,10 +2953,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>No E2E suite exists.</x:v>
+        <x:v>Playwright desktop/mobile Chromium: 11 passed, 1 desktop-only skip; homepage search, browse, auth gates, seller/admin sign-in and mobile overflow.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Add Playwright or equivalent after core routes stabilize.</x:v>
+        <x:v>Cover listing creation/contact, registration, dealer submission, moderation mutations and accessibility.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -10637,10 +10637,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F181" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G181" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="H181" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10661,10 +10661,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>No automated E2E suite.</x:v>
+        <x:v>PR #6 browser foundation passes 11 desktop/mobile Chromium cases; no submission or mutation journey yet.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Implement incrementally by module.</x:v>
+        <x:v>Automate registration through contact, listing creation, dealer registration and moderation changes.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -10684,10 +10684,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F182" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G182" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="H182" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10708,10 +10708,10 @@
         <x:v>Real/simulated devices; slow network</x:v>
       </x:c>
       <x:c r="N182" s="136" t="str">
-        <x:v>Responsive code exists; formal QA incomplete.</x:v>
+        <x:v>Simulated Android Chromium checks pass for homepage search, browse, seller/admin login, auth gates and width.</x:v>
       </x:c>
       <x:c r="O182" s="136" t="str">
-        <x:v>Create device checklist and execute before launch.</x:v>
+        <x:v>Test iPhone Safari and mobile upload/keyboard on hosted staging.</x:v>
       </x:c>
     </x:row>
     <x:row r="183">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6653225883140f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e5b4953da08409b"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12831,7 +12831,7 @@
         <x:v>Deliberate failure blocks merge; staging smoke passes.</x:v>
       </x:c>
       <x:c r="G23" s="141" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9d70d8bdede4975"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdaa1a575bbb4bf0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13009,10 +13009,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E7" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Playwright valid seller/admin login on desktop/mobile</x:v>
       </x:c>
       <x:c r="F7" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Partial pass: valid sign-in; invalid/banned cases pending</x:v>
       </x:c>
       <x:c r="G7" s="141" t="str">
         <x:v>Users in each state</x:v>
@@ -13529,10 +13529,10 @@
         <x:v>SEO unit + E2E</x:v>
       </x:c>
       <x:c r="E27" s="141" t="str">
-        <x:v>Automated partial</x:v>
+        <x:v>SEO checks plus Playwright unknown facet 404</x:v>
       </x:c>
       <x:c r="F27" s="141" t="str">
-        <x:v>37 SEO tests pass</x:v>
+        <x:v>Partial pass: unknown 404; reordered URL browser check pending</x:v>
       </x:c>
       <x:c r="G27" s="141" t="str">
         <x:v>Facet cases</x:v>
@@ -13997,10 +13997,10 @@
         <x:v>Visual regression</x:v>
       </x:c>
       <x:c r="E45" s="141" t="str">
-        <x:v>Manual deferred</x:v>
+        <x:v>Owner visual review plus Playwright mobile width check</x:v>
       </x:c>
       <x:c r="F45" s="141" t="str">
-        <x:v>Homepage visuals owner-approved and pushed; comprehensive cross-route responsive/branding QA pending</x:v>
+        <x:v>Partial pass: approved homepage; mobile width passes; Safari/cross-route QA pending</x:v>
       </x:c>
       <x:c r="G45" s="141" t="str">
         <x:v>PR #2 local preview</x:v>
@@ -14023,10 +14023,10 @@
         <x:v>E2E</x:v>
       </x:c>
       <x:c r="E46" s="141" t="str">
-        <x:v>Manual</x:v>
+        <x:v>Playwright desktop/mobile homepage search tabs</x:v>
       </x:c>
       <x:c r="F46" s="141" t="str">
-        <x:v>Awaiting automation</x:v>
+        <x:v>Passed: car/bike/parts navigation; deeper filter combinations pending</x:v>
       </x:c>
       <x:c r="G46" s="141" t="str">
         <x:v>Seeded taxonomy</x:v>
@@ -14257,10 +14257,10 @@
         <x:v>Deployment integration</x:v>
       </x:c>
       <x:c r="E55" s="141" t="str">
-        <x:v>Manual + repair</x:v>
+        <x:v>GitHub CI plus local clean isolated DB</x:v>
       </x:c>
       <x:c r="F55" s="141" t="str">
-        <x:v>Passed locally; Google-auth schema repair verified</x:v>
+        <x:v>Passed local and CI #36631593477: migrations, curated/demo seed, DB assertions</x:v>
       </x:c>
       <x:c r="G55" s="141" t="str">
         <x:v>Fresh PostgreSQL</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R258092b1c4f949e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3df76d77713649e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05e8cf9711ee43b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbca3d49a0c614e05"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Cover dealer registration in browser acceptance
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rfd9626648cc64d64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rd484d1c0a10f4c27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rea01f118d0ac4593"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R9e05219a75484dfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R3dad5851471c4e9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R537b13b82f414621"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rdc41449dc64c4131"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4a49ede30c604975"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R4af7da076971424d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Re8c87d200a404c69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R05350b5772114266"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R2e8104b5d81348ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Ra493e9500b4f4f1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Raacbd471dce447b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R333281003a734f29"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0bf85f93e3a1448a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8504975124378114</x:v>
+        <x:v>0.8512437810945275</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: CI passed; isolated DB tests 3/3, sweep 99 URLs/0 issues, desktop/mobile Chromium 11 passed. Persistent online staging remains open.</x:v>
+        <x:v>PR #6: CI passed; isolated DB tests 3/3, sweep 99-100 URLs/0 issues, desktop/mobile Chromium 13 passed including dealer registration. Persistent online staging remains open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44369242059c4d35"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d1764eff082458d"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Homepage PR #5 merged into main on 30 Sep 2026. Stage 6.2 PR #6 GitHub Actions run #36631593477 passed: seeded test DB, 3 database checks, 99-route sweep and desktop/mobile Chromium suite. Online staging, required branch check, external monitoring and deeper transaction/browser journeys remain open.</x:v>
+        <x:v>Homepage PR #5 merged into main on 30 Sep 2026. Stage 6.2 PR #6 GitHub Actions run #36631593477 passed. Local isolated DB tests 3/3, sweep 99-100 routes with no issues, and expanded desktop/mobile Chromium suite 13 passed. Online staging, required branch check, external monitoring and remaining transaction/browser journeys remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2932,7 +2932,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G17" s="137" t="n">
-        <x:v>0.55</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="H17" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2953,10 +2953,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Playwright desktop/mobile Chromium: 11 passed, 1 desktop-only skip; homepage search, browse, auth gates, seller/admin sign-in and mobile overflow.</x:v>
+        <x:v>Playwright desktop/mobile Chromium: 13 passed, 1 desktop-only skip; homepage search, browse, auth gates, seller/admin sign-in, dealer registration and mobile overflow.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Cover listing creation/contact, registration, dealer submission, moderation mutations and accessibility.</x:v>
+        <x:v>Cover listing creation/contact, buyer registration, moderation mutations and accessibility.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -10640,7 +10640,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G181" s="137" t="n">
-        <x:v>0.4</x:v>
+        <x:v>0.45</x:v>
       </x:c>
       <x:c r="H181" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10661,10 +10661,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>PR #6 browser foundation passes 11 desktop/mobile Chromium cases; no submission or mutation journey yet.</x:v>
+        <x:v>PR #6 browser foundation passes 13 desktop/mobile Chromium cases including dealer registration; car/bike/part submission and moderation mutations remain open.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Automate registration through contact, listing creation, dealer registration and moderation changes.</x:v>
+        <x:v>Automate buyer registration through contact, listing creation and moderation changes.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -10687,7 +10687,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G182" s="137" t="n">
-        <x:v>0.3</x:v>
+        <x:v>0.35</x:v>
       </x:c>
       <x:c r="H182" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10708,7 +10708,7 @@
         <x:v>Real/simulated devices; slow network</x:v>
       </x:c>
       <x:c r="N182" s="136" t="str">
-        <x:v>Simulated Android Chromium checks pass for homepage search, browse, seller/admin login, auth gates and width.</x:v>
+        <x:v>Simulated Android Chromium checks pass for homepage search, browse, seller/admin login, dealer registration, auth gates and width.</x:v>
       </x:c>
       <x:c r="O182" s="136" t="str">
         <x:v>Test iPhone Safari and mobile upload/keyboard on hosted staging.</x:v>
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e5b4953da08409b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3066350ebd54dcb"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdaa1a575bbb4bf0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51930aa36cab46f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13737,10 +13737,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E35" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Playwright desktop/mobile dealer registration</x:v>
       </x:c>
       <x:c r="F35" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Partial pass: new dealer dashboard and pending badge; duplicate slug case pending</x:v>
       </x:c>
       <x:c r="G35" s="141" t="str">
         <x:v>Authenticated individual</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3df76d77713649e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd862307333b7438c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbca3d49a0c614e05"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3707c2b31c044fc9"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Patch production dependencies and enforce audit in CI
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4a49ede30c604975"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R4af7da076971424d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Re8c87d200a404c69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R05350b5772114266"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R2e8104b5d81348ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Ra493e9500b4f4f1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Raacbd471dce447b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7bc28bed50c340f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rebe3ef796ff3497a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R45e9d74d555d4cc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R8717a4eecd404230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R17b821f99bac4106"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R38e6fbd815934d8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R56755dddb2ee4341"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0bf85f93e3a1448a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcb1e69580efd4cec"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1262,7 +1262,7 @@
       </x:c>
       <x:c r="B6" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>150</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="C6" s="88"/>
       <x:c r="D6" s="97" t="str">
@@ -1316,7 +1316,7 @@
       </x:c>
       <x:c r="B8" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C8" s="88"/>
       <x:c r="D8" s="97" t="str">
@@ -1326,7 +1326,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F8" s="99" t="str">
-        <x:v>build:safe passed 30 Sep; max First Load JS 128 kB</x:v>
+        <x:v>15.5.26 build:safe passed 30 Sep; max First Load JS 128 kB; production audit zero vulnerabilities</x:v>
       </x:c>
       <x:c r="G8" s="97" t="str">
         <x:v>Next functionality</x:v>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8512437810945275</x:v>
+        <x:v>0.8537313432835822</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1466,7 +1466,7 @@
       </x:c>
       <x:c r="B15" s="106" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>150</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="C15" s="107" t="str">
         <x:v>Implemented in current code and functionally available</x:v>
@@ -1504,7 +1504,7 @@
       </x:c>
       <x:c r="B17" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C17" s="110" t="str">
         <x:v>Foundation exists; end-to-end feature incomplete</x:v>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d1764eff082458d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red5844cb8aa04a07"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Homepage PR #5 merged into main on 30 Sep 2026. Stage 6.2 PR #6 GitHub Actions run #36631593477 passed. Local isolated DB tests 3/3, sweep 99-100 routes with no issues, and expanded desktop/mobile Chromium suite 13 passed. Online staging, required branch check, external monitoring and remaining transaction/browser journeys remain open.</x:v>
+        <x:v>Homepage PR #5 merged into main. Stage 6.2 PR #6 runs CI and isolated DB/browser acceptance. Security patch on 30 Sep removed all production dependency audit findings; local checks, lint, build, 100-route sweep and 13 Chromium cases pass. Online staging, branch protection, monitoring and deeper journeys remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2718,7 +2718,7 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>PR #6 GitHub Actions run #36631593477 passed migrations, seeds, DB tests, checks, lint, build, sweep and Chromium.</x:v>
+        <x:v>PR #6 CI passes migrations, seed, DB tests, checks, lint, build, sweep and Chromium. Production dependency audit added as a blocking job step.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
         <x:v>Mark check required in branch protection and demonstrate deliberate failure blocks merge.</x:v>
@@ -2976,10 +2976,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F18" s="136" t="str">
-        <x:v>Partially Implemented</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="G18" s="137" t="n">
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H18" s="136" t="str">
         <x:v>Critical</x:v>
@@ -3000,10 +3000,10 @@
         <x:v>npm audit review; regression build</x:v>
       </x:c>
       <x:c r="N18" s="136" t="str">
-        <x:v>Drizzle advisory was fixed; npm still reports high-severity advisories locally.</x:v>
+        <x:v>30 Sep 2026: Next.js 15.5.26, sharp 0.35.5 and patched PostCSS/js-yaml installed. npm audit --omit=dev reports zero vulnerabilities; checks, lint, build, 100-route sweep and 13 Chromium tests pass.</x:v>
       </x:c>
       <x:c r="O18" s="136" t="str">
-        <x:v>Audit each advisory and upgrade compatibly.</x:v>
+        <x:v>Monitor advisories in CI; four moderate development-only esbuild advisories await a compatible upstream Drizzle kit update.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3066350ebd54dcb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb3bb2062a534d98"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51930aa36cab46f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73e1f286ed694f06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd862307333b7438c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30bcd9bc1172473e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3707c2b31c044fc9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re62d544d1eae431f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Verify marketplace journeys and serve runtime uploads
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7bc28bed50c340f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rebe3ef796ff3497a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R45e9d74d555d4cc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R8717a4eecd404230"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R17b821f99bac4106"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R38e6fbd815934d8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R56755dddb2ee4341"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra68705532e0b4f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R6ea104ba3ef946df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rfcbce11842b34123"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R4a0af6ebb68a41a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R4037b2e6776f43b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rf64e659506744b50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Re27840f9030c4e0f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcb1e69580efd4cec"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1445000a422242de"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8537313432835822</x:v>
+        <x:v>0.856716417910448</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: CI passed; isolated DB tests 3/3, sweep 99-100 URLs/0 issues, desktop/mobile Chromium 13 passed including dealer registration. Persistent online staging remains open.</x:v>
+        <x:v>PR #6: CI and production audit pass; isolated DB tests 3/3, 100-route sweep 0 issues, expanded Chromium suite 23 passed with car/bike/part, buyer contact and admin approval.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red5844cb8aa04a07"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd677d50485c04a98"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Homepage PR #5 merged into main. Stage 6.2 PR #6 runs CI and isolated DB/browser acceptance. Security patch on 30 Sep removed all production dependency audit findings; local checks, lint, build, 100-route sweep and 13 Chromium cases pass. Online staging, branch protection, monitoring and deeper journeys remain open.</x:v>
+        <x:v>Stage 6.2 PR #6 has patched dependencies and production audit gate. Local checks, lint, build, 100-route sweep and 23 Chromium cases pass, including live upload/public image URL and car/bike/part publication, buyer lead and audited moderation. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2932,7 +2932,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G17" s="137" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="H17" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2953,10 +2953,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Playwright desktop/mobile Chromium: 13 passed, 1 desktop-only skip; homepage search, browse, auth gates, seller/admin sign-in, dealer registration and mobile overflow.</x:v>
+        <x:v>Desktop/mobile Chromium: 23 passed, 1 mobile-only skip. Real photo upload and public image URL, car/bike/part publication, buyer phone lead and audited admin approval now pass.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Cover listing creation/contact, buyer registration, moderation mutations and accessibility.</x:v>
+        <x:v>Add account registration, invalid/banned login, edit/delete, dealer verification and full moderation/inspection cases.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -10640,7 +10640,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G181" s="137" t="n">
-        <x:v>0.45</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="H181" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10661,10 +10661,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>PR #6 browser foundation passes 13 desktop/mobile Chromium cases including dealer registration; car/bike/part submission and moderation mutations remain open.</x:v>
+        <x:v>23 browser cases pass in Chromium with isolated PostgreSQL: seller publishes all three verticals, buyer contact logs lead, admin approval writes audit, dealer registration works.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Automate buyer registration through contact, listing creation and moderation changes.</x:v>
+        <x:v>Cover registration, seller edit/delete, negative permissions, inspection and remaining admin mutations.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -10687,7 +10687,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G182" s="137" t="n">
-        <x:v>0.35</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="H182" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10708,10 +10708,10 @@
         <x:v>Real/simulated devices; slow network</x:v>
       </x:c>
       <x:c r="N182" s="136" t="str">
-        <x:v>Simulated Android Chromium checks pass for homepage search, browse, seller/admin login, dealer registration, auth gates and width.</x:v>
+        <x:v>Simulated Android Chromium passes search, sign-in, dealer registration, all three listing publications, photo upload, phone reveal, moderation and viewport width.</x:v>
       </x:c>
       <x:c r="O182" s="136" t="str">
-        <x:v>Test iPhone Safari and mobile upload/keyboard on hosted staging.</x:v>
+        <x:v>Add simulated Safari/iPhone and mobile keyboard/upload checks; real-device review remains parked.</x:v>
       </x:c>
     </x:row>
     <x:row r="183">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb3bb2062a534d98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3761d31dc5de4316"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73e1f286ed694f06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb481e93baf6d4f78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13113,10 +13113,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E11" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Desktop/mobile Chromium publication with photo</x:v>
       </x:c>
       <x:c r="F11" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Passed: active car and detail redirect; optional-field boundaries remain open</x:v>
       </x:c>
       <x:c r="G11" s="141" t="str">
         <x:v>Seeded taxonomy and upload provider</x:v>
@@ -13191,10 +13191,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E14" s="141" t="str">
-        <x:v>Automated checks</x:v>
+        <x:v>Desktop/mobile Chromium publication with photo</x:v>
       </x:c>
       <x:c r="F14" s="141" t="str">
-        <x:v>Passed; final browser QA deferred</x:v>
+        <x:v>Passed: active bike and detail redirect; electric path remains open</x:v>
       </x:c>
       <x:c r="G14" s="141" t="str">
         <x:v>Bike CRUD complete</x:v>
@@ -13217,10 +13217,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E15" s="141" t="str">
-        <x:v>Automated checks</x:v>
+        <x:v>Desktop/mobile Chromium publication with photo</x:v>
       </x:c>
       <x:c r="F15" s="141" t="str">
-        <x:v>Passed; final browser QA deferred</x:v>
+        <x:v>Passed: active part and detail redirect; fitment cases remain open</x:v>
       </x:c>
       <x:c r="G15" s="141" t="str">
         <x:v>Parts CRUD complete</x:v>
@@ -13347,10 +13347,10 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E20" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Desktop/mobile upload plus public WebP URL</x:v>
       </x:c>
       <x:c r="F20" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Passed valid image end to end; size/count boundaries remain open</x:v>
       </x:c>
       <x:c r="G20" s="141" t="str">
         <x:v>Representative image fixtures</x:v>
@@ -13581,10 +13581,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E29" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Desktop/mobile buyer reveal plus database lead count</x:v>
       </x:c>
       <x:c r="F29" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Passed active phone reveal and lead log; inactive rejection remains open</x:v>
       </x:c>
       <x:c r="G29" s="141" t="str">
         <x:v>Active and inactive listings</x:v>
@@ -13945,10 +13945,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E43" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Desktop/mobile admin approval plus DB audit</x:v>
       </x:c>
       <x:c r="F43" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Partial pass: approve and audit; reject/remove and denial remain open</x:v>
       </x:c>
       <x:c r="G43" s="141" t="str">
         <x:v>Reported/flagged listings</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30bcd9bc1172473e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc428f6e17bd54c68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re62d544d1eae431f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26d0fba160ed4b95"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete car registration fields and clarify validation
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra68705532e0b4f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R6ea104ba3ef946df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rfcbce11842b34123"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R4a0af6ebb68a41a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R4037b2e6776f43b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rf64e659506744b50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Re27840f9030c4e0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbf30b5da46654fdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R1facf029a4754343"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Ra645e76a5c044f39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R5dc7621ba50044a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R6609b1646e304ec0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rb459bf9bc629490f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R67d794dbc7b64e70"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1445000a422242de"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R45892f4f24af4d8c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1262,7 +1262,7 @@
       </x:c>
       <x:c r="B6" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>151</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="C6" s="88"/>
       <x:c r="D6" s="97" t="str">
@@ -1316,7 +1316,7 @@
       </x:c>
       <x:c r="B8" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C8" s="88"/>
       <x:c r="D8" s="97" t="str">
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.856716417910448</x:v>
+        <x:v>0.8585572139303483</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1466,7 +1466,7 @@
       </x:c>
       <x:c r="B15" s="106" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>151</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="C15" s="107" t="str">
         <x:v>Implemented in current code and functionally available</x:v>
@@ -1504,7 +1504,7 @@
       </x:c>
       <x:c r="B17" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C17" s="110" t="str">
         <x:v>Foundation exists; end-to-end feature incomplete</x:v>
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: CI and production audit pass; isolated DB tests 3/3, 100-route sweep 0 issues, expanded Chromium suite 23 passed with car/bike/part, buyer contact and admin approval.</x:v>
+        <x:v>PR #6: car registration fields complete; 100-route sweep 0 issues, 23 Chromium tests pass (1 desktop skip), including registered car details persisted in DB. Broader negative-path QA remains.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd677d50485c04a98"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0367524ad9c4977"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6 has patched dependencies and production audit gate. Local checks, lint, build, 100-route sweep and 23 Chromium cases pass, including live upload/public image URL and car/bike/part publication, buyer lead and audited moderation. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: patched production dependencies, audit gate, car registration field completion, local checks/lint/build, 100-route sweep and 23 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -5091,10 +5091,10 @@
         <x:v>Signed V1</x:v>
       </x:c>
       <x:c r="F63" s="136" t="str">
-        <x:v>Partially Implemented</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="G63" s="137" t="n">
-        <x:v>0.65</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H63" s="136" t="str">
         <x:v>Medium</x:v>
@@ -5115,10 +5115,10 @@
         <x:v>Registered/unregistered; auction sheet; token year</x:v>
       </x:c>
       <x:c r="N63" s="136" t="str">
-        <x:v>Schema supports fields, but form does not expose registered city, token year or auction grade.</x:v>
+        <x:v>Car create/edit forms expose registered city, last token paid year and auction grade conditionally. Server rejects conflicting unregistered/auction values. Desktop and mobile browser publication confirmed these fields in isolated PostgreSQL.</x:v>
       </x:c>
       <x:c r="O63" s="136" t="str">
-        <x:v>Complete missing car fields and conditional UI.</x:v>
+        <x:v>Final owner review can be included in launch acceptance; no further implementation dependency.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -10170,7 +10170,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G171" s="137" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.92</x:v>
       </x:c>
       <x:c r="H171" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10191,10 +10191,10 @@
         <x:v>Tampered forms; oversized text; invalid IDs</x:v>
       </x:c>
       <x:c r="N171" s="136" t="str">
-        <x:v>Zod/server validation is broadly implemented; final cross-feature validation audit remains.</x:v>
+        <x:v>Car, bike and parts schema bounds now return field-specific messages; car registration and auction combinations reject contradictory submissions. Seller validation checks pass. Cross-feature tampering review remains.</x:v>
       </x:c>
       <x:c r="O171" s="136" t="str">
-        <x:v>Complete during final QA/hardening after functionality development.</x:v>
+        <x:v>Audit remaining forms and direct server-action inputs; add negative browser coverage for auth, listing edit/delete and admin permissions.</x:v>
       </x:c>
     </x:row>
     <x:row r="172">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3761d31dc5de4316"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62e5fa18049a43e4"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb481e93baf6d4f78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra970b3aac7f04911"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13139,10 +13139,10 @@
         <x:v>Unit + Integration</x:v>
       </x:c>
       <x:c r="E12" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Automated seller schema boundary checks plus desktop/mobile Chromium car publication and DB verification</x:v>
       </x:c>
       <x:c r="F12" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Partial pass: price/year/photo limits and registration/auction conflicts; invalid IDs and direct action tampering still open</x:v>
       </x:c>
       <x:c r="G12" s="141" t="str">
         <x:v>Invalid IDs, price, year, mileage, images</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc428f6e17bd54c68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbad464063ea54364"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26d0fba160ed4b95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfe779901a4644dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Reject foreign-origin listing uploads
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbf30b5da46654fdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R1facf029a4754343"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Ra645e76a5c044f39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R5dc7621ba50044a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R6609b1646e304ec0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rb459bf9bc629490f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R67d794dbc7b64e70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8cabcdd06d384e6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rc7b488d878a84671"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R8144cb79410d47ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R365fbde7828144a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Ra0b0edae36b74cc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R37a0a46ccaf148bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R593a737798e9484a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R45892f4f24af4d8c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8c9a304561434a95"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8585572139303483</x:v>
+        <x:v>0.8588059701492538</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: car registration fields complete; 100-route sweep 0 issues, 23 Chromium tests pass (1 desktop skip), including registered car details persisted in DB. Broader negative-path QA remains.</x:v>
+        <x:v>PR #6: car registration fields and upload Origin guard verified; 100-route sweep 0 issues, 23 Chromium tests pass (1 desktop skip), including registered car DB fields and foreign-origin 403. Broader negative-path QA remains.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0367524ad9c4977"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ae34e46213c47e6"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: patched production dependencies, audit gate, car registration field completion, local checks/lint/build, 100-route sweep and 23 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, local checks/lint/build, 100-route sweep and 23 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -4483,7 +4483,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G50" s="137" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="H50" s="136" t="str">
         <x:v>Critical</x:v>
@@ -4504,10 +4504,10 @@
         <x:v>Cross-origin forms; origin/host mismatch</x:v>
       </x:c>
       <x:c r="N50" s="136" t="str">
-        <x:v>Origin/session protections are implemented; final security assessment remains deferred.</x:v>
+        <x:v>Upload POST now compares Origin with the incoming Host and rejects mismatches. Authenticated desktop/mobile Chromium test confirms foreign-origin 403 while valid uploads still succeed. Next server actions keep their built-in origin/session protections.</x:v>
       </x:c>
       <x:c r="O50" s="136" t="str">
-        <x:v>Complete during final QA/hardening after functionality development.</x:v>
+        <x:v>Review remaining state-changing routes and proxy host configuration in staging; complete final cross-origin assessment.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62e5fa18049a43e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03ceb09b56cc4ac2"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra970b3aac7f04911"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8f7eaba69fa4f49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13347,10 +13347,10 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E20" s="141" t="str">
-        <x:v>Desktop/mobile upload plus public WebP URL</x:v>
+        <x:v>Desktop/mobile Chromium upload, public WebP URL and authenticated foreign-Origin rejection</x:v>
       </x:c>
       <x:c r="F20" s="141" t="str">
-        <x:v>Passed valid image end to end; size/count boundaries remain open</x:v>
+        <x:v>Partial pass: valid image end to end, foreign-origin 403; size/count boundaries remain open</x:v>
       </x:c>
       <x:c r="G20" s="141" t="str">
         <x:v>Representative image fixtures</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbad464063ea54364"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R061eca1c242f4837"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfe779901a4644dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ab8f6548d144dac"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Cover negative account access in browser acceptance
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8cabcdd06d384e6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rc7b488d878a84671"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R8144cb79410d47ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R365fbde7828144a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Ra0b0edae36b74cc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R37a0a46ccaf148bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R593a737798e9484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R006b632b9caa40d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R38070570db084b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rc1b74b155906467f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R982741669f2e456d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rad3217d3916644eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rdc09687bd0684bbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R8886cf653c794e0c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8c9a304561434a95"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R94fbba5100c14722"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8588059701492538</x:v>
+        <x:v>0.8590547263681593</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: car registration fields and upload Origin guard verified; 100-route sweep 0 issues, 23 Chromium tests pass (1 desktop skip), including registered car DB fields and foreign-origin 403. Broader negative-path QA remains.</x:v>
+        <x:v>PR #6: 100-route sweep 0 issues; 27 Chromium tests pass (1 desktop skip). Car registration, upload Origin guard and invalid/banned/unverified login plus duplicate registration are verified with isolated DB checks.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ae34e46213c47e6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reeb6e50cc47d4960"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, local checks/lint/build, 100-route sweep and 23 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, local checks/lint/build, 100-route sweep and 27 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2932,7 +2932,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G17" s="137" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.85</x:v>
       </x:c>
       <x:c r="H17" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2953,10 +2953,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 23 passed, 1 mobile-only skip. Real photo upload and public image URL, car/bike/part publication, buyer phone lead and audited admin approval now pass.</x:v>
+        <x:v>Desktop/mobile Chromium: 27 passed, 1 mobile-only skip. Real upload/public URL, three listing verticals, buyer lead, admin approval, registration fields, foreign-origin rejection, invalid/banned/unverified sign-in and duplicate registration pass with isolated DB checks.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Add account registration, invalid/banned login, edit/delete, dealer verification and full moderation/inspection cases.</x:v>
+        <x:v>Add valid registration, password reset, seller edit/delete, dealer verification, full moderation and inspection cases.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03ceb09b56cc4ac2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a2e597cc9d140ee"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8f7eaba69fa4f49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R427fcc31b8fd4a54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12983,10 +12983,10 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E6" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Desktop/mobile Chromium duplicate email registration plus DB user count</x:v>
       </x:c>
       <x:c r="F6" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Partial pass: duplicate account rejected without new user; malformed registration inputs remain open</x:v>
       </x:c>
       <x:c r="G6" s="141" t="str">
         <x:v>Existing account and malformed inputs</x:v>
@@ -13009,10 +13009,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E7" s="141" t="str">
-        <x:v>Playwright valid seller/admin login on desktop/mobile</x:v>
+        <x:v>Desktop/mobile Chromium valid, invalid, banned and unverified login plus DB session check</x:v>
       </x:c>
       <x:c r="F7" s="141" t="str">
-        <x:v>Partial pass: valid sign-in; invalid/banned cases pending</x:v>
+        <x:v>Passed: valid users sign in; invalid/banned denied; unverified denied until verification; no forbidden sessions</x:v>
       </x:c>
       <x:c r="G7" s="141" t="str">
         <x:v>Users in each state</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R061eca1c242f4837"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24020d77a4ed49a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ab8f6548d144dac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra519875061e34d32"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Verify seller ownership edits and media deletion
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R006b632b9caa40d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R38070570db084b80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rc1b74b155906467f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R982741669f2e456d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rad3217d3916644eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rdc09687bd0684bbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R8886cf653c794e0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd5f915fe86284b0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R043c316a0fb146dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rd2447cde80f6427f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Ra5cbb5c769ac4ef3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R505a088b35e6440e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rc8c8a8c34e454e8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R8ac3babf7c154a2b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R94fbba5100c14722"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5bd4c67bdda5498b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8590547263681593</x:v>
+        <x:v>0.8595522388059702</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: 100-route sweep 0 issues; 27 Chromium tests pass (1 desktop skip). Car registration, upload Origin guard and invalid/banned/unverified login plus duplicate registration are verified with isolated DB checks.</x:v>
+        <x:v>PR #6: 100-route sweep 0 issues; 31 Chromium tests pass (1 desktop skip). Auth negatives, cross-user edit denial, owner edit/delete and photo cleanup have isolated DB evidence.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reeb6e50cc47d4960"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf91f4f8c84c1418b"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, local checks/lint/build, 100-route sweep and 27 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, local checks/lint/build, 100-route sweep and 31 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2932,7 +2932,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G17" s="137" t="n">
-        <x:v>0.85</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H17" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2953,10 +2953,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 27 passed, 1 mobile-only skip. Real upload/public URL, three listing verticals, buyer lead, admin approval, registration fields, foreign-origin rejection, invalid/banned/unverified sign-in and duplicate registration pass with isolated DB checks.</x:v>
+        <x:v>Desktop/mobile Chromium: 31 passed, 1 mobile-only skip. Three listing verticals, buyer lead, admin approval, registration fields, foreign-origin rejection, auth negatives, cross-user edit denial, owner edit/delete and photo cleanup pass with isolated DB checks.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Add valid registration, password reset, seller edit/delete, dealer verification, full moderation and inspection cases.</x:v>
+        <x:v>Add valid registration, password reset, dealer verification, full moderation/inspection and remaining negative paths.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -10123,7 +10123,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G170" s="137" t="n">
-        <x:v>0.85</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H170" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10144,10 +10144,10 @@
         <x:v>IDOR; direct action calls; cross-user access</x:v>
       </x:c>
       <x:c r="N170" s="136" t="str">
-        <x:v>Authorization checks cover owner/admin workflows added through Stage 5; final matrix review remains.</x:v>
+        <x:v>Server ownership checks now have desktop/mobile browser coverage: another seller receives rendered not-found page and no edit controls; owner can edit price and delete own bike, with DB/media/public URL cleanup. Remaining direct-action IDOR matrix is open.</x:v>
       </x:c>
       <x:c r="O170" s="136" t="str">
-        <x:v>Complete during final QA/hardening after functionality development.</x:v>
+        <x:v>Cover direct cross-user action calls and private media references across remaining modules.</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a2e597cc9d140ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cea8b608a36478b"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R427fcc31b8fd4a54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8e12358fac84893"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13087,10 +13087,10 @@
         <x:v>Security integration</x:v>
       </x:c>
       <x:c r="E10" s="141" t="str">
-        <x:v>Automated checks</x:v>
+        <x:v>Automated feature checks plus desktop/mobile Chromium cross-user edit-page denial</x:v>
       </x:c>
       <x:c r="F10" s="141" t="str">
-        <x:v>Passed in feature checks; final matrix deferred</x:v>
+        <x:v>Partial pass: rendered not-found and no edit controls for another seller; direct action/media IDOR cases remain</x:v>
       </x:c>
       <x:c r="G10" s="141" t="str">
         <x:v>Two users with listings/uploads</x:v>
@@ -13243,10 +13243,10 @@
         <x:v>Integration + SEO</x:v>
       </x:c>
       <x:c r="E16" s="141" t="str">
-        <x:v>Automated checks</x:v>
+        <x:v>Automated checks plus desktop/mobile Chromium owner car edit with DB price/status assertion</x:v>
       </x:c>
       <x:c r="F16" s="141" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Passed owner price edit; facet and slug resync remain covered by feature checks</x:v>
       </x:c>
       <x:c r="G16" s="141" t="str">
         <x:v>Edit flow complete</x:v>
@@ -13269,10 +13269,10 @@
         <x:v>Integration + Security</x:v>
       </x:c>
       <x:c r="E17" s="141" t="str">
-        <x:v>Automated checks</x:v>
+        <x:v>Automated checks plus desktop/mobile Chromium bike deletion with DB, public URL and photo assertions</x:v>
       </x:c>
       <x:c r="F17" s="141" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Passed: row soft-deleted, photo links removed, public listing and stored image unavailable</x:v>
       </x:c>
       <x:c r="G17" s="141" t="str">
         <x:v>Delete policy complete</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24020d77a4ed49a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R435242b4af9a453f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra519875061e34d32"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea2c3cb3babd4259"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Verify dealer decisions and public badges
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd5f915fe86284b0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R043c316a0fb146dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rd2447cde80f6427f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Ra5cbb5c769ac4ef3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R505a088b35e6440e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rc8c8a8c34e454e8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R8ac3babf7c154a2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rce855659135d4083"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R0639b6fec92d4c2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R2a7cc1a0ba474756"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R6639d519be9245c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Ra58fb3fc323f4f19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R196c81ac391f4a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R3f8fcc4cbc6d48aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5bd4c67bdda5498b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R12d4bbf68f4448b5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8595522388059702</x:v>
+        <x:v>0.8596517412935324</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: 100-route sweep 0 issues; 31 Chromium tests pass (1 desktop skip). Auth negatives, cross-user edit denial, owner edit/delete and photo cleanup have isolated DB evidence.</x:v>
+        <x:v>PR #6: 100-route sweep 0 issues; 33 Chromium tests pass (1 desktop skip). Auth, ownership, media cleanup and dealer verify/revoke have isolated DB evidence.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf91f4f8c84c1418b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d123499763d4948"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, local checks/lint/build, 100-route sweep and 31 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, local checks/lint/build, 100-route sweep and 33 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2932,7 +2932,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G17" s="137" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.92</x:v>
       </x:c>
       <x:c r="H17" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2953,10 +2953,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 31 passed, 1 mobile-only skip. Three listing verticals, buyer lead, admin approval, registration fields, foreign-origin rejection, auth negatives, cross-user edit denial, owner edit/delete and photo cleanup pass with isolated DB checks.</x:v>
+        <x:v>Desktop/mobile Chromium: 33 passed, 1 mobile-only skip. Three listing verticals, buyer lead, admin approval, registration fields, foreign-origin rejection, auth negatives, cross-user edit denial, owner edit/delete/photo cleanup and dealer verify/revoke with badge/audit pass in isolated DB.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Add valid registration, password reset, dealer verification, full moderation/inspection and remaining negative paths.</x:v>
+        <x:v>Add valid registration, password reset, full moderation/inspection and remaining negative paths.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -8734,10 +8734,10 @@
         <x:v>Approve/revoke; non-admin; homepage/directory/detail badge</x:v>
       </x:c>
       <x:c r="N140" s="136" t="str">
-        <x:v>Dealer settings, logo, manual verification/revocation, badges and inventory management are implemented.</x:v>
+        <x:v>Manual dealer verification is implemented. Desktop/mobile Chromium now confirms admin grant and reasoned revocation, changed public verified badge, and new append-only audit entries in isolated PostgreSQL.</x:v>
       </x:c>
       <x:c r="O140" s="136" t="str">
-        <x:v>Retain in final regression and comprehensive browser QA.</x:v>
+        <x:v>Final live administrator review can be included in launch acceptance; provider/hosting setup is separate.</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1cea8b608a36478b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf70f4a91d9244e41"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8e12358fac84893"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b5cd86f54cf4b75"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13789,10 +13789,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E37" s="141" t="str">
-        <x:v>Automated checks</x:v>
+        <x:v>Automated checks plus desktop/mobile Chromium admin verify/revoke, public badge and DB audit assertions</x:v>
       </x:c>
       <x:c r="F37" s="141" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Passed: grant/revoke changes verified_at and public badge; both decisions append audit events</x:v>
       </x:c>
       <x:c r="G37" s="141" t="str">
         <x:v>Verification admin complete</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R435242b4af9a453f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc010f44568b344fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea2c3cb3babd4259"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffcf7a37e76a40bd"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Verify inspection and sell assistance journeys in browser
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rce855659135d4083"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R0639b6fec92d4c2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R2a7cc1a0ba474756"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R6639d519be9245c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Ra58fb3fc323f4f19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R196c81ac391f4a3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R3f8fcc4cbc6d48aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R9f23fb5ba3fc4629"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R6dd718dd1d0e4c2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R80bf8640d3e44622"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rae9b1345d66c46e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R1a5dde3afee74c3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rbb599ccba0724b42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R479c3ef91e9148e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R12d4bbf68f4448b5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfa3841d592054c9a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8596517412935324</x:v>
+        <x:v>0.8597512437810946</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: 100-route sweep 0 issues; 33 Chromium tests pass (1 desktop skip). Auth, ownership, media cleanup and dealer verify/revoke have isolated DB evidence.</x:v>
+        <x:v>PR #6: 100-route sweep 0 issues; 41 Chromium tests pass (1 desktop skip). Auth, ownership, dealer, inspection and Sell My Car Assistance have isolated DB evidence.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d123499763d4948"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14f537db4e2541ff"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, local checks/lint/build, 100-route sweep and 33 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, local checks/lint/build, 100-route sweep and 41 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2932,7 +2932,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G17" s="137" t="n">
-        <x:v>0.92</x:v>
+        <x:v>0.94</x:v>
       </x:c>
       <x:c r="H17" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2953,10 +2953,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 33 passed, 1 mobile-only skip. Three listing verticals, buyer lead, admin approval, registration fields, foreign-origin rejection, auth negatives, cross-user edit denial, owner edit/delete/photo cleanup and dealer verify/revoke with badge/audit pass in isolated DB.</x:v>
+        <x:v>Desktop/mobile Chromium: 41 passed, 1 desktop skip; 100-route sweep has 0 issues. Three listing verticals, auth/ownership/dealer, buyer lead, moderation approval, inspection and Sell My Car Assistance request/admin/customer histories pass against isolated PostgreSQL.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Add valid registration, password reset, full moderation/inspection and remaining negative paths.</x:v>
+        <x:v>Add valid registration, password reset, full moderation, listing-linked inspection and remaining negative paths.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -8875,10 +8875,10 @@
         <x:v>Auth redirect; validation; phone normalization; listing/no listing</x:v>
       </x:c>
       <x:c r="N143" s="136" t="str">
-        <x:v>Implemented.</x:v>
+        <x:v>Implemented and verified in desktop/mobile Chromium with isolated PostgreSQL: seller inspection request persists with an initial event; admin contact update appends a customer message and private note; customer sees the message but never the private note.</x:v>
       </x:c>
       <x:c r="O143" s="136" t="str">
-        <x:v>Add listing validity and abuse tests.</x:v>
+        <x:v>Listing-linked request, invalid transitions and final live browser acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
@@ -8922,10 +8922,10 @@
         <x:v>Valid/invalid transitions; admin auth</x:v>
       </x:c>
       <x:c r="N144" s="136" t="str">
-        <x:v>Inspection administration, customer-visible status and append-only follow-up history are implemented.</x:v>
+        <x:v>Implemented and verified in desktop/mobile Chromium with isolated PostgreSQL: seller inspection request persists with an initial event; admin contact update appends a customer message and private note; customer sees the message but never the private note.</x:v>
       </x:c>
       <x:c r="O144" s="136" t="str">
-        <x:v>Retain in final regression and comprehensive browser QA.</x:v>
+        <x:v>Listing-linked request, invalid transitions and final live browser acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
@@ -8969,10 +8969,10 @@
         <x:v>Admin/non-admin; filtering; status changes</x:v>
       </x:c>
       <x:c r="N145" s="136" t="str">
-        <x:v>Inspection administration, customer-visible status and append-only follow-up history are implemented.</x:v>
+        <x:v>Implemented and verified in desktop/mobile Chromium with isolated PostgreSQL: seller inspection request persists with an initial event; admin contact update appends a customer message and private note; customer sees the message but never the private note.</x:v>
       </x:c>
       <x:c r="O145" s="136" t="str">
-        <x:v>Retain in final regression and comprehensive browser QA.</x:v>
+        <x:v>Listing-linked request, invalid transitions and final live browser acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
@@ -9016,10 +9016,10 @@
         <x:v>Validation; auth/guest decision; duplicate; privacy</x:v>
       </x:c>
       <x:c r="N146" s="136" t="str">
-        <x:v>Sell My Car Assistance public submission and audited administration workflow are implemented.</x:v>
+        <x:v>Implemented and verified in desktop/mobile Chromium with isolated PostgreSQL: structured seller request and initial event persist; admin contact update appends a customer message and private note; customer sees the message but never the private note.</x:v>
       </x:c>
       <x:c r="O146" s="136" t="str">
-        <x:v>Retain in final regression and comprehensive browser QA.</x:v>
+        <x:v>Negative authorization/validation cases and final live browser acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="147">
@@ -9063,10 +9063,10 @@
         <x:v>Authorization; status changes; filtering</x:v>
       </x:c>
       <x:c r="N147" s="136" t="str">
-        <x:v>Sell My Car Assistance public submission and audited administration workflow are implemented.</x:v>
+        <x:v>Implemented and verified in desktop/mobile Chromium with isolated PostgreSQL: structured seller request and initial event persist; admin contact update appends a customer message and private note; customer sees the message but never the private note.</x:v>
       </x:c>
       <x:c r="O147" s="136" t="str">
-        <x:v>Retain in final regression and comprehensive browser QA.</x:v>
+        <x:v>Negative authorization/validation cases and final live browser acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf70f4a91d9244e41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf33c0b4efecc45be"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b5cd86f54cf4b75"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcd01539f6954366"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13815,10 +13815,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E38" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Desktop/mobile Chromium request without listing, normalized phone, DB reference and initial event</x:v>
       </x:c>
       <x:c r="F38" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Partial pass: no-listing request persists; linked listing and invalid reference still open</x:v>
       </x:c>
       <x:c r="G38" s="141" t="str">
         <x:v>Signed-in user and cities</x:v>
@@ -13841,10 +13841,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E39" s="141" t="str">
-        <x:v>Automated checks</x:v>
+        <x:v>Desktop/mobile Chromium admin status update, append-only event, customer visibility and private-note exclusion</x:v>
       </x:c>
       <x:c r="F39" s="141" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Partial pass: requested to contacted lifecycle and privacy verified; invalid transitions still open</x:v>
       </x:c>
       <x:c r="G39" s="141" t="str">
         <x:v>Inspection admin complete</x:v>
@@ -13867,10 +13867,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E40" s="141" t="str">
-        <x:v>Automated checks</x:v>
+        <x:v>Desktop/mobile Chromium structured request, DB fields, admin update, append-only event and customer privacy</x:v>
       </x:c>
       <x:c r="F40" s="141" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Partial pass: request/manage and customer history verified; negative cases still open</x:v>
       </x:c>
       <x:c r="G40" s="141" t="str">
         <x:v>Public/admin flows complete</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc010f44568b344fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd694e6709e8d4a5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffcf7a37e76a40bd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4048fa94a824715"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Verify moderation and account ban journeys
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R9f23fb5ba3fc4629"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R6dd718dd1d0e4c2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R80bf8640d3e44622"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rae9b1345d66c46e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R1a5dde3afee74c3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rbb599ccba0724b42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R479c3ef91e9148e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R727aa0fbd20d4535"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rdd2fe9d8db6542b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R525d2e528bab4199"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R90fa66bef2fb4996"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R8c1131c577234480"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R44eabc1833524639"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R8496a1d4cc104fc4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfa3841d592054c9a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc8759dd9c7a34143"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8597512437810946</x:v>
+        <x:v>0.8607960199004977</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: 100-route sweep 0 issues; 41 Chromium tests pass (1 desktop skip). Auth, ownership, dealer, inspection and Sell My Car Assistance have isolated DB evidence.</x:v>
+        <x:v>PR #6: 100-route sweep 0 issues; 45 Chromium tests pass (1 desktop skip). Listing, auth, dealer, inspection, assistance, moderation and ban/unban have isolated DB evidence.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14f537db4e2541ff"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra34d31910e0b44b7"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, local checks/lint/build, 100-route sweep and 41 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, local checks/lint/build, 100-route sweep and 45 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2932,7 +2932,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G17" s="137" t="n">
-        <x:v>0.94</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H17" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2953,10 +2953,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 41 passed, 1 desktop skip; 100-route sweep has 0 issues. Three listing verticals, auth/ownership/dealer, buyer lead, moderation approval, inspection and Sell My Car Assistance request/admin/customer histories pass against isolated PostgreSQL.</x:v>
+        <x:v>Desktop/mobile Chromium: 45 passed, 1 desktop skip; 100-route sweep has 0 issues. Listing, auth, ownership, dealer, buyer lead, inspection, assistance, admin hide/reinstate/remove and ban/unban journeys pass against isolated PostgreSQL.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Add valid registration, password reset, full moderation, listing-linked inspection and remaining negative paths.</x:v>
+        <x:v>Add valid registration, password reset, listing reports, listing-linked inspection and remaining negative/direct-action paths.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -4551,10 +4551,10 @@
         <x:v>Login and active-session ban cases</x:v>
       </x:c>
       <x:c r="N51" s="136" t="str">
-        <x:v>Session resolver checks isBanned; admin ban UI is missing.</x:v>
+        <x:v>Banned login is denied; desktop/mobile browser tests confirm admin ban revokes active sessions, unban appends an audit record and restored user can sign in. Admin ban/unban UI is implemented.</x:v>
       </x:c>
       <x:c r="O51" s="136" t="str">
-        <x:v>Build admin ban/unban management.</x:v>
+        <x:v>Retain provider-independent browser regression; final live acceptance remains open.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -9345,10 +9345,10 @@
         <x:v>Reason; repeated; direct URL; SEO</x:v>
       </x:c>
       <x:c r="N153" s="136" t="str">
-        <x:v>Action exists, but inactive detail remains public.</x:v>
+        <x:v>Admin controls implemented. Desktop/mobile browser tests confirm reasoned hide, reinstate and permanent removal with public visibility changes and audit entries; ban revokes sessions, restore permits login and both decisions append audit history.</x:v>
       </x:c>
       <x:c r="O153" s="136" t="str">
-        <x:v>Fix visibility and require/standardize removal reason.</x:v>
+        <x:v>Report resolution, direct-action authorization and final live acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="154">
@@ -9439,10 +9439,10 @@
         <x:v>Transition matrix; search/detail; concurrent actions</x:v>
       </x:c>
       <x:c r="N155" s="136" t="str">
-        <x:v>Admin listing edits/status transitions, audit history and user ban/unban controls are implemented.</x:v>
+        <x:v>Admin controls implemented. Desktop/mobile browser tests confirm reasoned hide, reinstate and permanent removal with public visibility changes and audit entries; ban revokes sessions, restore permits login and both decisions append audit history.</x:v>
       </x:c>
       <x:c r="O155" s="136" t="str">
-        <x:v>Retain in final regression and comprehensive browser QA.</x:v>
+        <x:v>Report resolution, direct-action authorization and final live acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="156">
@@ -9533,10 +9533,10 @@
         <x:v>Ban/unban; active session; listings; audit</x:v>
       </x:c>
       <x:c r="N157" s="136" t="str">
-        <x:v>Admin listing edits/status transitions, audit history and user ban/unban controls are implemented.</x:v>
+        <x:v>Admin controls implemented. Desktop/mobile browser tests confirm reasoned hide, reinstate and permanent removal with public visibility changes and audit entries; ban revokes sessions, restore permits login and both decisions append audit history.</x:v>
       </x:c>
       <x:c r="O157" s="136" t="str">
-        <x:v>Retain in final regression and comprehensive browser QA.</x:v>
+        <x:v>Report resolution, direct-action authorization and final live acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="158">
@@ -9580,10 +9580,10 @@
         <x:v>All action types; tamper/foreign keys</x:v>
       </x:c>
       <x:c r="N158" s="136" t="str">
-        <x:v>Admin listing edits/status transitions, audit history and user ban/unban controls are implemented.</x:v>
+        <x:v>Admin controls implemented. Desktop/mobile browser tests confirm reasoned hide, reinstate and permanent removal with public visibility changes and audit entries; ban revokes sessions, restore permits login and both decisions append audit history.</x:v>
       </x:c>
       <x:c r="O158" s="136" t="str">
-        <x:v>Retain in final regression and comprehensive browser QA.</x:v>
+        <x:v>Report resolution, direct-action authorization and final live acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="159">
@@ -10640,7 +10640,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G181" s="137" t="n">
-        <x:v>0.7</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H181" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10661,10 +10661,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>23 browser cases pass in Chromium with isolated PostgreSQL: seller publishes all three verticals, buyer contact logs lead, admin approval writes audit, dealer registration works.</x:v>
+        <x:v>Desktop/mobile Chromium: 45 passed, 1 desktop skip in isolated PostgreSQL. Seller posts/edits/deletes, buyer contact, dealer registration and verification, inspection, assistance, admin moderation and ban/unban pass; 100-route sweep reports 0 issues.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Cover registration, seller edit/delete, negative permissions, inspection and remaining admin mutations.</x:v>
+        <x:v>Cover valid registration, password reset, reports, linked inspection and remaining negative paths; add Safari/mobile device acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf33c0b4efecc45be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24ea6f83548d4dad"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcd01539f6954366"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a16bad54dad4c9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13945,10 +13945,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E43" s="141" t="str">
-        <x:v>Desktop/mobile admin approval plus DB audit</x:v>
+        <x:v>Desktop/mobile Chromium admin approve, hide, reinstate and permanent removal; DB audit and public visibility</x:v>
       </x:c>
       <x:c r="F43" s="141" t="str">
-        <x:v>Partial pass: approve and audit; reject/remove and denial remain open</x:v>
+        <x:v>Partial pass: moderation status/audit/visibility verified; reports and direct non-admin denial remain open</x:v>
       </x:c>
       <x:c r="G43" s="141" t="str">
         <x:v>Reported/flagged listings</x:v>
@@ -13971,10 +13971,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E44" s="141" t="str">
-        <x:v>Automated checks</x:v>
+        <x:v>Desktop/mobile Chromium ban, session revocation, unban, audit history and restored login</x:v>
       </x:c>
       <x:c r="F44" s="141" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Passed browser lifecycle and DB enforcement; retain direct-action authorization in security regression</x:v>
       </x:c>
       <x:c r="G44" s="141" t="str">
         <x:v>User admin complete</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd694e6709e8d4a5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ffe6f05579d4452"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4048fa94a824715"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03738c859e00448b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Honor five-report safety threshold and confirm submissions
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R727aa0fbd20d4535"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rdd2fe9d8db6542b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R525d2e528bab4199"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R90fa66bef2fb4996"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R8c1131c577234480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R44eabc1833524639"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R8496a1d4cc104fc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re1a6787d8a7545a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R2a594b87dffa4e31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R442d467104584acd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rcb188f6504bb43c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R75ce14ac698747ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R4c25411276184028"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rb35d9c2b2f904ac6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc8759dd9c7a34143"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf595bbbbdeb74282"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1262,7 +1262,7 @@
       </x:c>
       <x:c r="B6" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>152</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C6" s="88"/>
       <x:c r="D6" s="97" t="str">
@@ -1316,7 +1316,7 @@
       </x:c>
       <x:c r="B8" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C8" s="88"/>
       <x:c r="D8" s="97" t="str">
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8607960199004977</x:v>
+        <x:v>0.8626865671641791</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1466,7 +1466,7 @@
       </x:c>
       <x:c r="B15" s="106" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>152</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C15" s="107" t="str">
         <x:v>Implemented in current code and functionally available</x:v>
@@ -1504,7 +1504,7 @@
       </x:c>
       <x:c r="B17" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C17" s="110" t="str">
         <x:v>Foundation exists; end-to-end feature incomplete</x:v>
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: 100-route sweep 0 issues; 45 Chromium tests pass (1 desktop skip). Listing, auth, dealer, inspection, assistance, moderation and ban/unban have isolated DB evidence.</x:v>
+        <x:v>PR #6: 100-route sweep 0 issues; 47 Chromium tests pass (1 desktop skip). Listing, auth, dealer, assistance, moderation, bans and report safety hold have isolated DB evidence.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra34d31910e0b44b7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R743510ebd0bc40c5"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, local checks/lint/build, 100-route sweep and 45 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, five-report safety hold, local checks/lint/build, 100-route sweep and 47 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2932,7 +2932,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G17" s="137" t="n">
-        <x:v>0.95</x:v>
+        <x:v>0.96</x:v>
       </x:c>
       <x:c r="H17" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2953,10 +2953,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 45 passed, 1 desktop skip; 100-route sweep has 0 issues. Listing, auth, ownership, dealer, buyer lead, inspection, assistance, admin hide/reinstate/remove and ban/unban journeys pass against isolated PostgreSQL.</x:v>
+        <x:v>Desktop/mobile Chromium: 47 passed, 1 desktop skip; 100-route sweep has 0 issues. Listing, auth, dealer, assistance, moderation, ban/unban, and five-report safety hold with customer confirmation/admin resolution pass against isolated PostgreSQL.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Add valid registration, password reset, listing reports, listing-linked inspection and remaining negative/direct-action paths.</x:v>
+        <x:v>Add valid registration, password reset, authenticated reporting, report concurrency, listing-linked inspection and remaining negative/direct-action paths.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -9110,10 +9110,10 @@
         <x:v>Anonymous/auth; duplicate; invalid listing; all reasons</x:v>
       </x:c>
       <x:c r="N148" s="136" t="str">
-        <x:v>Implemented with user/anonymous uniqueness.</x:v>
+        <x:v>Anonymous report reason/comment, same-cookie duplicate suppression and database persistence verified in desktop/mobile Chromium. Server now rejects unavailable or nonexistent listing submissions with a user-facing response.</x:v>
       </x:c>
       <x:c r="O148" s="136" t="str">
-        <x:v>Add listing existence/status validation tests.</x:v>
+        <x:v>Add authenticated reporting, invalid reason and direct-request browser cases; final live acceptance remains open.</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
@@ -9157,10 +9157,10 @@
         <x:v>Cookie reuse/reset; concurrent reports; threshold</x:v>
       </x:c>
       <x:c r="N149" s="136" t="str">
-        <x:v>Implemented with threshold 5 and unique constraints.</x:v>
+        <x:v>One report per anonymous cookie/user is enforced by unique indexes; same-cookie duplicate browser test persists only one report. Listing row locking serializes concurrent submissions, and auto-hide waits for five open reports.</x:v>
       </x:c>
       <x:c r="O149" s="136" t="str">
-        <x:v>Review distributed abuse/rate limiting.</x:v>
+        <x:v>Add a concurrent fifth/sixth submission test and review distributed anonymous abuse/rate limiting.</x:v>
       </x:c>
     </x:row>
     <x:row r="150">
@@ -9180,10 +9180,10 @@
         <x:v>Signed V1</x:v>
       </x:c>
       <x:c r="F150" s="136" t="str">
-        <x:v>Partially Implemented</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="G150" s="137" t="n">
-        <x:v>0.65</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H150" s="136" t="str">
         <x:v>High</x:v>
@@ -9204,10 +9204,10 @@
         <x:v>Threshold 4/5/6; concurrent reports; sold reason</x:v>
       </x:c>
       <x:c r="N150" s="136" t="str">
-        <x:v>Current action sets pending_review and logs action remove.</x:v>
+        <x:v>Five open reports trigger one audited pending-review safety hold; first four leave the ad public. Reporter receives a confirmation page, and admin approval restores the ad and dismisses reports. Verified desktop/mobile Chromium with isolated PostgreSQL.</x:v>
       </x:c>
       <x:c r="O150" s="136" t="str">
-        <x:v>Align naming/transitions with Flagged status model.</x:v>
+        <x:v>Concurrent fifth/sixth submission and final live acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="151">
@@ -10640,7 +10640,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G181" s="137" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.92</x:v>
       </x:c>
       <x:c r="H181" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10661,10 +10661,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 45 passed, 1 desktop skip in isolated PostgreSQL. Seller posts/edits/deletes, buyer contact, dealer registration and verification, inspection, assistance, admin moderation and ban/unban pass; 100-route sweep reports 0 issues.</x:v>
+        <x:v>Desktop/mobile Chromium: 47 passed, 1 desktop skip in isolated PostgreSQL. Seller/buyer/dealer, inspection, assistance, moderation, ban/unban and anonymous report threshold/admin resolution pass; 100-route sweep reports 0 issues.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Cover valid registration, password reset, reports, linked inspection and remaining negative paths; add Safari/mobile device acceptance.</x:v>
+        <x:v>Cover valid registration, password reset, authenticated/concurrent reports, linked inspection and remaining negative paths; add Safari/mobile device acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24ea6f83548d4dad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37a370846865456b"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a16bad54dad4c9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26b62b1dc73d4fcf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13893,10 +13893,10 @@
         <x:v>Integration + Security</x:v>
       </x:c>
       <x:c r="E41" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Desktop/mobile Chromium anonymous report and same-cookie duplicate with isolated DB assertion</x:v>
       </x:c>
       <x:c r="F41" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Partial pass: anonymous duplicate suppressed; authenticated and invalid-direct-input paths remain open</x:v>
       </x:c>
       <x:c r="G41" s="141" t="str">
         <x:v>Same listing/user/cookie</x:v>
@@ -13919,10 +13919,10 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E42" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Desktop/mobile Chromium sequential reports 1-5, public visibility, one auto-queue, confirmation and admin resolution</x:v>
       </x:c>
       <x:c r="F42" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Partial pass: four active then fifth safety hold and one audit entry; simultaneous fifth/sixth remains open</x:v>
       </x:c>
       <x:c r="G42" s="141" t="str">
         <x:v>Four then concurrent fifth/sixth</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ffe6f05579d4452"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda2372ef7f214129"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03738c859e00448b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4887509c8de4650"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Verify concurrent report safety hold
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re1a6787d8a7545a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R2a594b87dffa4e31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R442d467104584acd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rcb188f6504bb43c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R75ce14ac698747ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R4c25411276184028"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rb35d9c2b2f904ac6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb637f2488d3941aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rff2b8c5fbfd54c5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R8d3d8ce4107743c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R9c42e8b7eac94b12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rb2c9ca40b6ec4c2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R6fa16ec431954579"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R4f3f67f77fca429c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf595bbbbdeb74282"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R643d062ba32544d9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R743510ebd0bc40c5"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3963e95ecc494502"/>
 </x:worksheet>
 </file>
 
@@ -2956,7 +2956,7 @@
         <x:v>Desktop/mobile Chromium: 47 passed, 1 desktop skip; 100-route sweep has 0 issues. Listing, auth, dealer, assistance, moderation, ban/unban, and five-report safety hold with customer confirmation/admin resolution pass against isolated PostgreSQL.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Add valid registration, password reset, authenticated reporting, report concurrency, listing-linked inspection and remaining negative/direct-action paths.</x:v>
+        <x:v>Add valid registration, password reset, authenticated reporting, listing-linked inspection and remaining negative/direct-action paths.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -9157,10 +9157,10 @@
         <x:v>Cookie reuse/reset; concurrent reports; threshold</x:v>
       </x:c>
       <x:c r="N149" s="136" t="str">
-        <x:v>One report per anonymous cookie/user is enforced by unique indexes; same-cookie duplicate browser test persists only one report. Listing row locking serializes concurrent submissions, and auto-hide waits for five open reports.</x:v>
+        <x:v>One report per anonymous cookie/user is enforced by unique indexes; same-cookie duplicate browser test persists only one report. Desktop/mobile Chromium simultaneously submitted fifth/sixth reports after four open reports: exactly five stayed open, one new queue event was written and the ad was held.</x:v>
       </x:c>
       <x:c r="O149" s="136" t="str">
-        <x:v>Add a concurrent fifth/sixth submission test and review distributed anonymous abuse/rate limiting.</x:v>
+        <x:v>Review distributed anonymous abuse/rate limiting and final live acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="150">
@@ -9207,7 +9207,7 @@
         <x:v>Five open reports trigger one audited pending-review safety hold; first four leave the ad public. Reporter receives a confirmation page, and admin approval restores the ad and dismisses reports. Verified desktop/mobile Chromium with isolated PostgreSQL.</x:v>
       </x:c>
       <x:c r="O150" s="136" t="str">
-        <x:v>Concurrent fifth/sixth submission and final live acceptance remain open.</x:v>
+        <x:v>Final live acceptance remains open.</x:v>
       </x:c>
     </x:row>
     <x:row r="151">
@@ -10664,7 +10664,7 @@
         <x:v>Desktop/mobile Chromium: 47 passed, 1 desktop skip in isolated PostgreSQL. Seller/buyer/dealer, inspection, assistance, moderation, ban/unban and anonymous report threshold/admin resolution pass; 100-route sweep reports 0 issues.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Cover valid registration, password reset, authenticated/concurrent reports, linked inspection and remaining negative paths; add Safari/mobile device acceptance.</x:v>
+        <x:v>Cover valid registration, password reset, authenticated reports, linked inspection and remaining negative paths; add Safari/mobile device acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37a370846865456b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b7adbe077894e97"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26b62b1dc73d4fcf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b0ee30a074a40cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13919,10 +13919,10 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E42" s="141" t="str">
-        <x:v>Desktop/mobile Chromium sequential reports 1-5, public visibility, one auto-queue, confirmation and admin resolution</x:v>
+        <x:v>Desktop/mobile Chromium sequential reports 1-5 and simultaneous fifth/sixth, public visibility, auto-queue, confirmation and admin resolution</x:v>
       </x:c>
       <x:c r="F42" s="141" t="str">
-        <x:v>Partial pass: four active then fifth safety hold and one audit entry; simultaneous fifth/sixth remains open</x:v>
+        <x:v>Passed: four remain public; fifth holds ad; concurrent fifth/sixth yield five open reports and one new queue event</x:v>
       </x:c>
       <x:c r="G42" s="141" t="str">
         <x:v>Four then concurrent fifth/sixth</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda2372ef7f214129"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6c8a480b264460d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4887509c8de4650"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb67cd1f588de431b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Verify email registration and password reset in browser
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb637f2488d3941aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rff2b8c5fbfd54c5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R8d3d8ce4107743c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R9c42e8b7eac94b12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rb2c9ca40b6ec4c2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R6fa16ec431954579"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R4f3f67f77fca429c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra938129411c14fdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rfc4f3b86a14c4c94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R0d2673005f3c4e07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R5bd72b9e265f4b5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rd4a028e2905c4c83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rdb938b60b79a48fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R806f83b882a446d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R643d062ba32544d9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9db48634ea6344e7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8626865671641791</x:v>
+        <x:v>0.8628358208955226</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: 100-route sweep 0 issues; 47 Chromium tests pass (1 desktop skip). Listing, auth, dealer, assistance, moderation, bans and report safety hold have isolated DB evidence.</x:v>
+        <x:v>PR #6: 100-route sweep 0 issues; 51 Chromium tests pass (1 desktop skip). Verified-email registration and password reset now have isolated DB/browser evidence alongside listing, dealer, assistance, moderation, bans and report safety hold.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3963e95ecc494502"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae44d6e75c904769"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, five-report safety hold, local checks/lint/build, 100-route sweep and 47 Chromium cases pass. Online staging, branch protection, monitoring and remaining edge journeys stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, five-report safety hold, verified-email registration and password-reset browser/DB acceptance; 100-route sweep and 51 Chromium cases pass. Online staging, provider configuration, branch protection, monitoring and remaining edge journeys stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2932,7 +2932,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G17" s="137" t="n">
-        <x:v>0.96</x:v>
+        <x:v>0.97</x:v>
       </x:c>
       <x:c r="H17" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2953,10 +2953,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 47 passed, 1 desktop skip; 100-route sweep has 0 issues. Listing, auth, dealer, assistance, moderation, ban/unban, and five-report safety hold with customer confirmation/admin resolution pass against isolated PostgreSQL.</x:v>
+        <x:v>Desktop/mobile Chromium: 51 passed, 1 desktop skip; 100-route sweep has 0 issues. Isolated PostgreSQL confirms verified-email registration, password-reset lifecycle, listings, dealer, assistance, moderation, ban/unban and report safety hold.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Add valid registration, password reset, authenticated reporting, listing-linked inspection and remaining negative/direct-action paths.</x:v>
+        <x:v>Add authenticated reporting, listing-linked inspection and remaining negative/direct-action paths; final live device acceptance remains open.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -4004,7 +4004,7 @@
         <x:v>User registration</x:v>
       </x:c>
       <x:c r="D40" s="136" t="str">
-        <x:v>Name, email, Pakistani mobile number and password registration</x:v>
+        <x:v>Name, email, optional Pakistani mobile number and password registration with verified email before sign-in</x:v>
       </x:c>
       <x:c r="E40" s="136" t="str">
         <x:v>Signed V1</x:v>
@@ -4028,16 +4028,16 @@
         <x:v>Users table</x:v>
       </x:c>
       <x:c r="L40" s="136" t="str">
-        <x:v>Valid unique users register and receive a session; invalid/duplicate data returns safe field errors.</x:v>
+        <x:v>Valid unique user receives verification email, verifies once and can then sign in; invalid/duplicate data returns safe field errors.</x:v>
       </x:c>
       <x:c r="M40" s="136" t="str">
         <x:v>Happy path; duplicates; invalid phone/email/password; DB failure</x:v>
       </x:c>
       <x:c r="N40" s="136" t="str">
-        <x:v>authenticateAction implements registration.</x:v>
+        <x:v>Desktop/mobile Chromium and isolated PostgreSQL confirm registration, email verification, one-use and expiry checks, and no session before verification; duplicate email and malformed name/password are rejected without a new user.</x:v>
       </x:c>
       <x:c r="O40" s="136" t="str">
-        <x:v>Add automated integration coverage.</x:v>
+        <x:v>Production email provider configuration and final live browser acceptance remain open; direct-action invalid email/phone and DB-failure cases remain in security regression.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -4363,10 +4363,10 @@
         <x:v>Known/unknown account; throttling; expiry</x:v>
       </x:c>
       <x:c r="N47" s="136" t="str">
-        <x:v>Account-management implementation includes session handling and secure password-reset flow; automated checks pass.</x:v>
+        <x:v>Desktop/mobile Chromium confirms recovery email link capture in isolated acceptance mode; unknown-account response remains non-enumerating in automated checks.</x:v>
       </x:c>
       <x:c r="O47" s="136" t="str">
-        <x:v>Retain in final regression and comprehensive browser QA.</x:v>
+        <x:v>Configure production email provider and complete live delivery acceptance; throttling remains in security regression.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -4410,10 +4410,10 @@
         <x:v>Token lifecycle; password policy; session revocation</x:v>
       </x:c>
       <x:c r="N48" s="136" t="str">
-        <x:v>Account-management implementation includes session handling and secure password-reset flow; automated checks pass.</x:v>
+        <x:v>Desktop/mobile Chromium and isolated PostgreSQL confirm a single-use reset link, hashed token, expiry denial, existing-session revocation, old-password denial and new-password sign-in.</x:v>
       </x:c>
       <x:c r="O48" s="136" t="str">
-        <x:v>Retain in final regression and comprehensive browser QA.</x:v>
+        <x:v>Production email delivery and final live browser acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -10640,7 +10640,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G181" s="137" t="n">
-        <x:v>0.92</x:v>
+        <x:v>0.94</x:v>
       </x:c>
       <x:c r="H181" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10661,10 +10661,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 47 passed, 1 desktop skip in isolated PostgreSQL. Seller/buyer/dealer, inspection, assistance, moderation, ban/unban and anonymous report threshold/admin resolution pass; 100-route sweep reports 0 issues.</x:v>
+        <x:v>Desktop/mobile Chromium: 51 passed, 1 desktop skip in isolated PostgreSQL. Verified-email registration and reset token expiry/reuse/session revocation join seller/buyer/dealer, inspection, assistance, moderation, ban/unban and report threshold; 100-route sweep reports 0 issues.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Cover valid registration, password reset, authenticated reports, linked inspection and remaining negative paths; add Safari/mobile device acceptance.</x:v>
+        <x:v>Cover authenticated reports, linked inspection and remaining negative/direct-action paths; add Safari/mobile device acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b7adbe077894e97"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5da0c83eee8d420c"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b0ee30a074a40cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc24fce980ace4cfc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12957,16 +12957,16 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E5" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Desktop/mobile Chromium registration, captured verification link and isolated DB/session assertions</x:v>
       </x:c>
       <x:c r="F5" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Passed: unverified user cannot sign in; one-use verification link activates account and permits sign-in; expired link fails</x:v>
       </x:c>
       <x:c r="G5" s="141" t="str">
         <x:v>Clean DB and valid unique data</x:v>
       </x:c>
       <x:c r="H5" s="141" t="str">
-        <x:v>User created, session issued, redirect correct</x:v>
+        <x:v>User created without session; verified email required before sign-in</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -12983,10 +12983,10 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E6" s="141" t="str">
-        <x:v>Desktop/mobile Chromium duplicate email registration plus DB user count</x:v>
+        <x:v>Desktop/mobile Chromium duplicate email, malformed name/password and DB user-count assertions</x:v>
       </x:c>
       <x:c r="F6" s="141" t="str">
-        <x:v>Partial pass: duplicate account rejected without new user; malformed registration inputs remain open</x:v>
+        <x:v>Partial pass: duplicate, short name and short password rejected without new users; malformed email/phone and direct-action cases remain</x:v>
       </x:c>
       <x:c r="G6" s="141" t="str">
         <x:v>Existing account and malformed inputs</x:v>
@@ -13061,10 +13061,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E9" s="141" t="str">
-        <x:v>Automated checks</x:v>
+        <x:v>Desktop/mobile Chromium reset link, isolated DB token/session assertions and invalid-token lifecycle</x:v>
       </x:c>
       <x:c r="F9" s="141" t="str">
-        <x:v>Passed; final browser QA deferred</x:v>
+        <x:v>Passed: hashed single-use token, expiry denial, session revocation, old-password denial and new-password sign-in</x:v>
       </x:c>
       <x:c r="G9" s="141" t="str">
         <x:v>Reset feature complete</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6c8a480b264460d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22f2e531f2e744c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb67cd1f588de431b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b2a4989fd8d4933"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Preserve car inspection links and verify signed-in reports
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra938129411c14fdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rfc4f3b86a14c4c94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R0d2673005f3c4e07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R5bd72b9e265f4b5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rd4a028e2905c4c83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rdb938b60b79a48fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R806f83b882a446d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf22c81e4d5494bbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Ra9a35ea0ced34c04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R5d2961894c4e4523"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R441925b9aadf4323"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rf74dce30b3404a8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R1576f650fed64296"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R4a43b7d2470b4474"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9db48634ea6344e7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcf6037e1db7e4e1e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8628358208955226</x:v>
+        <x:v>0.8629353233830847</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: 100-route sweep 0 issues; 51 Chromium tests pass (1 desktop skip). Verified-email registration and password reset now have isolated DB/browser evidence alongside listing, dealer, assistance, moderation, bans and report safety hold.</x:v>
+        <x:v>PR #6: clean isolated DB, 99-route sweep 0 issues, 55 Chromium tests pass (1 desktop skip). Verified registration/reset, listing-linked inspection, authenticated reports and core marketplace journeys have DB/browser evidence.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae44d6e75c904769"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba5f60be9c6047ee"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: patched dependencies, audit gate, car registration fields, upload Origin guard, five-report safety hold, verified-email registration and password-reset browser/DB acceptance; 100-route sweep and 51 Chromium cases pass. Online staging, provider configuration, branch protection, monitoring and remaining edge journeys stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: clean repeatable acceptance DB, 55 Chromium cases and 99-route sweep pass; verified registration/reset, linked inspection, authenticated reporting, report safety hold and core marketplace journeys have browser/DB evidence. Online staging, providers, branch protection, monitoring and remaining negative/live acceptance stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2932,7 +2932,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G17" s="137" t="n">
-        <x:v>0.97</x:v>
+        <x:v>0.98</x:v>
       </x:c>
       <x:c r="H17" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2953,10 +2953,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 51 passed, 1 desktop skip; 100-route sweep has 0 issues. Isolated PostgreSQL confirms verified-email registration, password-reset lifecycle, listings, dealer, assistance, moderation, ban/unban and report safety hold.</x:v>
+        <x:v>Desktop/mobile Chromium: 55 passed, 1 desktop skip against a freshly rebuilt isolated PostgreSQL database; 99-route sweep has 0 issues. Verified-email registration, password reset, listing-linked inspection, authenticated reporting and core marketplace journeys pass.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Add authenticated reporting, listing-linked inspection and remaining negative/direct-action paths; final live device acceptance remains open.</x:v>
+        <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -8875,10 +8875,10 @@
         <x:v>Auth redirect; validation; phone normalization; listing/no listing</x:v>
       </x:c>
       <x:c r="N143" s="136" t="str">
-        <x:v>Implemented and verified in desktop/mobile Chromium with isolated PostgreSQL: seller inspection request persists with an initial event; admin contact update appends a customer message and private note; customer sees the message but never the private note.</x:v>
+        <x:v>Desktop/mobile Chromium and isolated PostgreSQL confirm standalone and car-linked requests, preserved listing reference across sign-in, forged/unavailable reference rejection, initial append-only event and customer-visible admin updates without private notes.</x:v>
       </x:c>
       <x:c r="O143" s="136" t="str">
-        <x:v>Listing-linked request, invalid transitions and final live browser acceptance remain open.</x:v>
+        <x:v>Invalid lifecycle transitions and final live browser acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
@@ -8922,10 +8922,10 @@
         <x:v>Valid/invalid transitions; admin auth</x:v>
       </x:c>
       <x:c r="N144" s="136" t="str">
-        <x:v>Implemented and verified in desktop/mobile Chromium with isolated PostgreSQL: seller inspection request persists with an initial event; admin contact update appends a customer message and private note; customer sees the message but never the private note.</x:v>
+        <x:v>Desktop/mobile Chromium and isolated PostgreSQL confirm standalone and car-linked requests, preserved listing reference across sign-in, forged/unavailable reference rejection, initial append-only event and customer-visible admin updates without private notes.</x:v>
       </x:c>
       <x:c r="O144" s="136" t="str">
-        <x:v>Listing-linked request, invalid transitions and final live browser acceptance remain open.</x:v>
+        <x:v>Invalid lifecycle transitions and final live browser acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
@@ -8969,10 +8969,10 @@
         <x:v>Admin/non-admin; filtering; status changes</x:v>
       </x:c>
       <x:c r="N145" s="136" t="str">
-        <x:v>Implemented and verified in desktop/mobile Chromium with isolated PostgreSQL: seller inspection request persists with an initial event; admin contact update appends a customer message and private note; customer sees the message but never the private note.</x:v>
+        <x:v>Desktop/mobile Chromium and isolated PostgreSQL confirm standalone and car-linked requests, preserved listing reference across sign-in, forged/unavailable reference rejection, initial append-only event and customer-visible admin updates without private notes.</x:v>
       </x:c>
       <x:c r="O145" s="136" t="str">
-        <x:v>Listing-linked request, invalid transitions and final live browser acceptance remain open.</x:v>
+        <x:v>Invalid lifecycle transitions and final live browser acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
@@ -9110,10 +9110,10 @@
         <x:v>Anonymous/auth; duplicate; invalid listing; all reasons</x:v>
       </x:c>
       <x:c r="N148" s="136" t="str">
-        <x:v>Anonymous report reason/comment, same-cookie duplicate suppression and database persistence verified in desktop/mobile Chromium. Server now rejects unavailable or nonexistent listing submissions with a user-facing response.</x:v>
+        <x:v>Anonymous and signed-in reporting verified in desktop/mobile Chromium. Account-bound duplicate submissions remain one report across sessions; anonymous cookie duplicate also remains one. Invalid or unavailable listing submissions are rejected.</x:v>
       </x:c>
       <x:c r="O148" s="136" t="str">
-        <x:v>Add authenticated reporting, invalid reason and direct-request browser cases; final live acceptance remains open.</x:v>
+        <x:v>Add invalid reason/direct-request browser cases and final live acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
@@ -10640,7 +10640,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G181" s="137" t="n">
-        <x:v>0.94</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H181" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10661,10 +10661,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 51 passed, 1 desktop skip in isolated PostgreSQL. Verified-email registration and reset token expiry/reuse/session revocation join seller/buyer/dealer, inspection, assistance, moderation, ban/unban and report threshold; 100-route sweep reports 0 issues.</x:v>
+        <x:v>Desktop/mobile Chromium: 55 passed, 1 desktop skip. Linked car inspection survives sign-in, rejects forged references and writes a listing-linked event; signed-in report remains account-bound across sessions. Clean DB reseeding and 99-route sweep pass.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Cover authenticated reports, linked inspection and remaining negative/direct-action paths; add Safari/mobile device acceptance.</x:v>
+        <x:v>Cover remaining direct-action and validation negatives; add Safari/mobile device and live staging acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5da0c83eee8d420c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racc97dc957234a12"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc24fce980ace4cfc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc537dd728ff4f11"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13815,10 +13815,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E38" s="141" t="str">
-        <x:v>Desktop/mobile Chromium request without listing, normalized phone, DB reference and initial event</x:v>
+        <x:v>Desktop/mobile Chromium standalone and car-linked requests, sign-in continuity, forged-reference rejection, DB link and initial event</x:v>
       </x:c>
       <x:c r="F38" s="141" t="str">
-        <x:v>Partial pass: no-listing request persists; linked listing and invalid reference still open</x:v>
+        <x:v>Passed: valid listing link persists with request/event; forged and unavailable IDs fail without a request</x:v>
       </x:c>
       <x:c r="G38" s="141" t="str">
         <x:v>Signed-in user and cities</x:v>
@@ -13893,10 +13893,10 @@
         <x:v>Integration + Security</x:v>
       </x:c>
       <x:c r="E41" s="141" t="str">
-        <x:v>Desktop/mobile Chromium anonymous report and same-cookie duplicate with isolated DB assertion</x:v>
+        <x:v>Desktop/mobile Chromium anonymous and authenticated reports, cookie/account duplicate checks and isolated DB assertions</x:v>
       </x:c>
       <x:c r="F41" s="141" t="str">
-        <x:v>Partial pass: anonymous duplicate suppressed; authenticated and invalid-direct-input paths remain open</x:v>
+        <x:v>Partial pass: anonymous and account duplicates suppressed; invalid-reason/direct-request cases remain</x:v>
       </x:c>
       <x:c r="G41" s="141" t="str">
         <x:v>Same listing/user/cookie</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22f2e531f2e744c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55702cdf94c04279"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b2a4989fd8d4933"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4480eba60466437d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Align inspection wording with request-only scope
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf22c81e4d5494bbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Ra9a35ea0ced34c04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R5d2961894c4e4523"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R441925b9aadf4323"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rf74dce30b3404a8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R1576f650fed64296"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R4a43b7d2470b4474"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd146a34014c54fe3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Ree8b4f4971ac4293"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R5916c96ffea04d59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R4cf96acd33254a03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R0f36545227b64129"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rc9c0c49273e34e88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rffb019dd92cf4b31"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcf6037e1db7e4e1e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7907218bfb774602"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba5f60be9c6047ee"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fa66f19df034084"/>
 </x:worksheet>
 </file>
 
@@ -8875,7 +8875,7 @@
         <x:v>Auth redirect; validation; phone normalization; listing/no listing</x:v>
       </x:c>
       <x:c r="N143" s="136" t="str">
-        <x:v>Desktop/mobile Chromium and isolated PostgreSQL confirm standalone and car-linked requests, preserved listing reference across sign-in, forged/unavailable reference rejection, initial append-only event and customer-visible admin updates without private notes.</x:v>
+        <x:v>Desktop/mobile Chromium and isolated PostgreSQL confirm standalone and car-linked requests, preserved reference across sign-in, forged/unavailable reference rejection and initial event. Customer copy now describes an availability/follow-up request without promising an inspector, checklist or response time.</x:v>
       </x:c>
       <x:c r="O143" s="136" t="str">
         <x:v>Invalid lifecycle transitions and final live browser acceptance remain open.</x:v>
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racc97dc957234a12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6cbe3ac44b14f85"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc537dd728ff4f11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6de240c9ece64227"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55702cdf94c04279"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda61b5aa4d9b42f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4480eba60466437d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R542858d70bb2460b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Reject unsupported image providers and clarify configuration
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd146a34014c54fe3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Ree8b4f4971ac4293"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R5916c96ffea04d59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R4cf96acd33254a03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R0f36545227b64129"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rc9c0c49273e34e88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rffb019dd92cf4b31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6e471514a6a847fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rf97d412033e04558"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rc688b1f3cd644874"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rbc5618c7959a4b74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R979eedbcf4e846b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rd57910fcd2264da7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Ra05405ef1f0d4ed6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7907218bfb774602"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R154d1d5bd4f44e5d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1343,7 +1343,7 @@
       </x:c>
       <x:c r="B9" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Requires Correction")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C9" s="88"/>
       <x:c r="D9" s="97" t="str">
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8629353233830847</x:v>
+        <x:v>0.8671641791044776</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1523,7 +1523,7 @@
       </x:c>
       <x:c r="B18" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Requires Correction")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C18" s="110" t="str">
         <x:v>Implemented behavior is wrong or unsafe</x:v>
@@ -1561,7 +1561,7 @@
       </x:c>
       <x:c r="B20" s="111" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Out of Scope / Removed")</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C20" s="112" t="str">
         <x:v>Deliberately removed; do not build without signed change</x:v>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fa66f19df034084"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73de20822b644310"/>
 </x:worksheet>
 </file>
 
@@ -6243,7 +6243,7 @@
         <x:v>Upload/display/delete; credential failure; variants</x:v>
       </x:c>
       <x:c r="N87" s="136" t="str">
-        <x:v>Upload and display branches exist but have not been production-validated.</x:v>
+        <x:v>Cloudflare upload/display/delete branches exist; public delivery provider and delivery hash are now explicit in the environment template. Local checks pass; staging provider credentials and live media acceptance remain open.</x:v>
       </x:c>
       <x:c r="O87" s="136" t="str">
         <x:v>Configure staging and complete end-to-end media tests.</x:v>
@@ -6266,10 +6266,10 @@
         <x:v>Signed V1</x:v>
       </x:c>
       <x:c r="F88" s="136" t="str">
-        <x:v>Requires Correction</x:v>
+        <x:v>Out of Scope / Removed</x:v>
       </x:c>
       <x:c r="G88" s="137" t="n">
-        <x:v>0.15</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H88" s="136" t="str">
         <x:v>High</x:v>
@@ -6290,10 +6290,10 @@
         <x:v>Upload/display/delete; URL generation</x:v>
       </x:c>
       <x:c r="N88" s="136" t="str">
-        <x:v>S3 variables exist in .env.example, but storage.ts falls back to local for any non-cloudflare value.</x:v>
+        <x:v>Unsupported S3/R2 environment options were removed. Storage and delivery now reject unknown provider values instead of silently using local disk/URLs; the upload security check covers this failure mode.</x:v>
       </x:c>
       <x:c r="O88" s="136" t="str">
-        <x:v>Remove unsupported S3 config or implement it deliberately.</x:v>
+        <x:v>Cloudflare Images remains the documented durable production option; staging configuration and end-to-end provider acceptance are tracked in JW-083.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6cbe3ac44b14f85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9329a9151c894f11"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6de240c9ece64227"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd674343454ad4e5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda61b5aa4d9b42f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra83716b3980649c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R542858d70bb2460b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafcb6a707e6441cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Make abandoned upload cleanup retry safe
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6e471514a6a847fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rf97d412033e04558"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rc688b1f3cd644874"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rbc5618c7959a4b74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R979eedbcf4e846b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rd57910fcd2264da7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Ra05405ef1f0d4ed6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbfea781bbbec47fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rd6193a95a26d4726"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Reae190362abd4c92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R38742a19c55a486d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Raf0a88a479114583"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Red14af490cdc446e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R86cc3fbae82c4b14"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R154d1d5bd4f44e5d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcfb5318d65fd4636"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1316,7 +1316,7 @@
       </x:c>
       <x:c r="B8" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C8" s="88"/>
       <x:c r="D8" s="97" t="str">
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="B10" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C10" s="88"/>
       <x:c r="D10" s="97" t="str">
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8671641791044776</x:v>
+        <x:v>0.8716417910447762</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1504,7 +1504,7 @@
       </x:c>
       <x:c r="B17" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C17" s="110" t="str">
         <x:v>Foundation exists; end-to-end feature incomplete</x:v>
@@ -1542,7 +1542,7 @@
       </x:c>
       <x:c r="B19" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C19" s="110" t="str">
         <x:v>Not implemented</x:v>
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: clean isolated DB, 99-route sweep 0 issues, 55 Chromium tests pass (1 desktop skip). Verified registration/reset, listing-linked inspection, authenticated reports and core marketplace journeys have DB/browser evidence.</x:v>
+        <x:v>PR #6: clean isolated DB, 99-route sweep 0 issues, 57 Chromium tests pass (1 planned skip). Orphan cleanup, verified registration/reset, linked inspection, authenticated reports and core marketplace journeys have DB/browser evidence.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73de20822b644310"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc839689de1f4617"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: clean repeatable acceptance DB, 55 Chromium cases and 99-route sweep pass; verified registration/reset, linked inspection, authenticated reporting, report safety hold and core marketplace journeys have browser/DB evidence. Online staging, providers, branch protection, monitoring and remaining negative/live acceptance stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: clean repeatable acceptance DB, 57 Chromium cases and 99-route sweep pass; orphan cleanup, verified registration/reset, linked inspection, authenticated reporting, report safety hold and core marketplace journeys have browser/DB evidence. Online staging, providers, cron schedule, branch protection, monitoring and remaining negative/live acceptance stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2953,7 +2953,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 55 passed, 1 desktop skip against a freshly rebuilt isolated PostgreSQL database; 99-route sweep has 0 issues. Verified-email registration, password reset, listing-linked inspection, authenticated reporting and core marketplace journeys pass.</x:v>
+        <x:v>Desktop/mobile Chromium: 57 passed, 1 planned skip against a freshly rebuilt isolated PostgreSQL database; 99-route sweep has 0 issues. Orphan cleanup, verified registration/reset, linked inspection, authenticated reporting and core marketplace journeys pass.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
@@ -6125,10 +6125,10 @@
         <x:v>Signed V1</x:v>
       </x:c>
       <x:c r="F85" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G85" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H85" s="136" t="str">
         <x:v>Medium</x:v>
@@ -6149,10 +6149,10 @@
         <x:v>Age boundary; attached/unattached; failed delete</x:v>
       </x:c>
       <x:c r="N85" s="136" t="str">
-        <x:v>No cleanup mechanism exists.</x:v>
+        <x:v>Protected 24-hour orphan purge now locks unclaimed upload rows, deletes each stored object before its database row, retries failed storage deletions, and preserves claimed listing media. Desktop/mobile Chromium and isolated PostgreSQL acceptance pass.</x:v>
       </x:c>
       <x:c r="O85" s="136" t="str">
-        <x:v>Add scheduled cleanup after ownership binding.</x:v>
+        <x:v>Configure and monitor the production cron schedule under JW-197; verify live storage-provider cleanup in staging.</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -10661,7 +10661,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 55 passed, 1 desktop skip. Linked car inspection survives sign-in, rejects forged references and writes a listing-linked event; signed-in report remains account-bound across sessions. Clean DB reseeding and 99-route sweep pass.</x:v>
+        <x:v>Desktop/mobile Chromium: 57 passed, 1 planned skip. Orphan cleanup preserves claimed media and retries failed object removal; clean DB reseeding and 99-route sweep pass alongside core marketplace journeys.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Cover remaining direct-action and validation negatives; add Safari/mobile device and live staging acceptance.</x:v>
@@ -11601,7 +11601,7 @@
         <x:v>Authorized/unauthorized; missed run; retry</x:v>
       </x:c>
       <x:c r="N201" s="136" t="str">
-        <x:v>Protected endpoints exist; scheduler not configured.</x:v>
+        <x:v>Protected purge-expired endpoint now has browser/DB acceptance for orphan media cleanup. Production schedule, credentials, monitoring and alerting remain unconfigured.</x:v>
       </x:c>
       <x:c r="O201" s="136" t="str">
         <x:v>Configure in staging and monitor.</x:v>
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9329a9151c894f11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fbcdc42b4324c74"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd674343454ad4e5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91c9c173b16b413b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra83716b3980649c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64cfdb3acfef49bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafcb6a707e6441cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd0bd6dccb5349d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add recoverable browse loading and error states
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbfea781bbbec47fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rd6193a95a26d4726"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Reae190362abd4c92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R38742a19c55a486d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Raf0a88a479114583"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Red14af490cdc446e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R86cc3fbae82c4b14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4fc1a3525a9d4fd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R3b6fc0d7801841b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Re25aadfbb93941b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rc949f6411c364360"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rcf692c7fca4f4ba0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Ra02bf99ed5394be0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R7e5f2d8d1a694983"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcfb5318d65fd4636"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb7dd0379ec2c46ca"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8716417910447762</x:v>
+        <x:v>0.8733830845771147</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc839689de1f4617"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0655d479fc464231"/>
 </x:worksheet>
 </file>
 
@@ -7350,7 +7350,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G111" s="137" t="n">
-        <x:v>0.55</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H111" s="136" t="str">
         <x:v>High</x:v>
@@ -7371,10 +7371,10 @@
         <x:v>Empty DB; query failure; slow response</x:v>
       </x:c>
       <x:c r="N111" s="136" t="str">
-        <x:v>Empty state exists; explicit loading/error boundaries are absent.</x:v>
+        <x:v>Cars, bikes and parts browsing now have accessible loading skeletons scoped after URL validation, plus route-level recoverable error screens with retry and clear-filters actions. Actionable no-results state was already present; invalid URL 404 and canonical redirects remain protected.</x:v>
       </x:c>
       <x:c r="O111" s="136" t="str">
-        <x:v>Add route-level loading and error UI.</x:v>
+        <x:v>Exercise the error boundary with a controlled backend failure in isolated browser acceptance, then verify slow-network loading and retry on live devices.</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fbcdc42b4324c74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra79a15a8bde74ed9"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91c9c173b16b413b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf450fc8fdeef45b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64cfdb3acfef49bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e8a6f02baaf4c3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd0bd6dccb5349d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdad86e1451934e0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add shared authentication rate limits
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4fc1a3525a9d4fd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R3b6fc0d7801841b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Re25aadfbb93941b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rc949f6411c364360"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rcf692c7fca4f4ba0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Ra02bf99ed5394be0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R7e5f2d8d1a694983"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1315d9be6d044831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R26676e0c28a840e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R19241c014810497e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rb7a2873b209c44d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Raa718afc97d34651"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R261f0ba900ff4a48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rb4cc585271a14317"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb7dd0379ec2c46ca"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R343b59e2516c4d69"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1316,7 +1316,7 @@
       </x:c>
       <x:c r="B8" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C8" s="88"/>
       <x:c r="D8" s="97" t="str">
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="B10" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C10" s="88"/>
       <x:c r="D10" s="97" t="str">
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8733830845771147</x:v>
+        <x:v>0.8762686567164182</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1504,7 +1504,7 @@
       </x:c>
       <x:c r="B17" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C17" s="110" t="str">
         <x:v>Foundation exists; end-to-end feature incomplete</x:v>
@@ -1542,7 +1542,7 @@
       </x:c>
       <x:c r="B19" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C19" s="110" t="str">
         <x:v>Not implemented</x:v>
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: clean isolated DB, 99-route sweep 0 issues, 57 Chromium tests pass (1 planned skip). Orphan cleanup, verified registration/reset, linked inspection, authenticated reports and core marketplace journeys have DB/browser evidence.</x:v>
+        <x:v>PR #6: clean isolated DB, 99-route sweep 0 issues, 59 Chromium tests pass (1 planned skip). Atomic auth retry limiting, orphan cleanup, verified registration/reset, linked inspection and core marketplace journeys have DB/browser evidence.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0655d479fc464231"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c53e78382d84a3d"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: clean repeatable acceptance DB, 57 Chromium cases and 99-route sweep pass; orphan cleanup, verified registration/reset, linked inspection, authenticated reporting, report safety hold and core marketplace journeys have browser/DB evidence. Online staging, providers, cron schedule, branch protection, monitoring and remaining negative/live acceptance stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: clean repeatable acceptance DB, 59 Chromium cases and 99-route sweep pass; auth retry limits, orphan cleanup, verified registration/reset, linked inspection, report safety hold and core marketplace journeys have browser/DB evidence. Online staging, providers, public-write limits, cron schedule, branch protection, monitoring and remaining live acceptance stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2953,7 +2953,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 57 passed, 1 planned skip against a freshly rebuilt isolated PostgreSQL database; 99-route sweep has 0 issues. Orphan cleanup, verified registration/reset, linked inspection, authenticated reporting and core marketplace journeys pass.</x:v>
+        <x:v>Desktop/mobile Chromium: 59 passed, 1 planned skip against a fresh isolated PostgreSQL database; 99-route sweep has 0 issues. Auth retry limits, orphan cleanup, verified registration/reset, linked inspection, authenticated reporting and core journeys pass.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
@@ -4436,7 +4436,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G49" s="137" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.93</x:v>
       </x:c>
       <x:c r="H49" s="136" t="str">
         <x:v>Critical</x:v>
@@ -4457,10 +4457,10 @@
         <x:v>Burst; distributed attempts; reset window; proxy headers</x:v>
       </x:c>
       <x:c r="N49" s="136" t="str">
-        <x:v>Abuse controls exist on key flows, but a dedicated authentication rate-limit acceptance suite remains for final hardening.</x:v>
+        <x:v>PostgreSQL-backed atomic limits now cover sign-in, registration, password reset request/confirmation, verification resend/confirmation; successful sign-in clears the account attempt bucket. Concurrent DB test and desktop/mobile sign-in throttling browser acceptance pass. Reset/resend keep non-enumerating responses.</x:v>
       </x:c>
       <x:c r="O49" s="136" t="str">
-        <x:v>Complete during final QA/hardening after functionality development.</x:v>
+        <x:v>Cover Google OAuth start and verify trusted proxy IP headers, thresholds and alerting in staging.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -10214,10 +10214,10 @@
         <x:v>Signed V1</x:v>
       </x:c>
       <x:c r="F172" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G172" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="H172" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10238,10 +10238,10 @@
         <x:v>Per-IP/user; proxy spoof; reset; fail-open/closed</x:v>
       </x:c>
       <x:c r="N172" s="136" t="str">
-        <x:v>No general rate limiting exists.</x:v>
+        <x:v>Shared database rate-limit buckets and expiry cleanup now protect primary authentication actions across app instances. Atomic concurrency and user-facing login limit pass isolated DB/browser acceptance.</x:v>
       </x:c>
       <x:c r="O172" s="136" t="str">
-        <x:v>Implement before public launch.</x:v>
+        <x:v>Extend rate limits to public reports, uploads, lead events and other state-changing endpoints; validate proxy headers and production thresholds.</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -10661,7 +10661,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 57 passed, 1 planned skip. Orphan cleanup preserves claimed media and retries failed object removal; clean DB reseeding and 99-route sweep pass alongside core marketplace journeys.</x:v>
+        <x:v>Desktop/mobile Chromium: 59 passed, 1 planned skip. Atomic auth rate limiting and retry UI join orphan cleanup, verified registration/reset, linked inspection, moderation and core marketplace journeys; clean DB reseeding and 99-route sweep pass.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Cover remaining direct-action and validation negatives; add Safari/mobile device and live staging acceptance.</x:v>
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra79a15a8bde74ed9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6853d5548c414663"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf450fc8fdeef45b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0796548e5fcb4dd6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13009,10 +13009,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E7" s="141" t="str">
-        <x:v>Desktop/mobile Chromium valid, invalid, banned and unverified login plus DB session check</x:v>
+        <x:v>Desktop/mobile Chromium valid/invalid/banned/unverified login, DB sessions and repeated-failure retry limit; atomic DB concurrency check</x:v>
       </x:c>
       <x:c r="F7" s="141" t="str">
-        <x:v>Passed: valid users sign in; invalid/banned denied; unverified denied until verification; no forbidden sessions</x:v>
+        <x:v>Passed: only valid active users get sessions; repeated failures show a 15-minute retry limit in both viewports</x:v>
       </x:c>
       <x:c r="G7" s="141" t="str">
         <x:v>Users in each state</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e8a6f02baaf4c3c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R551d216ef45c4eab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdad86e1451934e0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re88f8b5903394879"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Limit public upload report and contact actions
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1315d9be6d044831"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R26676e0c28a840e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R19241c014810497e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rb7a2873b209c44d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Raa718afc97d34651"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R261f0ba900ff4a48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rb4cc585271a14317"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R15e217270e764baa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R97d96e6e51ff4fe5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R9e547433dd604d47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R0223c31a1726419f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R97e981751e054b69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Ra66d6224e4734b19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rdb2e2ae5de044ecc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R343b59e2516c4d69"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8bc8ee4c6ef3403d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8762686567164182</x:v>
+        <x:v>0.8787064676616916</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: clean isolated DB, 99-route sweep 0 issues, 59 Chromium tests pass (1 planned skip). Atomic auth retry limiting, orphan cleanup, verified registration/reset, linked inspection and core marketplace journeys have DB/browser evidence.</x:v>
+        <x:v>PR #6: clean isolated DB, 99-route sweep 0 issues, 63 Chromium tests pass (1 planned skip). Atomic auth, upload, contact and report limits join orphan cleanup, verified registration/reset and core marketplace browser/DB evidence.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c53e78382d84a3d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bef48bdb0a24d15"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: clean repeatable acceptance DB, 59 Chromium cases and 99-route sweep pass; auth retry limits, orphan cleanup, verified registration/reset, linked inspection, report safety hold and core marketplace journeys have browser/DB evidence. Online staging, providers, public-write limits, cron schedule, branch protection, monitoring and remaining live acceptance stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: clean repeatable acceptance DB, 63 Chromium cases and 99-route sweep pass; auth/public-write limits, orphan cleanup, verified registration/reset, linked inspection, report safety hold and core marketplace journeys have browser/DB evidence. Online staging, providers, cron schedule, proxy validation, branch protection, monitoring and remaining live acceptance stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2953,7 +2953,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 59 passed, 1 planned skip against a fresh isolated PostgreSQL database; 99-route sweep has 0 issues. Auth retry limits, orphan cleanup, verified registration/reset, linked inspection, authenticated reporting and core journeys pass.</x:v>
+        <x:v>Desktop/mobile Chromium: 63 passed, 1 planned skip against a fresh isolated PostgreSQL database; 99-route sweep has 0 issues. Auth, upload, contact and report limits join orphan cleanup, verified registration/reset, linked inspection and core journeys.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
@@ -4436,7 +4436,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G49" s="137" t="n">
-        <x:v>0.93</x:v>
+        <x:v>0.97</x:v>
       </x:c>
       <x:c r="H49" s="136" t="str">
         <x:v>Critical</x:v>
@@ -4457,10 +4457,10 @@
         <x:v>Burst; distributed attempts; reset window; proxy headers</x:v>
       </x:c>
       <x:c r="N49" s="136" t="str">
-        <x:v>PostgreSQL-backed atomic limits now cover sign-in, registration, password reset request/confirmation, verification resend/confirmation; successful sign-in clears the account attempt bucket. Concurrent DB test and desktop/mobile sign-in throttling browser acceptance pass. Reset/resend keep non-enumerating responses.</x:v>
+        <x:v>PostgreSQL-backed atomic limits cover sign-in, registration, reset and verification actions; Google sign-in start now limits configured IP requests. Successful sign-in clears the account attempt bucket. Concurrent DB and desktop/mobile browser retry tests pass.</x:v>
       </x:c>
       <x:c r="O49" s="136" t="str">
-        <x:v>Cover Google OAuth start and verify trusted proxy IP headers, thresholds and alerting in staging.</x:v>
+        <x:v>Verify Google provider path, trusted proxy IP headers, thresholds and alerting in staging.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -10217,7 +10217,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G172" s="137" t="n">
-        <x:v>0.4</x:v>
+        <x:v>0.85</x:v>
       </x:c>
       <x:c r="H172" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10238,10 +10238,10 @@
         <x:v>Per-IP/user; proxy spoof; reset; fail-open/closed</x:v>
       </x:c>
       <x:c r="N172" s="136" t="str">
-        <x:v>Shared database rate-limit buckets and expiry cleanup now protect primary authentication actions across app instances. Atomic concurrency and user-facing login limit pass isolated DB/browser acceptance.</x:v>
+        <x:v>Shared database limits now protect auth actions, Google sign-in start, image-upload requests, seller-contact events and listing reports. Desktop/mobile browser tests prove 429 upload response and blocked contact/report writes; atomic DB concurrency test passes. Existing image count/byte ceilings remain.</x:v>
       </x:c>
       <x:c r="O172" s="136" t="str">
-        <x:v>Extend rate limits to public reports, uploads, lead events and other state-changing endpoints; validate proxy headers and production thresholds.</x:v>
+        <x:v>Review remaining public write actions and validate proxy headers, limits, expiry recovery and alerts in staging.</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -10661,7 +10661,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 59 passed, 1 planned skip. Atomic auth rate limiting and retry UI join orphan cleanup, verified registration/reset, linked inspection, moderation and core marketplace journeys; clean DB reseeding and 99-route sweep pass.</x:v>
+        <x:v>Desktop/mobile Chromium: 63 passed, 1 planned skip. Atomic auth limits and browser-verified upload/contact/report denial join orphan cleanup, verified registration/reset, linked inspection, moderation and core marketplace journeys; clean DB and 99-route sweep pass.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Cover remaining direct-action and validation negatives; add Safari/mobile device and live staging acceptance.</x:v>
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6853d5548c414663"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b4bdd4be2ae40bf"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0796548e5fcb4dd6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02a45947be524964"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13347,10 +13347,10 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E20" s="141" t="str">
-        <x:v>Desktop/mobile Chromium upload, public WebP URL and authenticated foreign-Origin rejection</x:v>
+        <x:v>Desktop/mobile Chromium upload/public WebP URL, foreign-Origin 403 and request-bucket 429 before file read</x:v>
       </x:c>
       <x:c r="F20" s="141" t="str">
-        <x:v>Partial pass: valid image end to end, foreign-origin 403; size/count boundaries remain open</x:v>
+        <x:v>Partial pass: valid image and request limit enforced; individual size/count boundaries remain open</x:v>
       </x:c>
       <x:c r="G20" s="141" t="str">
         <x:v>Representative image fixtures</x:v>
@@ -13893,10 +13893,10 @@
         <x:v>Integration + Security</x:v>
       </x:c>
       <x:c r="E41" s="141" t="str">
-        <x:v>Desktop/mobile Chromium anonymous and authenticated reports, cookie/account duplicate checks and isolated DB assertions</x:v>
+        <x:v>Desktop/mobile Chromium anonymous/auth reports, duplicate cookie/account checks, rate-limit denial and DB assertions</x:v>
       </x:c>
       <x:c r="F41" s="141" t="str">
-        <x:v>Partial pass: anonymous and account duplicates suppressed; invalid-reason/direct-request cases remain</x:v>
+        <x:v>Partial pass: duplicates and excess report writes suppressed; invalid-reason/direct-request cases remain</x:v>
       </x:c>
       <x:c r="G41" s="141" t="str">
         <x:v>Same listing/user/cookie</x:v>
@@ -14153,10 +14153,10 @@
         <x:v>Security/load</x:v>
       </x:c>
       <x:c r="E51" s="141" t="str">
-        <x:v>Not available</x:v>
+        <x:v>Concurrent PostgreSQL bucket test plus desktop/mobile Chromium sign-in, upload, contact and report denial</x:v>
       </x:c>
       <x:c r="F51" s="141" t="str">
-        <x:v>Blocked by feature</x:v>
+        <x:v>Partial pass: limits trigger and block excess writes; staging proxy headers, expiry recovery and remaining actions open</x:v>
       </x:c>
       <x:c r="G51" s="141" t="str">
         <x:v>Rate limits complete</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R551d216ef45c4eab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fb8f629e45241c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re88f8b5903394879"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R031f9d4111ad4997"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Keep preview deployments out of search indexes
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R15e217270e764baa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R97d96e6e51ff4fe5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R9e547433dd604d47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R0223c31a1726419f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R97e981751e054b69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Ra66d6224e4734b19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rdb2e2ae5de044ecc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ref425fcc912d4044"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Raed11b3a50df4dc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Ra08e6443ce2e48de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rbaafb7f281724b0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R19d13b9d657c4ee0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R0b69b23635764384"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R1b95f0b6f37b480e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8bc8ee4c6ef3403d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R019223535bea4c9f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: clean isolated DB, 99-route sweep 0 issues, 63 Chromium tests pass (1 planned skip). Atomic auth, upload, contact and report limits join orphan cleanup, verified registration/reset and core marketplace browser/DB evidence.</x:v>
+        <x:v>PR #6: clean isolated DB, 99-route acceptance sweep 0 issues, 63 Chromium tests pass (1 planned skip). Latest local 97-route sweep found 0 issues; robots policy now blocks preview builds. Production hosting and provider acceptance remain open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bef48bdb0a24d15"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54cd5d46e4ea4174"/>
 </x:worksheet>
 </file>
 
@@ -9956,10 +9956,10 @@
         <x:v>Staging/production env render; robots fetch</x:v>
       </x:c>
       <x:c r="N166" s="136" t="str">
-        <x:v>robots.ts is environment-aware.</x:v>
+        <x:v>Robots policy now gives VERCEL_ENV precedence over NODE_ENV, so preview/development builds remain blocked even when built with NODE_ENV=production. Five environment-policy assertions pass; local 97-route sweep found 0 issues.</x:v>
       </x:c>
       <x:c r="O166" s="136" t="str">
-        <x:v>Verify actual hosting environment variables.</x:v>
+        <x:v>Verify robots.txt and canonical host on the selected production and staging deployments.</x:v>
       </x:c>
     </x:row>
     <x:row r="167">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b4bdd4be2ae40bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4e6e7f9d3314358"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02a45947be524964"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ae75af40ad34e76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fb8f629e45241c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1de4ed893f224783"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R031f9d4111ad4997"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56c411169b804499"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Limit inspection and sell assistance requests
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ref425fcc912d4044"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Raed11b3a50df4dc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Ra08e6443ce2e48de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rbaafb7f281724b0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R19d13b9d657c4ee0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R0b69b23635764384"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R1b95f0b6f37b480e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rff7df4d377df48cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R2f1029306bd8485f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R280f43c66ffd4cef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R8619bcfc306a4e48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R4019a50dd4e94573"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R09ed7dfea6c2457c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R61ffad7d32194849"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R019223535bea4c9f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R078fb41c90d34e1b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8787064676616916</x:v>
+        <x:v>0.8789552238805971</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54cd5d46e4ea4174"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R449847cf77b54a42"/>
 </x:worksheet>
 </file>
 
@@ -8875,7 +8875,7 @@
         <x:v>Auth redirect; validation; phone normalization; listing/no listing</x:v>
       </x:c>
       <x:c r="N143" s="136" t="str">
-        <x:v>Desktop/mobile Chromium and isolated PostgreSQL confirm standalone and car-linked requests, preserved reference across sign-in, forged/unavailable reference rejection and initial event. Customer copy now describes an availability/follow-up request without promising an inspector, checklist or response time.</x:v>
+        <x:v>Standalone and linked inspection requests, customer updates and append-only events pass desktop/mobile browser and isolated DB acceptance. A daily per-account/source request limit now blocks excess submissions without a row.</x:v>
       </x:c>
       <x:c r="O143" s="136" t="str">
         <x:v>Invalid lifecycle transitions and final live browser acceptance remain open.</x:v>
@@ -8969,7 +8969,7 @@
         <x:v>Admin/non-admin; filtering; status changes</x:v>
       </x:c>
       <x:c r="N145" s="136" t="str">
-        <x:v>Desktop/mobile Chromium and isolated PostgreSQL confirm standalone and car-linked requests, preserved listing reference across sign-in, forged/unavailable reference rejection, initial append-only event and customer-visible admin updates without private notes.</x:v>
+        <x:v>Structured Sell My Car Assistance request, linked listing and customer-visible follow-up pass desktop/mobile browser and isolated DB acceptance. A daily per-account/source limit now blocks excess submissions without a row.</x:v>
       </x:c>
       <x:c r="O145" s="136" t="str">
         <x:v>Invalid lifecycle transitions and final live browser acceptance remain open.</x:v>
@@ -10217,7 +10217,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G172" s="137" t="n">
-        <x:v>0.85</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H172" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10238,10 +10238,10 @@
         <x:v>Per-IP/user; proxy spoof; reset; fail-open/closed</x:v>
       </x:c>
       <x:c r="N172" s="136" t="str">
-        <x:v>Shared database limits now protect auth actions, Google sign-in start, image-upload requests, seller-contact events and listing reports. Desktop/mobile browser tests prove 429 upload response and blocked contact/report writes; atomic DB concurrency test passes. Existing image count/byte ceilings remain.</x:v>
+        <x:v>Shared database limits protect auth, Google sign-in start, uploads, seller contact, reports, inspection requests and Sell My Car Assistance requests. Desktop/mobile browser cases confirm excess manual-service requests show a retry message and insert no request row; fresh isolated DB and 99-route sweep pass.</x:v>
       </x:c>
       <x:c r="O172" s="136" t="str">
-        <x:v>Review remaining public write actions and validate proxy headers, limits, expiry recovery and alerts in staging.</x:v>
+        <x:v>Review seller listing publication and remaining writes; validate trusted proxy headers, thresholds, expiry recovery and alerts in staging.</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4e6e7f9d3314358"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30bec4bd6f61474a"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ae75af40ad34e76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0038401e97c74c8a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14153,10 +14153,10 @@
         <x:v>Security/load</x:v>
       </x:c>
       <x:c r="E51" s="141" t="str">
-        <x:v>Concurrent PostgreSQL bucket test plus desktop/mobile Chromium sign-in, upload, contact and report denial</x:v>
+        <x:v>Atomic PostgreSQL bucket test plus desktop/mobile sign-in, upload, contact, report, inspection and assistance denial</x:v>
       </x:c>
       <x:c r="F51" s="141" t="str">
-        <x:v>Partial pass: limits trigger and block excess writes; staging proxy headers, expiry recovery and remaining actions open</x:v>
+        <x:v>Partial pass: each covered limit blocks excess writes; staging proxy headers, expiry recovery and remaining actions open</x:v>
       </x:c>
       <x:c r="G51" s="141" t="str">
         <x:v>Rate limits complete</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1de4ed893f224783"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red7ed14a31fa49c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56c411169b804499"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51643a49b14c4456"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Limit listing publication bursts
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rff7df4d377df48cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R2f1029306bd8485f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R280f43c66ffd4cef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R8619bcfc306a4e48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R4019a50dd4e94573"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R09ed7dfea6c2457c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R61ffad7d32194849"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R22d0205908824507"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R64bbb663e7e249af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Reb85e28662e84750"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R09c1e3d958f64ab0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R3ba339b4b48849f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Red4591cb200b45af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rd293179874e94ad5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R078fb41c90d34e1b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re4c256248118476f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8789552238805971</x:v>
+        <x:v>0.8792039800995025</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: clean isolated DB, 99-route acceptance sweep 0 issues, 63 Chromium tests pass (1 planned skip). Latest local 97-route sweep found 0 issues; robots policy now blocks preview builds. Production hosting and provider acceptance remain open.</x:v>
+        <x:v>PR #6: fresh isolated DB, 99-route sweep 0 issues, 63 Chromium tests pass (1 planned skip). Auth and public-write limits include ad publication and manual service requests; production staging/provider acceptance remains open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R449847cf77b54a42"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R810b92e23e5b4448"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: clean repeatable acceptance DB, 63 Chromium cases and 99-route sweep pass; auth/public-write limits, orphan cleanup, verified registration/reset, linked inspection, report safety hold and core marketplace journeys have browser/DB evidence. Online staging, providers, cron schedule, proxy validation, branch protection, monitoring and remaining live acceptance stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: clean repeatable acceptance DB, 63 Chromium passes and 99-route sweep 0 issues. Auth, uploads, contact, reports, manual-service requests and ad publication have shared limits; inactive detail visibility is owner/admin gated. Online staging, providers, proxy validation, cron scheduling, branch protection and live acceptance stay open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -10050,10 +10050,10 @@
         <x:v>All statuses; canonical; sitemap/search exclusion</x:v>
       </x:c>
       <x:c r="N168" s="136" t="str">
-        <x:v>Metadata noindexes non-active, but private statuses still render publicly.</x:v>
+        <x:v>Current detail-route guard serves inactive listings only to the owner or admin. Browser acceptance confirms pending-review and removed ads return public 404; metadata noindexes non-active views.</x:v>
       </x:c>
       <x:c r="O168" s="136" t="str">
-        <x:v>Resolve with inactive visibility work.</x:v>
+        <x:v>Confirm sold and expired buyer experience with product policy, and run staging crawler acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="169">
@@ -10217,7 +10217,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G172" s="137" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H172" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10238,10 +10238,10 @@
         <x:v>Per-IP/user; proxy spoof; reset; fail-open/closed</x:v>
       </x:c>
       <x:c r="N172" s="136" t="str">
-        <x:v>Shared database limits protect auth, Google sign-in start, uploads, seller contact, reports, inspection requests and Sell My Car Assistance requests. Desktop/mobile browser cases confirm excess manual-service requests show a retry message and insert no request row; fresh isolated DB and 99-route sweep pass.</x:v>
+        <x:v>Shared PostgreSQL limits cover authentication, OAuth start, uploads, contact, reports, inspection, Sell My Car Assistance and all three listing publication flows. Desktop/mobile car browser tests confirm denied ad creates no listing, then normal publication recovers; fresh 63-pass acceptance and 99-route sweep pass.</x:v>
       </x:c>
       <x:c r="O172" s="136" t="str">
-        <x:v>Review seller listing publication and remaining writes; validate trusted proxy headers, thresholds, expiry recovery and alerts in staging.</x:v>
+        <x:v>Validate trusted proxy IP headers, thresholds, expiry recovery and security alerts in staging; review remaining account/dealer write actions.</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30bec4bd6f61474a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba663d9e31034c97"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0038401e97c74c8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e1e0400ffa148ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14153,10 +14153,10 @@
         <x:v>Security/load</x:v>
       </x:c>
       <x:c r="E51" s="141" t="str">
-        <x:v>Atomic PostgreSQL bucket test plus desktop/mobile sign-in, upload, contact, report, inspection and assistance denial</x:v>
+        <x:v>Atomic PostgreSQL bucket check plus desktop/mobile sign-in, upload, contact, report, inspection, assistance and car-publication denial</x:v>
       </x:c>
       <x:c r="F51" s="141" t="str">
-        <x:v>Partial pass: each covered limit blocks excess writes; staging proxy headers, expiry recovery and remaining actions open</x:v>
+        <x:v>Partial pass: limits block excess writes; denied car publication inserts no listing and recovers. Staging proxy and expiry acceptance open.</x:v>
       </x:c>
       <x:c r="G51" s="141" t="str">
         <x:v>Rate limits complete</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red7ed14a31fa49c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2c10943cb1e4360"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51643a49b14c4456"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77fd5ea249ec4c3b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Clarify validation errors across forms
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R22d0205908824507"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R64bbb663e7e249af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Reb85e28662e84750"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R09c1e3d958f64ab0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R3ba339b4b48849f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Red4591cb200b45af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rd293179874e94ad5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc1b253b70a524ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rcd69cc2b58744292"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rb14c31dda1354811"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R9afc2caff67b407f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R2ed483f54b6b40c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rb1aa4aecf1d54bb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R8ce369611d7c44ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re4c256248118476f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6cd824c891104c43"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8792039800995025</x:v>
+        <x:v>0.879452736318408</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R810b92e23e5b4448"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7212ad306ba748e6"/>
 </x:worksheet>
 </file>
 
@@ -10170,7 +10170,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G171" s="137" t="n">
-        <x:v>0.92</x:v>
+        <x:v>0.97</x:v>
       </x:c>
       <x:c r="H171" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10191,10 +10191,10 @@
         <x:v>Tampered forms; oversized text; invalid IDs</x:v>
       </x:c>
       <x:c r="N171" s="136" t="str">
-        <x:v>Car, bike and parts schema bounds now return field-specific messages; car registration and auction combinations reject contradictory submissions. Seller validation checks pass. Cross-feature tampering review remains.</x:v>
+        <x:v>Audited user-input Zod constraints across car, bike, parts, inspection, assistance, dealer, account and saved-search actions. Missing integer, bound and enum messages now explain corrections; malformed city/variant IDs have regression checks. Full check, lint, production build and 97-route local sweep pass.</x:v>
       </x:c>
       <x:c r="O171" s="136" t="str">
-        <x:v>Audit remaining forms and direct server-action inputs; add negative browser coverage for auth, listing edit/delete and admin permissions.</x:v>
+        <x:v>Complete direct server-action tampering/browser negative matrix for auth, edits, deletes and admin permissions in JW-166/JW-177.</x:v>
       </x:c>
     </x:row>
     <x:row r="172">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba663d9e31034c97"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c0e3c7494454b86"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e1e0400ffa148ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcee1bdbb55764fdd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2c10943cb1e4360"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb80be8a622024196"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77fd5ea249ec4c3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29e5d7a06bd440bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Audit public and seller accessibility
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc1b253b70a524ce4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rcd69cc2b58744292"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rb14c31dda1354811"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R9afc2caff67b407f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R2ed483f54b6b40c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rb1aa4aecf1d54bb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R8ce369611d7c44ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf53f7a51fb1a42ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rb703f89019e14b33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R70f0a8019ee44d96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R642dbf5a02244e88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rfe2ab65fb2304eb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R2a8d5d198f4e4c1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R7ab7228c93f342c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6cd824c891104c43"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3af6efd060314d34"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1316,7 +1316,7 @@
       </x:c>
       <x:c r="B8" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C8" s="88"/>
       <x:c r="D8" s="97" t="str">
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="B10" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C10" s="88"/>
       <x:c r="D10" s="97" t="str">
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.879452736318408</x:v>
+        <x:v>0.8839303482587066</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1504,7 +1504,7 @@
       </x:c>
       <x:c r="B17" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C17" s="110" t="str">
         <x:v>Foundation exists; end-to-end feature incomplete</x:v>
@@ -1542,7 +1542,7 @@
       </x:c>
       <x:c r="B19" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C19" s="110" t="str">
         <x:v>Not implemented</x:v>
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: fresh isolated DB, 99-route sweep 0 issues, 63 Chromium tests pass (1 planned skip). Auth and public-write limits include ad publication and manual service requests; production staging/provider acceptance remains open.</x:v>
+        <x:v>PR #6: fresh isolated DB, 99-route sweep 0 issues, 69 Chromium tests pass (1 planned skip). Automated axe-core scan covers 16 public/seller routes on desktop/mobile; manual and live staging acceptance remain open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7212ad306ba748e6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c2ab15f7f6e4a98"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: clean repeatable acceptance DB, 63 Chromium passes and 99-route sweep 0 issues. Auth, uploads, contact, reports, manual-service requests and ad publication have shared limits; inactive detail visibility is owner/admin gated. Online staging, providers, proxy validation, cron scheduling, branch protection and live acceptance stay open.</x:v>
+        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 69 Chromium passes, 1 planned skip and 99-route sweep 0 issues. Public/seller accessibility scan has no axe violations across 16 routes in desktop/mobile. Online staging, provider configuration, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2953,7 +2953,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 63 passed, 1 planned skip against a fresh isolated PostgreSQL database; 99-route sweep has 0 issues. Auth, upload, contact and report limits join orphan cleanup, verified registration/reset, linked inspection and core journeys.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks and 69 desktop/mobile Chromium cases pass, with 1 planned viewport skip. 99-route sweep has 0 issues. Public and seller accessibility scan covers 16 routes in both viewports; live/manual acceptance remains open.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
@@ -3919,7 +3919,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G38" s="137" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H38" s="136" t="str">
         <x:v>High</x:v>
@@ -3940,10 +3940,10 @@
         <x:v>axe; keyboard-only; zoom 200%; contrast</x:v>
       </x:c>
       <x:c r="N38" s="136" t="str">
-        <x:v>Shared shell has keyboard focus and skip link; decorative hero imagery has reduced-motion fallback. Owner approved homepage visuals and 936baee is pushed; comprehensive accessibility audit remains open.</x:v>
+        <x:v>Automated axe-core audit now covers 10 public and 6 signed-in seller routes on desktop and mobile with no violations. Form/file labels, map region semantics, sort control name and low-contrast text were corrected; keyboard skip link passes. Homepage visual approval remains recorded.</x:v>
       </x:c>
       <x:c r="O38" s="136" t="str">
-        <x:v>Run keyboard, screen-reader, contrast and reduced-motion acceptance across primary flows during final QA.</x:v>
+        <x:v>Complete manual screen-reader and real-device keyboard/reduced-motion review, then extend automated audit to dealer and administrator journeys.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -10661,7 +10661,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Desktop/mobile Chromium: 63 passed, 1 planned skip. Atomic auth limits and browser-verified upload/contact/report denial join orphan cleanup, verified registration/reset, linked inspection, moderation and core marketplace journeys; clean DB and 99-route sweep pass.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 69 desktop/mobile Chromium passes and 1 planned skip. 99-route sweep has 0 issues; automated accessibility coverage now spans 16 public/seller routes in both viewports.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Cover remaining direct-action and validation negatives; add Safari/mobile device and live staging acceptance.</x:v>
@@ -10731,10 +10731,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F183" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G183" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="H183" s="136" t="str">
         <x:v>High</x:v>
@@ -10755,10 +10755,10 @@
         <x:v>axe; keyboard; screen reader spot checks</x:v>
       </x:c>
       <x:c r="N183" s="136" t="str">
-        <x:v>Accessibility intent exists but no recorded audit.</x:v>
+        <x:v>Automated axe-core checks cover 16 public/seller routes across desktop and mobile, plus keyboard skip-link acceptance. Identified contrast, form-label and map-region issues were fixed. Production build remains below the 150 KB first-load JS cap.</x:v>
       </x:c>
       <x:c r="O183" s="136" t="str">
-        <x:v>Run per feature and final site-wide audit.</x:v>
+        <x:v>Audit dealer/admin and listing-detail journeys; complete manual screen-reader, keyboard, reduced-motion and real-device acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="184">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c0e3c7494454b86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80f27acab39b4be8"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcee1bdbb55764fdd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0dd0f7cf6374f7a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14049,10 +14049,10 @@
         <x:v>Automated + Manual</x:v>
       </x:c>
       <x:c r="E47" s="141" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Automated axe-core audit on 16 public/seller routes in desktop and mobile Chromium; keyboard skip-link test</x:v>
       </x:c>
       <x:c r="F47" s="141" t="str">
-        <x:v>Final accessibility QA</x:v>
+        <x:v>Partial pass: automated scan has no violations after contrast, label and map fixes; manual screen-reader, zoom, reduced-motion and real-device review open</x:v>
       </x:c>
       <x:c r="G47" s="141" t="str">
         <x:v>Feature-complete UI</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb80be8a622024196"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a3962b691ba49c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29e5d7a06bd440bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7afb88f1dfdb4478"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Audit dealer and admin accessibility
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf53f7a51fb1a42ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rb703f89019e14b33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R70f0a8019ee44d96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R642dbf5a02244e88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rfe2ab65fb2304eb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R2a8d5d198f4e4c1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R7ab7228c93f342c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R50ab073f5fd4435d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Reeb51718f67b412b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R7e077ebd1e9b4d00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R5a6847cdfe684e0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R1f70d83c3d3c4b93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rb6fa35a930894b0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rfcec917fb7c040f7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3af6efd060314d34"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Radf2d6a0ea7046b8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8839303482587066</x:v>
+        <x:v>0.8846766169154229</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: fresh isolated DB, 99-route sweep 0 issues, 69 Chromium tests pass (1 planned skip). Automated axe-core scan covers 16 public/seller routes on desktop/mobile; manual and live staging acceptance remain open.</x:v>
+        <x:v>PR #6: fresh isolated DB, 101-route sweep 0 issues, 73 Chromium tests pass (1 planned skip). Automated axe-core scan covers 24 public/seller/dealer/admin routes on desktop/mobile; manual and live staging acceptance remain open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c2ab15f7f6e4a98"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R044e1bf5344448e3"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 69 Chromium passes, 1 planned skip and 99-route sweep 0 issues. Public/seller accessibility scan has no axe violations across 16 routes in desktop/mobile. Online staging, provider configuration, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
+        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 73 Chromium passes, 1 planned skip and 101-route sweep 0 issues. Accessibility scan has no axe violations across 24 routes in desktop/mobile. Online staging, provider configuration, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2953,7 +2953,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks and 69 desktop/mobile Chromium cases pass, with 1 planned viewport skip. 99-route sweep has 0 issues. Public and seller accessibility scan covers 16 routes in both viewports; live/manual acceptance remains open.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks and 73 desktop/mobile Chromium cases pass, with 1 planned viewport skip. 101-route sweep has 0 issues. Accessibility scan covers 24 routes in both viewports; live/manual acceptance remains open.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
@@ -3919,7 +3919,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G38" s="137" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H38" s="136" t="str">
         <x:v>High</x:v>
@@ -3940,10 +3940,10 @@
         <x:v>axe; keyboard-only; zoom 200%; contrast</x:v>
       </x:c>
       <x:c r="N38" s="136" t="str">
-        <x:v>Automated axe-core audit now covers 10 public and 6 signed-in seller routes on desktop and mobile with no violations. Form/file labels, map region semantics, sort control name and low-contrast text were corrected; keyboard skip link passes. Homepage visual approval remains recorded.</x:v>
+        <x:v>Automated axe-core audit covers 24 public, seller, dealer and administrator routes on desktop/mobile with no violations. Form/file labels, map semantics, navigation naming and low-contrast text/buttons were corrected; keyboard skip link passes. Homepage visuals remain owner-approved.</x:v>
       </x:c>
       <x:c r="O38" s="136" t="str">
-        <x:v>Complete manual screen-reader and real-device keyboard/reduced-motion review, then extend automated audit to dealer and administrator journeys.</x:v>
+        <x:v>Complete manual screen-reader, zoom, keyboard and reduced-motion review on real devices during launch acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -10661,7 +10661,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 69 desktop/mobile Chromium passes and 1 planned skip. 99-route sweep has 0 issues; automated accessibility coverage now spans 16 public/seller routes in both viewports.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 73 desktop/mobile Chromium passes and 1 planned skip. 101-route sweep has 0 issues; automated accessibility coverage spans 24 public/seller/dealer/admin routes in both viewports.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Cover remaining direct-action and validation negatives; add Safari/mobile device and live staging acceptance.</x:v>
@@ -10734,7 +10734,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G183" s="137" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.85</x:v>
       </x:c>
       <x:c r="H183" s="136" t="str">
         <x:v>High</x:v>
@@ -10755,10 +10755,10 @@
         <x:v>axe; keyboard; screen reader spot checks</x:v>
       </x:c>
       <x:c r="N183" s="136" t="str">
-        <x:v>Automated axe-core checks cover 16 public/seller routes across desktop and mobile, plus keyboard skip-link acceptance. Identified contrast, form-label and map-region issues were fixed. Production build remains below the 150 KB first-load JS cap.</x:v>
+        <x:v>Automated axe-core audit covers 24 public, seller, dealer and administrator routes in both viewports; skip-link keyboard acceptance passes. Corrected form labels, navigation landmarks and contrast. Dealer registration scan uses independently seeded accounts. Manual assistive-technology/live-device acceptance remains open.</x:v>
       </x:c>
       <x:c r="O183" s="136" t="str">
-        <x:v>Audit dealer/admin and listing-detail journeys; complete manual screen-reader, keyboard, reduced-motion and real-device acceptance.</x:v>
+        <x:v>Add listing-detail and remaining account journeys to automated audit, then complete manual screen-reader, zoom, keyboard and reduced-motion acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="184">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80f27acab39b4be8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdf321d16a0b4aea"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0dd0f7cf6374f7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd1fa65834fe4df8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14049,10 +14049,10 @@
         <x:v>Automated + Manual</x:v>
       </x:c>
       <x:c r="E47" s="141" t="str">
-        <x:v>Automated axe-core audit on 16 public/seller routes in desktop and mobile Chromium; keyboard skip-link test</x:v>
+        <x:v>Automated axe-core audit on 24 public/seller/dealer/admin routes in desktop and mobile Chromium; keyboard skip-link test</x:v>
       </x:c>
       <x:c r="F47" s="141" t="str">
-        <x:v>Partial pass: automated scan has no violations after contrast, label and map fixes; manual screen-reader, zoom, reduced-motion and real-device review open</x:v>
+        <x:v>Partial pass: automated scan has no violations after contrast, label and landmark fixes; manual screen-reader, zoom, reduced-motion and real-device review open</x:v>
       </x:c>
       <x:c r="G47" s="141" t="str">
         <x:v>Feature-complete UI</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a3962b691ba49c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfc6a867fa6a4d36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7afb88f1dfdb4478"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3546346a4dee441e"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Audit listing detail and account accessibility
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R50ab073f5fd4435d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Reeb51718f67b412b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R7e077ebd1e9b4d00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R5a6847cdfe684e0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R1f70d83c3d3c4b93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rb6fa35a930894b0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rfcec917fb7c040f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R52731acb95654352"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R16deac47002d4a07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R8eeae9eb8a9b42a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Ra5c11396120b436b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rfed83a38b0964f39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rab70a54f57db4dc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R71f9ad797ab04ffc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Radf2d6a0ea7046b8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Reeb482a9cb05438c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8846766169154229</x:v>
+        <x:v>0.8850248756218908</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: fresh isolated DB, 101-route sweep 0 issues, 73 Chromium tests pass (1 planned skip). Automated axe-core scan covers 24 public/seller/dealer/admin routes on desktop/mobile; manual and live staging acceptance remain open.</x:v>
+        <x:v>PR #6: fresh isolated DB, 101-route sweep 0 issues, 75 Chromium tests pass (1 planned skip). Automated axe-core scan covers 34 routes on desktop/mobile; manual and live staging acceptance remain open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R044e1bf5344448e3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc90d549967db4d2e"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 73 Chromium passes, 1 planned skip and 101-route sweep 0 issues. Accessibility scan has no axe violations across 24 routes in desktop/mobile. Online staging, provider configuration, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
+        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 75 Chromium passes, 1 planned skip and 101-route sweep 0 issues. Accessibility scan has no axe violations across 34 routes in desktop/mobile. Online staging, provider configuration, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2953,7 +2953,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks and 73 desktop/mobile Chromium cases pass, with 1 planned viewport skip. 101-route sweep has 0 issues. Accessibility scan covers 24 routes in both viewports; live/manual acceptance remains open.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks and 75 desktop/mobile Chromium cases pass, with 1 planned viewport skip. 101-route sweep has 0 issues. Accessibility scan covers 34 routes in both viewports; live/manual acceptance remains open.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
@@ -3919,7 +3919,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G38" s="137" t="n">
-        <x:v>0.95</x:v>
+        <x:v>0.97</x:v>
       </x:c>
       <x:c r="H38" s="136" t="str">
         <x:v>High</x:v>
@@ -3940,10 +3940,10 @@
         <x:v>axe; keyboard-only; zoom 200%; contrast</x:v>
       </x:c>
       <x:c r="N38" s="136" t="str">
-        <x:v>Automated axe-core audit covers 24 public, seller, dealer and administrator routes on desktop/mobile with no violations. Form/file labels, map semantics, navigation naming and low-contrast text/buttons were corrected; keyboard skip link passes. Homepage visuals remain owner-approved.</x:v>
+        <x:v>Automated axe-core audit covers 34 public, seller, dealer, administrator and vehicle-detail routes on desktop/mobile with no violations. Forms, landmarks, listing detail CTA, recent-history text and customer histories now pass contrast/label checks. Keyboard skip link passes; homepage visuals remain owner-approved.</x:v>
       </x:c>
       <x:c r="O38" s="136" t="str">
-        <x:v>Complete manual screen-reader, zoom, keyboard and reduced-motion review on real devices during launch acceptance.</x:v>
+        <x:v>Complete manual screen-reader, keyboard, zoom and reduced-motion review on real devices during launch acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -10661,7 +10661,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 73 desktop/mobile Chromium passes and 1 planned skip. 101-route sweep has 0 issues; automated accessibility coverage spans 24 public/seller/dealer/admin routes in both viewports.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 75 desktop/mobile Chromium passes and 1 planned skip. 101-route sweep has 0 issues; automated accessibility coverage spans 34 public/seller/dealer/admin/vehicle-detail routes in both viewports.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Cover remaining direct-action and validation negatives; add Safari/mobile device and live staging acceptance.</x:v>
@@ -10734,7 +10734,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G183" s="137" t="n">
-        <x:v>0.85</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H183" s="136" t="str">
         <x:v>High</x:v>
@@ -10755,10 +10755,10 @@
         <x:v>axe; keyboard; screen reader spot checks</x:v>
       </x:c>
       <x:c r="N183" s="136" t="str">
-        <x:v>Automated axe-core audit covers 24 public, seller, dealer and administrator routes in both viewports; skip-link keyboard acceptance passes. Corrected form labels, navigation landmarks and contrast. Dealer registration scan uses independently seeded accounts. Manual assistive-technology/live-device acceptance remains open.</x:v>
+        <x:v>Automated axe-core audit covers 34 routes across public, seller, dealer, administrator and car/bike/part detail journeys in both viewports. Fixed low-contrast text and phone CTA, form labels and navigation landmarks. Manual assistive-technology/live-device acceptance remains open.</x:v>
       </x:c>
       <x:c r="O183" s="136" t="str">
-        <x:v>Add listing-detail and remaining account journeys to automated audit, then complete manual screen-reader, zoom, keyboard and reduced-motion acceptance.</x:v>
+        <x:v>Complete manual screen-reader, keyboard, zoom and reduced-motion acceptance, then extend automated scans to remaining conditional form states.</x:v>
       </x:c>
     </x:row>
     <x:row r="184">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdf321d16a0b4aea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc59edf3cd5854c1b"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd1fa65834fe4df8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R713239cf871f4d5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14049,7 +14049,7 @@
         <x:v>Automated + Manual</x:v>
       </x:c>
       <x:c r="E47" s="141" t="str">
-        <x:v>Automated axe-core audit on 24 public/seller/dealer/admin routes in desktop and mobile Chromium; keyboard skip-link test</x:v>
+        <x:v>Automated axe-core audit on 34 public/seller/dealer/admin/vehicle-detail routes in desktop and mobile Chromium; keyboard skip-link test</x:v>
       </x:c>
       <x:c r="F47" s="141" t="str">
         <x:v>Partial pass: automated scan has no violations after contrast, label and landmark fixes; manual screen-reader, zoom, reduced-motion and real-device review open</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfc6a867fa6a4d36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a6d5b44098143a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3546346a4dee441e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46986a95226c42ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Limit account and dealer setting writes
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R52731acb95654352"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R16deac47002d4a07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R8eeae9eb8a9b42a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Ra5c11396120b436b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rfed83a38b0964f39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rab70a54f57db4dc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R71f9ad797ab04ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R85e8320113f7430b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R7706b7c67f254f2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R0beb59f1f00548bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rac939bbad5a94205"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R6ebafa8cdb6b43f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R134b6a3e4a674e94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Recb7b7f6b43c44bc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Reeb482a9cb05438c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R18eed6b912ca49af"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8850248756218908</x:v>
+        <x:v>0.885174129353234</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: fresh isolated DB, 101-route sweep 0 issues, 75 Chromium tests pass (1 planned skip). Automated axe-core scan covers 34 routes on desktop/mobile; manual and live staging acceptance remain open.</x:v>
+        <x:v>PR #6: fresh isolated DB, 101-route sweep 0 issues, 79 Chromium tests pass (1 planned skip). Account/dealer settings limits and 34-route accessibility scan pass on desktop/mobile; live staging acceptance remains open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc90d549967db4d2e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ccac87b9b714250"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 75 Chromium passes, 1 planned skip and 101-route sweep 0 issues. Accessibility scan has no axe violations across 34 routes in desktop/mobile. Online staging, provider configuration, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
+        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 79 Chromium passes, 1 planned skip and 101-route sweep 0 issues. Shared write limits include account/dealer settings; 34-route accessibility audit passes. Online staging, provider configuration, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2953,7 +2953,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks and 75 desktop/mobile Chromium cases pass, with 1 planned viewport skip. 101-route sweep has 0 issues. Accessibility scan covers 34 routes in both viewports; live/manual acceptance remains open.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks and 79 desktop/mobile Chromium cases pass, with 1 planned viewport skip. 101-route sweep has 0 issues. Account/dealer settings limits and 34-route accessibility scan join core marketplace coverage; live/manual acceptance remains open.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
@@ -10217,7 +10217,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G172" s="137" t="n">
-        <x:v>0.95</x:v>
+        <x:v>0.98</x:v>
       </x:c>
       <x:c r="H172" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10238,10 +10238,10 @@
         <x:v>Per-IP/user; proxy spoof; reset; fail-open/closed</x:v>
       </x:c>
       <x:c r="N172" s="136" t="str">
-        <x:v>Shared PostgreSQL limits cover authentication, OAuth start, uploads, contact, reports, inspection, Sell My Car Assistance and all three listing publication flows. Desktop/mobile car browser tests confirm denied ad creates no listing, then normal publication recovers; fresh 63-pass acceptance and 99-route sweep pass.</x:v>
+        <x:v>Shared PostgreSQL limits now cover authentication, OAuth start, uploads, contact, reports, manual-service requests, ad publication, account profile/password/avatar and dealer registration/profile/logo. Fresh desktop/mobile browser tests verify denied account/dealer writes preserve database state; atomic concurrency DB test passes.</x:v>
       </x:c>
       <x:c r="O172" s="136" t="str">
-        <x:v>Validate trusted proxy IP headers, thresholds, expiry recovery and security alerts in staging; review remaining account/dealer write actions.</x:v>
+        <x:v>Validate trusted proxy IP headers, thresholds, expiry recovery and security alerts in staging; review remaining remove and administrator write actions.</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -10661,7 +10661,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 75 desktop/mobile Chromium passes and 1 planned skip. 101-route sweep has 0 issues; automated accessibility coverage spans 34 public/seller/dealer/admin/vehicle-detail routes in both viewports.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 79 desktop/mobile Chromium passes and 1 planned skip. 101-route sweep has 0 issues; account/dealer write-denial tests and 34-route accessibility audit pass in both viewports.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Cover remaining direct-action and validation negatives; add Safari/mobile device and live staging acceptance.</x:v>
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc59edf3cd5854c1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b783498d3ff45d3"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R713239cf871f4d5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf21d8a4d3af847cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14153,10 +14153,10 @@
         <x:v>Security/load</x:v>
       </x:c>
       <x:c r="E51" s="141" t="str">
-        <x:v>Atomic PostgreSQL bucket check plus desktop/mobile sign-in, upload, contact, report, inspection, assistance and car-publication denial</x:v>
+        <x:v>Atomic PostgreSQL bucket check plus desktop/mobile sign-in, upload, contact, report, inspection, assistance, car publication and account/dealer settings denial</x:v>
       </x:c>
       <x:c r="F51" s="141" t="str">
-        <x:v>Partial pass: limits block excess writes; denied car publication inserts no listing and recovers. Staging proxy and expiry acceptance open.</x:v>
+        <x:v>Partial pass: covered limits block excess writes; denied account/dealer profile, password and image changes preserve database state. Staging proxy, expiry and remaining actions open.</x:v>
       </x:c>
       <x:c r="G51" s="141" t="str">
         <x:v>Rate limits complete</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a6d5b44098143a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa86857f02ec4456"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46986a95226c42ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d2e3b6c4b4a46fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Verify profile photo lifecycle
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R85e8320113f7430b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R7706b7c67f254f2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R0beb59f1f00548bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rac939bbad5a94205"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R6ebafa8cdb6b43f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R134b6a3e4a674e94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Recb7b7f6b43c44bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rff16d8550d96479a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rfe25f64f38bb4f6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Ree3cbbf4853a4784"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rd89e3300d7bb4216"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R9a048496519949f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R1170b729af114264"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rc896e4d811c44c92"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R18eed6b912ca49af"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R45c3167394ec4481"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1262,7 +1262,7 @@
       </x:c>
       <x:c r="B6" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>153</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="C6" s="88"/>
       <x:c r="D6" s="97" t="str">
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="B10" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C10" s="88"/>
       <x:c r="D10" s="97" t="str">
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.885174129353234</x:v>
+        <x:v>0.8901492537313435</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1466,7 +1466,7 @@
       </x:c>
       <x:c r="B15" s="106" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>153</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="C15" s="107" t="str">
         <x:v>Implemented in current code and functionally available</x:v>
@@ -1542,7 +1542,7 @@
       </x:c>
       <x:c r="B19" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C19" s="110" t="str">
         <x:v>Not implemented</x:v>
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: fresh isolated DB, 101-route sweep 0 issues, 79 Chromium tests pass (1 planned skip). Account/dealer settings limits and 34-route accessibility scan pass on desktop/mobile; live staging acceptance remains open.</x:v>
+        <x:v>PR #6: fresh isolated DB, 101-route sweep 0 issues, 81 Chromium tests pass (1 planned skip). Avatar lifecycle, account/dealer limits and 34-route accessibility scan pass on desktop/mobile; live staging acceptance remains open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ccac87b9b714250"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc77900564644871"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 79 Chromium passes, 1 planned skip and 101-route sweep 0 issues. Shared write limits include account/dealer settings; 34-route accessibility audit passes. Online staging, provider configuration, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
+        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 81 Chromium passes, 1 planned skip and 101-route sweep 0 issues. Avatar lifecycle and shared write limits pass on desktop/mobile; 34-route accessibility audit passes. Online staging, providers, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2953,7 +2953,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks and 79 desktop/mobile Chromium cases pass, with 1 planned viewport skip. 101-route sweep has 0 issues. Account/dealer settings limits and 34-route accessibility scan join core marketplace coverage; live/manual acceptance remains open.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 81 desktop/mobile Chromium cases pass and 1 planned skip. 101-route sweep has 0 issues. Avatar upload/replacement/removal, account/dealer limits and 34-route accessibility audit pass; live/manual acceptance remains open.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
@@ -4856,10 +4856,10 @@
         <x:v>Signed V1</x:v>
       </x:c>
       <x:c r="F58" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="G58" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H58" s="136" t="str">
         <x:v>Low</x:v>
@@ -4880,10 +4880,10 @@
         <x:v>Upload types/size; authorization; replacement</x:v>
       </x:c>
       <x:c r="N58" s="136" t="str">
-        <x:v>avatarUrl column exists only.</x:v>
+        <x:v>Owner-only avatar upload, replacement and removal are implemented with validated image storage. Fresh desktop/mobile Chromium tests upload twice, confirm distinct stored keys and visible profile images, then remove the photo and verify the account row is cleared. Account image write limit denial is also browser-tested.</x:v>
       </x:c>
       <x:c r="O58" s="136" t="str">
-        <x:v>Implement with profile editing if retained in V1 UI.</x:v>
+        <x:v>Local behavior is complete; verify Cloudflare media cleanup after the production image provider is configured.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -10661,7 +10661,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 79 desktop/mobile Chromium passes and 1 planned skip. 101-route sweep has 0 issues; account/dealer write-denial tests and 34-route accessibility audit pass in both viewports.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 81 desktop/mobile Chromium passes and 1 planned skip. 101-route sweep has 0 issues; owner avatar upload/replacement/removal, account/dealer write-denial and 34-route accessibility audit pass in both viewports.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Cover remaining direct-action and validation negatives; add Safari/mobile device and live staging acceptance.</x:v>
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b783498d3ff45d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R816d21316b9e4297"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf21d8a4d3af847cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ab5aa30ea784da9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa86857f02ec4456"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2294e760e7141c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d2e3b6c4b4a46fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49a445f9c4e6460a"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add parts structured data and escape JSON-LD
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rff16d8550d96479a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rfe25f64f38bb4f6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Ree3cbbf4853a4784"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rd89e3300d7bb4216"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R9a048496519949f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R1170b729af114264"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rc896e4d811c44c92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R22ec360eabfa4321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R0331a5242faa40f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R2c86a82394854160"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rdd25fa81cd154468"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R7b162b7b0a9945e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rc552cf54326c4354"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R3c9bfd029e474750"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R45c3167394ec4481"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rec51a959dcbb46f2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8901492537313435</x:v>
+        <x:v>0.8908955223880599</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: fresh isolated DB, 101-route sweep 0 issues, 81 Chromium tests pass (1 planned skip). Avatar lifecycle, account/dealer limits and 34-route accessibility scan pass on desktop/mobile; live staging acceptance remains open.</x:v>
+        <x:v>PR #6: fresh isolated DB, 101-route sweep 0 issues, 83 Chromium tests pass (1 planned skip). Parts Product schema, avatar lifecycle, account/dealer limits and 34-route accessibility scan pass on desktop/mobile; live staging acceptance remains open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc77900564644871"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0364adef41042a4"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 81 Chromium passes, 1 planned skip and 101-route sweep 0 issues. Avatar lifecycle and shared write limits pass on desktop/mobile; 34-route accessibility audit passes. Online staging, providers, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
+        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 83 Chromium passes, 1 planned skip and 101-route sweep 0 issues. Parts Product schema, avatar lifecycle, shared write limits and 34-route accessibility audit pass. Online staging, providers, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2953,7 +2953,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 81 desktop/mobile Chromium cases pass and 1 planned skip. 101-route sweep has 0 issues. Avatar upload/replacement/removal, account/dealer limits and 34-route accessibility audit pass; live/manual acceptance remains open.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 83 desktop/mobile Chromium cases pass and 1 planned skip. 101-route sweep has 0 issues. Parts Product schema, avatar lifecycle, account/dealer limits and 34-route accessibility audit pass; live/manual acceptance remains open.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
@@ -9794,7 +9794,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G163" s="137" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H163" s="136" t="str">
         <x:v>High</x:v>
@@ -9815,10 +9815,10 @@
         <x:v>Schema.org validator; all verticals; production origin</x:v>
       </x:c>
       <x:c r="N163" s="136" t="str">
-        <x:v>Core JSON-LD exists; parts product-specific schema and production validation remain.</x:v>
+        <x:v>Car/bike Vehicle and auto-parts Product JSON-LD now render from visible listing data. Parts include PKR Offer price, condition, optional brand/category and city without checkout or shipping claims. Shared JSON-LD serialization escapes seller-controlled text so it cannot close the script element. Five new SEO assertions and desktop/mobile parts-detail browser checks pass.</x:v>
       </x:c>
       <x:c r="O163" s="136" t="str">
-        <x:v>Validate after deployment and add appropriate parts schema.</x:v>
+        <x:v>Run Google/schema.org rich-result validation against the selected public staging and production origins, including real media URLs.</x:v>
       </x:c>
     </x:row>
     <x:row r="164">
@@ -10661,7 +10661,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 81 desktop/mobile Chromium passes and 1 planned skip. 101-route sweep has 0 issues; owner avatar upload/replacement/removal, account/dealer write-denial and 34-route accessibility audit pass in both viewports.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 83 desktop/mobile Chromium passes and 1 planned skip. 101-route sweep has 0 issues; parts Product schema, avatar lifecycle, write-denial and 34-route accessibility audit pass in both viewports.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Cover remaining direct-action and validation negatives; add Safari/mobile device and live staging acceptance.</x:v>
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R816d21316b9e4297"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4d3f1f39a9e45fb"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ab5aa30ea784da9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4906b039604d4e72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14101,10 +14101,10 @@
         <x:v>Manual + automated schema</x:v>
       </x:c>
       <x:c r="E49" s="141" t="str">
-        <x:v>Not run</x:v>
+        <x:v>49 local SEO assertions plus desktop/mobile Chromium Product JSON-LD extraction from an active parts listing</x:v>
       </x:c>
       <x:c r="F49" s="141" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partial pass: Product type, canonical URL, PKR price, condition and classified-only offer verified; public rich-result validator and production origin/media checks remain</x:v>
       </x:c>
       <x:c r="G49" s="141" t="str">
         <x:v>Deployed staging URL</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2294e760e7141c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76c07f3e07a44eda"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49a445f9c4e6460a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3f4906439774c95"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Document V1 regression sign-off
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R22ec360eabfa4321"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R0331a5242faa40f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R2c86a82394854160"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rdd25fa81cd154468"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R7b162b7b0a9945e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rc552cf54326c4354"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R3c9bfd029e474750"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re2d066a131264cc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R5aabb5d1a0794ba8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R9733e773e3834b02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rff41a02c91da449a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rf5e2a372cdcb4c32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R8fff2e93fb364914"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R597ddfaa6a6c47ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rec51a959dcbb46f2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3c78041ef87e42a4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1316,7 +1316,7 @@
       </x:c>
       <x:c r="B8" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C8" s="88"/>
       <x:c r="D8" s="97" t="str">
@@ -1370,7 +1370,7 @@
       </x:c>
       <x:c r="B10" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C10" s="88"/>
       <x:c r="D10" s="97" t="str">
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8908955223880599</x:v>
+        <x:v>0.8953731343283585</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1504,7 +1504,7 @@
       </x:c>
       <x:c r="B17" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C17" s="110" t="str">
         <x:v>Foundation exists; end-to-end feature incomplete</x:v>
@@ -1542,7 +1542,7 @@
       </x:c>
       <x:c r="B19" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C19" s="110" t="str">
         <x:v>Not implemented</x:v>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0364adef41042a4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4619ee05c8764f7a"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 83 Chromium passes, 1 planned skip and 101-route sweep 0 issues. Parts Product schema, avatar lifecycle, shared write limits and 34-route accessibility audit pass. Online staging, providers, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
+        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 83 Chromium passes, 1 planned skip and 101-route sweep 0 issues. Parts Product schema, avatar lifecycle, write limits and 34-route accessibility audit pass. A linked V1 regression checklist now records release evidence and blockers. Online staging, providers, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -10872,10 +10872,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F186" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G186" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H186" s="136" t="str">
         <x:v>High</x:v>
@@ -10896,10 +10896,10 @@
         <x:v>Checklist review; defect retest</x:v>
       </x:c>
       <x:c r="N186" s="136" t="str">
-        <x:v>Process is informal.</x:v>
+        <x:v>docs/REGRESSION_CHECKLIST.md now defines a reusable release-candidate record, automated gate, module-by-module manual steps linked to Test Matrix IDs, expected evidence, defect retest and merge sign-off rules. Deployment guide links to it. Local automation is current, but live staging/provider/real-device evidence and reviewer signatures are not yet available.</x:v>
       </x:c>
       <x:c r="O186" s="136" t="str">
-        <x:v>Use this workbook's Test Matrix for feature sign-off.</x:v>
+        <x:v>Fill the checklist and Test Matrix with candidate-specific staging, Safari/real-device, provider and infrastructure evidence; obtain PR reviewer sign-off before merge.</x:v>
       </x:c>
     </x:row>
     <x:row r="187">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4d3f1f39a9e45fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6dce35a751643e3"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4906b039604d4e72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1576224de5234e6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76c07f3e07a44eda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re15be31192e94e5a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3f4906439774c95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc4a4c3aaae9421e"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add iPhone WebKit acceptance smoke
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re2d066a131264cc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R5aabb5d1a0794ba8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R9733e773e3834b02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rff41a02c91da449a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rf5e2a372cdcb4c32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R8fff2e93fb364914"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R597ddfaa6a6c47ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8ed0eb17e8594175"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R04541f9624524d36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R2b6e7f29dbbb4ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R3df7e105541342d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R63fb03dcbdba4103"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rcb44fa3772bb4322"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rb6be661385ac4feb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3c78041ef87e42a4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6072e333726747df"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8953731343283585</x:v>
+        <x:v>0.8963681592039803</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: fresh isolated DB, 101-route sweep 0 issues, 83 Chromium tests pass (1 planned skip). Parts Product schema, avatar lifecycle, account/dealer limits and 34-route accessibility scan pass on desktop/mobile; live staging acceptance remains open.</x:v>
+        <x:v>PR #6: fresh isolated DB, 101-route sweep 0 issues, 85 browser tests pass (1 planned skip), including two iPhone WebKit smoke cases. Parts schema, avatar lifecycle, write limits and 34-route Chromium accessibility scan pass; live staging/real-device acceptance remains open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4619ee05c8764f7a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4de7b0f3baac4a34"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 83 Chromium passes, 1 planned skip and 101-route sweep 0 issues. Parts Product schema, avatar lifecycle, write limits and 34-route accessibility audit pass. A linked V1 regression checklist now records release evidence and blockers. Online staging, providers, proxy validation, cron schedule, branch protection, manual accessibility and live acceptance remain open.</x:v>
+        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 85 browser passes across Chromium and iPhone WebKit smoke, 1 planned skip and 101-route sweep 0 issues. Regression checklist records evidence and blockers. Online staging, providers, proxy validation, cron schedule, branch protection, manual accessibility and real-device acceptance remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2953,7 +2953,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 83 desktop/mobile Chromium cases pass and 1 planned skip. 101-route sweep has 0 issues. Parts Product schema, avatar lifecycle, account/dealer limits and 34-route accessibility audit pass; live/manual acceptance remains open.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 85 browser cases pass and 1 planned skip across desktop/mobile Chromium and iPhone WebKit smoke. 101-route sweep has 0 issues. Parts schema, avatar lifecycle, write limits and 34-route Chromium accessibility audit pass; live/manual acceptance remains open.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
@@ -10661,7 +10661,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 83 desktop/mobile Chromium passes and 1 planned skip. 101-route sweep has 0 issues; parts Product schema, avatar lifecycle, write-denial and 34-route accessibility audit pass in both viewports.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 85 browser passes and 1 planned skip. 101-route sweep has 0 issues; core Chromium journeys plus iPhone WebKit navigation/search/sign-in/photo-upload smoke pass. Real-device and direct-action negative matrices remain open.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Cover remaining direct-action and validation negatives; add Safari/mobile device and live staging acceptance.</x:v>
@@ -10687,7 +10687,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G182" s="137" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="H182" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10708,10 +10708,10 @@
         <x:v>Real/simulated devices; slow network</x:v>
       </x:c>
       <x:c r="N182" s="136" t="str">
-        <x:v>Simulated Android Chromium passes search, sign-in, dealer registration, all three listing publications, photo upload, phone reveal, moderation and viewport width.</x:v>
+        <x:v>Simulated Android Chromium covers core seller, dealer, buyer and admin journeys. Added iPhone 13 WebKit smoke checks for mobile navigation, auto-parts search, responsive width, sign-in and car-photo upload; both pass in fresh isolated acceptance. Local HTTP production-mode WebKit needs a test-only session-cookie injection because Secure cookies require HTTPS. CI now installs WebKit alongside Chromium.</x:v>
       </x:c>
       <x:c r="O182" s="136" t="str">
-        <x:v>Add simulated Safari/iPhone and mobile keyboard/upload checks; real-device review remains parked.</x:v>
+        <x:v>Run real iPhone Safari and Android Chrome on HTTPS staging, including keyboard, camera/file picker, slow network and full posting/contact journeys; local WebKit smoke is not a real-device sign-off.</x:v>
       </x:c>
     </x:row>
     <x:row r="183">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6dce35a751643e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00d35e62c2394258"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1576224de5234e6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc19723a1944c4edd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13997,10 +13997,10 @@
         <x:v>Visual regression</x:v>
       </x:c>
       <x:c r="E45" s="141" t="str">
-        <x:v>Owner visual review plus Playwright mobile width check</x:v>
+        <x:v>Owner homepage review; desktop/mobile Chromium responsive checks; iPhone 13 WebKit navigation, search, width, sign-in and photo-upload smoke</x:v>
       </x:c>
       <x:c r="F45" s="141" t="str">
-        <x:v>Partial pass: approved homepage; mobile width passes; Safari/cross-route QA pending</x:v>
+        <x:v>Partial pass: Chromium and simulated WebKit smoke have no viewport overflow; real Safari/iPhone, camera/keyboard and broader staging QA remain open</x:v>
       </x:c>
       <x:c r="G45" s="141" t="str">
         <x:v>PR #2 local preview</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re15be31192e94e5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16b06ea4542640fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc4a4c3aaae9421e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R205bdaefc1824b85"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Verify cross-user sold and delete action denial
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8ed0eb17e8594175"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R04541f9624524d36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R2b6e7f29dbbb4ce4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R3df7e105541342d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R63fb03dcbdba4103"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rcb44fa3772bb4322"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rb6be661385ac4feb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R875ead88663a476d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R3b2925ec76354a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R89e9025b5c174ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R26835d4842e14d3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R9734a716b369401e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Re4b40b73c96a4e50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rf1482c56fb54411a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6072e333726747df"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0d9ada7319c040dc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8963681592039803</x:v>
+        <x:v>0.8965174129353236</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1617,7 +1617,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B24" s="115" t="str">
-        <x:v>Homepage review and merge — completed</x:v>
+        <x:v>Homepage review and merge - completed</x:v>
       </x:c>
       <x:c r="C24" s="107" t="str">
         <x:v>PR #5 reviewed and merged into main on 30 Sep 2026 (merge c1ef18d).</x:v>
@@ -1635,10 +1635,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B25" s="117" t="str">
-        <x:v>Stage 6.2 CI and acceptance — in progress</x:v>
+        <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: fresh isolated DB, 101-route sweep 0 issues, 85 browser tests pass (1 planned skip), including two iPhone WebKit smoke cases. Parts schema, avatar lifecycle, write limits and 34-route Chromium accessibility scan pass; live staging/real-device acceptance remains open.</x:v>
+        <x:v>PR #6: 87 local browser passes, 1 planned skip, 4 DB checks and 101-route sweep with 0 issues. Cross-user sold/delete replay passes. GitHub run 34 passed on rerun; the new test commit still needs CI. Live staging and real-device acceptance remain open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1674,7 +1674,7 @@
         <x:v>Complete remaining launch acceptance</x:v>
       </x:c>
       <x:c r="C27" s="110" t="str">
-        <x:v>Automate registration, listing submission/contact, dealer registration, moderation mutations and Safari mobile; verify live provider integrations.</x:v>
+        <x:v>Complete direct edit/media/admin denial tests, real-device and manual accessibility review, then validate live providers and production infrastructure.</x:v>
       </x:c>
       <x:c r="D27" s="88"/>
       <x:c r="E27" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4de7b0f3baac4a34"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R869a56cf97484cce"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: repeatable isolated DB, 85 browser passes across Chromium and iPhone WebKit smoke, 1 planned skip and 101-route sweep 0 issues. Regression checklist records evidence and blockers. Online staging, providers, proxy validation, cron schedule, branch protection, manual accessibility and real-device acceptance remain open.</x:v>
+        <x:v>Stage 6.2 PR #6: local isolated DB has 87 browser passes, 1 planned skip, 4 DB checks and 101-route sweep with 0 issues. Direct sold/delete replay is denied across users. GitHub run 34 passed on attempt 2; the new test commit awaits CI. Staging, providers, proxy/cron checks, branch protection and manual/real-device acceptance remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2718,7 +2718,7 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>PR #6 CI passes migrations, seed, DB tests, checks, lint, build, sweep and Chromium. Production dependency audit added as a blocking job step.</x:v>
+        <x:v>GitHub run 34 on 4f019d3 passes migrations, seed, DB checks, static checks, lint, build, sweep, Chromium/WebKit and production dependency audit on attempt 2. Attempt 1 had a missing ReportListing client manifest entry; the unchanged commit passed on rerun. New direct-action cases have local evidence; their pushed-commit CI must also pass.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
         <x:v>Mark check required in branch protection and demonstrate deliberate failure blocks merge.</x:v>
@@ -2953,7 +2953,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 85 browser cases pass and 1 planned skip across desktop/mobile Chromium and iPhone WebKit smoke. 101-route sweep has 0 issues. Parts schema, avatar lifecycle, write limits and 34-route Chromium accessibility audit pass; live/manual acceptance remains open.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 87 browser passes and 1 planned skip across desktop/mobile Chromium and iPhone WebKit smoke. 101-route sweep has 0 issues. Direct cross-user sold/delete requests preserve the target listing; live/manual acceptance remains open.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
@@ -10123,7 +10123,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G170" s="137" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.93</x:v>
       </x:c>
       <x:c r="H170" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10144,10 +10144,10 @@
         <x:v>IDOR; direct action calls; cross-user access</x:v>
       </x:c>
       <x:c r="N170" s="136" t="str">
-        <x:v>Server ownership checks now have desktop/mobile browser coverage: another seller receives rendered not-found page and no edit controls; owner can edit price and delete own bike, with DB/media/public URL cleanup. Remaining direct-action IDOR matrix is open.</x:v>
+        <x:v>Desktop/mobile Chromium now captures valid owner sold/delete server-action requests and replays them with a different seller session. Both actions leave the disposable listing active and undeleted. Cross-user edit-page denial and owner edit/delete success also pass. Direct edit, media and administrator denial matrices remain open.</x:v>
       </x:c>
       <x:c r="O170" s="136" t="str">
-        <x:v>Cover direct cross-user action calls and private media references across remaining modules.</x:v>
+        <x:v>Extend direct action denial to listing edits, upload attachment, administrator mutations and private media references.</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -10661,7 +10661,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 85 browser passes and 1 planned skip. 101-route sweep has 0 issues; core Chromium journeys plus iPhone WebKit navigation/search/sign-in/photo-upload smoke pass. Real-device and direct-action negative matrices remain open.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 87 browser passes and 1 planned skip. 101-route sweep has 0 issues. Cross-user sold/delete request replay joins core Chromium journeys and iPhone WebKit smoke. Direct edit/media/admin negatives and real-device acceptance remain open.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Cover remaining direct-action and validation negatives; add Safari/mobile device and live staging acceptance.</x:v>
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00d35e62c2394258"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R877d7da394204aba"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc19723a1944c4edd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdc830ee7e3043b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13087,10 +13087,10 @@
         <x:v>Security integration</x:v>
       </x:c>
       <x:c r="E10" s="141" t="str">
-        <x:v>Automated feature checks plus desktop/mobile Chromium cross-user edit-page denial</x:v>
+        <x:v>Desktop/mobile Chromium cross-user edit-page denial plus captured sold/delete server-action replay with another seller session</x:v>
       </x:c>
       <x:c r="F10" s="141" t="str">
-        <x:v>Partial pass: rendered not-found and no edit controls for another seller; direct action/media IDOR cases remain</x:v>
+        <x:v>Partial pass: another seller cannot open edit controls, mark sold or delete the target listing; direct edit/media/admin cases remain</x:v>
       </x:c>
       <x:c r="G10" s="141" t="str">
         <x:v>Two users with listings/uploads</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16b06ea4542640fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R910ed285e359446c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R205bdaefc1824b85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49f68ea4c5374f6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Verify action roles and transactional upload ownership
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R875ead88663a476d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R3b2925ec76354a60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R89e9025b5c174ca1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R26835d4842e14d3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R9734a716b369401e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Re4b40b73c96a4e50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rf1482c56fb54411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc32db3bfb7814e4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R499e60f14d4b46fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Re8dc22b92c064f4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R750cbeb333f14e58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rdef71ac6055841fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R96888cd6921d45be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R38fa10758db1433c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0d9ada7319c040dc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbce24f59a29c460b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1397,7 +1397,7 @@
       </x:c>
       <x:c r="B11" s="101" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8965174129353236</x:v>
+        <x:v>0.8974129353233832</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: 87 local browser passes, 1 planned skip, 4 DB checks and 101-route sweep with 0 issues. Cross-user sold/delete replay passes. GitHub run 34 passed on rerun; the new test commit still needs CI. Live staging and real-device acceptance remain open.</x:v>
+        <x:v>PR #6: 91 local browser passes, 1 planned skip, 5 DB checks and 101-route sweep with 0 issues. Owner/admin direct requests and upload-claim rollback are covered. Prior GitHub run 35 passed; current PR checks govern new commits. Live staging and real-device acceptance remain open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1674,7 +1674,7 @@
         <x:v>Complete remaining launch acceptance</x:v>
       </x:c>
       <x:c r="C27" s="110" t="str">
-        <x:v>Complete direct edit/media/admin denial tests, real-device and manual accessibility review, then validate live providers and production infrastructure.</x:v>
+        <x:v>Finish private-media/upload and dealer/service authorization cases, controlled failure recovery and performance/load checks; then complete live providers and real-device review.</x:v>
       </x:c>
       <x:c r="D27" s="88"/>
       <x:c r="E27" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R869a56cf97484cce"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref08f4bcbc104935"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: local isolated DB has 87 browser passes, 1 planned skip, 4 DB checks and 101-route sweep with 0 issues. Direct sold/delete replay is denied across users. GitHub run 34 passed on attempt 2; the new test commit awaits CI. Staging, providers, proxy/cron checks, branch protection and manual/real-device acceptance remain open.</x:v>
+        <x:v>Stage 6.2 PR #6: fresh local acceptance has 91 browser passes, 1 planned skip, 5 DB checks and 101-route sweep with 0 issues. Direct owner/admin permissions and upload-claim rollback are verified. Staging, providers, proxy/cron checks, branch protection, performance/load and manual/real-device acceptance remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2718,7 +2718,7 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>GitHub run 34 on 4f019d3 passes migrations, seed, DB checks, static checks, lint, build, sweep, Chromium/WebKit and production dependency audit on attempt 2. Attempt 1 had a missing ReportListing client manifest entry; the unchanged commit passed on rerun. New direct-action cases have local evidence; their pushed-commit CI must also pass.</x:v>
+        <x:v>GitHub run 35 on a739bcf passed migration, seed, DB checks, static checks, lint, build, sweep, Chromium/WebKit and production dependency audit. The preceding run 34 recovered from a client-manifest error on an unchanged-commit rerun. Current PR checks are authoritative for later commits; branch protection remains unverified.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
         <x:v>Mark check required in branch protection and demonstrate deliberate failure blocks merge.</x:v>
@@ -2885,7 +2885,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G16" s="137" t="n">
-        <x:v>0.45</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="H16" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2906,10 +2906,10 @@
         <x:v>Unit; integration; transaction tests</x:v>
       </x:c>
       <x:c r="N16" s="136" t="str">
-        <x:v>Node test runner validates seeded reference data, all three inventory verticals and taxonomy facet integrity on isolated PostgreSQL.</x:v>
+        <x:v>Five isolated PostgreSQL checks cover migrations/reference data, all inventory verticals, facet integrity, atomic rate limits and real upload-claim transactions. A mixed own/foreign upload batch rolls back all claims; duplicate keys and reuse fail, while a valid owner claim succeeds.</x:v>
       </x:c>
       <x:c r="O16" s="136" t="str">
-        <x:v>Add transactional success/validation/authorization/rollback tests for critical actions.</x:v>
+        <x:v>Extend transaction rollback and concurrency checks to publication, edits, moderation and service-request updates.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2953,7 +2953,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 87 browser passes and 1 planned skip across desktop/mobile Chromium and iPhone WebKit smoke. 101-route sweep has 0 issues. Direct cross-user sold/delete requests preserve the target listing; live/manual acceptance remains open.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 5 DB checks, 91 browser passes and 1 planned skip across desktop/mobile Chromium and iPhone WebKit smoke. 101-route sweep has 0 issues. Direct edit/sold/delete and admin denial include valid-session positive controls; live/manual acceptance remains open.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
@@ -10123,7 +10123,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G170" s="137" t="n">
-        <x:v>0.93</x:v>
+        <x:v>0.96</x:v>
       </x:c>
       <x:c r="H170" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10144,10 +10144,10 @@
         <x:v>IDOR; direct action calls; cross-user access</x:v>
       </x:c>
       <x:c r="N170" s="136" t="str">
-        <x:v>Desktop/mobile Chromium now captures valid owner sold/delete server-action requests and replays them with a different seller session. Both actions leave the disposable listing active and undeleted. Cross-user edit-page denial and owner edit/delete success also pass. Direct edit, media and administrator denial matrices remain open.</x:v>
+        <x:v>Desktop/mobile direct requests enforce ownership for edit, sold and delete; seller and anonymous requests cannot hide/remove listings or ban users. Database rows, photos and audit history stay unchanged on denial. Identical requests succeed with owner/admin sessions. Tests explicitly carry current cookies on local HTTP and wait for intercepted requests to abort before replay.</x:v>
       </x:c>
       <x:c r="O170" s="136" t="str">
-        <x:v>Extend direct action denial to listing edits, upload attachment, administrator mutations and private media references.</x:v>
+        <x:v>Cover HTTP upload-key attachment and private media reads, plus direct dealer and service-request mutations; complete live staging review.</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -10661,10 +10661,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 4 DB checks, 87 browser passes and 1 planned skip. 101-route sweep has 0 issues. Cross-user sold/delete request replay joins core Chromium journeys and iPhone WebKit smoke. Direct edit/media/admin negatives and real-device acceptance remain open.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 5 DB checks, 91 browser passes and 1 planned skip; 101-route sweep has 0 issues. Direct owner/admin action replay and upload-claim rollback join core marketplace, accessibility and WebKit smoke coverage.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Cover remaining direct-action and validation negatives; add Safari/mobile device and live staging acceptance.</x:v>
+        <x:v>Complete HTTP upload attachment, private-media and remaining dealer/service mutation negatives, then real-device and live-provider acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R877d7da394204aba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d409afd307f4953"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdc830ee7e3043b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd385c2e5528b44be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13087,10 +13087,10 @@
         <x:v>Security integration</x:v>
       </x:c>
       <x:c r="E10" s="141" t="str">
-        <x:v>Desktop/mobile Chromium cross-user edit-page denial plus captured sold/delete server-action replay with another seller session</x:v>
+        <x:v>Desktop/mobile direct edit, sold and delete replay with explicit actor sessions, plus matching owner success controls</x:v>
       </x:c>
       <x:c r="F10" s="141" t="str">
-        <x:v>Partial pass: another seller cannot open edit controls, mark sold or delete the target listing; direct edit/media/admin cases remain</x:v>
+        <x:v>Partial pass: unauthorized listing writes preserve data/photos; identical owner requests succeed. Private media reads and HTTP attachment cases remain.</x:v>
       </x:c>
       <x:c r="G10" s="141" t="str">
         <x:v>Two users with listings/uploads</x:v>
@@ -13399,10 +13399,10 @@
         <x:v>Security integration</x:v>
       </x:c>
       <x:c r="E22" s="141" t="str">
-        <x:v>Automated checks</x:v>
+        <x:v>Isolated PostgreSQL integration test of real upload-claim transactions: mixed ownership, duplicate/reused keys, valid owner claim</x:v>
       </x:c>
       <x:c r="F22" s="141" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Partial pass: foreign batch fails and rolls back the valid key; duplicates/reuse fail; owner claim succeeds. HTTP publication/edit attachment negative tests remain.</x:v>
       </x:c>
       <x:c r="G22" s="141" t="str">
         <x:v>Ownership binding implemented</x:v>
@@ -13945,10 +13945,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E43" s="141" t="str">
-        <x:v>Desktop/mobile Chromium admin approve, hide, reinstate and permanent removal; DB audit and public visibility</x:v>
+        <x:v>Desktop/mobile admin mutation success plus direct flag/remove replay by seller and anonymous visitor; database and audit assertions</x:v>
       </x:c>
       <x:c r="F43" s="141" t="str">
-        <x:v>Partial pass: moderation status/audit/visibility verified; reports and direct non-admin denial remain open</x:v>
+        <x:v>Local pass: unauthorized requests redirect without listing/audit changes; identical administrator requests hide/remove and append audit entries. Live acceptance remains.</x:v>
       </x:c>
       <x:c r="G43" s="141" t="str">
         <x:v>Reported/flagged listings</x:v>
@@ -13971,10 +13971,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E44" s="141" t="str">
-        <x:v>Desktop/mobile Chromium ban, session revocation, unban, audit history and restored login</x:v>
+        <x:v>Desktop/mobile ban/unban/session-revocation flow plus direct ban replay denied to seller/anonymous visitors with admin success control</x:v>
       </x:c>
       <x:c r="F44" s="141" t="str">
-        <x:v>Passed browser lifecycle and DB enforcement; retain direct-action authorization in security regression</x:v>
+        <x:v>Local pass: unauthorized ban leaves account/audit unchanged; admin ban succeeds and is audited. Live acceptance remains.</x:v>
       </x:c>
       <x:c r="G44" s="141" t="str">
         <x:v>User admin complete</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R910ed285e359446c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd20d86614e9b4916"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49f68ea4c5374f6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2d5c3ce97f549ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Protect local private media and verify photo attachment ownership
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc32db3bfb7814e4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R499e60f14d4b46fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Re8dc22b92c064f4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R750cbeb333f14e58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rdef71ac6055841fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R96888cd6921d45be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R38fa10758db1433c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R48914c09a22847db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rbe9a9efb0a084b56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R50a83d8642934fc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rcc14377553da454a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R553c7035dea64708"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R3bce93717e5b47d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rad68670e62ee4f74"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -888,7 +888,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbce24f59a29c460b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R772039b2c81149ce"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1638,7 +1638,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: 91 local browser passes, 1 planned skip, 5 DB checks and 101-route sweep with 0 issues. Owner/admin direct requests and upload-claim rollback are covered. Prior GitHub run 35 passed; current PR checks govern new commits. Live staging and real-device acceptance remain open.</x:v>
+        <x:v>PR #6: 93 local browser passes, 1 planned skip, 5 DB checks and 101-route sweep with 0 issues. Local photo privacy and foreign publish/edit attachment tests pass. Prior GitHub run 36 passed; current PR checks govern new commits. Live staging remains open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1674,7 +1674,7 @@
         <x:v>Complete remaining launch acceptance</x:v>
       </x:c>
       <x:c r="C27" s="110" t="str">
-        <x:v>Finish private-media/upload and dealer/service authorization cases, controlled failure recovery and performance/load checks; then complete live providers and real-device review.</x:v>
+        <x:v>Next: dealer/service authorization, controlled failure recovery and performance/load. Cloudflare private delivery, live providers and real-device review remain launch gates.</x:v>
       </x:c>
       <x:c r="D27" s="88"/>
       <x:c r="E27" s="88"/>
@@ -1773,7 +1773,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref08f4bcbc104935"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc39dbb8c584467d"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1880,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: fresh local acceptance has 91 browser passes, 1 planned skip, 5 DB checks and 101-route sweep with 0 issues. Direct owner/admin permissions and upload-claim rollback are verified. Staging, providers, proxy/cron checks, branch protection, performance/load and manual/real-device acceptance remain open.</x:v>
+        <x:v>Stage 6.2 PR #6: 93 local browser passes, 1 planned skip, 5 DB checks and 101-route sweep with 0 issues. Local media access and cross-user HTTP attachment verified. Cloudflare private delivery, staging, providers, proxy/cron, branch protection, performance/load and manual acceptance remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2718,7 +2718,7 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>GitHub run 35 on a739bcf passed migration, seed, DB checks, static checks, lint, build, sweep, Chromium/WebKit and production dependency audit. The preceding run 34 recovered from a client-manifest error on an unchanged-commit rerun. Current PR checks are authoritative for later commits; branch protection remains unverified.</x:v>
+        <x:v>GitHub run 36 on b32d457 passed all gates, including two-worker Chromium/WebKit acceptance. Current PR checks are authoritative for later commits; branch protection remains unverified.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
         <x:v>Mark check required in branch protection and demonstrate deliberate failure blocks merge.</x:v>
@@ -2953,7 +2953,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 5 DB checks, 91 browser passes and 1 planned skip across desktop/mobile Chromium and iPhone WebKit smoke. 101-route sweep has 0 issues. Direct edit/sold/delete and admin denial include valid-session positive controls; live/manual acceptance remains open.</x:v>
+        <x:v>Fresh isolated PostgreSQL acceptance: 5 DB checks, 93 browser passes and 1 planned skip across desktop/mobile Chromium and iPhone WebKit; 101-route sweep has 0 issues. Local media read authorization and HTTP foreign-photo attachment join prior owner/admin checks. Live/manual acceptance remains open.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
@@ -10144,10 +10144,10 @@
         <x:v>IDOR; direct action calls; cross-user access</x:v>
       </x:c>
       <x:c r="N170" s="136" t="str">
-        <x:v>Desktop/mobile direct requests enforce ownership for edit, sold and delete; seller and anonymous requests cannot hide/remove listings or ban users. Database rows, photos and audit history stay unchanged on denial. Identical requests succeed with owner/admin sessions. Tests explicitly carry current cookies on local HTTP and wait for intercepted requests to abort before replay.</x:v>
+        <x:v>Local photo GET/HEAD authorization now enforces listing visibility and pending-upload ownership, with owner/admin controls, no-store responses, blocked optimizer access and storage outside public/. Desktop/mobile HTTP publish/edit reject foreign photo keys without changing listing images; valid-owner replays pass. Legacy development photo compatibility is preserved.</x:v>
       </x:c>
       <x:c r="O170" s="136" t="str">
-        <x:v>Cover HTTP upload-key attachment and private media reads, plus direct dealer and service-request mutations; complete live staging review.</x:v>
+        <x:v>Complete dealer/service direct-mutation negatives. Cloudflare private/signed delivery implementation and live provider acceptance remain a launch gate; local media authorization does not protect direct Cloudflare URLs.</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -10661,10 +10661,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 5 DB checks, 91 browser passes and 1 planned skip; 101-route sweep has 0 issues. Direct owner/admin action replay and upload-claim rollback join core marketplace, accessibility and WebKit smoke coverage.</x:v>
+        <x:v>Local acceptance: 93 browser passes, 1 planned skip, 5 DB checks and 101-route sweep with 0 issues. Private local image GET/HEAD, optimizer denial, owner previews and foreign publish/edit photo keys are covered with positive controls.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Complete HTTP upload attachment, private-media and remaining dealer/service mutation negatives, then real-device and live-provider acceptance.</x:v>
+        <x:v>Complete dealer/service mutation negatives, controlled failure recovery and performance/load checks; Cloudflare private delivery and live/real-device acceptance remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -12309,7 +12309,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d409afd307f4953"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R515b95f34cd64dc5"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12864,7 +12864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd385c2e5528b44be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4f2b0ad305e48dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13087,10 +13087,10 @@
         <x:v>Security integration</x:v>
       </x:c>
       <x:c r="E10" s="141" t="str">
-        <x:v>Desktop/mobile direct edit, sold and delete replay with explicit actor sessions, plus matching owner success controls</x:v>
+        <x:v>Desktop/mobile direct listing actions plus local image GET/HEAD checks for pending, active and all inactive statuses; owner/admin success, foreign/anonymous denial and optimizer rejection</x:v>
       </x:c>
       <x:c r="F10" s="141" t="str">
-        <x:v>Partial pass: unauthorized listing writes preserve data/photos; identical owner requests succeed. Private media reads and HTTP attachment cases remain.</x:v>
+        <x:v>Local pass: private reads denied, active photos public, owner edit preview loads, no-store headers verified. Cloudflare private delivery remains pending.</x:v>
       </x:c>
       <x:c r="G10" s="141" t="str">
         <x:v>Two users with listings/uploads</x:v>
@@ -13399,10 +13399,10 @@
         <x:v>Security integration</x:v>
       </x:c>
       <x:c r="E22" s="141" t="str">
-        <x:v>Isolated PostgreSQL integration test of real upload-claim transactions: mixed ownership, duplicate/reused keys, valid owner claim</x:v>
+        <x:v>Real database rollback and desktop/mobile captured publish/edit HTTP requests replayed with another user's unclaimed key, followed by valid-owner positive controls</x:v>
       </x:c>
       <x:c r="F22" s="141" t="str">
-        <x:v>Partial pass: foreign batch fails and rolls back the valid key; duplicates/reuse fail; owner claim succeeds. HTTP publication/edit attachment negative tests remain.</x:v>
+        <x:v>Local pass: foreign publish creates no listing or claim; foreign edit preserves listing images; original owner payload succeeds. Production/provider acceptance remains.</x:v>
       </x:c>
       <x:c r="G22" s="141" t="str">
         <x:v>Ownership binding implemented</x:v>
@@ -14432,7 +14432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd20d86614e9b4916"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72de2db063214171"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14658,7 +14658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2d5c3ce97f549ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14d019580dd940a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Reconcile tracker progress and current acceptance evidence
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R48914c09a22847db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rbe9a9efb0a084b56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R50a83d8642934fc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rcc14377553da454a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R553c7035dea64708"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R3bce93717e5b47d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rad68670e62ee4f74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdb392ab5d74b4487"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R9e04d7112b764be9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rda246002cd7f40b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R2424cffe62d245a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rdb487aa56ef9452a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rc20d3f9971c941b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rbbcb403f7f8f4ce0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,8 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="0%"/>
+    <x:numFmt numFmtId="201" formatCode="0.0%"/>
   </x:numFmts>
   <x:fonts count="28">
     <x:font>
@@ -326,7 +327,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="142">
+  <x:cellXfs count="143">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -659,6 +660,7 @@
     <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="19" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -888,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R772039b2c81149ce"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8c7219f423794af3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1173,7 +1175,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="86" t="str">
-        <x:v>JaniWheels V1 Development Control Sheet</x:v>
+        <x:v>JaniWheels V1 Development Control Sheet — 3 October 2026</x:v>
       </x:c>
       <x:c r="B1" s="86"/>
       <x:c r="C1" s="86"/>
@@ -1187,7 +1189,7 @@
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="87" t="str">
-        <x:v>Use the Feature Tracker as the source of truth. Update Status, Completion, Priority, Owner and Next Action after each tested feature branch.</x:v>
+        <x:v>Completion is the equal-weight average of in-scope feature estimates, not effort spent or launch approval. Evidence, remaining gates and next actions are recorded in Feature Tracker.</x:v>
       </x:c>
       <x:c r="B2" s="87"/>
       <x:c r="C2" s="87"/>
@@ -1229,13 +1231,13 @@
       <x:c r="I4" s="89"/>
       <x:c r="J4" s="89"/>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="16.799999237060547" hidden="0" customHeight="1">
       <x:c r="A5" s="90" t="str">
         <x:v>In-scope feature rows</x:v>
       </x:c>
       <x:c r="B5" s="91" t="n">
-        <x:f>COUNTIFS('Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")</x:f>
-        <x:v>201</x:v>
+        <x:f>COUNTIFS('Feature Tracker'!$A$5:$A$215,"&lt;&gt;",'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request",'Feature Tracker'!$F$5:$F$215,"&lt;&gt;Out of Scope / Removed")</x:f>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="C5" s="88"/>
       <x:c r="D5" s="92" t="str">
@@ -1245,18 +1247,18 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F5" s="94" t="str">
-        <x:v>Full project check passed 30 Sep 2026</x:v>
+        <x:v>Passed on a96704b; CI run 37</x:v>
       </x:c>
       <x:c r="G5" s="92" t="str">
         <x:v>Current branch</x:v>
       </x:c>
       <x:c r="H5" s="93" t="str">
-        <x:v>codex/homepage-visuals (pushed)</x:v>
+        <x:v>codex/launch-quality-system; a96704b pushed</x:v>
       </x:c>
       <x:c r="I5" s="93"/>
       <x:c r="J5" s="94"/>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="16.799999237060547" hidden="0" customHeight="1">
       <x:c r="A6" s="95" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -1272,24 +1274,24 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F6" s="99" t="str">
-        <x:v>Zero warnings/errors on 30 Sep 2026</x:v>
+        <x:v>No warnings/errors; CI run 37</x:v>
       </x:c>
       <x:c r="G6" s="97" t="str">
-        <x:v>Stage 6.1</x:v>
+        <x:v>Current stage</x:v>
       </x:c>
       <x:c r="H6" s="98" t="str">
-        <x:v>Homepage visuals approved and pushed</x:v>
+        <x:v>Homepage merged via PR #5; Stage 6.2 active</x:v>
       </x:c>
       <x:c r="I6" s="98"/>
       <x:c r="J6" s="99"/>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A7" s="95" t="str">
         <x:v>Feature branch review</x:v>
       </x:c>
       <x:c r="B7" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Complete on Feature Branch - Awaiting Review")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="88"/>
       <x:c r="D7" s="97" t="str">
@@ -1299,24 +1301,24 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F7" s="99" t="str">
-        <x:v>12/12 checks + local signup success</x:v>
+        <x:v>Local signup/checks pass; live provider review open</x:v>
       </x:c>
       <x:c r="G7" s="97" t="str">
-        <x:v>Legal/content</x:v>
+        <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>936baee on origin/codex/homepage-visuals</x:v>
+        <x:v>PR #6 open; GitHub run 37 passed</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A8" s="95" t="str">
-        <x:v>Partially/Data layer</x:v>
+        <x:v>Partial / configuration</x:v>
       </x:c>
       <x:c r="B8" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>32</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C8" s="88"/>
       <x:c r="D8" s="97" t="str">
@@ -1326,18 +1328,18 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F8" s="99" t="str">
-        <x:v>15.5.26 build:safe passed 30 Sep; max First Load JS 128 kB; production audit zero vulnerabilities</x:v>
+        <x:v>Final build passed; max First Load JS 128 KB</x:v>
       </x:c>
       <x:c r="G8" s="97" t="str">
         <x:v>Next functionality</x:v>
       </x:c>
       <x:c r="H8" s="98" t="str">
-        <x:v>Persistent staging, required CI check and monitoring</x:v>
+        <x:v>Dealer/service negatives and controlled failure recovery</x:v>
       </x:c>
       <x:c r="I8" s="98"/>
       <x:c r="J8" s="99"/>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A9" s="95" t="str">
         <x:v>Requires correction</x:v>
       </x:c>
@@ -1350,37 +1352,37 @@
         <x:v>Database acceptance</x:v>
       </x:c>
       <x:c r="E9" s="98" t="str">
-        <x:v>Ongoing</x:v>
+        <x:v>Local passed</x:v>
       </x:c>
       <x:c r="F9" s="99" t="str">
-        <x:v>Run alongside each package</x:v>
+        <x:v>5 DB checks; live deployment acceptance open</x:v>
       </x:c>
       <x:c r="G9" s="97" t="str">
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Authenticated and populated browser/DB acceptance pending</x:v>
+        <x:v>93 local passes, 1 planned skip; real-device QA open</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A10" s="95" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="B10" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C10" s="88"/>
       <x:c r="D10" s="97" t="str">
         <x:v>Responsive/branding</x:v>
       </x:c>
       <x:c r="E10" s="98" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Partial pass</x:v>
       </x:c>
       <x:c r="F10" s="99" t="str">
-        <x:v>Shell checks pass; visual and accessibility acceptance pending</x:v>
+        <x:v>Owner homepage review + automated axe/viewport; manual review open</x:v>
       </x:c>
       <x:c r="G10" s="97" t="str">
         <x:v>Google Maps</x:v>
@@ -1391,29 +1393,29 @@
       <x:c r="I10" s="98"/>
       <x:c r="J10" s="99"/>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A11" s="100" t="str">
-        <x:v>Weighted completion</x:v>
-      </x:c>
-      <x:c r="B11" s="101" t="n">
-        <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request")/B5</x:f>
-        <x:v>0.8974129353233832</x:v>
+        <x:v>Overall completion</x:v>
+      </x:c>
+      <x:c r="B11" s="142" t="n">
+        <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request",'Feature Tracker'!$F$5:$F$215,"&lt;&gt;Out of Scope / Removed")/B5</x:f>
+        <x:v>0.9058500000000003</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
         <x:v>Security/load</x:v>
       </x:c>
       <x:c r="E11" s="103" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partial pass</x:v>
       </x:c>
       <x:c r="F11" s="104" t="str">
-        <x:v>Final hardening gate</x:v>
+        <x:v>Local security checks pass; formal review/load open</x:v>
       </x:c>
       <x:c r="G11" s="102" t="str">
         <x:v>Final QA blocker</x:v>
       </x:c>
       <x:c r="H11" s="103" t="str">
-        <x:v>Enable billing and verify live maps</x:v>
+        <x:v>Hosting/providers, Cloudflare privacy, load and final acceptance</x:v>
       </x:c>
       <x:c r="I11" s="103"/>
       <x:c r="J11" s="104"/>
@@ -1469,7 +1471,7 @@
         <x:v>154</x:v>
       </x:c>
       <x:c r="C15" s="107" t="str">
-        <x:v>Implemented in current code and functionally available</x:v>
+        <x:v>Implemented and available in current code; does not mean production launch approval</x:v>
       </x:c>
       <x:c r="D15" s="88"/>
       <x:c r="E15" s="88"/>
@@ -1485,10 +1487,10 @@
       </x:c>
       <x:c r="B16" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Complete on Feature Branch - Awaiting Review")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C16" s="110" t="str">
-        <x:v>Implemented in PR #2 but not yet merged</x:v>
+        <x:v>Implementation verified on feature branch; PR review/merge outstanding</x:v>
       </x:c>
       <x:c r="D16" s="88"/>
       <x:c r="E16" s="88"/>
@@ -1504,10 +1506,10 @@
       </x:c>
       <x:c r="B17" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>32</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C17" s="110" t="str">
-        <x:v>Foundation exists; end-to-end feature incomplete</x:v>
+        <x:v>Partly implemented or awaiting configuration/acceptance</x:v>
       </x:c>
       <x:c r="D17" s="88"/>
       <x:c r="E17" s="88"/>
@@ -1542,10 +1544,10 @@
       </x:c>
       <x:c r="B19" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C19" s="110" t="str">
-        <x:v>Not implemented</x:v>
+        <x:v>No implemented delivery for this feature; see row-specific prerequisites</x:v>
       </x:c>
       <x:c r="D19" s="88"/>
       <x:c r="E19" s="88"/>
@@ -1638,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: 93 local browser passes, 1 planned skip, 5 DB checks and 101-route sweep with 0 issues. Local photo privacy and foreign publish/edit attachment tests pass. Prior GitHub run 36 passed; current PR checks govern new commits. Live staging remains open.</x:v>
+        <x:v>PR #6: a96704b passed GitHub run 37. Local suite: 93 browser passes, 1 planned skip, 5 DB checks and 101 routes clean; final media recheck: 2 cases and 103 routes clean. Persistent staging remains open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1728,7 +1730,7 @@
         <x:v>Final browser acceptance</x:v>
       </x:c>
       <x:c r="C30" s="110" t="str">
-        <x:v>Execute all critical journeys end to end after functionality completion.</x:v>
+        <x:v>Complete remaining negative/failure cases and live provider/real-device journeys using the regression checklist. Core local browser suite already passes.</x:v>
       </x:c>
       <x:c r="D30" s="88"/>
       <x:c r="E30" s="88"/>
@@ -1773,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc39dbb8c584467d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6a3a37015154bf3"/>
 </x:worksheet>
 </file>
 
@@ -1880,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Stage 6.2 PR #6: 93 local browser passes, 1 planned skip, 5 DB checks and 101-route sweep with 0 issues. Local media access and cross-user HTTP attachment verified. Cloudflare private delivery, staging, providers, proxy/cron, branch protection, performance/load and manual acceptance remain open.</x:v>
+        <x:v>Reconciled 3 Oct 2026 against a96704b and successful GitHub run 37. Local acceptance: 93 browser passes, 1 planned skip, 5 DB checks; 101-route clean sweep and final 103-route media recheck. Framework complete pending PR #6 review; production gates remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2078,7 +2080,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B27" s="124" t="str">
-        <x:v>Update Status, Completion %, Evidence / Current State, Next Action and Owner on the same feature row.</x:v>
+        <x:v>Review Status, Completion estimate, Evidence, Next Action and Owner after every verified package. Estimates reflect feature acceptance, not commit/test counts or elapsed effort. Dashboard uses an equal-weight average excluding removed scope.</x:v>
       </x:c>
       <x:c r="C27" s="124"/>
       <x:c r="D27" s="124"/>
@@ -2180,7 +2182,7 @@
         <x:v>Latest master</x:v>
       </x:c>
       <x:c r="B36" s="130" t="str">
-        <x:v>Future updates must replace the same Library file so its version history and identity remain intact.</x:v>
+        <x:v>Maintain the repository master at docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx. Older exported/Library copies may be stale; no automatic Library synchronization is claimed.</x:v>
       </x:c>
       <x:c r="C36" s="130"/>
       <x:c r="D36" s="130"/>
@@ -2612,7 +2614,7 @@
         <x:v>Stage 0</x:v>
       </x:c>
       <x:c r="J10" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Backend</x:v>
       </x:c>
       <x:c r="K10" s="136" t="str">
         <x:v>Deployment decisions</x:v>
@@ -2624,10 +2626,10 @@
         <x:v>Boot with missing/valid variables; configuration audit</x:v>
       </x:c>
       <x:c r="N10" s="136" t="str">
-        <x:v>.env.example exists, but S3 variables are listed while S3 storage is not implemented.</x:v>
+        <x:v>Environment template now documents local/Cloudflare media and rejects unsupported provider values. a96704b moves local storage outside public/. The template still refers to a missing src/lib/env.ts and unused/future settings; comprehensive startup validation is not implemented.</x:v>
       </x:c>
       <x:c r="O10" s="136" t="str">
-        <x:v>Align the environment template with the selected production provider.</x:v>
+        <x:v>Audit documented variables against consumers and implement safe startup validation for required deployment settings.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2706,7 +2708,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J12" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>DevOps</x:v>
       </x:c>
       <x:c r="K12" s="136" t="str">
         <x:v>GitHub Actions</x:v>
@@ -2718,7 +2720,7 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>GitHub run 36 on b32d457 passed all gates, including two-worker Chromium/WebKit acceptance. Current PR checks are authoritative for later commits; branch protection remains unverified.</x:v>
+        <x:v>GitHub run 37 passed all quality/acceptance gates on a96704b: https://github.com/Tech-Orbit-Systems/JaniWheels/actions/runs/37035200489 . Branch protection and a deliberate failing-check merge block remain unverified.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
         <x:v>Mark check required in branch protection and demonstrate deliberate failure blocks merge.</x:v>
@@ -2859,10 +2861,10 @@
         <x:v>npm run sweep on every route-changing branch</x:v>
       </x:c>
       <x:c r="N15" s="136" t="str">
-        <x:v>scripts/sweep.ts covers principal route shapes.</x:v>
+        <x:v>Fresh isolated acceptance checks 101 URLs with zero issues. Final media rebuild follow-up checked 103 URLs with zero issues. GitHub run 37 passed on a96704b.</x:v>
       </x:c>
       <x:c r="O15" s="136" t="str">
-        <x:v>Extend as new routes are added.</x:v>
+        <x:v>Keep the sweep in CI and add routes as functionality grows.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2885,7 +2887,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G16" s="137" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="H16" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2894,7 +2896,7 @@
         <x:v>Stage 1</x:v>
       </x:c>
       <x:c r="J16" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="K16" s="136" t="str">
         <x:v>Test runner and isolated DB</x:v>
@@ -2906,7 +2908,7 @@
         <x:v>Unit; integration; transaction tests</x:v>
       </x:c>
       <x:c r="N16" s="136" t="str">
-        <x:v>Five isolated PostgreSQL checks cover migrations/reference data, all inventory verticals, facet integrity, atomic rate limits and real upload-claim transactions. A mixed own/foreign upload batch rolls back all claims; duplicate keys and reuse fail, while a valid owner claim succeeds.</x:v>
+        <x:v>Reviewed estimate 75%: automated framework and five isolated DB checks are operational, including concurrent rate limits and actual upload-claim rollback, duplicate/reuse/foreign-key denial. HTTP authorization suite also proves publish/edit denial and owner/admin success. Wider transaction failure/concurrency coverage is incomplete.</x:v>
       </x:c>
       <x:c r="O16" s="136" t="str">
         <x:v>Extend transaction rollback and concurrency checks to publication, edits, moderation and service-request updates.</x:v>
@@ -2929,10 +2931,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F17" s="136" t="str">
-        <x:v>Partially Implemented</x:v>
+        <x:v>Complete on Feature Branch - Awaiting Review</x:v>
       </x:c>
       <x:c r="G17" s="137" t="n">
-        <x:v>0.98</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H17" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2941,7 +2943,7 @@
         <x:v>Stage 1</x:v>
       </x:c>
       <x:c r="J17" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="K17" s="136" t="str">
         <x:v>Stable staging/test DB</x:v>
@@ -2953,10 +2955,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Fresh isolated PostgreSQL acceptance: 5 DB checks, 93 browser passes and 1 planned skip across desktop/mobile Chromium and iPhone WebKit; 101-route sweep has 0 issues. Local media read authorization and HTTP foreign-photo attachment join prior owner/admin checks. Live/manual acceptance remains open.</x:v>
+        <x:v>Framework acceptance criteria met on a96704b: isolated DB, desktop/mobile Chromium core journeys, iPhone WebKit smoke, 93 browser passes and one planned desktop-only skip; CI run 37 passed. PR #6 review remains open. Wider test coverage, real devices and deployment acceptance are separately tracked in JW-177/178/199.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Add remaining negative/direct-action authorization paths and final live device acceptance.</x:v>
+        <x:v>Review PR #6; retain regression coverage. Track additional cases in JW-177 rather than reopening the test-framework implementation.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -3966,7 +3968,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G39" s="137" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H39" s="136" t="str">
         <x:v>High</x:v>
@@ -3975,7 +3977,7 @@
         <x:v>Stage 0</x:v>
       </x:c>
       <x:c r="J39" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="K39" s="136" t="str">
         <x:v>Local branch preview</x:v>
@@ -3987,10 +3989,10 @@
         <x:v>1440, 1024, 768, 414, 390, 360 px</x:v>
       </x:c>
       <x:c r="N39" s="136" t="str">
-        <x:v>Owner approved homepage visual package and 936baee is pushed. Earlier 320px/1440px primary-route checks found no overflow; comprehensive cross-route responsive acceptance remains open.</x:v>
+        <x:v>Reviewed estimate 90%: owner-approved homepage merged via PR #5; automated desktop/mobile route checks and iPhone WebKit smoke pass, including overflow checks. Broader tablet, real-device, keyboard/camera and slow-network visual acceptance remains open.</x:v>
       </x:c>
       <x:c r="O39" s="136" t="str">
-        <x:v>Complete desktop/tablet/mobile visual acceptance across buyer, seller, dealer and admin flows.</x:v>
+        <x:v>Complete remaining tablet/real-device visual review and record issues by route.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -4081,10 +4083,10 @@
         <x:v>Valid; wrong password; unknown user; banned user</x:v>
       </x:c>
       <x:c r="N41" s="136" t="str">
-        <x:v>Implemented with dummy-hash timing protection.</x:v>
+        <x:v>Password login has timing protection and PostgreSQL rate limits. Desktop/mobile tests cover valid, invalid, banned and unverified accounts, retry limits and password-reset session revocation.</x:v>
       </x:c>
       <x:c r="O41" s="136" t="str">
-        <x:v>Add rate limiting and integration tests.</x:v>
+        <x:v>Retain CI regression; verify production cookie/origin/provider configuration at launch.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -4598,10 +4600,10 @@
         <x:v>Anonymous; normal user; admin; direct action call</x:v>
       </x:c>
       <x:c r="N52" s="136" t="str">
-        <x:v>Route and action both enforce admin access.</x:v>
+        <x:v>Administrator routes/actions check role. Direct hide/remove/ban HTTP replay rejects seller and anonymous actors without DB/audit changes; identical administrator payload succeeds. CI run 37 passed.</x:v>
       </x:c>
       <x:c r="O52" s="136" t="str">
-        <x:v>Add authorization integration tests.</x:v>
+        <x:v>Extend dealer/service direct-action authorization under JW-166; retain existing administrator regressions.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -4633,7 +4635,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J53" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Backend</x:v>
       </x:c>
       <x:c r="K53" s="136" t="str">
         <x:v>Production DB access</x:v>
@@ -4645,10 +4647,10 @@
         <x:v>Access test; audit review</x:v>
       </x:c>
       <x:c r="N53" s="136" t="str">
-        <x:v>Local admin was set manually; production admin not created.</x:v>
+        <x:v>Local administrator access exists. No dedicated bootstrap command or complete audited production-bootstrap runbook was found; production administrator creation remains open.</x:v>
       </x:c>
       <x:c r="O53" s="136" t="str">
-        <x:v>Create production runbook and initial admin at deployment.</x:v>
+        <x:v>Implement/document audited first-admin provisioning, then execute only against the chosen production environment.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -5846,7 +5848,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G79" s="137" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.85</x:v>
       </x:c>
       <x:c r="H79" s="136" t="str">
         <x:v>High</x:v>
@@ -5855,7 +5857,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J79" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Backend</x:v>
       </x:c>
       <x:c r="K79" s="136" t="str">
         <x:v>External cron scheduler</x:v>
@@ -5867,10 +5869,10 @@
         <x:v>TTL boundary; cron auth; search/detail behavior</x:v>
       </x:c>
       <x:c r="N79" s="136" t="str">
-        <x:v>Protected expire endpoint exists; scheduler and reactivation are missing.</x:v>
+        <x:v>Reviewed estimate 85%: protected expire-listings job and owner-only reactivateListingAction are implemented. Dashboard offers Reactivate for 30 days for sold/expired listings. Production scheduler, TTL boundary and full reactivation browser acceptance remain open.</x:v>
       </x:c>
       <x:c r="O79" s="136" t="str">
-        <x:v>Configure scheduler and define renewal flow.</x:v>
+        <x:v>Test expiry/reactivation boundaries and authorization; configure and monitor production scheduling under JW-197.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -6055,10 +6057,10 @@
         <x:v>9.9/10/10.1 MB; 29/30/31 files</x:v>
       </x:c>
       <x:c r="N83" s="136" t="str">
-        <x:v>Server and listing schema enforce limits.</x:v>
+        <x:v>API enforces per-file/count/content-length bounds and hourly user file/byte quotas; listing schema rejects excessive/duplicate keys. Browser request-bucket denial passes.</x:v>
       </x:c>
       <x:c r="O83" s="136" t="str">
-        <x:v>Add aggregate request-size protection.</x:v>
+        <x:v>Complete exact size/count and aggregate byte boundary tests in T-016; retain the implemented aggregate protection.</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -6102,10 +6104,10 @@
         <x:v>Key theft; cross-user attach; expired temp upload</x:v>
       </x:c>
       <x:c r="N84" s="136" t="str">
-        <x:v>Upload ownership controls were completed with the listing CRUD/security work.</x:v>
+        <x:v>Real DB transaction tests reject foreign, duplicate and reused keys. Desktop/mobile publish/edit HTTP replay with foreign photo keys is denied without listing/photo changes; valid owner controls succeed on a96704b.</x:v>
       </x:c>
       <x:c r="O84" s="136" t="str">
-        <x:v>Retain in final regression and comprehensive browser QA.</x:v>
+        <x:v>Retain passing ownership regressions; finish provider-specific private delivery under JW-083.</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -6196,10 +6198,10 @@
         <x:v>Absolute/relative path; restart; broken image sweep</x:v>
       </x:c>
       <x:c r="N86" s="136" t="str">
-        <x:v>UPLOAD_DIR fallback is implemented.</x:v>
+        <x:v>a96704b stores local media in absolute private .uploads; public/ storage is rejected. Existing development files were moved, legacy JPEG fixture decoding preserved, and local GET/HEAD ownership/status checks pass on desktop/mobile. No-store direct previews bypass the optimizer.</x:v>
       </x:c>
       <x:c r="O86" s="136" t="str">
-        <x:v>Keep local provider development-only.</x:v>
+        <x:v>Keep local provider development-only; follow migration guidance in docs/QUALITY.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -6231,7 +6233,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J87" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Backend</x:v>
       </x:c>
       <x:c r="K87" s="136" t="str">
         <x:v>Cloudflare credentials and delivery hash</x:v>
@@ -6243,10 +6245,10 @@
         <x:v>Upload/display/delete; credential failure; variants</x:v>
       </x:c>
       <x:c r="N87" s="136" t="str">
-        <x:v>Cloudflare upload/display/delete branches exist; public delivery provider and delivery hash are now explicit in the environment template. Local checks pass; staging provider credentials and live media acceptance remain open.</x:v>
+        <x:v>Cloudflare upload/delete adapter and direct delivery URLs exist. a96704b protects local reads only; Cloudflare private/signed delivery is not implemented or verified. Live upload/display/delete and configuration failure acceptance remain open.</x:v>
       </x:c>
       <x:c r="O87" s="136" t="str">
-        <x:v>Configure staging and complete end-to-end media tests.</x:v>
+        <x:v>Implement provider-appropriate private delivery before production use; configure staging and verify media lifecycle.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -6263,13 +6265,13 @@
         <x:v>R2/S3 storage option advertised in environment documentation</x:v>
       </x:c>
       <x:c r="E88" s="136" t="str">
-        <x:v>Signed V1</x:v>
+        <x:v>Excluded / Change Request</x:v>
       </x:c>
       <x:c r="F88" s="136" t="str">
         <x:v>Out of Scope / Removed</x:v>
       </x:c>
       <x:c r="G88" s="137" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H88" s="136" t="str">
         <x:v>High</x:v>
@@ -6290,10 +6292,10 @@
         <x:v>Upload/display/delete; URL generation</x:v>
       </x:c>
       <x:c r="N88" s="136" t="str">
-        <x:v>Unsupported S3/R2 environment options were removed. Storage and delivery now reject unknown provider values instead of silently using local disk/URLs; the upload security check covers this failure mode.</x:v>
+        <x:v>S3/R2 option was removed from the environment template and unsupported providers fail explicitly. This excluded alternative contributes neither numerator nor denominator to overall completion.</x:v>
       </x:c>
       <x:c r="O88" s="136" t="str">
-        <x:v>Cloudflare Images remains the documented durable production option; staging configuration and end-to-end provider acceptance are tracked in JW-083.</x:v>
+        <x:v>No V1 S3 implementation. Cloudflare provider work remains in JW-083.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -6325,7 +6327,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J89" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="K89" s="136" t="str">
         <x:v>Production image provider</x:v>
@@ -6337,10 +6339,10 @@
         <x:v>LCP; mobile bandwidth; broken URLs; alt text</x:v>
       </x:c>
       <x:c r="N89" s="136" t="str">
-        <x:v>Next Image and Cloudflare width paths are used; production validation remains.</x:v>
+        <x:v>Uploaded images are re-encoded as WebP. Local media now uses direct unoptimized no-store requests to preserve authorization; static site images retain Next optimization. Cloudflare width delivery exists but production dimensions, bandwidth and visual quality are unverified.</x:v>
       </x:c>
       <x:c r="O89" s="136" t="str">
-        <x:v>Run Lighthouse and real-device tests.</x:v>
+        <x:v>Verify production image transformations and private delivery together; measure mobile media bandwidth/LCP.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -7841,10 +7843,10 @@
         <x:v>Valid/invalid listing ID; non-car listing</x:v>
       </x:c>
       <x:c r="N121" s="136" t="str">
-        <x:v>Implemented for cars.</x:v>
+        <x:v>Desktop/mobile car-linked inspection acceptance preserves listing reference across sign-in and stores the request/event; forged or unavailable IDs fail without creating a request.</x:v>
       </x:c>
       <x:c r="O121" s="136" t="str">
-        <x:v>Validate listing ownership/status in inspection action.</x:v>
+        <x:v>Retain passing linked-request tests; complete remaining service action negatives under JW-166.</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -8381,10 +8383,10 @@
         <x:v>Signed V1</x:v>
       </x:c>
       <x:c r="F133" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G133" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="H133" s="136" t="str">
         <x:v>High</x:v>
@@ -8393,7 +8395,7 @@
         <x:v>Stage 3</x:v>
       </x:c>
       <x:c r="J133" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Backend</x:v>
       </x:c>
       <x:c r="K133" s="136" t="str">
         <x:v>Email provider and saved searches</x:v>
@@ -8405,10 +8407,10 @@
         <x:v>Match accuracy; frequency; duplicates; delivery failure; unsubscribe</x:v>
       </x:c>
       <x:c r="N133" s="136" t="str">
-        <x:v>No alert job/provider/template exists.</x:v>
+        <x:v>Reviewed estimate 40%: saved-search alert preferences and authenticated matching cron exist; unique outbox records deduplicate listing/search pairs. No delivery worker/template or delivered_at updater was found. Matching currently reads the first result page, so overflow and retry correctness need acceptance.</x:v>
       </x:c>
       <x:c r="O133" s="136" t="str">
-        <x:v>Choose email provider and build notification worker.</x:v>
+        <x:v>Implement delivery worker, email template/retry/control flow and complete matching/overflow/deduplication tests, then configure provider and scheduler.</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -8452,10 +8454,10 @@
         <x:v>Happy path; duplicate user; duplicate slug; invalid data</x:v>
       </x:c>
       <x:c r="N134" s="136" t="str">
-        <x:v>Implemented.</x:v>
+        <x:v>Dealer registration and owner settings/logo are implemented. Desktop/mobile acceptance creates a dealer/dashboard and verifies account/dealer write limits. Duplicate-slug edge acceptance remains in T-031.</x:v>
       </x:c>
       <x:c r="O134" s="136" t="str">
-        <x:v>Add integration tests and logo support.</x:v>
+        <x:v>Complete remaining registration edge cases and live provider acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
@@ -8487,7 +8489,7 @@
         <x:v>Stage 4</x:v>
       </x:c>
       <x:c r="J135" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="K135" s="136" t="str">
         <x:v>Dealer data</x:v>
@@ -8499,10 +8501,10 @@
         <x:v>Verified/unverified; zero listings; pagination</x:v>
       </x:c>
       <x:c r="N135" s="136" t="str">
-        <x:v>Dealer directory/storefront behavior is implemented; comprehensive browser acceptance remains deferred.</x:v>
+        <x:v>Directory/storefront code and route/accessibility checks pass; admin verification/revocation changes public badges with DB audit assertions. Exact inventory-count, mixed-state and pagination checks remain open.</x:v>
       </x:c>
       <x:c r="O135" s="136" t="str">
-        <x:v>Complete during final QA/hardening after functionality development.</x:v>
+        <x:v>Complete T-032 with deterministic mixed-status dealer inventory.</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
@@ -8546,10 +8548,10 @@
         <x:v>Unknown slug; empty inventory; pagination; mobile</x:v>
       </x:c>
       <x:c r="N136" s="136" t="str">
-        <x:v>Implemented for car inventory.</x:v>
+        <x:v>Storefront queries active listings across verticals and passes row.vertical to ListingCard, supporting cars, bikes and parts. Public route/accessibility checks pass; deterministic count and pagination acceptance remains in T-032.</x:v>
       </x:c>
       <x:c r="O136" s="136" t="str">
-        <x:v>Extend to bike/parts if dealers may list them.</x:v>
+        <x:v>Verify mixed-vertical inventory/counts and pagination in T-032; no bike/parts extension is required.</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
@@ -10029,7 +10031,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G168" s="137" t="n">
-        <x:v>0.55</x:v>
+        <x:v>0.85</x:v>
       </x:c>
       <x:c r="H168" s="136" t="str">
         <x:v>High</x:v>
@@ -10038,7 +10040,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J168" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="K168" s="136" t="str">
         <x:v>Status lifecycle</x:v>
@@ -10050,10 +10052,10 @@
         <x:v>All statuses; canonical; sitemap/search exclusion</x:v>
       </x:c>
       <x:c r="N168" s="136" t="str">
-        <x:v>Current detail-route guard serves inactive listings only to the owner or admin. Browser acceptance confirms pending-review and removed ads return public 404; metadata noindexes non-active views.</x:v>
+        <x:v>Reviewed estimate 85%: docs/PROJECT.md and shared visibility policy define active-only public details; inactive owner/admin views are noindexed. Static policy checks and public pending/removed browser denial pass. Media GET/HEAD checks now cover every inactive status. Full listing lifecycle/crawler deployment acceptance remains.</x:v>
       </x:c>
       <x:c r="O168" s="136" t="str">
-        <x:v>Confirm sold and expired buyer experience with product policy, and run staging crawler acceptance.</x:v>
+        <x:v>Test sold/expired detail, search and sitemap transitions end to end on staging; preserve the documented active-only public policy.</x:v>
       </x:c>
     </x:row>
     <x:row r="169">
@@ -10132,7 +10134,7 @@
         <x:v>Stage 1</x:v>
       </x:c>
       <x:c r="J170" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="K170" s="136" t="str">
         <x:v>All CRUD actions</x:v>
@@ -10355,10 +10357,10 @@
         <x:v>Signed V1</x:v>
       </x:c>
       <x:c r="F175" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G175" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="H175" s="136" t="str">
         <x:v>High</x:v>
@@ -10367,7 +10369,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J175" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Backend</x:v>
       </x:c>
       <x:c r="K175" s="136" t="str">
         <x:v>Privacy policy and operations</x:v>
@@ -10379,10 +10381,10 @@
         <x:v>Retention job; account deletion; backup implications</x:v>
       </x:c>
       <x:c r="N175" s="136" t="str">
-        <x:v>Only expired-session purge exists.</x:v>
+        <x:v>Reviewed estimate 30%: purge-expired removes expired sessions, reset/verification tokens, old rate-limit buckets and abandoned uploads. Orphan storage cleanup has browser/DB acceptance. Account/report/service-record retention, deletion tooling and backup implications remain undefined/incomplete.</x:v>
       </x:c>
       <x:c r="O175" s="136" t="str">
-        <x:v>Define policy and implement necessary tools.</x:v>
+        <x:v>Document retention decisions and implement account/report/service deletion workflows; verify backup handling and scheduled execution.</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
@@ -10402,10 +10404,10 @@
         <x:v>Signed V1</x:v>
       </x:c>
       <x:c r="F176" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G176" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="H176" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10414,7 +10416,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J176" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="K176" s="136" t="str">
         <x:v>Feature-complete staging</x:v>
@@ -10426,10 +10428,10 @@
         <x:v>OWASP review; dependency; auth; IDOR; upload; headers</x:v>
       </x:c>
       <x:c r="N176" s="136" t="str">
-        <x:v>No formal review has been completed.</x:v>
+        <x:v>Reviewed estimate 40%: local review/regressions cover ownership, admin replay, upload content/origin/rate limits, private local reads and dependency audit. CI run 37 passes. Formal infrastructure assessment, remaining action negatives and Cloudflare privacy are not complete; this is not launch security sign-off.</x:v>
       </x:c>
       <x:c r="O176" s="136" t="str">
-        <x:v>Schedule after V1 feature completion.</x:v>
+        <x:v>Finish dealer/service/private-provider assessment and infrastructure review; close critical/high findings with regression evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="177">
@@ -10640,7 +10642,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G181" s="137" t="n">
-        <x:v>0.95</x:v>
+        <x:v>0.97</x:v>
       </x:c>
       <x:c r="H181" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10649,7 +10651,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J181" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="K181" s="136" t="str">
         <x:v>E2E framework</x:v>
@@ -10661,10 +10663,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Local acceptance: 93 browser passes, 1 planned skip, 5 DB checks and 101-route sweep with 0 issues. Private local image GET/HEAD, optimizer denial, owner previews and foreign publish/edit photo keys are covered with positive controls.</x:v>
+        <x:v>Reviewed estimate 97% for core local functional coverage: 93 browser passes, one planned skip, five DB checks and 101-route clean sweep; final media rebuild added a 103-route clean sweep and two focused passes. GitHub run 37 passes on a96704b. Dealer/service direct mutation negatives and controlled failure recovery remain.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Complete dealer/service mutation negatives, controlled failure recovery and performance/load checks; Cloudflare private delivery and live/real-device acceptance remain.</x:v>
+        <x:v>Complete remaining local negative/failure cases. Real-device and production acceptance remain separate JW-178/199 gates.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -10790,7 +10792,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J184" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="K184" s="136" t="str">
         <x:v>Production-like media/data</x:v>
@@ -10802,7 +10804,7 @@
         <x:v>Bundle report; Lighthouse; 4G profile</x:v>
       </x:c>
       <x:c r="N184" s="136" t="str">
-        <x:v>30 Sep production build passes with max First Load JS 128 kB, below the 150 kB project ceiling; Sep 9 changes removed duplicate account queries and unused homepage counts. Staging Web Vitals/load acceptance remains open.</x:v>
+        <x:v>a96704b production build has maximum First Load JS 128 KB, below 150 KB. Production media/Web Vitals and representative query/load acceptance remain open.</x:v>
       </x:c>
       <x:c r="O184" s="136" t="str">
         <x:v>Measure Core Web Vitals and browse query/load behavior on production-like staging before launch.</x:v>
@@ -11354,7 +11356,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J196" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>DevOps</x:v>
       </x:c>
       <x:c r="K196" s="136" t="str">
         <x:v>Cloudflare or implemented provider</x:v>
@@ -11366,10 +11368,10 @@
         <x:v>Upload/display/delete; cache; failure</x:v>
       </x:c>
       <x:c r="N196" s="136" t="str">
-        <x:v>Local provider is not production-safe.</x:v>
+        <x:v>Cloudflare adapter exists under JW-083, but no durable staging/production media service is verified. Local storage is development-only; private/signed Cloudflare delivery is an unresolved implementation gate.</x:v>
       </x:c>
       <x:c r="O196" s="136" t="str">
-        <x:v>Configure and validate selected provider.</x:v>
+        <x:v>Complete JW-083 private delivery and configure durable storage; verify upload/read/delete across deployment and restart.</x:v>
       </x:c>
     </x:row>
     <x:row r="197">
@@ -12309,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R515b95f34cd64dc5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R091215728ac74949"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12356,7 +12358,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="139" t="str">
-        <x:v>Development-first sequence: implement -&gt; automated checks + database acceptance -&gt; local commit -&gt; explicit approval before push/merge. Comprehensive browser, branding and responsive QA occur after functionality is complete.</x:v>
+        <x:v>Verified development is committed, pushed and recorded automatically under owner authorization. PR review and main merge remain separate. Local browser/DB acceptance runs alongside packages; live/real-device launch acceptance remains open.</x:v>
       </x:c>
       <x:c r="B2" s="139"/>
       <x:c r="C2" s="139"/>
@@ -12687,13 +12689,13 @@
         <x:v>feature/saved-search-alerts</x:v>
       </x:c>
       <x:c r="E17" s="141" t="str">
-        <x:v>Users manage saved filters and receive deduplicated consented alerts.</x:v>
+        <x:v>Saved-search management, alert preferences and deduplicated match outbox exist; delivery worker, templates, retry/control and full matching acceptance remain.</x:v>
       </x:c>
       <x:c r="F17" s="141" t="str">
-        <x:v>Match and delivery tests pass.</x:v>
+        <x:v>Automated matching/overflow/deduplication and delivered-email acceptance pass with configured provider/scheduler.</x:v>
       </x:c>
       <x:c r="G17" s="141" t="str">
-        <x:v>Completed</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -12822,10 +12824,10 @@
         <x:v>CI, automated testing and staging</x:v>
       </x:c>
       <x:c r="D23" s="141" t="str">
-        <x:v>chore/launch-quality-system</x:v>
+        <x:v>codex/launch-quality-system</x:v>
       </x:c>
       <x:c r="E23" s="141" t="str">
-        <x:v>PR checks, staging, E2E and monitoring are operational.</x:v>
+        <x:v>PR #6 / a96704b: CI run 37 passes, 93 local browser cases and 5 DB checks. Persistent staging, monitoring and required-check enforcement remain open.</x:v>
       </x:c>
       <x:c r="F23" s="141" t="str">
         <x:v>Deliberate failure blocks merge; staging smoke passes.</x:v>
@@ -12845,16 +12847,16 @@
         <x:v>Production infrastructure and hardening</x:v>
       </x:c>
       <x:c r="D24" s="141" t="str">
-        <x:v>chore/production-readiness</x:v>
+        <x:v>codex/production-readiness (planned)</x:v>
       </x:c>
       <x:c r="E24" s="141" t="str">
-        <x:v>DB/media/backups/cron/logs/domain/security/load tests are complete.</x:v>
+        <x:v>Local hardening has started: upload ownership/privacy, action authorization and cleanup. Production DB/media/backups/cron/logs/domain, formal security/load and live acceptance remain open.</x:v>
       </x:c>
       <x:c r="F24" s="141" t="str">
         <x:v>Formal launch checklist has no open critical/high issue.</x:v>
       </x:c>
       <x:c r="G24" s="141" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12864,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4f2b0ad305e48dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1a63ac5e5d64c3a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13295,10 +13297,10 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E18" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Desktop/mobile direct mark-sold owner success and foreign-user denial with DB state checks; shared visibility assertions</x:v>
       </x:c>
       <x:c r="F18" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Partial pass: mark-sold authorization verified; cron TTL, reactivation and complete search/contact/SEO lifecycle remain</x:v>
       </x:c>
       <x:c r="G18" s="141" t="str">
         <x:v>Active listing and cron secret</x:v>
@@ -13347,7 +13349,7 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E20" s="141" t="str">
-        <x:v>Desktop/mobile Chromium upload/public WebP URL, foreign-Origin 403 and request-bucket 429 before file read</x:v>
+        <x:v>Desktop/mobile upload WebP, owner-only pending GET/HEAD, foreign-Origin 403 and request-bucket 429; source size/count/quota guards</x:v>
       </x:c>
       <x:c r="F20" s="141" t="str">
         <x:v>Partial pass: valid image and request limit enforced; individual size/count boundaries remain open</x:v>
@@ -13373,10 +13375,10 @@
         <x:v>Security</x:v>
       </x:c>
       <x:c r="E21" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Automated check:uploads decodes/re-encodes valid images, rejects magic-byte-only fake and unsafe keys, preserves safe legacy conversion</x:v>
       </x:c>
       <x:c r="F21" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Partial pass: fake image/key rejection and WebP conversion verified; comprehensive oversized, SVG/executable/polyglot HTTP matrix remains</x:v>
       </x:c>
       <x:c r="G21" s="141" t="str">
         <x:v>SVG/executable/polyglot fixtures</x:v>
@@ -13711,13 +13713,13 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E34" s="141" t="str">
-        <x:v>Automated checks</x:v>
+        <x:v>Saved-search UI/static checks plus matching cron and unique outbox in source; no email delivery worker exists</x:v>
       </x:c>
       <x:c r="F34" s="141" t="str">
-        <x:v>Feature passed; delivery provider configuration pending</x:v>
+        <x:v>Partial implementation only: full match/overflow/dedupe/retry and delivered-email acceptance pending</x:v>
       </x:c>
       <x:c r="G34" s="141" t="str">
-        <x:v>Saved search/alerts complete</x:v>
+        <x:v>Implement delivery worker and configure email provider/scheduler</x:v>
       </x:c>
       <x:c r="H34" s="141" t="str">
         <x:v>Exact filters, no duplicate alerts</x:v>
@@ -14003,7 +14005,7 @@
         <x:v>Partial pass: Chromium and simulated WebKit smoke have no viewport overflow; real Safari/iPhone, camera/keyboard and broader staging QA remain open</x:v>
       </x:c>
       <x:c r="G45" s="141" t="str">
-        <x:v>PR #2 local preview</x:v>
+        <x:v>Owner-approved homepage merged in PR #5; PR #6 local acceptance</x:v>
       </x:c>
       <x:c r="H45" s="141" t="str">
         <x:v>No overflow/clipping; approved layout</x:v>
@@ -14179,10 +14181,10 @@
         <x:v>Security review</x:v>
       </x:c>
       <x:c r="E52" s="141" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Local authorization replay, upload/content/origin/rate-limit/private-read regressions and CI dependency audit</x:v>
       </x:c>
       <x:c r="F52" s="141" t="str">
-        <x:v>Pre-launch</x:v>
+        <x:v>Partial pass locally; formal infrastructure review, remaining action negatives and Cloudflare private delivery open</x:v>
       </x:c>
       <x:c r="G52" s="141" t="str">
         <x:v>Feature-complete staging</x:v>
@@ -14260,7 +14262,7 @@
         <x:v>GitHub CI plus local clean isolated DB</x:v>
       </x:c>
       <x:c r="F55" s="141" t="str">
-        <x:v>Passed local and CI #36631593477: migrations, curated/demo seed, DB assertions</x:v>
+        <x:v>Passed local isolated migrations/seed and CI run 37 on a96704b</x:v>
       </x:c>
       <x:c r="G55" s="141" t="str">
         <x:v>Fresh PostgreSQL</x:v>
@@ -14309,10 +14311,10 @@
         <x:v>Integration/Operational</x:v>
       </x:c>
       <x:c r="E57" s="141" t="str">
-        <x:v>Manual partial</x:v>
+        <x:v>Local orphan-purge authentication and DB/file preservation acceptance; protected expire/alert jobs present</x:v>
       </x:c>
       <x:c r="F57" s="141" t="str">
-        <x:v>Pending scheduler</x:v>
+        <x:v>Partial pass: orphan cleanup verified; expiry/alert edge cases, production scheduler and monitoring remain</x:v>
       </x:c>
       <x:c r="G57" s="141" t="str">
         <x:v>Configured CRON_SECRET</x:v>
@@ -14432,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72de2db063214171"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf04f24465c545d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14592,7 +14594,7 @@
         <x:v>Removed / Do Not Build</x:v>
       </x:c>
       <x:c r="D12" s="141" t="str">
-        <x:v>Password auth; secure email reset to be designed</x:v>
+        <x:v>Google-first and verified-email authentication with secure email reset; SMS OTP remains excluded</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -14658,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14d019580dd940a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1caedf44c0ee4e5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Verify dealer and service permissions and listing reactivation
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdb392ab5d74b4487"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R9e04d7112b764be9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rda246002cd7f40b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R2424cffe62d245a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rdb487aa56ef9452a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rc20d3f9971c941b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rbbcb403f7f8f4ce0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rccbf8fe74e0c4d57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R1cb305b1849c4049"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R0e611caff5e54e9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R5492dd8b08d1440a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R93ea17b2712d410f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rb2f5dab66f2e4018"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R273d74f389eb4dff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8c7219f423794af3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R597df881ea9948f2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1253,7 +1253,7 @@
         <x:v>Current branch</x:v>
       </x:c>
       <x:c r="H5" s="93" t="str">
-        <x:v>codex/launch-quality-system; a96704b pushed</x:v>
+        <x:v>codex/launch-quality-system; PR #6</x:v>
       </x:c>
       <x:c r="I5" s="93"/>
       <x:c r="J5" s="94"/>
@@ -1334,7 +1334,7 @@
         <x:v>Next functionality</x:v>
       </x:c>
       <x:c r="H8" s="98" t="str">
-        <x:v>Dealer/service negatives and controlled failure recovery</x:v>
+        <x:v>Controlled failure/recovery, provider privacy and alert delivery</x:v>
       </x:c>
       <x:c r="I8" s="98"/>
       <x:c r="J8" s="99"/>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>93 local passes, 1 planned skip; real-device QA open</x:v>
+        <x:v>101 local passes, 1 planned skip; live/device QA open</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1399,7 +1399,7 @@
       </x:c>
       <x:c r="B11" s="142" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request",'Feature Tracker'!$F$5:$F$215,"&lt;&gt;Out of Scope / Removed")/B5</x:f>
-        <x:v>0.9058500000000003</x:v>
+        <x:v>0.9064000000000001</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>PR #6: a96704b passed GitHub run 37. Local suite: 93 browser passes, 1 planned skip, 5 DB checks and 101 routes clean; final media recheck: 2 cases and 103 routes clean. Persistent staging remains open.</x:v>
+        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 5 DB checks and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Dealer/service negatives and expiry/reactivation pass. Current PR checks govern the latest commit; production staging remains open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1676,7 +1676,7 @@
         <x:v>Complete remaining launch acceptance</x:v>
       </x:c>
       <x:c r="C27" s="110" t="str">
-        <x:v>Next: dealer/service authorization, controlled failure recovery and performance/load. Cloudflare private delivery, live providers and real-device review remain launch gates.</x:v>
+        <x:v>Next: controlled failure/recovery, Cloudflare private delivery, email-alert worker and retention/configuration work. Production providers, load and real-device acceptance remain open.</x:v>
       </x:c>
       <x:c r="D27" s="88"/>
       <x:c r="E27" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6a3a37015154bf3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d467b3342934bc7"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Reconciled 3 Oct 2026 against a96704b and successful GitHub run 37. Local acceptance: 93 browser passes, 1 planned skip, 5 DB checks; 101-route clean sweep and final 103-route media recheck. Framework complete pending PR #6 review; production gates remain open.</x:v>
+        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 5 DB checks and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Dealer/service replay and expiry/reactivation are verified. Each finished package is committed/pushed with this master tracker; PR review/merge and live launch gates remain separate.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2955,7 +2955,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Framework acceptance criteria met on a96704b: isolated DB, desktop/mobile Chromium core journeys, iPhone WebKit smoke, 93 browser passes and one planned desktop-only skip; CI run 37 passed. PR #6 review remains open. Wider test coverage, real devices and deployment acceptance are separately tracked in JW-177/178/199.</x:v>
+        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 5 DB checks and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Framework remains verified on feature branch awaiting PR #6 review; additional live/device acceptance remains separately tracked.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Review PR #6; retain regression coverage. Track additional cases in JW-177 rather than reopening the test-framework implementation.</x:v>
@@ -5848,7 +5848,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G79" s="137" t="n">
-        <x:v>0.85</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H79" s="136" t="str">
         <x:v>High</x:v>
@@ -5869,10 +5869,10 @@
         <x:v>TTL boundary; cron auth; search/detail behavior</x:v>
       </x:c>
       <x:c r="N79" s="136" t="str">
-        <x:v>Reviewed estimate 85%: protected expire-listings job and owner-only reactivateListingAction are implemented. Dashboard offers Reactivate for 30 days for sold/expired listings. Production scheduler, TTL boundary and full reactivation browser acceptance remain open.</x:v>
+        <x:v>Expiry/reactivation local acceptance passes in desktop/mobile: unauthenticated cron denied, due active fixture expires, future fixture remains active, foreign/anonymous reactivation denied, owner receives a fresh 30-day window, and active/rejected/removed requests do not extend it.</x:v>
       </x:c>
       <x:c r="O79" s="136" t="str">
-        <x:v>Test expiry/reactivation boundaries and authorization; configure and monitor production scheduling under JW-197.</x:v>
+        <x:v>Configure and monitor production expiry scheduling; run full live search/contact/SEO lifecycle acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -10146,10 +10146,10 @@
         <x:v>IDOR; direct action calls; cross-user access</x:v>
       </x:c>
       <x:c r="N170" s="136" t="str">
-        <x:v>Local photo GET/HEAD authorization now enforces listing visibility and pending-upload ownership, with owner/admin controls, no-store responses, blocked optimizer access and storage outside public/. Desktop/mobile HTTP publish/edit reject foreign photo keys without changing listing images; valid-owner replays pass. Legacy development photo compatibility is preserved.</x:v>
+        <x:v>Local photo/action coverage includes direct dealer verify/revoke and inspection/assistance update replay: non-admin/anonymous actors cannot mutate records/audits; owners also cannot perform service-admin changes. Identical administrator payload succeeds. Customer records/private notes remain isolated. Prior owner listing/media regressions pass.</x:v>
       </x:c>
       <x:c r="O170" s="136" t="str">
-        <x:v>Complete dealer/service direct-mutation negatives. Cloudflare private/signed delivery implementation and live provider acceptance remain a launch gate; local media authorization does not protect direct Cloudflare URLs.</x:v>
+        <x:v>Complete remaining action/edge/concurrency matrix and provider/infrastructure security review; Cloudflare private delivery remains in JW-083.</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -10642,7 +10642,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G181" s="137" t="n">
-        <x:v>0.97</x:v>
+        <x:v>0.98</x:v>
       </x:c>
       <x:c r="H181" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10663,10 +10663,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Reviewed estimate 97% for core local functional coverage: 93 browser passes, one planned skip, five DB checks and 101-route clean sweep; final media rebuild added a 103-route clean sweep and two focused passes. GitHub run 37 passes on a96704b. Dealer/service direct mutation negatives and controlled failure recovery remain.</x:v>
+        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 5 DB checks and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Eight new desktop/mobile cases cover dealer/service authorization and expiry/reactivation.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Complete remaining local negative/failure cases. Real-device and production acceptance remain separate JW-178/199 gates.</x:v>
+        <x:v>Next: controlled backend failure/retry recovery, deeper conditional/edge cases and live acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R091215728ac74949"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0024eb3f37e467d"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1a63ac5e5d64c3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8be86ef6d4044925"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13297,10 +13297,10 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E18" s="141" t="str">
-        <x:v>Desktop/mobile direct mark-sold owner success and foreign-user denial with DB state checks; shared visibility assertions</x:v>
+        <x:v>Desktop/mobile expiry cron, due/future fixtures, direct reactivation replay and owner positive control</x:v>
       </x:c>
       <x:c r="F18" s="141" t="str">
-        <x:v>Partial pass: mark-sold authorization verified; cron TTL, reactivation and complete search/contact/SEO lifecycle remain</x:v>
+        <x:v>Local pass: cron auth, expiry selection, owner-only fresh 30-day window and active/rejected/removed no-op checked; complete live search/contact/SEO lifecycle and scheduler remain</x:v>
       </x:c>
       <x:c r="G18" s="141" t="str">
         <x:v>Active listing and cron secret</x:v>
@@ -13791,10 +13791,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E37" s="141" t="str">
-        <x:v>Automated checks plus desktop/mobile Chromium admin verify/revoke, public badge and DB audit assertions</x:v>
+        <x:v>Desktop/mobile verification/revocation public-badge/audit flow plus direct seller/anonymous replay with identical administrator controls</x:v>
       </x:c>
       <x:c r="F37" s="141" t="str">
-        <x:v>Passed: grant/revoke changes verified_at and public badge; both decisions append audit events</x:v>
+        <x:v>Local pass: unauthorized verify/revoke leaves dealer and audit unchanged; admin decisions succeed with exactly one audit each</x:v>
       </x:c>
       <x:c r="G37" s="141" t="str">
         <x:v>Verification admin complete</x:v>
@@ -13843,10 +13843,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E39" s="141" t="str">
-        <x:v>Desktop/mobile Chromium admin status update, append-only event, customer visibility and private-note exclusion</x:v>
+        <x:v>Desktop/mobile creation/customer history plus direct administration replay by owner, foreign seller and anonymous visitor; admin positive control and unchanged DB/audit checks</x:v>
       </x:c>
       <x:c r="F39" s="141" t="str">
-        <x:v>Partial pass: requested to contacted lifecycle and privacy verified; invalid transitions still open</x:v>
+        <x:v>Local pass for covered paths: unauthorized writes, invalid status jump, missing customer message and terminal-state reopening rejected; valid admin update audited; customer isolation/private-note exclusion pass. Remaining intermediate transitions/live acceptance open.</x:v>
       </x:c>
       <x:c r="G39" s="141" t="str">
         <x:v>Inspection admin complete</x:v>
@@ -13869,10 +13869,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E40" s="141" t="str">
-        <x:v>Desktop/mobile Chromium structured request, DB fields, admin update, append-only event and customer privacy</x:v>
+        <x:v>Desktop/mobile creation/customer history plus direct administration replay by owner, foreign seller and anonymous visitor; admin positive control and unchanged DB/audit checks</x:v>
       </x:c>
       <x:c r="F40" s="141" t="str">
-        <x:v>Partial pass: request/manage and customer history verified; negative cases still open</x:v>
+        <x:v>Local pass for covered paths: unauthorized writes, invalid status jump, missing customer message and terminal-state reopening rejected; valid admin update audited; customer isolation/private-note exclusion pass. Remaining intermediate transitions/live acceptance open.</x:v>
       </x:c>
       <x:c r="G40" s="141" t="str">
         <x:v>Public/admin flows complete</x:v>
@@ -14311,10 +14311,10 @@
         <x:v>Integration/Operational</x:v>
       </x:c>
       <x:c r="E57" s="141" t="str">
-        <x:v>Local orphan-purge authentication and DB/file preservation acceptance; protected expire/alert jobs present</x:v>
+        <x:v>Local orphan-purge and expiry cron authentication; due/future expiry selection and owner reactivation browser/DB acceptance</x:v>
       </x:c>
       <x:c r="F57" s="141" t="str">
-        <x:v>Partial pass: orphan cleanup verified; expiry/alert edge cases, production scheduler and monitoring remain</x:v>
+        <x:v>Local cleanup/expiry checks pass; production scheduling, monitoring and saved-alert edge cases remain</x:v>
       </x:c>
       <x:c r="G57" s="141" t="str">
         <x:v>Configured CRON_SECRET</x:v>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf04f24465c545d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R553907c3a87c492f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1caedf44c0ee4e5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd90ae8fceb24bf4"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add audited first-administrator bootstrap with transaction acceptance
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rccbf8fe74e0c4d57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R1cb305b1849c4049"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R0e611caff5e54e9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R5492dd8b08d1440a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R93ea17b2712d410f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rb2f5dab66f2e4018"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R273d74f389eb4dff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8a8d927b0e5441fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R168a5a2ca24847f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R9983a95bf4ae4a52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rb92f78b18a7e4d3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rdaab815de5d54438"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rf3b9dea079514c58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rec1968df43ab488c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R597df881ea9948f2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9240569413954047"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1355,7 +1355,7 @@
         <x:v>Local passed</x:v>
       </x:c>
       <x:c r="F9" s="99" t="str">
-        <x:v>5 DB checks; live deployment acceptance open</x:v>
+        <x:v>6 DB checks; live deployment acceptance open</x:v>
       </x:c>
       <x:c r="G9" s="97" t="str">
         <x:v>Browser QA</x:v>
@@ -1399,7 +1399,7 @@
       </x:c>
       <x:c r="B11" s="142" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request",'Feature Tracker'!$F$5:$F$215,"&lt;&gt;Out of Scope / Removed")/B5</x:f>
-        <x:v>0.9064000000000001</x:v>
+        <x:v>0.9076500000000002</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 5 DB checks and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Dealer/service negatives and expiry/reactivation pass. Current PR checks govern the latest commit; production staging remains open.</x:v>
+        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 6 DB checks (baseline + bootstrap) and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Initial-admin tool/runbook also verified. Current PR checks govern the latest commit; production staging remains open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d467b3342934bc7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4d946bc9c754639"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 5 DB checks and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Dealer/service replay and expiry/reactivation are verified. Each finished package is committed/pushed with this master tracker; PR review/merge and live launch gates remain separate.</x:v>
+        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 6 DB checks (baseline + bootstrap) and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Admin bootstrap tool/runbook is verified; actual production provisioning remains open. Cloudflare privacy, alerts, retention, failure/load and live acceptance remain.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2887,7 +2887,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G16" s="137" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="H16" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2908,10 +2908,10 @@
         <x:v>Unit; integration; transaction tests</x:v>
       </x:c>
       <x:c r="N16" s="136" t="str">
-        <x:v>Reviewed estimate 75%: automated framework and five isolated DB checks are operational, including concurrent rate limits and actual upload-claim rollback, duplicate/reuse/foreign-key denial. HTTP authorization suite also proves publish/edit denial and owner/admin success. Wider transaction failure/concurrency coverage is incomplete.</x:v>
+        <x:v>Six isolated PostgreSQL checks now include first-admin dry run, eligibility, audit-failure rollback, concurrent first-admin attempts, idempotency and session revocation, alongside reference/facet/rate-limit/upload-claim checks. Browser authorization cases also preserve DB/audit state.</x:v>
       </x:c>
       <x:c r="O16" s="136" t="str">
-        <x:v>Extend transaction rollback and concurrency checks to publication, edits, moderation and service-request updates.</x:v>
+        <x:v>Extend transaction fault/concurrency checks to remaining moderation/service and delivery workflows.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2955,7 +2955,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 5 DB checks and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Framework remains verified on feature branch awaiting PR #6 review; additional live/device acceptance remains separately tracked.</x:v>
+        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 6 DB checks (5 baseline plus bootstrap transaction acceptance) and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Dealer/service and expiry cases pass; first-admin CLI is verified separately without modifying production accounts.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Review PR #6; retain regression coverage. Track additional cases in JW-177 rather than reopening the test-framework implementation.</x:v>
@@ -4626,7 +4626,7 @@
         <x:v>Launch Configuration Pending</x:v>
       </x:c>
       <x:c r="G53" s="137" t="n">
-        <x:v>0.7</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H53" s="136" t="str">
         <x:v>Critical</x:v>
@@ -4635,7 +4635,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J53" s="136" t="str">
-        <x:v>Backend</x:v>
+        <x:v>DevOps</x:v>
       </x:c>
       <x:c r="K53" s="136" t="str">
         <x:v>Production DB access</x:v>
@@ -4647,10 +4647,10 @@
         <x:v>Access test; audit review</x:v>
       </x:c>
       <x:c r="N53" s="136" t="str">
-        <x:v>Local administrator access exists. No dedicated bootstrap command or complete audited production-bootstrap runbook was found; production administrator creation remains open.</x:v>
+        <x:v>Preview-first operator CLI and docs/ADMIN_BOOTSTRAP.md implemented. Explicit database-name confirmation, verified/unbanned unique account checks, no second-admin bootstrap, serialized concurrent attempts, atomic audit and session revocation, rollback and idempotency pass in isolated migrated-table tests. No production account was changed.</x:v>
       </x:c>
       <x:c r="O53" s="136" t="str">
-        <x:v>Implement/document audited first-admin provisioning, then execute only against the chosen production environment.</x:v>
+        <x:v>At deployment, select the named verified owner, preview/apply on the intended production DB, reauthenticate and record operator/access review.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -10663,7 +10663,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 5 DB checks and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Eight new desktop/mobile cases cover dealer/service authorization and expiry/reactivation.</x:v>
+        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 6 DB checks (5 baseline plus bootstrap transaction acceptance) and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Dealer/service and expiry cases pass; first-admin CLI is verified separately without modifying production accounts.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Next: controlled backend failure/retry recovery, deeper conditional/edge cases and live acceptance.</x:v>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0024eb3f37e467d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78aafc563f104f5c"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8be86ef6d4044925"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56a701ced3464cf7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R553907c3a87c492f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5152192ca2dd4974"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd90ae8fceb24bf4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73c6da61f4794101"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Refresh failed browse requests and verify database recovery
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8a8d927b0e5441fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R168a5a2ca24847f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R9983a95bf4ae4a52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rb92f78b18a7e4d3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rdaab815de5d54438"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rf3b9dea079514c58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rec1968df43ab488c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rce77cd41a2e34245"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R8dd8b80b84ee45f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rc8f1be3fd49049a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R24fff1d2176846a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R9ad9185b9ed940dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R0bf6326441dc46d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R2d757358e30442ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9240569413954047"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6b5f9bbf7aff4cd2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1247,7 +1247,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F5" s="94" t="str">
-        <x:v>Passed on a96704b; CI run 37</x:v>
+        <x:v>Latest local checks passed; see current PR checks for CI</x:v>
       </x:c>
       <x:c r="G5" s="92" t="str">
         <x:v>Current branch</x:v>
@@ -1274,7 +1274,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F6" s="99" t="str">
-        <x:v>No warnings/errors; CI run 37</x:v>
+        <x:v>No local warnings/errors; see current PR checks for CI</x:v>
       </x:c>
       <x:c r="G6" s="97" t="str">
         <x:v>Current stage</x:v>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6 open; GitHub run 37 passed</x:v>
+        <x:v>PR #6 open; current head CI governs review</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1334,7 +1334,7 @@
         <x:v>Next functionality</x:v>
       </x:c>
       <x:c r="H8" s="98" t="str">
-        <x:v>Controlled failure/recovery, provider privacy and alert delivery</x:v>
+        <x:v>Cloudflare private delivery, alert worker and retention</x:v>
       </x:c>
       <x:c r="I8" s="98"/>
       <x:c r="J8" s="99"/>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>101 local passes, 1 planned skip; live/device QA open</x:v>
+        <x:v>101 baseline + 3 recovery passes; 1 planned skip</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1399,7 +1399,7 @@
       </x:c>
       <x:c r="B11" s="142" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request",'Feature Tracker'!$F$5:$F$215,"&lt;&gt;Out of Scope / Removed")/B5</x:f>
-        <x:v>0.9076500000000002</x:v>
+        <x:v>0.9079500000000003</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 6 DB checks (baseline + bootstrap) and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Initial-admin tool/runbook also verified. Current PR checks govern the latest commit; production staging remains open.</x:v>
+        <x:v>101 ordinary browser passes + 3 targeted recovery passes (separate runs), 1 planned skip; 6 DB checks; latest sweep 103 URLs, zero issues. Check/lint/final build pass; max First Load JS 128 KB. Initial-admin bootstrap and database-failure recovery verified. PR review and production acceptance remain open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1676,7 +1676,7 @@
         <x:v>Complete remaining launch acceptance</x:v>
       </x:c>
       <x:c r="C27" s="110" t="str">
-        <x:v>Next: controlled failure/recovery, Cloudflare private delivery, email-alert worker and retention/configuration work. Production providers, load and real-device acceptance remain open.</x:v>
+        <x:v>Next: Cloudflare private delivery, email-alert worker and retention/configuration. Production providers, load, slow-network and real-device acceptance remain open.</x:v>
       </x:c>
       <x:c r="D27" s="88"/>
       <x:c r="E27" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4d946bc9c754639"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0143b1fee95343c3"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 6 DB checks (baseline + bootstrap) and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Admin bootstrap tool/runbook is verified; actual production provisioning remains open. Cloudflare privacy, alerts, retention, failure/load and live acceptance remain.</x:v>
+        <x:v>101 ordinary browser passes + 3 targeted recovery passes (separate runs), 1 planned skip; 6 DB checks; latest sweep 103 URLs, zero issues. Check/lint/final build pass; max First Load JS 128 KB. Each package includes the updated master tracker and is committed/pushed. Production admin provisioning, providers, privacy, alerts, retention and live launch gates remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2955,7 +2955,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 6 DB checks (5 baseline plus bootstrap transaction acceptance) and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Dealer/service and expiry cases pass; first-admin CLI is verified separately without modifying production accounts.</x:v>
+        <x:v>101 ordinary browser passes + 3 targeted recovery passes (separate runs), 1 planned skip; 6 DB checks; latest sweep 103 URLs, zero issues. Check/lint/final build pass; max First Load JS 128 KB. Framework awaits PR #6 review; current head CI is authoritative.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Review PR #6; retain regression coverage. Track additional cases in JW-177 rather than reopening the test-framework implementation.</x:v>
@@ -7352,7 +7352,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G111" s="137" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H111" s="136" t="str">
         <x:v>High</x:v>
@@ -7373,10 +7373,10 @@
         <x:v>Empty DB; query failure; slow response</x:v>
       </x:c>
       <x:c r="N111" s="136" t="str">
-        <x:v>Cars, bikes and parts browsing now have accessible loading skeletons scoped after URL validation, plus route-level recoverable error screens with retry and clear-filters actions. Actionable no-results state was already present; invalid URL 404 and canonical redirects remain protected.</x:v>
+        <x:v>Cars, bikes and parts friendly error/clear-filter controls and post-restoration retry pass with real database-read fault injection. Fixed Try again retaining failed server data by refreshing before boundary reset. Three targeted browser cases pass on final build.</x:v>
       </x:c>
       <x:c r="O111" s="136" t="str">
-        <x:v>Exercise the error boundary with a controlled backend failure in isolated browser acceptance, then verify slow-network loading and retry on live devices.</x:v>
+        <x:v>Complete slow-network, provider-outage and real-device/loading acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -10642,7 +10642,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G181" s="137" t="n">
-        <x:v>0.98</x:v>
+        <x:v>0.99</x:v>
       </x:c>
       <x:c r="H181" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10663,10 +10663,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Clean isolated acceptance: 101 browser passes, 1 planned skip, 6 DB checks (5 baseline plus bootstrap transaction acceptance) and 101-route sweep with zero issues. Check, lint and build pass; max First Load JS 128 KB. Dealer/service and expiry cases pass; first-admin CLI is verified separately without modifying production accounts.</x:v>
+        <x:v>101 ordinary browser passes + 3 targeted recovery passes (separate runs), 1 planned skip; 6 DB checks; latest sweep 103 URLs, zero issues. Check/lint/final build pass; max First Load JS 128 KB. Recovery project is isolated after normal browser projects; forced database failure is restored in cleanup.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Next: controlled backend failure/retry recovery, deeper conditional/edge cases and live acceptance.</x:v>
+        <x:v>Remaining conditional/edge, provider, slow-network and live-device acceptance; CI on latest head governs PR review.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78aafc563f104f5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdeb9b895c7264867"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56a701ced3464cf7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa62385ffe4447ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5152192ca2dd4974"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4211c38cbb94489b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73c6da61f4794101"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdab0bcae51d496b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete autonomous launch hardening and reconcile remaining gates
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rce77cd41a2e34245"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R8dd8b80b84ee45f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rc8f1be3fd49049a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R24fff1d2176846a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R9ad9185b9ed940dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R0bf6326441dc46d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R2d757358e30442ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R883223235ae34cb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rb16a3fd7607b4d08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R90e8436a34774ffe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Ra1ba5ab418a0437b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R14c2ccf3dc734c18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rcfdcdcc00cd8486b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rf1e3d907a0cd4f23"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6b5f9bbf7aff4cd2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2305f5278d914b1a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1247,7 +1247,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F5" s="94" t="str">
-        <x:v>Latest local checks passed; see current PR checks for CI</x:v>
+        <x:v>Local passed; check current CI</x:v>
       </x:c>
       <x:c r="G5" s="92" t="str">
         <x:v>Current branch</x:v>
@@ -1264,7 +1264,7 @@
       </x:c>
       <x:c r="B6" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>154</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="C6" s="88"/>
       <x:c r="D6" s="97" t="str">
@@ -1274,7 +1274,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F6" s="99" t="str">
-        <x:v>No local warnings/errors; see current PR checks for CI</x:v>
+        <x:v>No local lint warnings/errors</x:v>
       </x:c>
       <x:c r="G6" s="97" t="str">
         <x:v>Current stage</x:v>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6 open; current head CI governs review</x:v>
+        <x:v>PR #6 open; prior run 41 passed; latest-head CI pending</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1318,7 +1318,7 @@
       </x:c>
       <x:c r="B8" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C8" s="88"/>
       <x:c r="D8" s="97" t="str">
@@ -1334,7 +1334,7 @@
         <x:v>Next functionality</x:v>
       </x:c>
       <x:c r="H8" s="98" t="str">
-        <x:v>Cloudflare private delivery, alert worker and retention</x:v>
+        <x:v>Live providers/hosting, retention and verification decisions</x:v>
       </x:c>
       <x:c r="I8" s="98"/>
       <x:c r="J8" s="99"/>
@@ -1355,13 +1355,13 @@
         <x:v>Local passed</x:v>
       </x:c>
       <x:c r="F9" s="99" t="str">
-        <x:v>6 DB checks; live deployment acceptance open</x:v>
+        <x:v>7 DB checks pass; live deployment checks remain</x:v>
       </x:c>
       <x:c r="G9" s="97" t="str">
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>101 baseline + 3 recovery passes; 1 planned skip</x:v>
+        <x:v>6 new + 2 report retests + 3 recovery pass; see evidence</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1372,7 +1372,7 @@
       </x:c>
       <x:c r="B10" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>11</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C10" s="88"/>
       <x:c r="D10" s="97" t="str">
@@ -1399,7 +1399,7 @@
       </x:c>
       <x:c r="B11" s="142" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request",'Feature Tracker'!$F$5:$F$215,"&lt;&gt;Out of Scope / Removed")/B5</x:f>
-        <x:v>0.9079500000000003</x:v>
+        <x:v>0.9262</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1468,7 +1468,7 @@
       </x:c>
       <x:c r="B15" s="106" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>154</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="C15" s="107" t="str">
         <x:v>Implemented and available in current code; does not mean production launch approval</x:v>
@@ -1506,7 +1506,7 @@
       </x:c>
       <x:c r="B17" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C17" s="110" t="str">
         <x:v>Partly implemented or awaiting configuration/acceptance</x:v>
@@ -1544,7 +1544,7 @@
       </x:c>
       <x:c r="B19" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>11</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C19" s="110" t="str">
         <x:v>No implemented delivery for this feature; see row-specific prerequisites</x:v>
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>101 ordinary browser passes + 3 targeted recovery passes (separate runs), 1 planned skip; 6 DB checks; latest sweep 103 URLs, zero issues. Check/lint/final build pass; max First Load JS 128 KB. Initial-admin bootstrap and database-failure recovery verified. PR review and production acceptance remain open.</x:v>
+        <x:v>Private media, alert worker, environment validation, dealer/tablet fixes and readiness implemented. 7 DB checks and focused browser tests pass; 101 routes have zero issues. Local full-run resource failure was retested successfully; current-head CI governs review.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1676,7 +1676,7 @@
         <x:v>Complete remaining launch acceptance</x:v>
       </x:c>
       <x:c r="C27" s="110" t="str">
-        <x:v>Next: Cloudflare private delivery, email-alert worker and retention/configuration. Production providers, load, slow-network and real-device acceptance remain open.</x:v>
+        <x:v>Remaining: hosting/HTTPS and production DB; live Cloudflare/Resend/Google/Maps acceptance; backups, schedules and external monitoring; retention/individual-seller/measurement decisions; staging load and real-device review. Review PR #6 before merge.</x:v>
       </x:c>
       <x:c r="D27" s="88"/>
       <x:c r="E27" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0143b1fee95343c3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01234bc362fe42b7"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>101 ordinary browser passes + 3 targeted recovery passes (separate runs), 1 planned skip; 6 DB checks; latest sweep 103 URLs, zero issues. Check/lint/final build pass; max First Load JS 128 KB. Each package includes the updated master tracker and is committed/pushed. Production admin provisioning, providers, privacy, alerts, retention and live launch gates remain open.</x:v>
+        <x:v>Autonomous package: private Cloudflare delivery, alert worker, deployment validation, dealer/tablet fixes, readiness/log hooks, retention inventory and local performance baselines. Required local gates and targeted retests pass. No live messages, provider provisioning or destructive retention actions performed. Tracker preserves external configuration and owner-decision gaps; current-head CI and PR review remain separate.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2602,10 +2602,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F10" s="136" t="str">
-        <x:v>Partially Implemented</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="G10" s="137" t="n">
-        <x:v>0.7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H10" s="136" t="str">
         <x:v>High</x:v>
@@ -2626,10 +2626,10 @@
         <x:v>Boot with missing/valid variables; configuration audit</x:v>
       </x:c>
       <x:c r="N10" s="136" t="str">
-        <x:v>Environment template now documents local/Cloudflare media and rejects unsupported provider values. a96704b moves local storage outside public/. The template still refers to a missing src/lib/env.ts and unused/future settings; comprehensive startup validation is not implemented.</x:v>
+        <x:v>Runtime startup validation and stricter launch CLI implemented and tested. Checks origins, PostgreSQL URL, non-placeholder secret, provider alignment, private-media variables, OAuth pairs and unsafe upload paths without printing values. Removed unused Typesense settings. Current local config passes; launch check correctly reports missing HTTPS/live email/durable media and cron-secret requirements.</x:v>
       </x:c>
       <x:c r="O10" s="136" t="str">
-        <x:v>Audit documented variables against consumers and implement safe startup validation for required deployment settings.</x:v>
+        <x:v>Run npm run check:deployment with the selected deployment configuration; live services remain separately tracked.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2887,7 +2887,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G16" s="137" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H16" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2908,10 +2908,10 @@
         <x:v>Unit; integration; transaction tests</x:v>
       </x:c>
       <x:c r="N16" s="136" t="str">
-        <x:v>Six isolated PostgreSQL checks now include first-admin dry run, eligibility, audit-failure rollback, concurrent first-admin attempts, idempotency and session revocation, alongside reference/facet/rate-limit/upload-claim checks. Browser authorization cases also preserve DB/audit state.</x:v>
+        <x:v>Seven isolated PostgreSQL checks pass, including 105-match alert overflow, queue deduplication, concurrent delivery, immutable retry payloads, opt-out/ban/email changes and expired retry-window suppression, plus bootstrap rollback/serialization and existing ownership/reference/rate-limit checks.</x:v>
       </x:c>
       <x:c r="O16" s="136" t="str">
-        <x:v>Extend transaction fault/concurrency checks to remaining moderation/service and delivery workflows.</x:v>
+        <x:v>Retain the clean CI gate and extend tests when remaining provider/retention decisions are implemented.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2955,7 +2955,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>101 ordinary browser passes + 3 targeted recovery passes (separate runs), 1 planned skip; 6 DB checks; latest sweep 103 URLs, zero issues. Check/lint/final build pass; max First Load JS 128 KB. Framework awaits PR #6 review; current head CI is authoritative.</x:v>
+        <x:v>Browser framework includes six new dealer/tablet/readiness/cron-routing cases. Current targeted runs: 6 launch-gap, 2 report-flow and 3 recovery passes. Earlier full local run had 100 passes and one Chrome resource failure; failed case now passes in both viewports. Latest sweep 101 URLs, zero issues. Current pushed-head CI remains authoritative.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Review PR #6; retain regression coverage. Track additional cases in JW-177 rather than reopening the test-framework implementation.</x:v>
@@ -3968,7 +3968,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G39" s="137" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H39" s="136" t="str">
         <x:v>High</x:v>
@@ -3989,10 +3989,10 @@
         <x:v>1440, 1024, 768, 414, 390, 360 px</x:v>
       </x:c>
       <x:c r="N39" s="136" t="str">
-        <x:v>Reviewed estimate 90%: owner-approved homepage merged via PR #5; automated desktop/mobile route checks and iPhone WebKit smoke pass, including overflow checks. Broader tablet, real-device, keyboard/camera and slow-network visual acceptance remains open.</x:v>
+        <x:v>Desktop/mobile dealer checks and tablet 1024x768 checks pass across home, cars, bikes, parts, dealers and login at 200% text size. Fixed header/footer overflow. Reduced-motion hero/sell visuals are static. Owner-approved homepage remains in place.</x:v>
       </x:c>
       <x:c r="O39" s="136" t="str">
-        <x:v>Complete remaining tablet/real-device visual review and record issues by route.</x:v>
+        <x:v>Real-device, camera/file picker, screen-reader and slow-network HTTPS acceptance remain parked for launch.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -4823,7 +4823,7 @@
         <x:v>Stage 4</x:v>
       </x:c>
       <x:c r="J57" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Product Owner</x:v>
       </x:c>
       <x:c r="K57" s="136" t="str">
         <x:v>Verification fields and admin UI</x:v>
@@ -4835,10 +4835,10 @@
         <x:v>Grant/revoke; badge accuracy; audit log</x:v>
       </x:c>
       <x:c r="N57" s="136" t="str">
-        <x:v>Phone verification timestamp exists but no seller verification workflow/UI.</x:v>
+        <x:v>Manual dealer verification is implemented separately. docs/PROJECT.md explicitly keeps entered phone numbers unverified; individual-seller badge meaning and evidence requirements are not defined. Do not repurpose phone_verified_at or imply SMS/identity verification.</x:v>
       </x:c>
       <x:c r="O57" s="136" t="str">
-        <x:v>Clarify badge field and implement admin controls.</x:v>
+        <x:v>Owner must define individual-seller badge semantics and acceptable manual evidence before adding a public claim.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -6221,10 +6221,10 @@
         <x:v>Signed V1</x:v>
       </x:c>
       <x:c r="F87" s="136" t="str">
-        <x:v>Partially Implemented</x:v>
+        <x:v>Launch Configuration Pending</x:v>
       </x:c>
       <x:c r="G87" s="137" t="n">
-        <x:v>0.65</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H87" s="136" t="str">
         <x:v>Critical</x:v>
@@ -6245,10 +6245,10 @@
         <x:v>Upload/display/delete; credential failure; variants</x:v>
       </x:c>
       <x:c r="N87" s="136" t="str">
-        <x:v>Cloudflare upload/delete adapter and direct delivery URLs exist. a96704b protects local reads only; Cloudflare private/signed delivery is not implemented or verified. Live upload/display/delete and configuration failure acceptance remain open.</x:v>
+        <x:v>Private Cloudflare UUID uploads, response privacy verification, server-only 60-second signing and authorized no-store proxy delivery implemented. Mock provider covers upload/signing/read/delete/configuration and upstream failure. Local shared visibility browser cases pass. docs/PRIVATE_MEDIA.md records old custom-ID migration and variant restrictions. Cloudflare credentials are absent locally.</x:v>
       </x:c>
       <x:c r="O87" s="136" t="str">
-        <x:v>Implement provider-appropriate private delivery before production use; configure staging and verify media lifecycle.</x:v>
+        <x:v>Provide/configure Cloudflare account, token, signing key, hash and private variant; migrate any old public custom IDs and run live upload/read/delete/access acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -6318,7 +6318,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G89" s="137" t="n">
-        <x:v>0.7</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="H89" s="136" t="str">
         <x:v>High</x:v>
@@ -6339,10 +6339,10 @@
         <x:v>LCP; mobile bandwidth; broken URLs; alt text</x:v>
       </x:c>
       <x:c r="N89" s="136" t="str">
-        <x:v>Uploaded images are re-encoded as WebP. Local media now uses direct unoptimized no-store requests to preserve authorization; static site images retain Next optimization. Cloudflare width delivery exists but production dimensions, bandwidth and visual quality are unverified.</x:v>
+        <x:v>Both providers deliver bounded WebP through the authorization endpoint; static assets retain Next optimization. Public provider/optimizer bypasses are removed. Cloudflare private variant and application bandwidth/processing need live measurement; no production media-performance claim.</x:v>
       </x:c>
       <x:c r="O89" s="136" t="str">
-        <x:v>Verify production image transformations and private delivery together; measure mobile media bandwidth/LCP.</x:v>
+        <x:v>Measure real image dimensions, transfer size, LCP and proxy capacity on HTTPS staging; configure bounded private variants.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -7399,7 +7399,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G112" s="137" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="H112" s="136" t="str">
         <x:v>Critical</x:v>
@@ -7420,10 +7420,10 @@
         <x:v>EXPLAIN ANALYZE; 20k listings; 500 concurrent users</x:v>
       </x:c>
       <x:c r="N112" s="136" t="str">
-        <x:v>Indexes are designed; no load/query-plan test has been run.</x:v>
+        <x:v>Rollback-only 10,000-car query-plan sample identified and fixed newest-first index ordering. Final local sample: recent 0.077 ms via listings_recent_idx; city+price 0.103 ms; city count 1.033 ms. See docs/LOCAL_QUERY_PLAN_REPORT.md. Single-run core queries are not full browse/load acceptance.</x:v>
       </x:c>
       <x:c r="O112" s="136" t="str">
-        <x:v>Seed production-like volume and load test.</x:v>
+        <x:v>Repeat full browse joins, deep pagination and concurrent queries on representative staging data and hosting.</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -7878,7 +7878,7 @@
         <x:v>Stage 3</x:v>
       </x:c>
       <x:c r="J122" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Product Owner</x:v>
       </x:c>
       <x:c r="K122" s="136" t="str">
         <x:v>Database</x:v>
@@ -7890,10 +7890,10 @@
         <x:v>Repeated/bot/owner; DB failure; concurrency</x:v>
       </x:c>
       <x:c r="N122" s="136" t="str">
-        <x:v>Basic counter exists and explicitly counts crawler hits.</x:v>
+        <x:v>Raw view counter remains a render counter including repeats/crawlers. docs/OPERATIONS.md explicitly excludes it from unique-visitor and conversion-rate claims.</x:v>
       </x:c>
       <x:c r="O122" s="136" t="str">
-        <x:v>Define view policy and use daily unique aggregation if needed.</x:v>
+        <x:v>Define whether V1 needs unique human views and its privacy/identity policy before changing counting semantics.</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
@@ -8383,10 +8383,10 @@
         <x:v>Signed V1</x:v>
       </x:c>
       <x:c r="F133" s="136" t="str">
-        <x:v>Partially Implemented</x:v>
+        <x:v>Launch Configuration Pending</x:v>
       </x:c>
       <x:c r="G133" s="137" t="n">
-        <x:v>0.4</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H133" s="136" t="str">
         <x:v>High</x:v>
@@ -8407,10 +8407,10 @@
         <x:v>Match accuracy; frequency; duplicates; delivery failure; unsubscribe</x:v>
       </x:c>
       <x:c r="N133" s="136" t="str">
-        <x:v>Reviewed estimate 40%: saved-search alert preferences and authenticated matching cron exist; unique outbox records deduplicate listing/search pairs. No delivery worker/template or delivered_at updater was found. Matching currently reads the first result page, so overflow and retry correctness need acceptance.</x:v>
+        <x:v>Implemented bounded overflow-safe matching and leased delivery worker, immutable email payload/idempotency key, retry/backoff, verified/unbanned recipient checks, current-email/active-listing checks, opt-out suppression and 23-hour reconciliation cutoff. Seven-check DB suite passes with mock sends; no live emails sent. Missing Resend API key/sender confirmed. See docs/ALERT_DELIVERY.md.</x:v>
       </x:c>
       <x:c r="O133" s="136" t="str">
-        <x:v>Implement delivery worker, email template/retry/control flow and complete matching/overflow/deduplication tests, then configure provider and scheduler.</x:v>
+        <x:v>Configure verified Resend sender and credentials, schedule queue/delivery, reconcile initial backlog and verify controlled mailbox/bounce/provider-outage behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -8477,10 +8477,10 @@
         <x:v>Signed V1</x:v>
       </x:c>
       <x:c r="F135" s="136" t="str">
-        <x:v>Partially Implemented</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="G135" s="137" t="n">
-        <x:v>0.9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H135" s="136" t="str">
         <x:v>High</x:v>
@@ -8501,10 +8501,10 @@
         <x:v>Verified/unverified; zero listings; pagination</x:v>
       </x:c>
       <x:c r="N135" s="136" t="str">
-        <x:v>Directory/storefront code and route/accessibility checks pass; admin verification/revocation changes public badges with DB audit assertions. Exact inventory-count, mixed-state and pagination checks remain open.</x:v>
+        <x:v>Desktop/mobile deterministic inventory acceptance passes: 26 active ads, 25+1 disjoint pages, total count independent of page size, stable ordering, invalid page fallback, inactive inventory denial and banned dealer exclusion. Fixed missing storefront pagination and truncated total.</x:v>
       </x:c>
       <x:c r="O135" s="136" t="str">
-        <x:v>Complete T-032 with deterministic mixed-status dealer inventory.</x:v>
+        <x:v>Include dealer inventory in routine release regression; live/device acceptance remains in launch QA.</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
@@ -9890,7 +9890,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G165" s="137" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H165" s="136" t="str">
         <x:v>Medium</x:v>
@@ -9911,10 +9911,10 @@
         <x:v>Build with/without DB; deployment preview</x:v>
       </x:c>
       <x:c r="N165" s="136" t="str">
-        <x:v>Sitemap is force-dynamic, but build still requires DB for page data in this workspace.</x:v>
+        <x:v>docs/DEPLOYMENT.md now explicitly requires a reachable migrated isolated CI or staging/build database; clean migrations, seeds and production build pass. Demo seeds are forbidden against production. Sitemap remains dynamic.</x:v>
       </x:c>
       <x:c r="O165" s="136" t="str">
-        <x:v>Define staging/build database requirements.</x:v>
+        <x:v>Configure the selected build/staging database and verify deployment-network access and sitemap origin.</x:v>
       </x:c>
     </x:row>
     <x:row r="166">
@@ -10360,7 +10360,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G175" s="137" t="n">
-        <x:v>0.3</x:v>
+        <x:v>0.35</x:v>
       </x:c>
       <x:c r="H175" s="136" t="str">
         <x:v>High</x:v>
@@ -10369,7 +10369,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J175" s="136" t="str">
-        <x:v>Backend</x:v>
+        <x:v>Product Owner / DevOps</x:v>
       </x:c>
       <x:c r="K175" s="136" t="str">
         <x:v>Privacy policy and operations</x:v>
@@ -10381,10 +10381,10 @@
         <x:v>Retention job; account deletion; backup implications</x:v>
       </x:c>
       <x:c r="N175" s="136" t="str">
-        <x:v>Reviewed estimate 30%: purge-expired removes expired sessions, reset/verification tokens, old rate-limit buckets and abandoned uploads. Orphan storage cleanup has browser/DB acceptance. Account/report/service-record retention, deletion tooling and backup implications remain undefined/incomplete.</x:v>
+        <x:v>Existing session/token/rate-bucket/orphan cleanup remains. Added a read-only retention inventory with aggregate counts/oldest dates and explicit account/report/service/audit/alert/backup policy decisions in docs/RETENTION_DECISIONS.md. Inventory ran on isolated DB; no customer records exported/deleted.</x:v>
       </x:c>
       <x:c r="O175" s="136" t="str">
-        <x:v>Document retention decisions and implement account/report/service deletion workflows; verify backup handling and scheduled execution.</x:v>
+        <x:v>Approve retention periods, legal holds, anonymization and backup replay rules before destructive lifecycle tooling.</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
@@ -10407,7 +10407,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G176" s="137" t="n">
-        <x:v>0.4</x:v>
+        <x:v>0.55</x:v>
       </x:c>
       <x:c r="H176" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10428,10 +10428,10 @@
         <x:v>OWASP review; dependency; auth; IDOR; upload; headers</x:v>
       </x:c>
       <x:c r="N176" s="136" t="str">
-        <x:v>Reviewed estimate 40%: local review/regressions cover ownership, admin replay, upload content/origin/rate limits, private local reads and dependency audit. CI run 37 passes. Formal infrastructure assessment, remaining action negatives and Cloudflare privacy are not complete; this is not launch security sign-off.</x:v>
+        <x:v>Private provider signing/configuration failures now have mock coverage; cron prototype-name routing is rejected and cron errors no longer expose exception text. Readiness failures are generic; runtime validation redacts values. Alert eligibility/lease/retry controls pass DB tests. Infrastructure/provider and formal review remain open.</x:v>
       </x:c>
       <x:c r="O176" s="136" t="str">
-        <x:v>Finish dealer/service/private-provider assessment and infrastructure review; close critical/high findings with regression evidence.</x:v>
+        <x:v>Review final PR and live provider/proxy/storage/log configuration; close high/critical launch findings.</x:v>
       </x:c>
     </x:row>
     <x:row r="177">
@@ -10663,10 +10663,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>101 ordinary browser passes + 3 targeted recovery passes (separate runs), 1 planned skip; 6 DB checks; latest sweep 103 URLs, zero issues. Check/lint/final build pass; max First Load JS 128 KB. Recovery project is isolated after normal browser projects; forced database failure is restored in cleanup.</x:v>
+        <x:v>Current local evidence: 7 DB checks, static checks/lint/build pass, 101-URL sweep zero issues. Six new launch-gap, two report-flow and three recovery tests pass. Prior full run: 100 passes, one Chrome ERR_INSUFFICIENT_RESOURCES failure (now retested), one planned skip, recovery dependencies not run. About 110 distinct cases have passing local evidence across separate runs; do not label this one full run.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Remaining conditional/edge, provider, slow-network and live-device acceptance; CI on latest head governs PR review.</x:v>
+        <x:v>Current-head clean CI and final provider/real-device/staging acceptance govern sign-off.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -10736,7 +10736,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G183" s="137" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H183" s="136" t="str">
         <x:v>High</x:v>
@@ -10757,10 +10757,10 @@
         <x:v>axe; keyboard; screen reader spot checks</x:v>
       </x:c>
       <x:c r="N183" s="136" t="str">
-        <x:v>Automated axe-core audit covers 34 routes across public, seller, dealer, administrator and car/bike/part detail journeys in both viewports. Fixed low-contrast text and phone CTA, form labels and navigation landmarks. Manual assistive-technology/live-device acceptance remains open.</x:v>
+        <x:v>Existing 34-route axe coverage is supplemented by 200% text sizing at tablet width across six routes and reduced-motion checks. Header/footer overflow found and fixed; desktop/mobile projects pass.</x:v>
       </x:c>
       <x:c r="O183" s="136" t="str">
-        <x:v>Complete manual screen-reader, keyboard, zoom and reduced-motion acceptance, then extend automated scans to remaining conditional form states.</x:v>
+        <x:v>Manual screen-reader, real-device and browser zoom acceptance remain for launch.</x:v>
       </x:c>
     </x:row>
     <x:row r="184">
@@ -10783,7 +10783,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G184" s="137" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H184" s="136" t="str">
         <x:v>High</x:v>
@@ -10804,10 +10804,10 @@
         <x:v>Bundle report; Lighthouse; 4G profile</x:v>
       </x:c>
       <x:c r="N184" s="136" t="str">
-        <x:v>a96704b production build has maximum First Load JS 128 KB, below 150 KB. Production media/Web Vitals and representative query/load acceptance remain open.</x:v>
+        <x:v>Production build remains under the 150 KB JS budget (maximum 128 KB). Local 100-request concurrency-five smoke: zero failures, p50 253 ms, p95 517 ms, max 839 ms. 10,000-row query sample verifies the newest-first index. Reports clearly distinguish local samples from production acceptance.</x:v>
       </x:c>
       <x:c r="O184" s="136" t="str">
-        <x:v>Measure Core Web Vitals and browse query/load behavior on production-like staging before launch.</x:v>
+        <x:v>Measure real media/Web Vitals and representative staging capacity before launch.</x:v>
       </x:c>
     </x:row>
     <x:row r="185">
@@ -10827,10 +10827,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F185" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G185" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="H185" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10851,10 +10851,10 @@
         <x:v>Ramp/soak/spike; query plans; pool limits</x:v>
       </x:c>
       <x:c r="N185" s="136" t="str">
-        <x:v>No load test performed.</x:v>
+        <x:v>Added repeatable loopback-only 100-request concurrency-five HTTP load smoke; zero failures. Synthetic 10,000-row query fixtures roll back. These are local baselines, not the required 500-user ramp/soak.</x:v>
       </x:c>
       <x:c r="O185" s="136" t="str">
-        <x:v>Create dataset and execute before launch.</x:v>
+        <x:v>Run representative 500-user ramp/soak with monitoring on the selected staging infrastructure.</x:v>
       </x:c>
     </x:row>
     <x:row r="186">
@@ -11368,10 +11368,10 @@
         <x:v>Upload/display/delete; cache; failure</x:v>
       </x:c>
       <x:c r="N196" s="136" t="str">
-        <x:v>Cloudflare adapter exists under JW-083, but no durable staging/production media service is verified. Local storage is development-only; private/signed Cloudflare delivery is an unresolved implementation gate.</x:v>
+        <x:v>Private Cloudflare delivery code and mock-provider checks are implemented under JW-083. No account/token/signing key/hash/variant is configured locally; durable staging/production storage and old-object migration are unverified.</x:v>
       </x:c>
       <x:c r="O196" s="136" t="str">
-        <x:v>Complete JW-083 private delivery and configure durable storage; verify upload/read/delete across deployment and restart.</x:v>
+        <x:v>Configure Cloudflare and verify private media lifecycle and persistence across deployment/restart.</x:v>
       </x:c>
     </x:row>
     <x:row r="197">
@@ -11485,10 +11485,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F199" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G199" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="H199" s="136" t="str">
         <x:v>Critical</x:v>
@@ -11509,10 +11509,10 @@
         <x:v>Synthetic error; alert delivery; PII review</x:v>
       </x:c>
       <x:c r="N199" s="136" t="str">
-        <x:v>Only console logging exists.</x:v>
+        <x:v>Next request-error hook emits structured timestamp/method/route-template/category events without request bodies, query strings, cookies or exception messages. Operator runbook documents host collection, access controls and review of separate framework/provider logs.</x:v>
       </x:c>
       <x:c r="O199" s="136" t="str">
-        <x:v>Configure structured logs and error monitoring.</x:v>
+        <x:v>Configure hosted log retention, aggregation and actionable error alerts; test an end-to-end staging alert.</x:v>
       </x:c>
     </x:row>
     <x:row r="200">
@@ -11532,10 +11532,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F200" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G200" s="137" t="n">
-        <x:v>0</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="H200" s="136" t="str">
         <x:v>High</x:v>
@@ -11556,10 +11556,10 @@
         <x:v>Failure simulation; alert escalation</x:v>
       </x:c>
       <x:c r="N200" s="136" t="str">
-        <x:v>Not configured.</x:v>
+        <x:v>Added uncached/noindex /api/health readiness endpoint with DB check and generic 503 failures; success/failure redaction unit checks and desktop/mobile HTTP checks pass.</x:v>
       </x:c>
       <x:c r="O200" s="136" t="str">
-        <x:v>Add after staging is live.</x:v>
+        <x:v>Attach the selected external uptime monitor to HTTPS staging/production and verify notifications.</x:v>
       </x:c>
     </x:row>
     <x:row r="201">
@@ -11629,7 +11629,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G202" s="137" t="n">
-        <x:v>0.4</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="H202" s="136" t="str">
         <x:v>Medium</x:v>
@@ -11638,7 +11638,7 @@
         <x:v>Stage 6</x:v>
       </x:c>
       <x:c r="J202" s="136" t="str">
-        <x:v>Unassigned</x:v>
+        <x:v>Product Owner / DevOps</x:v>
       </x:c>
       <x:c r="K202" s="136" t="str">
         <x:v>Analytics decision/privacy policy</x:v>
@@ -11650,10 +11650,10 @@
         <x:v>Event accuracy; consent; duplicate events</x:v>
       </x:c>
       <x:c r="N202" s="136" t="str">
-        <x:v>Lead events exist; no approved site analytics configuration shown.</x:v>
+        <x:v>docs/OPERATIONS.md defines basic V1 database measures, raw-view limitations and alert acceptance semantics. No external tracker or new analytics identifiers introduced; advanced analytics remains out of scope.</x:v>
       </x:c>
       <x:c r="O202" s="136" t="str">
-        <x:v>Define basic V1 measurement plan.</x:v>
+        <x:v>Approve unique-visitor/consent requirements if needed and configure the chosen operational measurement/reporting process.</x:v>
       </x:c>
     </x:row>
     <x:row r="203">
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdeb9b895c7264867"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re643fa0749274a9d"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12689,13 +12689,13 @@
         <x:v>feature/saved-search-alerts</x:v>
       </x:c>
       <x:c r="E17" s="141" t="str">
-        <x:v>Saved-search management, alert preferences and deduplicated match outbox exist; delivery worker, templates, retry/control and full matching acceptance remain.</x:v>
+        <x:v>Saved-search management plus bounded overflow-safe matching and leased immutable email delivery, retries and eligibility controls implemented and DB-tested with mock sends; provider/scheduler/mailbox acceptance remain.</x:v>
       </x:c>
       <x:c r="F17" s="141" t="str">
         <x:v>Automated matching/overflow/deduplication and delivered-email acceptance pass with configured provider/scheduler.</x:v>
       </x:c>
       <x:c r="G17" s="141" t="str">
-        <x:v>Partially Implemented</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -12850,7 +12850,7 @@
         <x:v>codex/production-readiness (planned)</x:v>
       </x:c>
       <x:c r="E24" s="141" t="str">
-        <x:v>Local hardening has started: upload ownership/privacy, action authorization and cleanup. Production DB/media/backups/cron/logs/domain, formal security/load and live acceptance remain open.</x:v>
+        <x:v>Private-media code, delivery worker, deployment validation, readiness/error events, retention inventory and local query/load baselines implemented. Live hosting/DB/media/mail/backups/cron/monitoring and final security/load acceptance remain.</x:v>
       </x:c>
       <x:c r="F24" s="141" t="str">
         <x:v>Formal launch checklist has no open critical/high issue.</x:v>
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa62385ffe4447ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8482079cb5c04d3f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13765,10 +13765,10 @@
         <x:v>DB integration + E2E</x:v>
       </x:c>
       <x:c r="E36" s="141" t="str">
-        <x:v>Route sweep partial</x:v>
+        <x:v>Desktop/mobile deterministic dealer fixture with 26 active and four inactive listings; pagination, counts, invalid page and banned owner checks</x:v>
       </x:c>
       <x:c r="F36" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Passed local: correct 26 total, disjoint 25+1 pages, inactive detail 404 and banned storefront/directory exclusion</x:v>
       </x:c>
       <x:c r="G36" s="141" t="str">
         <x:v>Mixed dealer listing states</x:v>
@@ -14233,10 +14233,10 @@
         <x:v>Load</x:v>
       </x:c>
       <x:c r="E54" s="141" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Local bounded smoke and rollback-only query-plan fixtures implemented; 500-user staging ramp/soak not run</x:v>
       </x:c>
       <x:c r="F54" s="141" t="str">
-        <x:v>Pre-launch</x:v>
+        <x:v>Partial: 100 requests at concurrency five, zero failures; staging 500-user capacity remains open</x:v>
       </x:c>
       <x:c r="G54" s="141" t="str">
         <x:v>Production-like staging</x:v>
@@ -14259,10 +14259,10 @@
         <x:v>Deployment integration</x:v>
       </x:c>
       <x:c r="E55" s="141" t="str">
-        <x:v>GitHub CI plus local clean isolated DB</x:v>
+        <x:v>Clean isolated migrations/seeding, seven DB checks and current local production build</x:v>
       </x:c>
       <x:c r="F55" s="141" t="str">
-        <x:v>Passed local isolated migrations/seed and CI run 37 on a96704b</x:v>
+        <x:v>Local passed; prior CI run 41 passed; inspect current head for newest migrations/build</x:v>
       </x:c>
       <x:c r="G55" s="141" t="str">
         <x:v>Fresh PostgreSQL</x:v>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4211c38cbb94489b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd836e8b2fba4999"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdab0bcae51d496b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a1d42826397458a"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Isolate saved-alert retry keys across environments
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R883223235ae34cb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rb16a3fd7607b4d08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R90e8436a34774ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Ra1ba5ab418a0437b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R14c2ccf3dc734c18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rcfdcdcc00cd8486b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rf1e3d907a0cd4f23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3a794ce6a12242b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rf224af8e304b439d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rbfd847c6cda64544"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R9aafa6fdbb6740ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rd337dba245f1433d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Ree3720479bbf4c7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R36ae3ee487b44fe4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2305f5278d914b1a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R41d53e89a5084631"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1247,7 +1247,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F5" s="94" t="str">
-        <x:v>Local passed; check current CI</x:v>
+        <x:v>Local + CI passed</x:v>
       </x:c>
       <x:c r="G5" s="92" t="str">
         <x:v>Current branch</x:v>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6 open; prior run 41 passed; latest-head CI pending</x:v>
+        <x:v>PR #6 open; run 42 passed on 254e171; current head checks govern</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>6 new + 2 report retests + 3 recovery pass; see evidence</x:v>
+        <x:v>Full CI acceptance passed; live/device gates open</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>Private media, alert worker, environment validation, dealer/tablet fixes and readiness implemented. 7 DB checks and focused browser tests pass; 101 routes have zero issues. Local full-run resource failure was retested successfully; current-head CI governs review.</x:v>
+        <x:v>GitHub run 42 passed on 254e171: migrations, DB tests, check, lint, build, route sweep, full browser acceptance and production dependency audit. Subsequent alert UUID retry fix passed targeted local DB acceptance/check/lint/build. PR #6 review and current-head CI remain merge gates. Production/provider/device acceptance remains open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01234bc362fe42b7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R403a6448fc074c24"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Autonomous package: private Cloudflare delivery, alert worker, deployment validation, dealer/tablet fixes, readiness/log hooks, retention inventory and local performance baselines. Required local gates and targeted retests pass. No live messages, provider provisioning or destructive retention actions performed. Tracker preserves external configuration and owner-decision gaps; current-head CI and PR review remain separate.</x:v>
+        <x:v>GitHub acceptance run 42 passed on 254e171, including audit, migrations, database tests, check/lint/build, route sweep and browser tests. Alert UUID review fix passes targeted local DB acceptance and required local checks. Each completed package is committed and pushed with this master tracker; PR review/merge, production credentials, owner policy and real-device gates remain separate.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2955,7 +2955,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Browser framework includes six new dealer/tablet/readiness/cron-routing cases. Current targeted runs: 6 launch-gap, 2 report-flow and 3 recovery passes. Earlier full local run had 100 passes and one Chrome resource failure; failed case now passes in both viewports. Latest sweep 101 URLs, zero issues. Current pushed-head CI remains authoritative.</x:v>
+        <x:v>GitHub run 42 passed the complete acceptance pipeline on 254e171: dependency audit, migrations, seed, DB tests, check, lint, build, sweep and browser tests. PR #6 remains open for review; current head checks govern merge.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Review PR #6; retain regression coverage. Track additional cases in JW-177 rather than reopening the test-framework implementation.</x:v>
@@ -8407,10 +8407,10 @@
         <x:v>Match accuracy; frequency; duplicates; delivery failure; unsubscribe</x:v>
       </x:c>
       <x:c r="N133" s="136" t="str">
-        <x:v>Implemented bounded overflow-safe matching and leased delivery worker, immutable email payload/idempotency key, retry/backoff, verified/unbanned recipient checks, current-email/active-listing checks, opt-out suppression and 23-hour reconciliation cutoff. Seven-check DB suite passes with mock sends; no live emails sent. Missing Resend API key/sender confirmed. See docs/ALERT_DELIVERY.md.</x:v>
+        <x:v>Overflow matching, deduplication, concurrent delivery, immutable retry payload/key, eligibility changes and 23-hour retry-window suppression pass in DB acceptance. GitHub run 42 passed the complete acceptance pipeline on 254e171. Subsequent review fix persists random UUID provider keys to avoid staging/production collisions; targeted DB test, check, lint and build pass locally. No live email sent.</x:v>
       </x:c>
       <x:c r="O133" s="136" t="str">
-        <x:v>Configure verified Resend sender and credentials, schedule queue/delivery, reconcile initial backlog and verify controlled mailbox/bounce/provider-outage behavior.</x:v>
+        <x:v>Configure verified Resend sender and credentials, schedule queue/delivery, review initial backlog and complete controlled mailbox, outage and deliverability acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -10663,7 +10663,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Current local evidence: 7 DB checks, static checks/lint/build pass, 101-URL sweep zero issues. Six new launch-gap, two report-flow and three recovery tests pass. Prior full run: 100 passes, one Chrome ERR_INSUFFICIENT_RESOURCES failure (now retested), one planned skip, recovery dependencies not run. About 110 distinct cases have passing local evidence across separate runs; do not label this one full run.</x:v>
+        <x:v>Clean GitHub run 42 on 254e171 passed full browser acceptance, DB tests and route sweep, plus audit/check/lint/build. This supersedes the earlier locally resource-limited combined run. Local targeted alert UUID retry regression also passes; real-provider/device and production load acceptance remain open.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Current-head clean CI and final provider/real-device/staging acceptance govern sign-off.</x:v>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re643fa0749274a9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cd68bf20cdd4c96"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8482079cb5c04d3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa78f65d738c41da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14262,7 +14262,7 @@
         <x:v>Clean isolated migrations/seeding, seven DB checks and current local production build</x:v>
       </x:c>
       <x:c r="F55" s="141" t="str">
-        <x:v>Local passed; prior CI run 41 passed; inspect current head for newest migrations/build</x:v>
+        <x:v>Local migrations and seven DB acceptance tests pass; clean GitHub run 42 on 254e171 also passed migration, seed and DB acceptance. Production database deployment and rollback rehearsal remain open.</x:v>
       </x:c>
       <x:c r="G55" s="141" t="str">
         <x:v>Fresh PostgreSQL</x:v>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd836e8b2fba4999"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b8f001ac6e34bc3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a1d42826397458a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e8775fb475c4709"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Record completed PR review and passing acceptance evidence
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3a794ce6a12242b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rf224af8e304b439d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rbfd847c6cda64544"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R9aafa6fdbb6740ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rd337dba245f1433d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Ree3720479bbf4c7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R36ae3ee487b44fe4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8251b599a86e4b91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rd237775a496245ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R9a8d6f54dc7a453a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R3b8f7040fa1449a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R686944cf1e5f4cda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R69e3d2b91214412c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R4b9a8b029e2f4542"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R41d53e89a5084631"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5207cd1180ca40ad"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6 open; run 42 passed on 254e171; current head checks govern</x:v>
+        <x:v>PR #6: agent review done; run 43 passed on 0569081; merge separate</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Full CI acceptance passed; live/device gates open</x:v>
+        <x:v>Full CI passed; real-device/provider gates open</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>GitHub run 42 passed on 254e171: migrations, DB tests, check, lint, build, route sweep, full browser acceptance and production dependency audit. Subsequent alert UUID retry fix passed targeted local DB acceptance/check/lint/build. PR #6 review and current-head CI remain merge gates. Production/provider/device acceptance remains open.</x:v>
+        <x:v>Application head 0569081 passed full GitHub run 43: audit, migrations, DB tests, check, lint, build, route sweep and browser tests. Agent self-review completed with no additional blocking regression identified; see docs/PR6_REVIEW.md. Review closeout changes docs/tracker only. Maintainer approval/main merge and live launch acceptance remain separate.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1676,7 +1676,7 @@
         <x:v>Complete remaining launch acceptance</x:v>
       </x:c>
       <x:c r="C27" s="110" t="str">
-        <x:v>Remaining: hosting/HTTPS and production DB; live Cloudflare/Resend/Google/Maps acceptance; backups, schedules and external monitoring; retention/individual-seller/measurement decisions; staging load and real-device review. Review PR #6 before merge.</x:v>
+        <x:v>Remaining gates require hosting/provider access, owner retention/verification decisions, HTTPS real-device/screen-reader acceptance and production-like load testing. PR #6 agent review is complete; main merge is separate. Details and required inputs: docs/PR6_REVIEW.md.</x:v>
       </x:c>
       <x:c r="D27" s="88"/>
       <x:c r="E27" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R403a6448fc074c24"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33ef1836ab804494"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>GitHub acceptance run 42 passed on 254e171, including audit, migrations, database tests, check/lint/build, route sweep and browser tests. Alert UUID review fix passes targeted local DB acceptance and required local checks. Each completed package is committed and pushed with this master tracker; PR review/merge, production credentials, owner policy and real-device gates remain separate.</x:v>
+        <x:v>Application head 0569081 passed full GitHub run 43. Agent self-review completed and recorded in docs/PR6_REVIEW.md; no additional blocking regression identified. Review closeout is docs/tracker only. Independent maintainer approval/main merge, live providers, owner policy decisions and real-device/load acceptance remain separate gates.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2955,10 +2955,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>GitHub run 42 passed the complete acceptance pipeline on 254e171: dependency audit, migrations, seed, DB tests, check, lint, build, sweep and browser tests. PR #6 remains open for review; current head checks govern merge.</x:v>
+        <x:v>Full GitHub run 43 passed on 0569081: audit, migrations, seed, DB tests, check, lint, build, sweep and browser acceptance. Agent self-review completed; no additional blocking regression identified. See docs/PR6_REVIEW.md. Maintainer approval/main merge remains separate.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Review PR #6; retain regression coverage. Track additional cases in JW-177 rather than reopening the test-framework implementation.</x:v>
+        <x:v>Maintainer review/merge decision and required repository checks; live acceptance remains tracked separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -8407,7 +8407,7 @@
         <x:v>Match accuracy; frequency; duplicates; delivery failure; unsubscribe</x:v>
       </x:c>
       <x:c r="N133" s="136" t="str">
-        <x:v>Overflow matching, deduplication, concurrent delivery, immutable retry payload/key, eligibility changes and 23-hour retry-window suppression pass in DB acceptance. GitHub run 42 passed the complete acceptance pipeline on 254e171. Subsequent review fix persists random UUID provider keys to avoid staging/production collisions; targeted DB test, check, lint and build pass locally. No live email sent.</x:v>
+        <x:v>Overflow, deduplication, concurrent delivery, immutable UUID retry identity, opt-out/eligibility and retry-window tests pass. Full GitHub run 43 on 0569081 passed, including the cross-environment retry-key fix. No live email sent.</x:v>
       </x:c>
       <x:c r="O133" s="136" t="str">
         <x:v>Configure verified Resend sender and credentials, schedule queue/delivery, review initial backlog and complete controlled mailbox, outage and deliverability acceptance.</x:v>
@@ -10663,7 +10663,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Clean GitHub run 42 on 254e171 passed full browser acceptance, DB tests and route sweep, plus audit/check/lint/build. This supersedes the earlier locally resource-limited combined run. Local targeted alert UUID retry regression also passes; real-provider/device and production load acceptance remain open.</x:v>
+        <x:v>Full GitHub run 43 passed on 0569081, including DB and browser acceptance, sweep, audit/check/lint/build. Agent review found no additional blocking regression in reviewed changes. Live/provider/real-device acceptance remains open.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Current-head clean CI and final provider/real-device/staging acceptance govern sign-off.</x:v>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cd68bf20cdd4c96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfb8003d4ed342a2"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa78f65d738c41da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e094b05eb3b4a05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14262,7 +14262,7 @@
         <x:v>Clean isolated migrations/seeding, seven DB checks and current local production build</x:v>
       </x:c>
       <x:c r="F55" s="141" t="str">
-        <x:v>Local migrations and seven DB acceptance tests pass; clean GitHub run 42 on 254e171 also passed migration, seed and DB acceptance. Production database deployment and rollback rehearsal remain open.</x:v>
+        <x:v>Local migrations/seven DB acceptance tests pass; full GitHub run 43 on 0569081 passed fresh migration, seed and DB acceptance. Production database deployment and rollback rehearsal remain open.</x:v>
       </x:c>
       <x:c r="G55" s="141" t="str">
         <x:v>Fresh PostgreSQL</x:v>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b8f001ac6e34bc3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47bf664d1fdd444f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e8775fb475c4709"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R352d2442d2df4d45"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Record approved B1 seller badge scope decision
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8251b599a86e4b91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rd237775a496245ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R9a8d6f54dc7a453a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R3b8f7040fa1449a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R686944cf1e5f4cda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R69e3d2b91214412c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R4b9a8b029e2f4542"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5312edaa44224833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R5be7687a33f144ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Ra6d1309520a94290"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rfa9406aee0ca4b3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R3c8819a97a414358"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Raa04f910a0ac4a59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R5cc02daa92c241dc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5207cd1180ca40ad"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R04a8acfffe874e6a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1237,7 +1237,7 @@
       </x:c>
       <x:c r="B5" s="91" t="n">
         <x:f>COUNTIFS('Feature Tracker'!$A$5:$A$215,"&lt;&gt;",'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request",'Feature Tracker'!$F$5:$F$215,"&lt;&gt;Out of Scope / Removed")</x:f>
-        <x:v>200</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="C5" s="88"/>
       <x:c r="D5" s="92" t="str">
@@ -1334,7 +1334,7 @@
         <x:v>Next functionality</x:v>
       </x:c>
       <x:c r="H8" s="98" t="str">
-        <x:v>Live providers/hosting, retention and verification decisions</x:v>
+        <x:v>Live hosting/providers and client retention decision</x:v>
       </x:c>
       <x:c r="I8" s="98"/>
       <x:c r="J8" s="99"/>
@@ -1372,7 +1372,7 @@
       </x:c>
       <x:c r="B10" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C10" s="88"/>
       <x:c r="D10" s="97" t="str">
@@ -1399,7 +1399,7 @@
       </x:c>
       <x:c r="B11" s="142" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request",'Feature Tracker'!$F$5:$F$215,"&lt;&gt;Out of Scope / Removed")/B5</x:f>
-        <x:v>0.9262</x:v>
+        <x:v>0.930854271356784</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1544,7 +1544,7 @@
       </x:c>
       <x:c r="B19" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Pending")</x:f>
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C19" s="110" t="str">
         <x:v>No implemented delivery for this feature; see row-specific prerequisites</x:v>
@@ -1563,7 +1563,7 @@
       </x:c>
       <x:c r="B20" s="111" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Out of Scope / Removed")</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C20" s="112" t="str">
         <x:v>Deliberately removed; do not build without signed change</x:v>
@@ -1676,7 +1676,7 @@
         <x:v>Complete remaining launch acceptance</x:v>
       </x:c>
       <x:c r="C27" s="110" t="str">
-        <x:v>Remaining gates require hosting/provider access, owner retention/verification decisions, HTTPS real-device/screen-reader acceptance and production-like load testing. PR #6 agent review is complete; main merge is separate. Details and required inputs: docs/PR6_REVIEW.md.</x:v>
+        <x:v>B1 approved 4 October: no ordinary-seller badge; JW-053 removed from V1. Retention decision A awaits client confirmation. Remaining gates: hosting/provider access, HTTPS real-device/screen-reader acceptance, production-like load and main merge decision.</x:v>
       </x:c>
       <x:c r="D27" s="88"/>
       <x:c r="E27" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33ef1836ab804494"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff4f8f83d7a34f89"/>
 </x:worksheet>
 </file>
 
@@ -4808,10 +4808,10 @@
         <x:v>Admin-controlled verified seller status and badge</x:v>
       </x:c>
       <x:c r="E57" s="136" t="str">
-        <x:v>Signed V1</x:v>
+        <x:v>Excluded / Change Request</x:v>
       </x:c>
       <x:c r="F57" s="136" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Out of Scope / Removed</x:v>
       </x:c>
       <x:c r="G57" s="137" t="n">
         <x:v>0</x:v>
@@ -4835,10 +4835,10 @@
         <x:v>Grant/revoke; badge accuracy; audit log</x:v>
       </x:c>
       <x:c r="N57" s="136" t="str">
-        <x:v>Manual dealer verification is implemented separately. docs/PROJECT.md explicitly keeps entered phone numbers unverified; individual-seller badge meaning and evidence requirements are not defined. Do not repurpose phone_verified_at or imply SMS/identity verification.</x:v>
+        <x:v>Owner approved B1 on 4 October 2026: no ordinary-seller Verified Seller badge in V1. Removed by explicit owner decision, not implemented. Email/phone/vehicle ownership claims must not be inferred. Audited manual dealer verification remains separately implemented.</x:v>
       </x:c>
       <x:c r="O57" s="136" t="str">
-        <x:v>Owner must define individual-seller badge semantics and acceptable manual evidence before adding a public claim.</x:v>
+        <x:v>No V1 implementation required. Any future individual-seller badge requires a new approved verification process and scope decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfb8003d4ed342a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a7c489511c64567"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e094b05eb3b4a05"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R266e724d08a94f1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47bf664d1fdd444f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c1105466e4f45e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R352d2442d2df4d45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14de4ec440264d74"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Implement approved account retention and recovery policy
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5312edaa44224833"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R5be7687a33f144ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Ra6d1309520a94290"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rfa9406aee0ca4b3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R3c8819a97a414358"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Raa04f910a0ac4a59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R5cc02daa92c241dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Red436dfd7a42468d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R9ae71f0a3ecc44ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rf88d032a75f84dff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R85236752210d42bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R3a47c3eaf4c84c3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Ra1d18c9ac3214569"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rc9abda3f7827484b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R04a8acfffe874e6a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1a278880e6c74122"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1247,7 +1247,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F5" s="94" t="str">
-        <x:v>Local + CI passed</x:v>
+        <x:v>Local check/build passed; current PR CI pending</x:v>
       </x:c>
       <x:c r="G5" s="92" t="str">
         <x:v>Current branch</x:v>
@@ -1274,7 +1274,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F6" s="99" t="str">
-        <x:v>No local lint warnings/errors</x:v>
+        <x:v>No lint warnings/errors</x:v>
       </x:c>
       <x:c r="G6" s="97" t="str">
         <x:v>Current stage</x:v>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6: agent review done; run 43 passed on 0569081; merge separate</x:v>
+        <x:v>PR #6 open; retention added; merge separate</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1334,7 +1334,7 @@
         <x:v>Next functionality</x:v>
       </x:c>
       <x:c r="H8" s="98" t="str">
-        <x:v>Live hosting/providers and client retention decision</x:v>
+        <x:v>Live hosting/providers, backup and retention rollout</x:v>
       </x:c>
       <x:c r="I8" s="98"/>
       <x:c r="J8" s="99"/>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Full CI passed; real-device/provider gates open</x:v>
+        <x:v>9 DB + 4 retention browser passes; live gates open</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1399,7 +1399,7 @@
       </x:c>
       <x:c r="B11" s="142" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request",'Feature Tracker'!$F$5:$F$215,"&lt;&gt;Out of Scope / Removed")/B5</x:f>
-        <x:v>0.930854271356784</x:v>
+        <x:v>0.9346231155778895</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>Application head 0569081 passed full GitHub run 43: audit, migrations, DB tests, check, lint, build, route sweep and browser tests. Agent self-review completed with no additional blocking regression identified; see docs/PR6_REVIEW.md. Review closeout changes docs/tracker only. Maintainer approval/main merge and live launch acceptance remain separate.</x:v>
+        <x:v>5 October retention milestone: 9 isolated DB tests, 4 targeted desktop/mobile browser passes, check/lint/build and 101-route sweep zero issues. Max First Load JS 128 KB. Account recovery, complaint holds, calendar retention, early deletion, provider retries and restore replay verified. Current PR CI governs full regression acceptance; production/device gates remain.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1676,7 +1676,7 @@
         <x:v>Complete remaining launch acceptance</x:v>
       </x:c>
       <x:c r="C27" s="110" t="str">
-        <x:v>B1 approved 4 October: no ordinary-seller badge; JW-053 removed from V1. Retention decision A awaits client confirmation. Remaining gates: hosting/provider access, HTTPS real-device/screen-reader acceptance, production-like load and main merge decision.</x:v>
+        <x:v>A and B1 approved. Approved retention development implemented and local DB updated. Next: configure production hosting/DB/media/mail, scheduling and monitoring; verify 30-day backups/deletion replay, HTTPS real-device/screen-reader and production-like load; main merge remains separate.</x:v>
       </x:c>
       <x:c r="D27" s="88"/>
       <x:c r="E27" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff4f8f83d7a34f89"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3f846a2e6954d62"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>Application head 0569081 passed full GitHub run 43. Agent self-review completed and recorded in docs/PR6_REVIEW.md; no additional blocking regression identified. Review closeout is docs/tracker only. Independent maintainer approval/main merge, live providers, owner policy decisions and real-device/load acceptance remain separate gates.</x:v>
+        <x:v>5 October: approved A retention development implemented and locally verified; workflow remains commit/push/update tracker automatically after verification. Local: 9 DB, 4 targeted retention browser cases and 101-route sweep zero issues; check/lint/build pass. Full current PR CI and production provider/backup/device acceptance remain separate.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -10313,7 +10313,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G174" s="137" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="H174" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10334,10 +10334,10 @@
         <x:v>Legal review; link availability; consent flows</x:v>
       </x:c>
       <x:c r="N174" s="136" t="str">
-        <x:v>Privacy Policy is live and linked. A final provider/data-retention review and any required consent UI remain for launch hardening.</x:v>
+        <x:v>Published privacy policy now states client-approved account recovery, 12/24-month retention, 90-day activity and 30-day backup policy, necessary holds and no inactivity-only account deletion. Closure/recovery linked in account settings and locally accepted on desktop/mobile. Final live provider disclosures/consent acceptance remains.</x:v>
       </x:c>
       <x:c r="O174" s="136" t="str">
-        <x:v>Validate final provider disclosures and consent requirements before production launch.</x:v>
+        <x:v>Validate actual provider disclosures, legal/consent requirements and production privacy operation before launch.</x:v>
       </x:c>
     </x:row>
     <x:row r="175">
@@ -10360,7 +10360,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G175" s="137" t="n">
-        <x:v>0.35</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H175" s="136" t="str">
         <x:v>High</x:v>
@@ -10381,10 +10381,10 @@
         <x:v>Retention job; account deletion; backup implications</x:v>
       </x:c>
       <x:c r="N175" s="136" t="str">
-        <x:v>Existing session/token/rate-bucket/orphan cleanup remains. Added a read-only retention inventory with aggregate counts/oldest dates and explicit account/report/service/audit/alert/backup policy decisions in docs/RETENTION_DECISIONS.md. Inventory ran on isolated DB; no customer records exported/deleted.</x:v>
+        <x:v>Client approved decision A exactly on 4 October 2026. Implemented immediate account hide/session revocation/alert stop, authenticated 30-day recovery, 12-month listing/service redaction, 24-month resolved evidence retention, 90-day payload clearing/anonymous usage aggregation, accountable complaint holds with 90-day review, approved early deletion, retryable media queue and independent restore ledger/replay. 5 October local acceptance: 9 DB tests, 4 desktop/mobile retention browser tests, 101-route sweep zero issues; check/lint/build pass. Normal local migrations applied. Production cleanup not run.</x:v>
       </x:c>
       <x:c r="O175" s="136" t="str">
-        <x:v>Approve retention periods, legal holds, anonymization and backup replay rules before destructive lifecycle tooling.</x:v>
+        <x:v>Configure authenticated cleanup/media/export scheduling and exact DB guard; verify live provider deletion, actual rolling 30-day backups, restricted hold records and mandatory restore replay drill before launch.</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a7c489511c64567"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b16984665464ed2"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R266e724d08a94f1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R414e54593fb548d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c1105466e4f45e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6ba15bedf2d48c8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14de4ec440264d74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b288106d69a4c4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Prevent restored deletion ledgers from reusing record identities
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Red436dfd7a42468d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R9ae71f0a3ecc44ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rf88d032a75f84dff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R85236752210d42bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R3a47c3eaf4c84c3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Ra1d18c9ac3214569"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rc9abda3f7827484b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rabf5e68fd91542e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R08934402cce04a4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Ra224a4ac3811484f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R98dc6a706a654ea5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R767d59477bc14722"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Re1bbbbe08b7441e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R7615466d24404a9d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1a278880e6c74122"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R78e006b3081a4669"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1247,7 +1247,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F5" s="94" t="str">
-        <x:v>Local check/build passed; current PR CI pending</x:v>
+        <x:v>Local passed; CI run 46 passed; latest PR checks govern</x:v>
       </x:c>
       <x:c r="G5" s="92" t="str">
         <x:v>Current branch</x:v>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6 open; retention added; merge separate</x:v>
+        <x:v>PR #6 open; full run 46 passed; latest head checks govern</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1355,13 +1355,13 @@
         <x:v>Local passed</x:v>
       </x:c>
       <x:c r="F9" s="99" t="str">
-        <x:v>7 DB checks pass; live deployment checks remain</x:v>
+        <x:v>9 DB checks pass; live deployment checks remain</x:v>
       </x:c>
       <x:c r="G9" s="97" t="str">
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>9 DB + 4 retention browser passes; live gates open</x:v>
+        <x:v>Full CI run 46 passed; 4 new retention cases; live gates open</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>5 October retention milestone: 9 isolated DB tests, 4 targeted desktop/mobile browser passes, check/lint/build and 101-route sweep zero issues. Max First Load JS 128 KB. Account recovery, complaint holds, calendar retention, early deletion, provider retries and restore replay verified. Current PR CI governs full regression acceptance; production/device gates remain.</x:v>
+        <x:v>5 October: application 279bd8b passed full GitHub run 46, including audit, migrations, 9 DB tests, check/lint/build, route sweep and full browser regression. Four targeted retention desktop/mobile cases also pass locally. Additional restore-ID reservation test passes; latest PR checks govern the updated head. Max First Load JS 128 KB. Production provider/backup/device acceptance remains.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3f846a2e6954d62"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8966540965245cb"/>
 </x:worksheet>
 </file>
 
@@ -10381,7 +10381,7 @@
         <x:v>Retention job; account deletion; backup implications</x:v>
       </x:c>
       <x:c r="N175" s="136" t="str">
-        <x:v>Client approved decision A exactly on 4 October 2026. Implemented immediate account hide/session revocation/alert stop, authenticated 30-day recovery, 12-month listing/service redaction, 24-month resolved evidence retention, 90-day payload clearing/anonymous usage aggregation, accountable complaint holds with 90-day review, approved early deletion, retryable media queue and independent restore ledger/replay. 5 October local acceptance: 9 DB tests, 4 desktop/mobile retention browser tests, 101-route sweep zero issues; check/lint/build pass. Normal local migrations applied. Production cleanup not run.</x:v>
+        <x:v>Decision A approved exactly. Implemented 30-day authenticated recovery, immediate public hide/session revocation/alerts stop, 12/24-month calendar retention, 90-day payload clearing/anonymous totals, necessary complaint holds with review, approved early deletion, retryable media queue and independent restore ledger. Local: 9 DB checks, 4 desktop/mobile retention cases, 101-route sweep zero issues, check/lint/build pass. Full GitHub run 46 passed on 279bd8b. Additional restore sequence-ID reservation fix passes both retention DB cases; latest PR checks govern the updated head. Normal local migrations applied; production cleanup not run.</x:v>
       </x:c>
       <x:c r="O175" s="136" t="str">
         <x:v>Configure authenticated cleanup/media/export scheduling and exact DB guard; verify live provider deletion, actual rolling 30-day backups, restricted hold records and mandatory restore replay drill before launch.</x:v>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b16984665464ed2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R125ac9a28a934561"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12850,7 +12850,7 @@
         <x:v>codex/production-readiness (planned)</x:v>
       </x:c>
       <x:c r="E24" s="141" t="str">
-        <x:v>Private-media code, delivery worker, deployment validation, readiness/error events, retention inventory and local query/load baselines implemented. Live hosting/DB/media/mail/backups/cron/monitoring and final security/load acceptance remain.</x:v>
+        <x:v>Private media, alert worker, deployment validation/readiness/error events, client-approved retention/closure/recovery/holds/early deletion/media retry/deletion replay and local query/load baselines implemented. Run 46 full CI passed; latest PR checks govern updated head. Live hosting/DB/media/mail/backups/cron/monitoring, restore drill and final security/load acceptance remain.</x:v>
       </x:c>
       <x:c r="F24" s="141" t="str">
         <x:v>Formal launch checklist has no open critical/high issue.</x:v>
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R414e54593fb548d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2500f561729c4e51"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14285,10 +14285,10 @@
         <x:v>Operational</x:v>
       </x:c>
       <x:c r="E56" s="141" t="str">
-        <x:v>Not run</x:v>
+        <x:v>Local deletion replay and ID-reservation pass; production backup drill not run</x:v>
       </x:c>
       <x:c r="F56" s="141" t="str">
-        <x:v>Pre-launch</x:v>
+        <x:v>Pre-launch: configure actual 30-day backups, current ledger/hold recovery and production-like restore smoke</x:v>
       </x:c>
       <x:c r="G56" s="141" t="str">
         <x:v>Production-like backup</x:v>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6ba15bedf2d48c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbef5d6b901d84a3b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b288106d69a4c4b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53355879638a4140"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Close local security lifecycle search and operations gaps
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rabf5e68fd91542e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R08934402cce04a4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Ra224a4ac3811484f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R98dc6a706a654ea5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R767d59477bc14722"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Re1bbbbe08b7441e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R7615466d24404a9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R05d40645a3c04c9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R2ce7ccc08bc94cc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rc0a69308994f45ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R591709f00eb3459c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R3f2f7839cbde40f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R6f1b4b7399bf44ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Raa9a66fc6bd4496f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R78e006b3081a4669"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Red60ef7747f04bed"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1264,7 +1264,7 @@
       </x:c>
       <x:c r="B6" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>156</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="C6" s="88"/>
       <x:c r="D6" s="97" t="str">
@@ -1318,7 +1318,7 @@
       </x:c>
       <x:c r="B8" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C8" s="88"/>
       <x:c r="D8" s="97" t="str">
@@ -1334,7 +1334,7 @@
         <x:v>Next functionality</x:v>
       </x:c>
       <x:c r="H8" s="98" t="str">
-        <x:v>Live hosting/providers, backup and retention rollout</x:v>
+        <x:v>Production access/providers and independent launch acceptance</x:v>
       </x:c>
       <x:c r="I8" s="98"/>
       <x:c r="J8" s="99"/>
@@ -1355,13 +1355,13 @@
         <x:v>Local passed</x:v>
       </x:c>
       <x:c r="F9" s="99" t="str">
-        <x:v>9 DB checks pass; live deployment checks remain</x:v>
+        <x:v>13 isolated DB cases; live acceptance open</x:v>
       </x:c>
       <x:c r="G9" s="97" t="str">
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Full CI run 46 passed; 4 new retention cases; live gates open</x:v>
+        <x:v>6 new local browser cases; 13 DB checks; latest CI governs</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1399,7 +1399,7 @@
       </x:c>
       <x:c r="B11" s="142" t="n">
         <x:f>SUMIFS('Feature Tracker'!$G$5:$G$215,'Feature Tracker'!$E$5:$E$215,"&lt;&gt;Excluded / Change Request",'Feature Tracker'!$F$5:$F$215,"&lt;&gt;Out of Scope / Removed")/B5</x:f>
-        <x:v>0.9346231155778895</x:v>
+        <x:v>0.9415075376884421</x:v>
       </x:c>
       <x:c r="C11" s="88"/>
       <x:c r="D11" s="102" t="str">
@@ -1468,7 +1468,7 @@
       </x:c>
       <x:c r="B15" s="106" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>156</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="C15" s="107" t="str">
         <x:v>Implemented and available in current code; does not mean production launch approval</x:v>
@@ -1506,7 +1506,7 @@
       </x:c>
       <x:c r="B17" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Partially Implemented")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Data Layer Only")+COUNTIF('Feature Tracker'!$F$5:$F$215,"Launch Configuration Pending")</x:f>
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C17" s="110" t="str">
         <x:v>Partly implemented or awaiting configuration/acceptance</x:v>
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>5 October: application 279bd8b passed full GitHub run 46, including audit, migrations, 9 DB tests, check/lint/build, route sweep and full browser regression. Four targeted retention desktop/mobile cases also pass locally. Additional restore-ID reservation test passes; latest PR checks govern the updated head. Max First Load JS 128 KB. Production provider/backup/device acceptance remains.</x:v>
+        <x:v>5 October autonomous closeout: local check/lint/build, 101-route sweep, 6 new desktop/mobile action cases and 13 DB checks pass. Security/lifecycle gaps, paginated browse performance and private aggregate operations report addressed. Prior full CI run 47 passed; latest-head CI governs review. Production/provider/device acceptance remains.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1676,7 +1676,7 @@
         <x:v>Complete remaining launch acceptance</x:v>
       </x:c>
       <x:c r="C27" s="110" t="str">
-        <x:v>A and B1 approved. Approved retention development implemented and local DB updated. Next: configure production hosting/DB/media/mail, scheduling and monitoring; verify 30-day backups/deletion replay, HTTPS real-device/screen-reader and production-like load; main merge remains separate.</x:v>
+        <x:v>Application work completed where access permits. Owner steps and handoff are in docs/OWNER_LAUNCH_ACTIONS.md: hosting/DB/DNS, Cloudflare/Resend, enabled Google configuration, backups/ledger/monitoring, independent PR review and protected main, actual devices and representative 500-user staging load. A/B1 remain approved.</x:v>
       </x:c>
       <x:c r="D27" s="88"/>
       <x:c r="E27" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8966540965245cb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59f14799e7e644d0"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>5 October: approved A retention development implemented and locally verified; workflow remains commit/push/update tracker automatically after verification. Local: 9 DB, 4 targeted retention browser cases and 101-route sweep zero issues; check/lint/build pass. Full current PR CI and production provider/backup/device acceptance remain separate.</x:v>
+        <x:v>5 October: autonomous security/lifecycle/search/operations package added with local check/lint/build, sweep and DB/browser verification. Master tracker preserves production/provider/device gaps. See OWNER_LAUNCH_ACTIONS.md for access/test handoff; feature push is separate from review/main merge.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2884,10 +2884,10 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F16" s="136" t="str">
-        <x:v>Partially Implemented</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="G16" s="137" t="n">
-        <x:v>0.9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H16" s="136" t="str">
         <x:v>Critical</x:v>
@@ -2908,10 +2908,10 @@
         <x:v>Unit; integration; transaction tests</x:v>
       </x:c>
       <x:c r="N16" s="136" t="str">
-        <x:v>Seven isolated PostgreSQL checks pass, including 105-match alert overflow, queue deduplication, concurrent delivery, immutable retry payloads, opt-out/ban/email changes and expired retry-window suppression, plus bootstrap rollback/serialization and existing ownership/reference/rate-limit checks.</x:v>
+        <x:v>Isolated PostgreSQL integration framework covers publishing facets, ownership, bootstrap rollback/concurrency, alerts retries/overflow, retention/replay, aggregate reporting, origin guards, limiter recovery and sorted browse pagination. 13 DB cases; provider and production acceptance remain in their own rows.</x:v>
       </x:c>
       <x:c r="O16" s="136" t="str">
-        <x:v>Retain the clean CI gate and extend tests when remaining provider/retention decisions are implemented.</x:v>
+        <x:v>Maintain regression coverage as product/provider changes occur; no framework implementation gap remains.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -4485,7 +4485,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G50" s="137" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H50" s="136" t="str">
         <x:v>Critical</x:v>
@@ -4506,10 +4506,10 @@
         <x:v>Cross-origin forms; origin/host mismatch</x:v>
       </x:c>
       <x:c r="N50" s="136" t="str">
-        <x:v>Upload POST now compares Origin with the incoming Host and rejects mismatches. Authenticated desktop/mobile Chromium test confirms foreign-origin 403 while valid uploads still succeed. Next server actions keep their built-in origin/session protections.</x:v>
+        <x:v>Configured scheme/host/port Origin checks reject foreign, opaque, path/userinfo and spoofed-Host origins; cross-site Fetch Metadata rejected. Browser direct seller action cross-origin replay rejected. Next server-action protection and upload route guard retained.</x:v>
       </x:c>
       <x:c r="O50" s="136" t="str">
-        <x:v>Review remaining state-changing routes and proxy host configuration in staging; complete final cross-origin assessment.</x:v>
+        <x:v>Verify trusted proxy/public origin configuration and cross-origin rejection on HTTPS staging.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -7352,7 +7352,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G111" s="137" t="n">
-        <x:v>0.95</x:v>
+        <x:v>0.97</x:v>
       </x:c>
       <x:c r="H111" s="136" t="str">
         <x:v>High</x:v>
@@ -7373,10 +7373,10 @@
         <x:v>Empty DB; query failure; slow response</x:v>
       </x:c>
       <x:c r="N111" s="136" t="str">
-        <x:v>Cars, bikes and parts friendly error/clear-filter controls and post-restoration retry pass with real database-read fault injection. Fixed Try again retaining failed server data by refreshing before boundary reset. Three targeted browser cases pass on final build.</x:v>
+        <x:v>Existing real DB failure/recovery acceptance retained; delayed seller action shows pending state and disables repeat clicks in desktop/mobile. Explicit exhausted write-limit notice displayed.</x:v>
       </x:c>
       <x:c r="O111" s="136" t="str">
-        <x:v>Complete slow-network, provider-outage and real-device/loading acceptance.</x:v>
+        <x:v>Real slow-network/device and live provider-outage acceptance remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -7399,7 +7399,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G112" s="137" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H112" s="136" t="str">
         <x:v>Critical</x:v>
@@ -7420,10 +7420,10 @@
         <x:v>EXPLAIN ANALYZE; 20k listings; 500 concurrent users</x:v>
       </x:c>
       <x:c r="N112" s="136" t="str">
-        <x:v>Rollback-only 10,000-car query-plan sample identified and fixed newest-first index ordering. Final local sample: recent 0.077 ms via listings_recent_idx; city+price 0.103 ms; city count 1.033 ms. See docs/LOCAL_QUERY_PLAN_REPORT.md. Single-run core queries are not full browse/load acceptance.</x:v>
+        <x:v>Pagination now precedes browse enrichment; indexed correlated primary photo replaces full-image aggregate. Rollback-only 20,000-ad full-query benchmark covers car/bike/part first and offset-5000 pages; first-page 127-152 ms to 1.4-2.4 ms, deep pages 141-221 ms to 34-44 ms locally. DB compares six sorts/two pages/all verticals including NULL/ties and duplicate-position photo. See LOCAL_QUERY_PLAN_REPORT.md.</x:v>
       </x:c>
       <x:c r="O112" s="136" t="str">
-        <x:v>Repeat full browse joins, deep pagination and concurrent queries on representative staging data and hosting.</x:v>
+        <x:v>Repeat concurrent full-query benchmark on representative HTTPS staging host/data; local query measurements are not 500-user capacity acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -10031,7 +10031,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G168" s="137" t="n">
-        <x:v>0.85</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H168" s="136" t="str">
         <x:v>High</x:v>
@@ -10052,10 +10052,10 @@
         <x:v>All statuses; canonical; sitemap/search exclusion</x:v>
       </x:c>
       <x:c r="N168" s="136" t="str">
-        <x:v>Reviewed estimate 85%: docs/PROJECT.md and shared visibility policy define active-only public details; inactive owner/admin views are noindexed. Static policy checks and public pending/removed browser denial pass. Media GET/HEAD checks now cover every inactive status. Full listing lifecycle/crawler deployment acceptance remains.</x:v>
+        <x:v>Desktop/mobile seller acceptance checks sold ad anonymous detail 404, exclusion from recent search and sitemap, seller deletion preserving approved private photos, owner photo denial/admin positive control, and stale sold action unable to resurrect removed ad.</x:v>
       </x:c>
       <x:c r="O168" s="136" t="str">
-        <x:v>Test sold/expired detail, search and sitemap transitions end to end on staging; preserve the documented active-only public policy.</x:v>
+        <x:v>Verify expiry/sold/deleted lifecycle and live provider visibility on staging with configured scheduling.</x:v>
       </x:c>
     </x:row>
     <x:row r="169">
@@ -10125,7 +10125,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G170" s="137" t="n">
-        <x:v>0.96</x:v>
+        <x:v>0.98</x:v>
       </x:c>
       <x:c r="H170" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10146,10 +10146,10 @@
         <x:v>IDOR; direct action calls; cross-user access</x:v>
       </x:c>
       <x:c r="N170" s="136" t="str">
-        <x:v>Local photo/action coverage includes direct dealer verify/revoke and inspection/assistance update replay: non-admin/anonymous actors cannot mutate records/audits; owners also cannot perform service-admin changes. Identical administrator payload succeeds. Customer records/private notes remain isolated. Prior owner listing/media regressions pass.</x:v>
+        <x:v>New direct-action cases cover shared write limits, foreign Origin, invalid admin enums/IDs/reason length, triple concurrent identical removal with one audit, stale seller action, private deleted media and complaint-hold edit preserving fields/photos. Row locks and conditional status updates protect concurrent transitions; prior auth/provider/mock acceptance retained.</x:v>
       </x:c>
       <x:c r="O170" s="136" t="str">
-        <x:v>Complete remaining action/edge/concurrency matrix and provider/infrastructure security review; Cloudflare private delivery remains in JW-083.</x:v>
+        <x:v>Independent final PR security review and live provider/proxy/storage acceptance; actual devices remain separate.</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -10172,7 +10172,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G171" s="137" t="n">
-        <x:v>0.97</x:v>
+        <x:v>0.99</x:v>
       </x:c>
       <x:c r="H171" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10193,10 +10193,10 @@
         <x:v>Tampered forms; oversized text; invalid IDs</x:v>
       </x:c>
       <x:c r="N171" s="136" t="str">
-        <x:v>Audited user-input Zod constraints across car, bike, parts, inspection, assistance, dealer, account and saved-search actions. Missing integer, bound and enum messages now explain corrections; malformed city/variant IDs have regression checks. Full check, lint, production build and 97-route local sweep pass.</x:v>
+        <x:v>Runtime moderation/listing/user/dealer decision checks added beyond TypeScript types. Direct browser action invalid enum/negative ID/oversize reason cases preserve DB state; complaint-hold edit returns clear error without changing evidence.</x:v>
       </x:c>
       <x:c r="O171" s="136" t="str">
-        <x:v>Complete direct server-action tampering/browser negative matrix for auth, edits, deletes and admin permissions in JW-166/JW-177.</x:v>
+        <x:v>Retain local negative regression; verify final live integrations/configuration before sign-off.</x:v>
       </x:c>
     </x:row>
     <x:row r="172">
@@ -10219,7 +10219,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G172" s="137" t="n">
-        <x:v>0.98</x:v>
+        <x:v>0.99</x:v>
       </x:c>
       <x:c r="H172" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10240,10 +10240,10 @@
         <x:v>Per-IP/user; proxy spoof; reset; fail-open/closed</x:v>
       </x:c>
       <x:c r="N172" s="136" t="str">
-        <x:v>Shared PostgreSQL limits now cover authentication, OAuth start, uploads, contact, reports, manual-service requests, ad publication, account profile/password/avatar and dealer registration/profile/logo. Fresh desktop/mobile browser tests verify denied account/dealer writes preserve database state; atomic concurrency DB test passes.</x:v>
+        <x:v>Shared seller/admin write quotas cover edits, sold/delete/reactivation/resubmission, moderation, bans, dealer verification, manual services, retention holds and avatar/logo removal. Exhaustion preserves state/audit, next-window recovery DB check passes; quota notices displayed.</x:v>
       </x:c>
       <x:c r="O172" s="136" t="str">
-        <x:v>Validate trusted proxy IP headers, thresholds, expiry recovery and security alerts in staging; review remaining remove and administrator write actions.</x:v>
+        <x:v>Validate trusted proxy IP handling, production thresholds and operational alerts on staging.</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -10381,10 +10381,10 @@
         <x:v>Retention job; account deletion; backup implications</x:v>
       </x:c>
       <x:c r="N175" s="136" t="str">
-        <x:v>Decision A approved exactly. Implemented 30-day authenticated recovery, immediate public hide/session revocation/alerts stop, 12/24-month calendar retention, 90-day payload clearing/anonymous totals, necessary complaint holds with review, approved early deletion, retryable media queue and independent restore ledger. Local: 9 DB checks, 4 desktop/mobile retention cases, 101-route sweep zero issues, check/lint/build pass. Full GitHub run 46 passed on 279bd8b. Additional restore sequence-ID reservation fix passes both retention DB cases; latest PR checks govern the updated head. Normal local migrations applied; production cleanup not run.</x:v>
+        <x:v>Approved A retention package retained. Ordinary seller delete now preserves photo references/files for approved retention and denies owner public media access; edited removed photos use durable deletion queue. Authenticated retention-media cron drains bounded retry queue with enabled/exact-DB guard.</x:v>
       </x:c>
       <x:c r="O175" s="136" t="str">
-        <x:v>Configure authenticated cleanup/media/export scheduling and exact DB guard; verify live provider deletion, actual rolling 30-day backups, restricted hold records and mandatory restore replay drill before launch.</x:v>
+        <x:v>Configure live cleanup/media/ledger scheduling, provider deletion, 30-day rolling backups and independent ledger restore replay; no live-provider or production cleanup sign-off claimed.</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
@@ -10407,7 +10407,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G176" s="137" t="n">
-        <x:v>0.55</x:v>
+        <x:v>0.85</x:v>
       </x:c>
       <x:c r="H176" s="136" t="str">
         <x:v>Critical</x:v>
@@ -10428,10 +10428,10 @@
         <x:v>OWASP review; dependency; auth; IDOR; upload; headers</x:v>
       </x:c>
       <x:c r="N176" s="136" t="str">
-        <x:v>Private provider signing/configuration failures now have mock coverage; cron prototype-name routing is rejected and cron errors no longer expose exception text. Readiness failures are generic; runtime validation redacts values. Alert eligibility/lease/retry controls pass DB tests. Infrastructure/provider and formal review remain open.</x:v>
+        <x:v>Local application review addressed stale state writes, moderation duplicate audit races, tampered runtime decisions, complaint-evidence edits, upload Origin spoofing, deleted-photo privacy and write-limit gaps. Targeted DB/browser evidence recorded; independent review and infrastructure/provider review still open.</x:v>
       </x:c>
       <x:c r="O176" s="136" t="str">
-        <x:v>Review final PR and live provider/proxy/storage/log configuration; close high/critical launch findings.</x:v>
+        <x:v>Independent PR review and staging provider/proxy/log/storage security assessment; close any high/critical launch finding.</x:v>
       </x:c>
     </x:row>
     <x:row r="177">
@@ -10663,10 +10663,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Full GitHub run 43 passed on 0569081, including DB and browser acceptance, sweep, audit/check/lint/build. Agent review found no additional blocking regression in reviewed changes. Live/provider/real-device acceptance remains open.</x:v>
+        <x:v>Local new autonomous closeout package: 6 desktop/mobile action cases plus 13 isolated DB checks (including search sorts/pagination). Existing full CI run 47 passed before this package; latest-head full regression governs PR sign-off.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Current-head clean CI and final provider/real-device/staging acceptance govern sign-off.</x:v>
+        <x:v>Latest-head CI, independent review, live provider/staging/device acceptance remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -11488,7 +11488,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G199" s="137" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="H199" s="136" t="str">
         <x:v>Critical</x:v>
@@ -11509,10 +11509,10 @@
         <x:v>Synthetic error; alert delivery; PII review</x:v>
       </x:c>
       <x:c r="N199" s="136" t="str">
-        <x:v>Next request-error hook emits structured timestamp/method/route-template/category events without request bodies, query strings, cookies or exception messages. Operator runbook documents host collection, access controls and review of separate framework/provider logs.</x:v>
+        <x:v>Structured cron completion/failure events and read-only operations report expose retry/backlog/overdue-hold signals alongside readiness/runtime error events. Reports exclude personal customer payloads and secrets.</x:v>
       </x:c>
       <x:c r="O199" s="136" t="str">
-        <x:v>Configure hosted log retention, aggregation and actionable error alerts; test an end-to-end staging alert.</x:v>
+        <x:v>Configure hosted log retention/aggregation, monitoring recipients and end-to-end staging notifications.</x:v>
       </x:c>
     </x:row>
     <x:row r="200">
@@ -11629,7 +11629,7 @@
         <x:v>Partially Implemented</x:v>
       </x:c>
       <x:c r="G202" s="137" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="H202" s="136" t="str">
         <x:v>Medium</x:v>
@@ -11650,10 +11650,10 @@
         <x:v>Event accuracy; consent; duplicate events</x:v>
       </x:c>
       <x:c r="N202" s="136" t="str">
-        <x:v>docs/OPERATIONS.md defines basic V1 database measures, raw-view limitations and alert acceptance semantics. No external tracker or new analytics identifiers introduced; advanced analytics remains out of scope.</x:v>
+        <x:v>Read-only exact-database operator report supplies inventory, raw render/contact totals, anonymous retained monthly contacts, service/report status, email backlog and retention queues. DB redaction/read-only checks pass. Definitions explicitly distinguish renders from humans, contacts from sales and provider acceptance from delivery.</x:v>
       </x:c>
       <x:c r="O202" s="136" t="str">
-        <x:v>Approve unique-visitor/consent requirements if needed and configure the chosen operational measurement/reporting process.</x:v>
+        <x:v>Configure production operational reporting process. Recommendation: keep clearly labelled existing V1 counts; unique-human tracking needs a separate privacy/method decision if desired.</x:v>
       </x:c>
     </x:row>
     <x:row r="203">
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R125ac9a28a934561"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9d34a4990fe4618"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2500f561729c4e51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31f0041c35774305"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13791,10 +13791,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E37" s="141" t="str">
-        <x:v>Desktop/mobile verification/revocation public-badge/audit flow plus direct seller/anonymous replay with identical administrator controls</x:v>
+        <x:v>Dealer/service authorization retained; direct admin decision tampering and three concurrent removal replays</x:v>
       </x:c>
       <x:c r="F37" s="141" t="str">
-        <x:v>Local pass: unauthorized verify/revoke leaves dealer and audit unchanged; admin decisions succeed with exactly one audit each</x:v>
+        <x:v>Local desktop/mobile negatives preserve state; authorized concurrent removal yields one audit; independent/live security acceptance remains</x:v>
       </x:c>
       <x:c r="G37" s="141" t="str">
         <x:v>Verification admin complete</x:v>
@@ -14311,10 +14311,10 @@
         <x:v>Integration/Operational</x:v>
       </x:c>
       <x:c r="E57" s="141" t="str">
-        <x:v>Local orphan-purge and expiry cron authentication; due/future expiry selection and owner reactivation browser/DB acceptance</x:v>
+        <x:v>Authenticated retention/media workers, lifecycle visibility, limiter exhaustion/recovery, stale sold replay and complaint-evidence edit guards</x:v>
       </x:c>
       <x:c r="F57" s="141" t="str">
-        <x:v>Local cleanup/expiry checks pass; production scheduling, monitoring and saved-alert edge cases remain</x:v>
+        <x:v>Local DB/browser pass; production schedules/provider deletion/backups/ledger restore rehearsal remain</x:v>
       </x:c>
       <x:c r="G57" s="141" t="str">
         <x:v>Configured CRON_SECRET</x:v>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbef5d6b901d84a3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8483b59a0d74a89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53355879638a4140"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra128337099dc498a"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Record full CI closeout and owner launch acceptance handoff
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R05d40645a3c04c9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R2ce7ccc08bc94cc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rc0a69308994f45ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R591709f00eb3459c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R3f2f7839cbde40f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R6f1b4b7399bf44ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Raa9a66fc6bd4496f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R049445080ab84b8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R45720f57a7d24d9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R1ab30b67c8a64794"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Ra8a1043321d8490a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R0d2b22a78d2f47c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R1d1d4b1fef054d93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R6658e22c94db422d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Red60ef7747f04bed"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbe62405a13ae4b6e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1247,7 +1247,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F5" s="94" t="str">
-        <x:v>Local passed; CI run 46 passed; latest PR checks govern</x:v>
+        <x:v>Application 1e0a071: full CI run 49 passed; latest head checks govern</x:v>
       </x:c>
       <x:c r="G5" s="92" t="str">
         <x:v>Current branch</x:v>
@@ -1274,7 +1274,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F6" s="99" t="str">
-        <x:v>No lint warnings/errors</x:v>
+        <x:v>Run 49 check/lint passed; no warnings/errors</x:v>
       </x:c>
       <x:c r="G6" s="97" t="str">
         <x:v>Current stage</x:v>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6 open; full run 46 passed; latest head checks govern</x:v>
+        <x:v>PR #6 open; application 1e0a071 full run 49 passed</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>6 new local browser cases; 13 DB checks; latest CI governs</x:v>
+        <x:v>CI 120 browser passes, 1 planned skip; 13 DB checks</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>5 October autonomous closeout: local check/lint/build, 101-route sweep, 6 new desktop/mobile action cases and 13 DB checks pass. Security/lifecycle gaps, paginated browse performance and private aggregate operations report addressed. Prior full CI run 47 passed; latest-head CI governs review. Production/provider/device acceptance remains.</x:v>
+        <x:v>5 October: application 1e0a071 passed full GitHub run 49: audit, migrations, 13 DB cases, check/lint/build, 101-route sweep and 120 browser passes with 1 planned skip (Chromium/mobile/WebKit/recovery). Google-prefetch/redirect and WebKit-origin findings from run 48 fixed. Maximum First Load JS 128 KB. Production/provider/device acceptance remains; latest head checks govern PR review.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59f14799e7e644d0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6c97646da834dc7"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>5 October: autonomous security/lifecycle/search/operations package added with local check/lint/build, sweep and DB/browser verification. Master tracker preserves production/provider/device gaps. See OWNER_LAUNCH_ACTIONS.md for access/test handoff; feature push is separate from review/main merge.</x:v>
+        <x:v>5 October application 1e0a071 passed full CI run 49: audit/migrations, 13 DB checks, check/lint/build, 101-route sweep, 120 browser passes and 1 planned skip. Master tracker is 94.2%; live deployment/provider/device gaps remain. Owner steps are in OWNER_LAUNCH_ACTIONS.md. Feature push, independent PR review and main merge are separate.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2720,7 +2720,7 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>GitHub run 37 passed all quality/acceptance gates on a96704b: https://github.com/Tech-Orbit-Systems/JaniWheels/actions/runs/37035200489 . Branch protection and a deliberate failing-check merge block remain unverified.</x:v>
+        <x:v>Application 1e0a071 passed full GitHub run 49: production dependency audit, migrations/seed, 13 isolated DB checks, check/lint/build, route sweep and complete browser suite. Branch protection/required-check enforcement remains a repository-admin launch gate.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
         <x:v>Mark check required in branch protection and demonstrate deliberate failure blocks merge.</x:v>
@@ -2955,7 +2955,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Full GitHub run 43 passed on 0569081: audit, migrations, seed, DB tests, check, lint, build, sweep and browser acceptance. Agent self-review completed; no additional blocking regression identified. See docs/PR6_REVIEW.md. Maintainer approval/main merge remains separate.</x:v>
+        <x:v>Full CI run 49 passes on application 1e0a071; includes new seller lifecycle/admin tampering/concurrency/held edit cases plus retention, Chromium/mobile/WebKit and recovery acceptance. Independent PR #6 review/main merge remain open.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Maintainer review/merge decision and required repository checks; live acceptance remains tracked separately.</x:v>
@@ -4459,7 +4459,7 @@
         <x:v>Burst; distributed attempts; reset window; proxy headers</x:v>
       </x:c>
       <x:c r="N49" s="136" t="str">
-        <x:v>PostgreSQL-backed atomic limits cover sign-in, registration, reset and verification actions; Google sign-in start now limits configured IP requests. Successful sign-in clears the account attempt bucket. Concurrent DB and desktop/mobile browser retry tests pass.</x:v>
+        <x:v>Local/CI auth limiter and next-window recovery checks pass. Google auth initiation no longer prefetches; unavailable redirect uses configured site origin. Live Google provider, proxy thresholds and alerts remain.</x:v>
       </x:c>
       <x:c r="O49" s="136" t="str">
         <x:v>Verify Google provider path, trusted proxy IP headers, thresholds and alerting in staging.</x:v>
@@ -10663,7 +10663,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Local new autonomous closeout package: 6 desktop/mobile action cases plus 13 isolated DB checks (including search sorts/pagination). Existing full CI run 47 passed before this package; latest-head full regression governs PR sign-off.</x:v>
+        <x:v>Application 1e0a071 full CI run 49 passes: 120 browser passes, 1 planned skip, 13 isolated DB checks, check/lint/build and 101-route sweep. Run 48 Google-prefetch/redirect and WebKit-origin findings fixed; independent final review and live provider/device acceptance remain.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Latest-head CI, independent review, live provider/staging/device acceptance remain.</x:v>
@@ -10710,7 +10710,7 @@
         <x:v>Real/simulated devices; slow network</x:v>
       </x:c>
       <x:c r="N182" s="136" t="str">
-        <x:v>Simulated Android Chromium covers core seller, dealer, buyer and admin journeys. Added iPhone 13 WebKit smoke checks for mobile navigation, auto-parts search, responsive width, sign-in and car-photo upload; both pass in fresh isolated acceptance. Local HTTP production-mode WebKit needs a test-only session-cookie injection because Secure cookies require HTTPS. CI now installs WebKit alongside Chromium.</x:v>
+        <x:v>Full Linux CI run 49 passes mobile Chromium and WebKit navigation/photo upload. Windows local WebKit photo upload passes; navigation timed out waiting for stable Auto Parts tab while local suites ran concurrently. Actual iPhone Safari/Android Chrome HTTPS, camera, keyboard, slow-network and assistive acceptance remain required; no real-device sign-off claimed.</x:v>
       </x:c>
       <x:c r="O182" s="136" t="str">
         <x:v>Run real iPhone Safari and Android Chrome on HTTPS staging, including keyboard, camera/file picker, slow network and full posting/contact journeys; local WebKit smoke is not a real-device sign-off.</x:v>
@@ -10898,7 +10898,7 @@
         <x:v>Checklist review; defect retest</x:v>
       </x:c>
       <x:c r="N186" s="136" t="str">
-        <x:v>docs/REGRESSION_CHECKLIST.md now defines a reusable release-candidate record, automated gate, module-by-module manual steps linked to Test Matrix IDs, expected evidence, defect retest and merge sign-off rules. Deployment guide links to it. Local automation is current, but live staging/provider/real-device evidence and reviewer signatures are not yet available.</x:v>
+        <x:v>Candidate 1e0a071 passes full CI run 49, including Chromium/mobile/WebKit and recovery, 13 DB cases and 101-route sweep. Tracker links provider/device/staging gates to owner handoff; this does not substitute independent review or live acceptance.</x:v>
       </x:c>
       <x:c r="O186" s="136" t="str">
         <x:v>Fill the checklist and Test Matrix with candidate-specific staging, Safari/real-device, provider and infrastructure evidence; obtain PR reviewer sign-off before merge.</x:v>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9d34a4990fe4618"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcb576a952434f07"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12827,7 +12827,7 @@
         <x:v>codex/launch-quality-system</x:v>
       </x:c>
       <x:c r="E23" s="141" t="str">
-        <x:v>PR #6 / a96704b: CI run 37 passes, 93 local browser cases and 5 DB checks. Persistent staging, monitoring and required-check enforcement remain open.</x:v>
+        <x:v>PR #6 / application 1e0a071: full CI run 49 passes with 120 browser cases, 1 planned skip, 13 DB checks, check/lint/build and 101-route sweep. Persistent staging, monitoring, independent review and required-check enforcement remain open.</x:v>
       </x:c>
       <x:c r="F23" s="141" t="str">
         <x:v>Deliberate failure blocks merge; staging smoke passes.</x:v>
@@ -12850,7 +12850,7 @@
         <x:v>codex/production-readiness (planned)</x:v>
       </x:c>
       <x:c r="E24" s="141" t="str">
-        <x:v>Private media, alert worker, deployment validation/readiness/error events, client-approved retention/closure/recovery/holds/early deletion/media retry/deletion replay and local query/load baselines implemented. Run 46 full CI passed; latest PR checks govern updated head. Live hosting/DB/media/mail/backups/cron/monitoring, restore drill and final security/load acceptance remain.</x:v>
+        <x:v>Approved A/B1 application work includes retention/replay/holds/private media queues, resilient alerts, runtime readiness/errors, action security, 20,000-ad paginated browse benchmark and aggregate operations reporting. Full CI run 49 passed on 1e0a071. Live hosting/DB/media/mail/backups/cron/monitoring, restore drill and final device/security/500-user staging acceptance require owner access; see OWNER_LAUNCH_ACTIONS.md.</x:v>
       </x:c>
       <x:c r="F24" s="141" t="str">
         <x:v>Formal launch checklist has no open critical/high issue.</x:v>
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31f0041c35774305"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc81ada66c8c44a29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8483b59a0d74a89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80b72375a5a241d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra128337099dc498a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44ef904321234489"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Keep tracker verification labels readable
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R049445080ab84b8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R45720f57a7d24d9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R1ab30b67c8a64794"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Ra8a1043321d8490a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R0d2b22a78d2f47c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R1d1d4b1fef054d93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R6658e22c94db422d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R29311298ca084b5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Ra4d40a6a26aa40e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rc78d2a4139ef4d48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rdac6e0246a5e4c4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R9f589d9ff8b54932"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rd73672bee39844f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R44bd971088584827"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbe62405a13ae4b6e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbf5f6587720d40fb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1247,7 +1247,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F5" s="94" t="str">
-        <x:v>Application 1e0a071: full CI run 49 passed; latest head checks govern</x:v>
+        <x:v>Code CI 49 passed</x:v>
       </x:c>
       <x:c r="G5" s="92" t="str">
         <x:v>Current branch</x:v>
@@ -1274,7 +1274,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F6" s="99" t="str">
-        <x:v>Run 49 check/lint passed; no warnings/errors</x:v>
+        <x:v>No warnings/errors</x:v>
       </x:c>
       <x:c r="G6" s="97" t="str">
         <x:v>Current stage</x:v>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6c97646da834dc7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44466c8ca3ad4a8d"/>
 </x:worksheet>
 </file>
 
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcb576a952434f07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9cc05921d2a4e2b"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc81ada66c8c44a29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21345c642c554909"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80b72375a5a241d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80df6fbf4b7545b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44ef904321234489"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e433b91c1f34e8b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Document external deployment handoff and update tracker
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R29311298ca084b5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Ra4d40a6a26aa40e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rc78d2a4139ef4d48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rdac6e0246a5e4c4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R9f589d9ff8b54932"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rd73672bee39844f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R44bd971088584827"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc8f6ca1317ed42db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rb35ad624071f41f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R93a13bfb57ab4dcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rc1fd546fda994eb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Raf683c7beb6c45ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R843aa0f6c5004c0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R89f46c29db44469b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbf5f6587720d40fb"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3e4b9f9a53db453d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44466c8ca3ad4a8d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40adf2abc4e14d42"/>
 </x:worksheet>
 </file>
 
@@ -1858,7 +1858,7 @@
         <x:v>Active package</x:v>
       </x:c>
       <x:c r="B7" s="127" t="str">
-        <x:v>Stage 6.2 CI and isolated DB/browser acceptance in PR #6; persistent online staging remains open</x:v>
+        <x:v>Stage 6.2 code/CI complete on feature branch; external deployment team owns hosting, provider, DNS and live acceptance per docs/DEPLOYMENT_HANDOFF.md</x:v>
       </x:c>
       <x:c r="C7" s="127"/>
       <x:c r="D7" s="127"/>
@@ -11274,10 +11274,10 @@
         <x:v>Deployment smoke; restart; rollback</x:v>
       </x:c>
       <x:c r="N194" s="136" t="str">
-        <x:v>No production deployment is documented as complete.</x:v>
+        <x:v>Deployment assigned to an external team by the owner on 8 Oct 2026. docs/DEPLOYMENT_HANDOFF.md provides the reviewed-source, runtime, environment, migration, provider, DNS and acceptance package. No production deployment is documented as complete.</x:v>
       </x:c>
       <x:c r="O194" s="136" t="str">
-        <x:v>Select and configure hosting.</x:v>
+        <x:v>External team: provision hosting and deploy reviewed main SHA; return URL, commit, smoke, rollback and monitoring evidence.</x:v>
       </x:c>
     </x:row>
     <x:row r="195">
@@ -11415,10 +11415,10 @@
         <x:v>DNS; SSL; www/non-www; canonical tags</x:v>
       </x:c>
       <x:c r="N197" s="136" t="str">
-        <x:v>Domain exists, but application production deployment is not verified.</x:v>
+        <x:v>8 Oct 2026 DNS check: ns91.host.com.pk/ns92.host.com.pk; apex resolves to existing cPanel server 5.101.140.80. Owner confirms Coming Soon site and no old website/mailbox data needs migration. Production HTTPS application is not deployed or verified.</x:v>
       </x:c>
       <x:c r="O197" s="136" t="str">
-        <x:v>Configure after hosting selection.</x:v>
+        <x:v>External team: recheck active DNS at cutover, update apex/www to selected host and verify TLS, redirects and canonical URL.</x:v>
       </x:c>
     </x:row>
     <x:row r="198">
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9cc05921d2a4e2b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36dfe24c25cc4b1f"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21345c642c554909"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0749018aca44385"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80df6fbf4b7545b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e061ef8fa2b48dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e433b91c1f34e8b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73907cdb0b324232"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Record passing PR security and acceptance checks
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc8f6ca1317ed42db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rb35ad624071f41f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R93a13bfb57ab4dcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rc1fd546fda994eb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Raf683c7beb6c45ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R843aa0f6c5004c0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R89f46c29db44469b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re6699fca42b14745"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Re6b8536de15d4891"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R1b3969804d634043"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R82fc3d66ea4c4de3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R45dca29a222a4c3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rcd456fd78696451d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R7b0780abdb9a40e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3e4b9f9a53db453d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4fd17d213dda443e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40adf2abc4e14d42"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40646a89d4cd40ba"/>
 </x:worksheet>
 </file>
 
@@ -3002,7 +3002,7 @@
         <x:v>npm audit review; regression build</x:v>
       </x:c>
       <x:c r="N18" s="136" t="str">
-        <x:v>30 Sep 2026: Next.js 15.5.26, sharp 0.35.5 and patched PostCSS/js-yaml installed. npm audit --omit=dev reports zero vulnerabilities; checks, lint, build, 100-route sweep and 13 Chromium tests pass.</x:v>
+        <x:v>30 Sep 2026: Next.js 15.5.26, sharp 0.35.5 and patched PostCSS/js-yaml installed; earlier package, route and browser checks passed. 8 Oct 2026: patched source-map-js to 1.2.2 for GHSA-68fv-2mgg-jv7q. Production npm audit reports zero vulnerabilities; local lint and build pass. GitHub PR #6 quality and acceptance CI passed.</x:v>
       </x:c>
       <x:c r="O18" s="136" t="str">
         <x:v>Monitor advisories in CI; four moderate development-only esbuild advisories await a compatible upstream Drizzle kit update.</x:v>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36dfe24c25cc4b1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ea48c28fdd84b33"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0749018aca44385"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29cc9e38566c4a00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e061ef8fa2b48dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa6748b535094d45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73907cdb0b324232"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e0a22bc84554641"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Fix independent review defects and preserve restore decisions
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re6699fca42b14745"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Re6b8536de15d4891"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R1b3969804d634043"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R82fc3d66ea4c4de3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R45dca29a222a4c3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rcd456fd78696451d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R7b0780abdb9a40e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd7770fee55ed453f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rd8fe32c4a7754124"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rbd6bb26b72634b9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rab25cf0420714878"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R57a37cc0187043c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R5b532c28b5f74d80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R4fc15565156d449a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4fd17d213dda443e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R890bb75dff8a46f6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1175,7 +1175,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="86" t="str">
-        <x:v>JaniWheels V1 Development Control Sheet — 3 October 2026</x:v>
+        <x:v>JaniWheels V1 Development Control Sheet - 8 October 2026</x:v>
       </x:c>
       <x:c r="B1" s="86"/>
       <x:c r="C1" s="86"/>
@@ -1247,7 +1247,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F5" s="94" t="str">
-        <x:v>Code CI 49 passed</x:v>
+        <x:v>Local checks passed</x:v>
       </x:c>
       <x:c r="G5" s="92" t="str">
         <x:v>Current branch</x:v>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6 open; application 1e0a071 full run 49 passed</x:v>
+        <x:v>PR #6 open; independent re-review of fixes required</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1328,7 +1328,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F8" s="99" t="str">
-        <x:v>Final build passed; max First Load JS 128 KB</x:v>
+        <x:v>Review-fix build passed; max JS 128 KB</x:v>
       </x:c>
       <x:c r="G8" s="97" t="str">
         <x:v>Next functionality</x:v>
@@ -1355,13 +1355,13 @@
         <x:v>Local passed</x:v>
       </x:c>
       <x:c r="F9" s="99" t="str">
-        <x:v>13 isolated DB cases; live acceptance open</x:v>
+        <x:v>18 isolated DB cases passed; live acceptance open</x:v>
       </x:c>
       <x:c r="G9" s="97" t="str">
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>CI 120 browser passes, 1 planned skip; 13 DB checks</x:v>
+        <x:v>Local review regressions pass; latest CI governs full suite</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1409,13 +1409,13 @@
         <x:v>Partial pass</x:v>
       </x:c>
       <x:c r="F11" s="104" t="str">
-        <x:v>Local security checks pass; formal review/load open</x:v>
+        <x:v>Fixes verified; re-review open</x:v>
       </x:c>
       <x:c r="G11" s="102" t="str">
         <x:v>Final QA blocker</x:v>
       </x:c>
       <x:c r="H11" s="103" t="str">
-        <x:v>Hosting/providers, Cloudflare privacy, load and final acceptance</x:v>
+        <x:v>Updated PR review, providers, load and final acceptance</x:v>
       </x:c>
       <x:c r="I11" s="103"/>
       <x:c r="J11" s="104"/>
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>5 October: application 1e0a071 passed full GitHub run 49: audit, migrations, 13 DB cases, check/lint/build, 101-route sweep and 120 browser passes with 1 planned skip (Chromium/mobile/WebKit/recovery). Google-prefetch/redirect and WebKit-origin findings from run 48 fixed. Maximum First Load JS 128 KB. Production/provider/device acceptance remains; latest head checks govern PR review.</x:v>
+        <x:v>8 October: nine confirmed independent-review defects and one ban-policy risk repaired. Regression cases cover restore/deletion, cancelled alerts, quota races/reactivation, taxonomy/location, closed dealers, redirects, logging and banned inventory. Local verification and latest exact-head CI are recorded in PR6_REVIEW_RESPONSE.md. Independent re-review, protected main and persistent staging remain open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40646a89d4cd40ba"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34534f3ff43a4207"/>
 </x:worksheet>
 </file>
 
@@ -2269,7 +2269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="133" t="str">
-        <x:v>Repository reconciliation: 30 Sep 2026 | Homepage visuals approved by owner; commit 936baee pushed to origin/codex/homepage-visuals | Full checks, lint and build passed | Final cross-route browser/DB and live Google Maps acceptance remain open</x:v>
+        <x:v>8 October 2026: independent PR #6 findings repaired on the feature branch. Updated-head independent review and merge remain pending. See PR6_REVIEW_RESPONSE.md for numbered dispositions and verification. Live deployment/provider/device gates remain open.</x:v>
       </x:c>
       <x:c r="B2" s="133"/>
       <x:c r="C2" s="133"/>
@@ -2720,10 +2720,10 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>Application 1e0a071 passed full GitHub run 49: production dependency audit, migrations/seed, 13 isolated DB checks, check/lint/build, route sweep and complete browser suite. Branch protection/required-check enforcement remains a repository-admin launch gate.</x:v>
+        <x:v>8 Oct: baseline e4170b2 CI passed. Independent review found 9 defects and 1 policy risk; fixes and regression evidence in PR6_REVIEW_RESPONSE.md. New head requires CI and re-review.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
-        <x:v>Mark check required in branch protection and demonstrate deliberate failure blocks merge.</x:v>
+        <x:v>Require green updated-head CI, independent re-review and branch protection before main merge; persistent staging remains.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2908,7 +2908,7 @@
         <x:v>Unit; integration; transaction tests</x:v>
       </x:c>
       <x:c r="N16" s="136" t="str">
-        <x:v>Isolated PostgreSQL integration framework covers publishing facets, ownership, bootstrap rollback/concurrency, alerts retries/overflow, retention/replay, aggregate reporting, origin guards, limiter recovery and sorted browse pagination. 13 DB cases; provider and production acceptance remain in their own rows.</x:v>
+        <x:v>8 Oct: 18 isolated DB regressions cover publication quota races, curated taxonomy/area ownership, restore moderation/alert suppression, safe logging and banned-owner alerts.</x:v>
       </x:c>
       <x:c r="O16" s="136" t="str">
         <x:v>Maintain regression coverage as product/provider changes occur; no framework implementation gap remains.</x:v>
@@ -2955,7 +2955,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Full CI run 49 passes on application 1e0a071; includes new seller lifecycle/admin tampering/concurrency/held edit cases plus retention, Chromium/mobile/WebKit and recovery acceptance. Independent PR #6 review/main merge remain open.</x:v>
+        <x:v>8 Oct: browser regressions added for seller-delete backup replay, quota reactivation, authenticated redirect, banned detail/media/contact and closed verified-dealer homepage. Final coverage in PR6_REVIEW_RESPONSE.md.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>Maintainer review/merge decision and required repository checks; live acceptance remains tracked separately.</x:v>
@@ -3519,7 +3519,7 @@
         <x:v>Verified/unverified/empty data cases</x:v>
       </x:c>
       <x:c r="N29" s="136" t="str">
-        <x:v>Homepage redesign is present in current branch ancestry and automated project checks pass; final branding/responsive acceptance is intentionally deferred.</x:v>
+        <x:v>8 Oct review #3: verified homepage dealers require an open, unbanned owner. Close/restore/ban browser regression checks homepage, storefront and directory; counts use public inventory eligibility.</x:v>
       </x:c>
       <x:c r="O29" s="136" t="str">
         <x:v>Retain in final regression and comprehensive browser QA.</x:v>
@@ -4271,7 +4271,7 @@
         <x:v>Open-redirect payloads; valid internal paths</x:v>
       </x:c>
       <x:c r="N45" s="136" t="str">
-        <x:v>safeNext is implemented.</x:v>
+        <x:v>8 Oct review #8: seven auth paths share bounded same-origin return-path validation. Backslash, encoded slash/control and foreign targets reject to /. Authenticated HTTP and helper regressions cover valid local paths.</x:v>
       </x:c>
       <x:c r="O45" s="136" t="str">
         <x:v>Add unit tests.</x:v>
@@ -4553,7 +4553,7 @@
         <x:v>Login and active-session ban cases</x:v>
       </x:c>
       <x:c r="N51" s="136" t="str">
-        <x:v>Banned login is denied; desktop/mobile browser tests confirm admin ban revokes active sessions, unban appends an audit record and restored user can sign in. Admin ban/unban UI is implemented.</x:v>
+        <x:v>8 Oct risk #10: banned inventory excluded from public search/detail/media/contact, saved/recent ads, sitemap, linked inspection and alerts. Unban exposes only still-active ads. Distinct seller/buyer alert regression passes.</x:v>
       </x:c>
       <x:c r="O51" s="136" t="str">
         <x:v>Retain provider-independent browser regression; final live acceptance remains open.</x:v>
@@ -5023,7 +5023,7 @@
         <x:v>Cascade; empty states; invalid IDs; cache</x:v>
       </x:c>
       <x:c r="N61" s="136" t="str">
-        <x:v>Implemented through /api/taxonomy.</x:v>
+        <x:v>8 Oct review #6: car/bike publication validates active curated make/model/variant and matching vertical. Forged, invalid or inactive supplied variants cannot fall back to custom text. DB rollback and valid publication tested.</x:v>
       </x:c>
       <x:c r="O61" s="136" t="str">
         <x:v>Add integration/E2E tests.</x:v>
@@ -5352,7 +5352,7 @@
         <x:v>Boundary 2/3/4; concurrent submits; sold/expired</x:v>
       </x:c>
       <x:c r="N68" s="136" t="str">
-        <x:v>Cars, bikes and parts publishing flows are implemented with instant publication, seller limits and synchronized facets.</x:v>
+        <x:v>8 Oct review #5: all vertical creation, reactivation and rejected-ad resubmission serialize on the owner row and check 3 live ads in the transaction. Concurrent publication permits only one final slot; real dealer profile exemption tested.</x:v>
       </x:c>
       <x:c r="O68" s="136" t="str">
         <x:v>Retain in final regression and comprehensive browser QA.</x:v>
@@ -5728,7 +5728,7 @@
         <x:v>Owner/non-owner; related images/reports; repeat delete</x:v>
       </x:c>
       <x:c r="N76" s="136" t="str">
-        <x:v>Owner listing CRUD, image management, lifecycle controls and inactive-listing privacy are implemented.</x:v>
+        <x:v>8 Oct review #1: seller deletion writes a seller-delete ledger receipt atomically. Backup replay hides the ad idempotently; retained photos stay private with admin evidence access. Retention expiry/holds remain authoritative.</x:v>
       </x:c>
       <x:c r="O76" s="136" t="str">
         <x:v>Retain in final regression and comprehensive browser QA.</x:v>
@@ -7655,7 +7655,7 @@
         <x:v>Active/inactive/missing; anonymous/auth; phone formats</x:v>
       </x:c>
       <x:c r="N117" s="136" t="str">
-        <x:v>Implemented with lead logging.</x:v>
+        <x:v>8 Oct: contact action rejects inactive/deleted ads and banned/closed/anonymized owners. Browser regression replays a previously captured reveal after ban and checks no phone disclosure.</x:v>
       </x:c>
       <x:c r="O117" s="136" t="str">
         <x:v>Add rate limiting/anti-scraping.</x:v>
@@ -7702,7 +7702,7 @@
         <x:v>Insert failure; repeat clicks; concurrency</x:v>
       </x:c>
       <x:c r="N118" s="136" t="str">
-        <x:v>Implemented transaction with failure isolation.</x:v>
+        <x:v>8 Oct review #9: handled lead errors log fixed event plus safe SQLSTATE only, never raw query/message/parameters. Source bounded to known values; private marker logging regression passes.</x:v>
       </x:c>
       <x:c r="O118" s="136" t="str">
         <x:v>Define deduplication policy and test.</x:v>
@@ -8407,7 +8407,7 @@
         <x:v>Match accuracy; frequency; duplicates; delivery failure; unsubscribe</x:v>
       </x:c>
       <x:c r="N133" s="136" t="str">
-        <x:v>Overflow, deduplication, concurrent delivery, immutable UUID retry identity, opt-out/eligibility and retry-window tests pass. Full GitHub run 43 on 0569081 passed, including the cross-environment retry-key fix. No live email sent.</x:v>
+        <x:v>8 Oct review #4/risk #10: closure replay suppresses old undelivered alerts before preference restore. Banned listing owners cannot match or deliver to another buyer. DB regressions pass; live mail/scheduling remain.</x:v>
       </x:c>
       <x:c r="O133" s="136" t="str">
         <x:v>Configure verified Resend sender and credentials, schedule queue/delivery, review initial backlog and complete controlled mailbox, outage and deliverability acceptance.</x:v>
@@ -9535,7 +9535,7 @@
         <x:v>Ban/unban; active session; listings; audit</x:v>
       </x:c>
       <x:c r="N157" s="136" t="str">
-        <x:v>Admin controls implemented. Desktop/mobile browser tests confirm reasoned hide, reinstate and permanent removal with public visibility changes and audit entries; ban revokes sessions, restore permits login and both decisions append audit history.</x:v>
+        <x:v>8 Oct risk #10: manual bans preserve inventory but hide public ads/media/contact and alert matches. Existing session revocation/audit rules retained. Unban cannot revive removed ads.</x:v>
       </x:c>
       <x:c r="O157" s="136" t="str">
         <x:v>Report resolution, direct-action authorization and final live acceptance remain open.</x:v>
@@ -10381,10 +10381,10 @@
         <x:v>Retention job; account deletion; backup implications</x:v>
       </x:c>
       <x:c r="N175" s="136" t="str">
-        <x:v>Approved A retention package retained. Ordinary seller delete now preserves photo references/files for approved retention and denies owner public media access; edited removed photos use durable deletion queue. Authenticated retention-media cron drains bounded retry queue with enabled/exact-DB guard.</x:v>
+        <x:v>8 Oct reviews #1/#2/#4: atomic seller-delete receipts, receipt-aware idempotent replay, later moderator rejection preserved, cancelled alerts suppressed. Approved A windows/holds unchanged. Production backup/restore drill remains.</x:v>
       </x:c>
       <x:c r="O175" s="136" t="str">
-        <x:v>Configure live cleanup/media/ledger scheduling, provider deletion, 30-day rolling backups and independent ledger restore replay; no live-provider or production cleanup sign-off claimed.</x:v>
+        <x:v>Independent review of repaired replay; deployment owner must export protected current ledger and rehearse restore before clearing maintenance.</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
@@ -11509,7 +11509,7 @@
         <x:v>Synthetic error; alert delivery; PII review</x:v>
       </x:c>
       <x:c r="N199" s="136" t="str">
-        <x:v>Structured cron completion/failure events and read-only operations report expose retry/backlog/overdue-hold signals alongside readiness/runtime error events. Reports exclude personal customer payloads and secrets.</x:v>
+        <x:v>8 Oct review #9: shared safe handled-error logger used for lead, auth delivery, view count, upload/storage and cron failures. Marker regression confirms query/PII omission. External log sink/alerts require deployment setup.</x:v>
       </x:c>
       <x:c r="O199" s="136" t="str">
         <x:v>Configure hosted log retention/aggregation, monitoring recipients and end-to-end staging notifications.</x:v>
@@ -12261,7 +12261,7 @@
         <x:v>Privacy/security review; DB acceptance; create/edit/detail tests; final responsive browser QA</x:v>
       </x:c>
       <x:c r="N215" t="str">
-        <x:v>Privacy-safe map storage and approximate public output are merged on main. Regression checks passed 30 Sep. Google Maps configuration exists locally; billing and live browser acceptance remain unresolved.</x:v>
+        <x:v>8 Oct review #7: each car/bike/part publication validates area belongs to selected city before claiming photos. All three rollback regressions pass. Existing approximate-location privacy retained; live Google Maps billing/provider acceptance remains.</x:v>
       </x:c>
       <x:c r="O215" t="str">
         <x:v>Enable billing without exposing the key; test car/bike/parts create, edit and public detail, then verify exact coordinates remain private.</x:v>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ea48c28fdd84b33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra817772d876d4db5"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12827,7 +12827,7 @@
         <x:v>codex/launch-quality-system</x:v>
       </x:c>
       <x:c r="E23" s="141" t="str">
-        <x:v>PR #6 / application 1e0a071: full CI run 49 passes with 120 browser cases, 1 planned skip, 13 DB checks, check/lint/build and 101-route sweep. Persistent staging, monitoring, independent review and required-check enforcement remain open.</x:v>
+        <x:v>8 Oct: independent PR #6 findings repaired and regression coverage expanded. Verify updated-head check/lint/build, 18 DB cases, 101-route sweep and browser suite in PR6_REVIEW_RESPONSE.md. Independent re-review, protected main and persistent staging remain open.</x:v>
       </x:c>
       <x:c r="F23" s="141" t="str">
         <x:v>Deliberate failure blocks merge; staging smoke passes.</x:v>
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29cc9e38566c4a00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf46f3ec21c24039"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13271,10 +13271,10 @@
         <x:v>Integration + Security</x:v>
       </x:c>
       <x:c r="E17" s="141" t="str">
-        <x:v>Automated checks plus desktop/mobile Chromium bike deletion with DB, public URL and photo assertions</x:v>
+        <x:v>Desktop/mobile seller deletion plus atomic ledger receipt, pre-delete backup replay repeated twice, retained evidence and anonymous/admin media authorization.</x:v>
       </x:c>
       <x:c r="F17" s="141" t="str">
-        <x:v>Passed: row soft-deleted, photo links removed, public listing and stored image unavailable</x:v>
+        <x:v>Regression covers public detail/media denial after replay and retained private photos for approved retention/admin evidence access.</x:v>
       </x:c>
       <x:c r="G17" s="141" t="str">
         <x:v>Delete policy complete</x:v>
@@ -13583,10 +13583,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E29" s="141" t="str">
-        <x:v>Desktop/mobile buyer reveal plus database lead count</x:v>
+        <x:v>Active buyer reveal/lead logging, inactive rejection and captured action replay after owner ban. Safe handled-error marker regression.</x:v>
       </x:c>
       <x:c r="F29" s="141" t="str">
-        <x:v>Passed active phone reveal and lead log; inactive rejection remains open</x:v>
+        <x:v>Active reveal remains available; inactive/banned owners cannot disclose phone. Raw query/message/parameters excluded from handled error logs.</x:v>
       </x:c>
       <x:c r="G29" s="141" t="str">
         <x:v>Active and inactive listings</x:v>
@@ -13713,13 +13713,13 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E34" s="141" t="str">
-        <x:v>Saved-search UI/static checks plus matching cron and unique outbox in source; no email delivery worker exists</x:v>
+        <x:v>Isolated DB overflow/dedupe/retry/concurrency, closure replay suppression and banned listing owner versus separate buyer. Local transport mocks; live provider/scheduler remain.</x:v>
       </x:c>
       <x:c r="F34" s="141" t="str">
-        <x:v>Partial implementation only: full match/overflow/dedupe/retry and delivered-email acceptance pending</x:v>
+        <x:v>Local DB delivery/matching acceptance passes, including cancelled alerts and banned inventory. Live email delivery/mailbox acceptance pending.</x:v>
       </x:c>
       <x:c r="G34" s="141" t="str">
-        <x:v>Implement delivery worker and configure email provider/scheduler</x:v>
+        <x:v>Deployment owner configures live email provider/scheduler and mailbox acceptance.</x:v>
       </x:c>
       <x:c r="H34" s="141" t="str">
         <x:v>Exact filters, no duplicate alerts</x:v>
@@ -13973,10 +13973,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E44" s="141" t="str">
-        <x:v>Desktop/mobile ban/unban/session-revocation flow plus direct ban replay denied to seller/anonymous visitors with admin success control</x:v>
+        <x:v>Existing authorization/session/audit tests plus banned public detail GET, image GET/HEAD, contact replay, discovery/sitemap and unban without reviving removed inventory.</x:v>
       </x:c>
       <x:c r="F44" s="141" t="str">
-        <x:v>Local pass: unauthorized ban leaves account/audit unchanged; admin ban succeeds and is audited. Live acceptance remains.</x:v>
+        <x:v>Local regressions cover admin access and banned inventory visibility. Independent updated-head review and production acceptance remain.</x:v>
       </x:c>
       <x:c r="G44" s="141" t="str">
         <x:v>User admin complete</x:v>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa6748b535094d45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcebee35feacc47cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e0a22bc84554641"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97f562a755ac4e54"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Patch Next.js security advisories and record CI gate
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd7770fee55ed453f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rd8fe32c4a7754124"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rbd6bb26b72634b9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rab25cf0420714878"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R57a37cc0187043c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R5b532c28b5f74d80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R4fc15565156d449a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6b2fd448aeed4998"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rba1d1b60c0924154"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rc6739781a8e1421e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R4b0a2b894e6043c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Re12a385de21848b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R8c3d2c12deeb44fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Reec68566e90f4c8e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R890bb75dff8a46f6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R74b205742e6f43d5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>8 October: nine confirmed independent-review defects and one ban-policy risk repaired. Regression cases cover restore/deletion, cancelled alerts, quota races/reactivation, taxonomy/location, closed dealers, redirects, logging and banned inventory. Local verification and latest exact-head CI are recorded in PR6_REVIEW_RESPONSE.md. Independent re-review, protected main and persistent staging remain open.</x:v>
+        <x:v>8 October: nine independent-review defects and ban-policy risk repaired; quota resubmission and input-preservation regressions pass. Next.js 15.5.27 security patch addresses the run 55 audit failure. Local verification and exact-head CI are recorded in PR6_REVIEW_RESPONSE.md. Updated independent review and deployment gates remain open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34534f3ff43a4207"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffe77b5a84b242dd"/>
 </x:worksheet>
 </file>
 
@@ -2720,7 +2720,7 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>8 Oct: baseline e4170b2 CI passed. Independent review found 9 defects and 1 policy risk; fixes and regression evidence in PR6_REVIEW_RESPONSE.md. New head requires CI and re-review.</x:v>
+        <x:v>8 Oct: review fixes pushed in 7c9a1e1; run 55 stopped at production dependency audit before tests. Next.js/security lint packages updated to 15.5.27. Latest exact-head CI and independent re-review remain required; see PR6_REVIEW_RESPONSE.md.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
         <x:v>Require green updated-head CI, independent re-review and branch protection before main merge; persistent staging remains.</x:v>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra817772d876d4db5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86e4738d9a9945d8"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf46f3ec21c24039"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf380115744664a33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcebee35feacc47cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f298aa1da30481b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97f562a755ac4e54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b2a78e9ed074faa"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Stabilize accessibility fixtures and record review verification
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6b2fd448aeed4998"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rba1d1b60c0924154"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rc6739781a8e1421e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R4b0a2b894e6043c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Re12a385de21848b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R8c3d2c12deeb44fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Reec68566e90f4c8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R19adabaf842e46b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R48f51482978c40f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rbaea67dc94e046be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R420894db814c45c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R9612a07a587b4093"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rf4c45e679b8244d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Re1e7b0af6c22465d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R74b205742e6f43d5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3dbfc6b9f3af493f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Local review regressions pass; latest CI governs full suite</x:v>
+        <x:v>CI 56 green; one fixture race repaired; latest CI governs full suite</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>8 October: nine independent-review defects and ban-policy risk repaired; quota resubmission and input-preservation regressions pass. Next.js 15.5.27 security patch addresses the run 55 audit failure. Local verification and exact-head CI are recorded in PR6_REVIEW_RESPONSE.md. Updated independent review and deployment gates remain open.</x:v>
+        <x:v>8 October: nine independent-review defects and ban-policy risk repaired. Next.js 15.5.27 production audit clean. CI 56 green: 18 DB tests, 101 URLs, 127 browser passes plus one retry-pass and one planned skip. Accessibility fixture race repaired. Latest exact-head CI, independent re-review and deployment gates remain authoritative.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffe77b5a84b242dd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5a646649c8f461c"/>
 </x:worksheet>
 </file>
 
@@ -2720,7 +2720,7 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>8 Oct: review fixes pushed in 7c9a1e1; run 55 stopped at production dependency audit before tests. Next.js/security lint packages updated to 15.5.27. Latest exact-head CI and independent re-review remain required; see PR6_REVIEW_RESPONSE.md.</x:v>
+        <x:v>8 Oct: review fixes 7c9a1e1 and Next.js 15.5.27 patch df422a7 pushed. CI run 56 passed: audit, 18 DB cases, checks/lint/build, 101 URLs and browser suite (127 pass, 1 retry-pass, 1 planned skip). Accessibility fixture race repaired; latest exact-head CI and independent re-review required.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
         <x:v>Require green updated-head CI, independent re-review and branch protection before main merge; persistent staging remains.</x:v>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86e4738d9a9945d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd74cedf4011e49f3"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf380115744664a33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra91f42de3d05497c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f298aa1da30481b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5000dc7f95104623"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b2a78e9ed074faa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc84f48443a584cc1"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Fix vehicle edit taxonomy and closure lock order
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R19adabaf842e46b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R48f51482978c40f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rbaea67dc94e046be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R420894db814c45c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R9612a07a587b4093"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rf4c45e679b8244d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Re1e7b0af6c22465d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6ea0fc8e99c04cd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R362e770fe60946bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R32bcba5c7dd149bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rac8374e947ac4a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R2e531974485e4afc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R8dc1388e7e544825"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R80c461d235fe4ea4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3dbfc6b9f3af493f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Refb1a353c3d642e2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6 open; independent re-review of fixes required</x:v>
+        <x:v>PR #6: fresh review found two P2 defects; local fixes verified; latest CI and re-review pending</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>CI 56 green; one fixture race repaired; latest CI governs full suite</x:v>
+        <x:v>Targeted car/bike/closure 6/6 and media 2/2 passed; full latest-head CI pending</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1409,7 +1409,7 @@
         <x:v>Partial pass</x:v>
       </x:c>
       <x:c r="F11" s="104" t="str">
-        <x:v>Fixes verified; re-review open</x:v>
+        <x:v>Two P2 fixes locally verified; independent re-review pending</x:v>
       </x:c>
       <x:c r="G11" s="102" t="str">
         <x:v>Final QA blocker</x:v>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5a646649c8f461c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf917c488a3214eda"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>5 October application 1e0a071 passed full CI run 49: audit/migrations, 13 DB checks, check/lint/build, 101-route sweep, 120 browser passes and 1 planned skip. Master tracker is 94.2%; live deployment/provider/device gaps remain. Owner steps are in OWNER_LAUNCH_ACTIONS.md. Feature push, independent PR review and main merge are separate.</x:v>
+        <x:v>8 October fresh review of 5918a8a found two P2 defects. Vehicle edit taxonomy and retention lock order are repaired on the feature branch. Check/lint/build, 18 isolated DB tests, 101-route sweep and 8 targeted desktop/mobile cases pass. Full latest-head CI and independent re-review remain pending. Live deployment/provider/device gaps remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2269,7 +2269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="133" t="str">
-        <x:v>8 October 2026: independent PR #6 findings repaired on the feature branch. Updated-head independent review and merge remain pending. See PR6_REVIEW_RESPONSE.md for numbered dispositions and verification. Live deployment/provider/device gates remain open.</x:v>
+        <x:v>8 October 2026: fresh PR #6 review found two P2 defects on 5918a8a. Vehicle edit taxonomy and lock-order fixes passed targeted local checks; latest-head CI and independent re-review remain pending. Live deployment/provider/device gates remain open.</x:v>
       </x:c>
       <x:c r="B2" s="133"/>
       <x:c r="C2" s="133"/>
@@ -5681,10 +5681,10 @@
         <x:v>Owner/non-owner/admin; each vertical; validation; SEO redirect</x:v>
       </x:c>
       <x:c r="N75" s="136" t="str">
-        <x:v>Owner listing CRUD, image management, lifecycle controls and inactive-listing privacy are implemented.</x:v>
+        <x:v>8 Oct fresh review: car/bike edits reject inactive make/model/variant and forged IDs; valid curated edits persist. Retention advisory lock precedes owner lock. Desktop/mobile targeted regressions 6/6.</x:v>
       </x:c>
       <x:c r="O75" s="136" t="str">
-        <x:v>Retain in final regression and comprehensive browser QA.</x:v>
+        <x:v>Full latest-head CI and independent re-review pending; retain broader browser, provider and real-device acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd74cedf4011e49f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73cc9ecd34c04bcd"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra91f42de3d05497c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re503da5f7f084a19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13089,10 +13089,10 @@
         <x:v>Security integration</x:v>
       </x:c>
       <x:c r="E10" s="141" t="str">
-        <x:v>Desktop/mobile direct listing actions plus local image GET/HEAD checks for pending, active and all inactive statuses; owner/admin success, foreign/anonymous denial and optimizer rejection</x:v>
+        <x:v>Desktop/mobile listing and media authorization, local image GET/HEAD and optimizer checks; owner edit preview is scrolled into view before lazy-image load assertion</x:v>
       </x:c>
       <x:c r="F10" s="141" t="str">
-        <x:v>Local pass: private reads denied, active photos public, owner edit preview loads, no-store headers verified. Cloudflare private delivery remains pending.</x:v>
+        <x:v>Local pass: private reads denied and active photos public; media authorization 2/2 after lazy-image fixture repair. Cloudflare private delivery remains pending.</x:v>
       </x:c>
       <x:c r="G10" s="141" t="str">
         <x:v>Two users with listings/uploads</x:v>
@@ -13245,10 +13245,10 @@
         <x:v>Integration + SEO</x:v>
       </x:c>
       <x:c r="E16" s="141" t="str">
-        <x:v>Automated checks plus desktop/mobile Chromium owner car edit with DB price/status assertion</x:v>
+        <x:v>Desktop/mobile car and bike edit actions: inactive make/model/variant, forged IDs, valid curated edits and concurrent account closure; DB facet checks</x:v>
       </x:c>
       <x:c r="F16" s="141" t="str">
-        <x:v>Passed owner price edit; facet and slug resync remain covered by feature checks</x:v>
+        <x:v>Local pass: 6/6 focused edit/closure cases; invalid taxonomy leaves ads unchanged, valid curated edits persist. Facet/slug checks pass; latest-head CI and real-device acceptance pending.</x:v>
       </x:c>
       <x:c r="G16" s="141" t="str">
         <x:v>Edit flow complete</x:v>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5000dc7f95104623"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0822c4bdc69b4edb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc84f48443a584cc1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R558949ec8c0c417c"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Finish closure lock ordering across correction and view count
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6ea0fc8e99c04cd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R362e770fe60946bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R32bcba5c7dd149bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rac8374e947ac4a50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R2e531974485e4afc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R8dc1388e7e544825"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R80c461d235fe4ea4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3f2df8605658479c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rd516281027d34ef1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Re661754c8c6b4d8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R9d75228ea8f3463c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R25f49cfa7ff946ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Ra2b27d4d674a4f4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R1571af75238542f5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Refb1a353c3d642e2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8450100daee44561"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6: fresh review found two P2 defects; local fixes verified; latest CI and re-review pending</x:v>
+        <x:v>PR #6: both fresh-review P2 defects repaired; local gates passed; CI and re-review pending</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1355,13 +1355,13 @@
         <x:v>Local passed</x:v>
       </x:c>
       <x:c r="F9" s="99" t="str">
-        <x:v>18 isolated DB cases passed; live acceptance open</x:v>
+        <x:v>19 isolated DB cases passed; live acceptance open</x:v>
       </x:c>
       <x:c r="G9" s="97" t="str">
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Targeted car/bike/closure 6/6 and media 2/2 passed; full latest-head CI pending</x:v>
+        <x:v>Latest code: 19 DB, 101 routes, edit/closure 6/6 and media 2/2; CI pending</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf917c488a3214eda"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1ed3fcc5c70453f"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>8 October fresh review of 5918a8a found two P2 defects. Vehicle edit taxonomy and retention lock order are repaired on the feature branch. Check/lint/build, 18 isolated DB tests, 101-route sweep and 8 targeted desktop/mobile cases pass. Full latest-head CI and independent re-review remain pending. Live deployment/provider/device gaps remain open.</x:v>
+        <x:v>8 October fresh review of 5918a8a found two P2 defects. Vehicle edits reject inactive/forged taxonomy. Edit, correction and closure use consistent lock order; migration 0018 removes view-count seller-lock inversion. Latest local check/lint/build, 19 DB tests, 101-route sweep and 8 targeted desktop/mobile cases pass. Full latest-head CI and independent re-review remain pending. Live deployment/provider/device gaps remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2269,7 +2269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="133" t="str">
-        <x:v>8 October 2026: fresh PR #6 review found two P2 defects on 5918a8a. Vehicle edit taxonomy and lock-order fixes passed targeted local checks; latest-head CI and independent re-review remain pending. Live deployment/provider/device gates remain open.</x:v>
+        <x:v>8 October 2026: fresh PR #6 review found two P2 defects on 5918a8a. Vehicle edit taxonomy and edit/correction/view-count closure lock-order fixes passed local gates: 19 DB tests, 101 routes and 8 targeted browser cases. Latest-head CI and independent re-review remain pending. Live deployment/provider/device gates remain open.</x:v>
       </x:c>
       <x:c r="B2" s="133"/>
       <x:c r="C2" s="133"/>
@@ -5681,7 +5681,7 @@
         <x:v>Owner/non-owner/admin; each vertical; validation; SEO redirect</x:v>
       </x:c>
       <x:c r="N75" s="136" t="str">
-        <x:v>8 Oct fresh review: car/bike edits reject inactive make/model/variant and forged IDs; valid curated edits persist. Retention advisory lock precedes owner lock. Desktop/mobile targeted regressions 6/6.</x:v>
+        <x:v>8 Oct fresh review: car/bike edits reject inactive make/model/variant and forged IDs; valid curated edits persist. Edit and rejected-ad correction take retention lock before owner lock; migration 0018 avoids view-count seller-lock inversion. Desktop/mobile 6/6 and controlled closure/view-count DB regression pass.</x:v>
       </x:c>
       <x:c r="O75" s="136" t="str">
         <x:v>Full latest-head CI and independent re-review pending; retain broader browser, provider and real-device acceptance.</x:v>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73cc9ecd34c04bcd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5d290c1d2b04af6"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re503da5f7f084a19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ec68d80a3ed4b70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13245,10 +13245,10 @@
         <x:v>Integration + SEO</x:v>
       </x:c>
       <x:c r="E16" s="141" t="str">
-        <x:v>Desktop/mobile car and bike edit actions: inactive make/model/variant, forged IDs, valid curated edits and concurrent account closure; DB facet checks</x:v>
+        <x:v>Desktop/mobile car and bike edits: inactive make/model/variant, forged IDs, valid curated edits and concurrent closure; DB facet checks and controlled view-count/closure lock barrier</x:v>
       </x:c>
       <x:c r="F16" s="141" t="str">
-        <x:v>Local pass: 6/6 focused edit/closure cases; invalid taxonomy leaves ads unchanged, valid curated edits persist. Facet/slug checks pass; latest-head CI and real-device acceptance pending.</x:v>
+        <x:v>Latest local pass: 6/6 focused edit/closure browser cases and 19/19 DB cases, including view-count/closure barrier. Invalid taxonomy leaves ads unchanged; valid curated edits persist. Latest-head CI and real-device acceptance pending.</x:v>
       </x:c>
       <x:c r="G16" s="141" t="str">
         <x:v>Edit flow complete</x:v>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0822c4bdc69b4edb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50b9398aead54269"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R558949ec8c0c417c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8325b1312d65454d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Serialize moderation with closure and validate variant IDs
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3f2df8605658479c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rd516281027d34ef1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Re661754c8c6b4d8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R9d75228ea8f3463c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R25f49cfa7ff946ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Ra2b27d4d674a4f4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R1571af75238542f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdbbeae8b7cf045e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R0cdeef88622c48b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R444addfb44de4f3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Ra4cb348fe2ed4bbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Re94a8e8b046942f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R75c07b816a674626"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rb747cd702a964ec3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8450100daee44561"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3e9a69fceb3443d8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6: both fresh-review P2 defects repaired; local gates passed; CI and re-review pending</x:v>
+        <x:v>PR #6: second fresh review found admin/closure P2 deadlock and malformed-ID P3; local fixes pass, latest CI/re-review pending</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Latest code: 19 DB, 101 routes, edit/closure 6/6 and media 2/2; CI pending</x:v>
+        <x:v>Head 73c1974 CI 59 green; new local fixes: 19 DB, 101 routes, 8 admin race, 6 vehicle, 2 reports; new CI pending</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1ed3fcc5c70453f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4719b27bccec4c1f"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>8 October fresh review of 5918a8a found two P2 defects. Vehicle edits reject inactive/forged taxonomy. Edit, correction and closure use consistent lock order; migration 0018 removes view-count seller-lock inversion. Latest local check/lint/build, 19 DB tests, 101-route sweep and 8 targeted desktop/mobile cases pass. Full latest-head CI and independent re-review remain pending. Live deployment/provider/device gaps remain open.</x:v>
+        <x:v>8 October second fresh review of 73c1974: admin approve/reinstate versus closure P2 deadlock and malformed variant-ID P3 confirmed. Moderation and report auto-hide now lock owner before listing and recheck locked state. Car/bike create/edit reject malformed or out-of-range variant IDs while preserving deliberate empty-ID fallback. Local check/lint/build, 19 DB tests, 101-route sweep, 8 deterministic admin/closure, 6 vehicle and 2 report browser cases pass. New exact-head CI and independent re-review pending; live provider/deployment/device gates remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2269,7 +2269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="133" t="str">
-        <x:v>8 October 2026: fresh PR #6 review found two P2 defects on 5918a8a. Vehicle edit taxonomy and edit/correction/view-count closure lock-order fixes passed local gates: 19 DB tests, 101 routes and 8 targeted browser cases. Latest-head CI and independent re-review remain pending. Live deployment/provider/device gates remain open.</x:v>
+        <x:v>8 October 2026: second fresh PR #6 review of 73c1974 found admin/closure P2 and malformed-ID P3. Owner-before-listing moderation and strict car/bike variant parsing pass local gates: 19 DB, 101 routes, 8 deterministic admin races, 6 vehicle and 2 report browser cases. New exact-head CI and independent re-review pending. Live deployment/provider/device gates remain open.</x:v>
       </x:c>
       <x:c r="B2" s="133"/>
       <x:c r="C2" s="133"/>
@@ -5681,10 +5681,10 @@
         <x:v>Owner/non-owner/admin; each vertical; validation; SEO redirect</x:v>
       </x:c>
       <x:c r="N75" s="136" t="str">
-        <x:v>8 Oct fresh review: car/bike edits reject inactive make/model/variant and forged IDs; valid curated edits persist. Edit and rejected-ad correction take retention lock before owner lock; migration 0018 avoids view-count seller-lock inversion. Desktop/mobile 6/6 and controlled closure/view-count DB regression pass.</x:v>
+        <x:v>Second fresh review: car/bike create/edit now reject malformed and &gt;2147483647 variant IDs with field errors; deliberate empty custom fallback remains. Approve/reinstate and report auto-hide lock seller before listing and recheck status. Desktop/mobile admin/closure 8/8, vehicle 6/6 and report auto-hide 2/2; 19 DB cases pass.</x:v>
       </x:c>
       <x:c r="O75" s="136" t="str">
-        <x:v>Full latest-head CI and independent re-review pending; retain broader browser, provider and real-device acceptance.</x:v>
+        <x:v>New exact-head CI and independent re-review pending; local WebKit, live providers, real devices and production acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5d290c1d2b04af6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dc492b3f759408d"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ec68d80a3ed4b70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fa9cae348764745"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13245,10 +13245,10 @@
         <x:v>Integration + SEO</x:v>
       </x:c>
       <x:c r="E16" s="141" t="str">
-        <x:v>Desktop/mobile car and bike edits: inactive make/model/variant, forged IDs, valid curated edits and concurrent closure; DB facet checks and controlled view-count/closure lock barrier</x:v>
+        <x:v>Car/bike malformed variant IDs with custom labels, overflow boundary, empty fallback and curated edit; deterministic admin approve/reinstate versus closure in both lock schedules; report auto-hide flow</x:v>
       </x:c>
       <x:c r="F16" s="141" t="str">
-        <x:v>Latest local pass: 6/6 focused edit/closure browser cases and 19/19 DB cases, including view-count/closure barrier. Invalid taxonomy leaves ads unchanged; valid curated edits persist. Latest-head CI and real-device acceptance pending.</x:v>
+        <x:v>Local pass: 8/8 forced admin/closure, 6/6 vehicle edit/closure and 2/2 report auto-hide desktop/mobile cases; 19/19 DB, 101 routes, check/lint/build. No unexpected Flight error, partial audit or closed-owner public ad. New CI/re-review pending.</x:v>
       </x:c>
       <x:c r="G16" s="141" t="str">
         <x:v>Edit flow complete</x:v>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50b9398aead54269"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R978a9fe611e54bc5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8325b1312d65454d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11cf66df439b45aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Prevent reciprocal report deadlocks
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdbbeae8b7cf045e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R0cdeef88622c48b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R444addfb44de4f3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Ra4cb348fe2ed4bbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Re94a8e8b046942f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R75c07b816a674626"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rb747cd702a964ec3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6769d35439974fbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R7f5bda62d2c34914"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R484627434c3d4106"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rd7413b6589e24c9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R6a5c34e0690d4f4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R0a3c315b99064d15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R5ded8a67c74f4989"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3e9a69fceb3443d8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4252ec3a44be4e9b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6: second fresh review found admin/closure P2 deadlock and malformed-ID P3; local fixes pass, latest CI/re-review pending</x:v>
+        <x:v>PR #6: third review found reciprocal-report P2 deadlock; local lock fix and regressions pass, new CI/re-review pending</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Head 73c1974 CI 59 green; new local fixes: 19 DB, 101 routes, 8 admin race, 6 vehicle, 2 reports; new CI pending</x:v>
+        <x:v>Head 082c2d2 CI 60 green; new local fix: 19 DB, 101 routes, reciprocal 4/4, report/closure 4/4, admin/closure 8/8; new CI pending</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4719b27bccec4c1f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5dfd4be76134cb1"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>8 October second fresh review of 73c1974: admin approve/reinstate versus closure P2 deadlock and malformed variant-ID P3 confirmed. Moderation and report auto-hide now lock owner before listing and recheck locked state. Car/bike create/edit reject malformed or out-of-range variant IDs while preserving deliberate empty-ID fallback. Local check/lint/build, 19 DB tests, 101-route sweep, 8 deterministic admin/closure, 6 vehicle and 2 report browser cases pass. New exact-head CI and independent re-review pending; live provider/deployment/device gates remain open.</x:v>
+        <x:v>9 October third review of 082c2d2: reciprocal authenticated reports can deadlock through reporter FK KEY SHARE after target-owner FOR UPDATE. Report path now uses owner NO KEY UPDATE, retaining closure serialization and eligibility recheck. Local 19 DB, check/lint/build, 101 routes, reciprocal 4/4, report/closure 4/4 and admin/closure 8/8 desktop/mobile cases pass. Prior admin/closure and malformed variant findings independently resolved. New exact-head CI and re-review pending; live provider/deployment/device gates remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2269,7 +2269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="133" t="str">
-        <x:v>8 October 2026: second fresh PR #6 review of 73c1974 found admin/closure P2 and malformed-ID P3. Owner-before-listing moderation and strict car/bike variant parsing pass local gates: 19 DB, 101 routes, 8 deterministic admin races, 6 vehicle and 2 report browser cases. New exact-head CI and independent re-review pending. Live deployment/provider/device gates remain open.</x:v>
+        <x:v>9 October 2026: third PR #6 review of 082c2d2 confirmed reciprocal-report P2 deadlock. Report owner NO KEY UPDATE permits reporter FK KEY SHARE while serializing closure. Local gates: 19 DB, 101 routes, 4 reciprocal, 4 report/closure and 8 admin/closure browser cases; check/lint/build pass. New exact-head CI and independent re-review pending. Live deployment/provider/device gates remain open.</x:v>
       </x:c>
       <x:c r="B2" s="133"/>
       <x:c r="C2" s="133"/>
@@ -5681,10 +5681,10 @@
         <x:v>Owner/non-owner/admin; each vertical; validation; SEO redirect</x:v>
       </x:c>
       <x:c r="N75" s="136" t="str">
-        <x:v>Second fresh review: car/bike create/edit now reject malformed and &gt;2147483647 variant IDs with field errors; deliberate empty custom fallback remains. Approve/reinstate and report auto-hide lock seller before listing and recheck status. Desktop/mobile admin/closure 8/8, vehicle 6/6 and report auto-hide 2/2; 19 DB cases pass.</x:v>
+        <x:v>Third review: reciprocal authenticated reports no longer invert target-owner lock against reporter FK. Forced listing barrier verifies both fourth and fifth reports, exactly one queue audit per hidden ad and retry dedup (4/4 desktop/mobile). Report/closure both orders 4/4; earlier admin/closure 8/8. Car/bike strict variant-ID fix remains verified.</x:v>
       </x:c>
       <x:c r="O75" s="136" t="str">
-        <x:v>New exact-head CI and independent re-review pending; local WebKit, live providers, real devices and production acceptance remain open.</x:v>
+        <x:v>Replacement-head CI and independent re-review pending; local WebKit, live providers, real devices and production acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dc492b3f759408d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d6c22a61cf84bce"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fa9cae348764745"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdf3e11537794ec5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13245,10 +13245,10 @@
         <x:v>Integration + SEO</x:v>
       </x:c>
       <x:c r="E16" s="141" t="str">
-        <x:v>Car/bike malformed variant IDs with custom labels, overflow boundary, empty fallback and curated edit; deterministic admin approve/reinstate versus closure in both lock schedules; report auto-hide flow</x:v>
+        <x:v>Reciprocal authenticated reporters with 3 or 4 prior reports and forced listing barrier; fifth-report auto-hide/audit, duplicate retry, report/closure both orders, admin/closure both orders</x:v>
       </x:c>
       <x:c r="F16" s="141" t="str">
-        <x:v>Local pass: 8/8 forced admin/closure, 6/6 vehicle edit/closure and 2/2 report auto-hide desktop/mobile cases; 19/19 DB, 101 routes, check/lint/build. No unexpected Flight error, partial audit or closed-owner public ad. New CI/re-review pending.</x:v>
+        <x:v>Local pass: reciprocal 4/4, report/closure 4/4 and admin/closure 8/8 desktop/mobile cases; 19/19 DB, 101 routes, check/lint/build. Both fifth reports and audits commit without unexpected Flight error. New CI/re-review pending.</x:v>
       </x:c>
       <x:c r="G16" s="141" t="str">
         <x:v>Edit flow complete</x:v>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R978a9fe611e54bc5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80cb931f063e4729"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11cf66df439b45aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d3175fa00db46d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Avoid reciprocal admin moderation FK deadlocks
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6769d35439974fbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R7f5bda62d2c34914"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R484627434c3d4106"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rd7413b6589e24c9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R6a5c34e0690d4f4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R0a3c315b99064d15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R5ded8a67c74f4989"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb0f542b58baa4b32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rbf6187c199bb458f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rd8f3ce27539744df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R3285753608b84912"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R7a233a1a8c8147c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rb3d918324dbc4169"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R22603cc687e1438a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4252ec3a44be4e9b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb7a70f7f1692451c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6: third review found reciprocal-report P2 deadlock; local lock fix and regressions pass, new CI/re-review pending</x:v>
+        <x:v>PR #6: fourth review found reciprocal admin moderation P2 deadlock; local lock fix and regressions pass, new CI/re-review pending</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Head 082c2d2 CI 60 green; new local fix: 19 DB, 101 routes, reciprocal 4/4, report/closure 4/4, admin/closure 8/8; new CI pending</x:v>
+        <x:v>Head d5aff99 CI 61 green; new local fix: 19 DB, 101 routes, reciprocal 8/8, closure 16/16, check/lint/build; new CI pending</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5dfd4be76134cb1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dd1ca54a59a40f4"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>9 October third review of 082c2d2: reciprocal authenticated reports can deadlock through reporter FK KEY SHARE after target-owner FOR UPDATE. Report path now uses owner NO KEY UPDATE, retaining closure serialization and eligibility recheck. Local 19 DB, check/lint/build, 101 routes, reciprocal 4/4, report/closure 4/4 and admin/closure 8/8 desktop/mobile cases pass. Prior admin/closure and malformed variant findings independently resolved. New exact-head CI and re-review pending; live provider/deployment/device gates remain open.</x:v>
+        <x:v>9 October fourth review of d5aff99: reciprocal admin approve/reinstate of admin-owned ads can deadlock through moderator FK KEY SHARE after target-owner FOR UPDATE. Shared moderation owner lock now uses NO KEY UPDATE, retaining closure serialization and eligibility recheck. Local 19 DB, check/lint/build, 101 routes, reciprocal admin/report 8/8 and closure 16/16 desktop/mobile cases pass. Prior reciprocal-report P2 independently resolved. New exact-head CI and re-review pending; live provider/deployment/device gates remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2269,7 +2269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="133" t="str">
-        <x:v>9 October 2026: third PR #6 review of 082c2d2 confirmed reciprocal-report P2 deadlock. Report owner NO KEY UPDATE permits reporter FK KEY SHARE while serializing closure. Local gates: 19 DB, 101 routes, 4 reciprocal, 4 report/closure and 8 admin/closure browser cases; check/lint/build pass. New exact-head CI and independent re-review pending. Live deployment/provider/device gates remain open.</x:v>
+        <x:v>9 October 2026: fourth PR #6 review of d5aff99 found reciprocal admin moderation P2 deadlock. Shared owner NO KEY UPDATE permits moderator FK KEY SHARE while serializing closure. Local gates: 19 DB, 101 routes, 8 reciprocal and 16 closure browser cases; check/lint/build pass. New exact-head CI and independent re-review pending. Live deployment/provider/device gates remain open.</x:v>
       </x:c>
       <x:c r="B2" s="133"/>
       <x:c r="C2" s="133"/>
@@ -5681,7 +5681,7 @@
         <x:v>Owner/non-owner/admin; each vertical; validation; SEO redirect</x:v>
       </x:c>
       <x:c r="N75" s="136" t="str">
-        <x:v>Third review: reciprocal authenticated reports no longer invert target-owner lock against reporter FK. Forced listing barrier verifies both fourth and fifth reports, exactly one queue audit per hidden ad and retry dedup (4/4 desktop/mobile). Report/closure both orders 4/4; earlier admin/closure 8/8. Car/bike strict variant-ID fix remains verified.</x:v>
+        <x:v>Fourth review: reciprocal admin-owned approve/reinstate no longer deadlock through moderator FK. Forced listing barrier verifies both decisions, two active ads and exactly one audit per ad (4/4 desktop/mobile). Reciprocal reports 4/4; admin/report/edit closure and account lifecycle 16/16. Previous reciprocal-report P2 independently resolved.</x:v>
       </x:c>
       <x:c r="O75" s="136" t="str">
         <x:v>Replacement-head CI and independent re-review pending; local WebKit, live providers, real devices and production acceptance remain open.</x:v>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d6c22a61cf84bce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R679b69ffbeff4c78"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdf3e11537794ec5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R653e9e1e42614b0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13245,10 +13245,10 @@
         <x:v>Integration + SEO</x:v>
       </x:c>
       <x:c r="E16" s="141" t="str">
-        <x:v>Reciprocal authenticated reporters with 3 or 4 prior reports and forced listing barrier; fifth-report auto-hide/audit, duplicate retry, report/closure both orders, admin/closure both orders</x:v>
+        <x:v>Reciprocal admin-owned approve and reinstate with forced listing barrier and exactly one audit; reciprocal authenticated reporters at threshold and duplicate retry; admin/report/edit closure forced schedules and account lifecycle</x:v>
       </x:c>
       <x:c r="F16" s="141" t="str">
-        <x:v>Local pass: reciprocal 4/4, report/closure 4/4 and admin/closure 8/8 desktop/mobile cases; 19/19 DB, 101 routes, check/lint/build. Both fifth reports and audits commit without unexpected Flight error. New CI/re-review pending.</x:v>
+        <x:v>Local pass: reciprocal admin/report 8/8 and closure 16/16 desktop/mobile cases; 19/19 DB, 101 routes, check/lint/build. Both admin decisions and reports commit without unexpected Flight error. New CI/re-review pending.</x:v>
       </x:c>
       <x:c r="G16" s="141" t="str">
         <x:v>Edit flow complete</x:v>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80cb931f063e4729"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc584c69ba20541f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d3175fa00db46d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7726643259554836"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Make alert retry acceptance timing deterministic
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb0f542b58baa4b32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rbf6187c199bb458f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rd8f3ce27539744df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R3285753608b84912"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R7a233a1a8c8147c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rb3d918324dbc4169"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R22603cc687e1438a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re761878a33c54b90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R6b1b200f1fc34441"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rbf1391c44287465c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rd91eacb9f9db4930"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Re397921e87554941"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R6f5a809d77d84764"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R7624b3cfbca0443f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb7a70f7f1692451c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rabf404bb02b548cd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Head d5aff99 CI 61 green; new local fix: 19 DB, 101 routes, reciprocal 8/8, closure 16/16, check/lint/build; new CI pending</x:v>
+        <x:v>Head d5aff99 CI 61 green; fix local: 19 DB, 101 routes, reciprocal 8/8, closure 16/16, check/lint/build. CI 62 stopped on alert retry test timing race; test corrected, isolated DB 19/19 pass; replacement CI pending.</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dd1ca54a59a40f4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44766281758f4ebe"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>9 October fourth review of d5aff99: reciprocal admin approve/reinstate of admin-owned ads can deadlock through moderator FK KEY SHARE after target-owner FOR UPDATE. Shared moderation owner lock now uses NO KEY UPDATE, retaining closure serialization and eligibility recheck. Local 19 DB, check/lint/build, 101 routes, reciprocal admin/report 8/8 and closure 16/16 desktop/mobile cases pass. Prior reciprocal-report P2 independently resolved. New exact-head CI and re-review pending; live provider/deployment/device gates remain open.</x:v>
+        <x:v>9 October fourth review of d5aff99: reciprocal admin approve/reinstate of admin-owned ads deadlocked through moderator FK KEY SHARE after owner FOR UPDATE. Shared moderation owner lock now uses NO KEY UPDATE, preserving closure serialization. Local 19 DB, check/lint/build, 101 routes, reciprocal admin/report 8/8 and closure 16/16 desktop/mobile cases pass. CI 62 stopped on pre-existing alert retry test timing race; forced retry now has a past due time and fresh isolated DB 19/19 pass. Replacement CI and independent re-review pending; live provider/deployment/device gates remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2269,7 +2269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="133" t="str">
-        <x:v>9 October 2026: fourth PR #6 review of d5aff99 found reciprocal admin moderation P2 deadlock. Shared owner NO KEY UPDATE permits moderator FK KEY SHARE while serializing closure. Local gates: 19 DB, 101 routes, 8 reciprocal and 16 closure browser cases; check/lint/build pass. New exact-head CI and independent re-review pending. Live deployment/provider/device gates remain open.</x:v>
+        <x:v>9 October 2026: fourth PR #6 review of d5aff99 found reciprocal admin moderation P2 deadlock. Shared owner NO KEY UPDATE permits moderator FK KEY SHARE while serializing closure. Local 19 DB, 101 routes, 8 reciprocal and 16 closure browser cases, check/lint/build pass. CI 62 stopped on alert retry test timing race; corrected and isolated DB 19/19 pass. Replacement CI and independent re-review pending. Live deployment/provider/device gates remain open.</x:v>
       </x:c>
       <x:c r="B2" s="133"/>
       <x:c r="C2" s="133"/>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R679b69ffbeff4c78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a51e01d39414dd4"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12866,7 +12866,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R653e9e1e42614b0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eeed321dc964e07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13248,7 +13248,7 @@
         <x:v>Reciprocal admin-owned approve and reinstate with forced listing barrier and exactly one audit; reciprocal authenticated reporters at threshold and duplicate retry; admin/report/edit closure forced schedules and account lifecycle</x:v>
       </x:c>
       <x:c r="F16" s="141" t="str">
-        <x:v>Local pass: reciprocal admin/report 8/8 and closure 16/16 desktop/mobile cases; 19/19 DB, 101 routes, check/lint/build. Both admin decisions and reports commit without unexpected Flight error. New CI/re-review pending.</x:v>
+        <x:v>Local pass: reciprocal admin/report 8/8 and closure 16/16 desktop/mobile; 19/19 DB, 101 routes, check/lint/build. Both admin decisions and reports commit without unexpected Flight error. CI 62 stopped on alert retry test timing race; corrected and isolated DB 19/19 pass. Replacement CI/re-review pending.</x:v>
       </x:c>
       <x:c r="G16" s="141" t="str">
         <x:v>Edit flow complete</x:v>
@@ -14434,7 +14434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc584c69ba20541f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5846b1f59b3d47bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14660,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7726643259554836"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83c92cb47079446c"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
test: close local acceptance backlog
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re761878a33c54b90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R6b1b200f1fc34441"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="Rbf1391c44287465c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Rd91eacb9f9db4930"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Re397921e87554941"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R6f5a809d77d84764"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R7624b3cfbca0443f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd4f27787aefa4591"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R07f997ed19184bb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R4a3584fc8c244911"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R6ba96df6d4dc49d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R2fbce3abf6154475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Re66142b2618147a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R83370b6e705648c9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rabf404bb02b548cd"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R436e060765b649ee"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1175,7 +1175,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="86" t="str">
-        <x:v>JaniWheels V1 Development Control Sheet - 8 October 2026</x:v>
+        <x:v>JaniWheels V1 Development Control Sheet - 10 October 2026</x:v>
       </x:c>
       <x:c r="B1" s="86"/>
       <x:c r="C1" s="86"/>
@@ -1253,7 +1253,7 @@
         <x:v>Current branch</x:v>
       </x:c>
       <x:c r="H5" s="93" t="str">
-        <x:v>codex/launch-quality-system; PR #6</x:v>
+        <x:v>codex/local-acceptance-backlog; PR pending</x:v>
       </x:c>
       <x:c r="I5" s="93"/>
       <x:c r="J5" s="94"/>
@@ -1280,7 +1280,7 @@
         <x:v>Current stage</x:v>
       </x:c>
       <x:c r="H6" s="98" t="str">
-        <x:v>Homepage merged via PR #5; Stage 6.2 active</x:v>
+        <x:v>PR #6 merged; Stage 6.2 local test backlog verified on feature branch</x:v>
       </x:c>
       <x:c r="I6" s="98"/>
       <x:c r="J6" s="99"/>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6: fourth review found reciprocal admin moderation P2 deadlock; local lock fix and regressions pass, new CI/re-review pending</x:v>
+        <x:v>PR #6 merged after independent review. New local package CI/review pending.</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1334,7 +1334,7 @@
         <x:v>Next functionality</x:v>
       </x:c>
       <x:c r="H8" s="98" t="str">
-        <x:v>Production access/providers and independent launch acceptance</x:v>
+        <x:v>Hosting, production DB/backups, live providers, real-device and production acceptance</x:v>
       </x:c>
       <x:c r="I8" s="98"/>
       <x:c r="J8" s="99"/>
@@ -1355,13 +1355,13 @@
         <x:v>Local passed</x:v>
       </x:c>
       <x:c r="F9" s="99" t="str">
-        <x:v>19 isolated DB cases passed; live acceptance open</x:v>
+        <x:v>22 isolated DB tests passed; live acceptance open</x:v>
       </x:c>
       <x:c r="G9" s="97" t="str">
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Head d5aff99 CI 61 green; fix local: 19 DB, 101 routes, reciprocal 8/8, closure 16/16, check/lint/build. CI 62 stopped on alert retry test timing race; test corrected, isolated DB 19/19 pass; replacement CI pending.</x:v>
+        <x:v>Local: 22 DB, 101 routes, 166 browser pass/1 planned skip; checks/build pass. CI pending.</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1415,7 +1415,7 @@
         <x:v>Final QA blocker</x:v>
       </x:c>
       <x:c r="H11" s="103" t="str">
-        <x:v>Updated PR review, providers, load and final acceptance</x:v>
+        <x:v>Latest-head CI/review plus deployment, provider, device and load acceptance</x:v>
       </x:c>
       <x:c r="I11" s="103"/>
       <x:c r="J11" s="104"/>
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>8 October: nine independent-review defects and ban-policy risk repaired. Next.js 15.5.27 production audit clean. CI 56 green: 18 DB tests, 101 URLs, 127 browser passes plus one retry-pass and one planned skip. Accessibility fixture race repaired. Latest exact-head CI, independent re-review and deployment gates remain authoritative.</x:v>
+        <x:v>10 October: PR #6 merged after independent re-review. Local acceptance backlog T-004, T-019/020, T-022/023/024, T-031 and T-035/036 now has deterministic DB and desktop/mobile browser evidence. Stage 6.2 still needs staging/live provider, production infrastructure, real-device and load acceptance.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44766281758f4ebe"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28c24a69da76441a"/>
 </x:worksheet>
 </file>
 
@@ -1858,7 +1858,7 @@
         <x:v>Active package</x:v>
       </x:c>
       <x:c r="B7" s="127" t="str">
-        <x:v>Stage 6.2 code/CI complete on feature branch; external deployment team owns hosting, provider, DNS and live acceptance per docs/DEPLOYMENT_HANDOFF.md</x:v>
+        <x:v>Stage 6.2 local test backlog covered on codex/local-acceptance-backlog; external deployment team owns hosting, providers, DNS and live acceptance per docs/DEPLOYMENT_HANDOFF.md</x:v>
       </x:c>
       <x:c r="C7" s="127"/>
       <x:c r="D7" s="127"/>
@@ -1870,7 +1870,7 @@
         <x:v>Current branch</x:v>
       </x:c>
       <x:c r="B8" s="127" t="str">
-        <x:v>codex/launch-quality-system (pushed; PR #6 open)</x:v>
+        <x:v>codex/local-acceptance-backlog (local package; CI/review pending)</x:v>
       </x:c>
       <x:c r="C8" s="127"/>
       <x:c r="D8" s="127"/>
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>9 October fourth review of d5aff99: reciprocal admin approve/reinstate of admin-owned ads deadlocked through moderator FK KEY SHARE after owner FOR UPDATE. Shared moderation owner lock now uses NO KEY UPDATE, preserving closure serialization. Local 19 DB, check/lint/build, 101 routes, reciprocal admin/report 8/8 and closure 16/16 desktop/mobile cases pass. CI 62 stopped on pre-existing alert retry test timing race; forced retry now has a past due time and fresh isolated DB 19/19 pass. Replacement CI and independent re-review pending; live provider/deployment/device gates remain open.</x:v>
+        <x:v>10 October: PR #6 merged at 117ef9b following independent re-review with no new actionable finding. Local backlog package adds exact seeded car/bike facet and multi-page sort assertions plus desktop/mobile session, URL canonicalization, detail/photo, dealer slug and complete service-transition checks. 22 DB and 166 browser cases pass with one planned skip; route sweep, check, lint and build pass. New branch CI/review and live deployment/provider/device gates remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2269,7 +2269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="133" t="str">
-        <x:v>9 October 2026: fourth PR #6 review of d5aff99 found reciprocal admin moderation P2 deadlock. Shared owner NO KEY UPDATE permits moderator FK KEY SHARE while serializing closure. Local 19 DB, 101 routes, 8 reciprocal and 16 closure browser cases, check/lint/build pass. CI 62 stopped on alert retry test timing race; corrected and isolated DB 19/19 pass. Replacement CI and independent re-review pending. Live deployment/provider/device gates remain open.</x:v>
+        <x:v>10 October 2026: PR #6 merged at 117ef9b after independent review. Stage 6.2 local test backlog covered by 22 isolated DB cases, desktop/mobile browser journeys (166 pass, 1 planned skip), 101-route sweep, check/lint/build. New branch CI/review and staging/live provider, infrastructure, load and real-device gates remain open.</x:v>
       </x:c>
       <x:c r="B2" s="133"/>
       <x:c r="C2" s="133"/>
@@ -2720,10 +2720,10 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>8 Oct: review fixes 7c9a1e1 and Next.js 15.5.27 patch df422a7 pushed. CI run 56 passed: audit, 18 DB cases, checks/lint/build, 101 URLs and browser suite (127 pass, 1 retry-pass, 1 planned skip). Accessibility fixture race repaired; latest exact-head CI and independent re-review required.</x:v>
+        <x:v>PR #6 latest-head CI #63 green and independently re-reviewed with no new actionable findings, then merged at 117ef9b. Local acceptance branch adds 3 seeded search DB cases and 12 desktop/mobile browser cases; local 22 DB, 166 browser passes, 1 planned skip, check/lint/build and 101-route sweep pass. New branch CI pending.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
-        <x:v>Require green updated-head CI, independent re-review and branch protection before main merge; persistent staging remains.</x:v>
+        <x:v>Require green new-head CI and independent review; confirm branch protection. Persistent staging and live acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2955,10 +2955,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>8 Oct: browser regressions added for seller-delete backup replay, quota reactivation, authenticated redirect, banned detail/media/contact and closed verified-dealer homepage. Final coverage in PR6_REVIEW_RESPONSE.md.</x:v>
+        <x:v>Local desktop/mobile automation now covers logout, expired/tampered sessions, canonical/unknown facets, three-vertical detail/photo delivery, duplicate dealer slugs and every inspection/assistance intermediate transition with audit/customer privacy. Full local suite: 166 pass, 1 planned skip; 22 DB cases pass.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>Maintainer review/merge decision and required repository checks; live acceptance remains tracked separately.</x:v>
+        <x:v>New branch CI and maintainer review; live provider, staging and real-device acceptance remain separately tracked.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -10663,10 +10663,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>Application 1e0a071 full CI run 49 passes: 120 browser passes, 1 planned skip, 13 isolated DB checks, check/lint/build and 101-route sweep. Run 48 Google-prefetch/redirect and WebKit-origin findings fixed; independent final review and live provider/device acceptance remain.</x:v>
+        <x:v>10 Oct local candidate: full desktop/mobile Chromium plus WebKit smoke and recovery suite 166 pass, 1 planned skip; 22 isolated DB cases, 101 routes, check/lint/build pass. New branch CI/review and live provider/device acceptance remain.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Latest-head CI, independent review, live provider/staging/device acceptance remain.</x:v>
+        <x:v>Latest-head CI and independent review; staging, live provider and real-device acceptance remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -10898,10 +10898,10 @@
         <x:v>Checklist review; defect retest</x:v>
       </x:c>
       <x:c r="N186" s="136" t="str">
-        <x:v>Candidate 1e0a071 passes full CI run 49, including Chromium/mobile/WebKit and recovery, 13 DB cases and 101-route sweep. Tracker links provider/device/staging gates to owner handoff; this does not substitute independent review or live acceptance.</x:v>
+        <x:v>Test Matrix now records deterministic local evidence for nine previously open rows. Clean candidate: 22 DB, 166 browser pass/1 planned skip, 101 routes, check/lint/build. No live-provider or real-device sign-off claimed.</x:v>
       </x:c>
       <x:c r="O186" s="136" t="str">
-        <x:v>Fill the checklist and Test Matrix with candidate-specific staging, Safari/real-device, provider and infrastructure evidence; obtain PR reviewer sign-off before merge.</x:v>
+        <x:v>Obtain branch review and record candidate-specific staging, live provider, real-device, production infrastructure and load evidence before launch sign-off.</x:v>
       </x:c>
     </x:row>
     <x:row r="187">
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a51e01d39414dd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2360629eb7024562"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12835,6 +12835,9 @@
       <x:c r="G23" s="141" t="str">
         <x:v>In Progress</x:v>
       </x:c>
+      <x:c r="H23" t="str">
+        <x:v>Local acceptance backlog verified; new branch CI/review plus live deployment/provider/device/load gates remain.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="88" t="str">
@@ -12866,7 +12869,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eeed321dc964e07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0b436774a914404"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13037,10 +13040,10 @@
         <x:v>Integration + Security</x:v>
       </x:c>
       <x:c r="E8" s="141" t="str">
-        <x:v>Manual only</x:v>
+        <x:v>Desktop/mobile browser: logout revokes DB session; replayed, expired and tampered cookies cannot reopen seller dashboard.</x:v>
       </x:c>
       <x:c r="F8" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Local pass (desktop/mobile); live session configuration pending deployment acceptance.</x:v>
       </x:c>
       <x:c r="G8" s="141" t="str">
         <x:v>Active/expired/tampered tokens</x:v>
@@ -13427,10 +13430,10 @@
         <x:v>DB integration</x:v>
       </x:c>
       <x:c r="E23" s="141" t="str">
-        <x:v>SEO only partial</x:v>
+        <x:v>Seeded DB integration: 15 car facet/combination cases compare exact IDs and totals with independent SQL, including two-feature intersection and empty result.</x:v>
       </x:c>
       <x:c r="F23" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Local pass; live inventory/search acceptance pending.</x:v>
       </x:c>
       <x:c r="G23" s="141" t="str">
         <x:v>Seeded deterministic listings</x:v>
@@ -13453,10 +13456,10 @@
         <x:v>DB integration</x:v>
       </x:c>
       <x:c r="E24" s="141" t="str">
-        <x:v>SEO only partial</x:v>
+        <x:v>Seeded DB integration: 10 bike facet/combination cases compare exact IDs and totals with independent SQL.</x:v>
       </x:c>
       <x:c r="F24" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Local pass; live inventory/search acceptance pending.</x:v>
       </x:c>
       <x:c r="G24" s="141" t="str">
         <x:v>Seeded bike listings</x:v>
@@ -13505,10 +13508,10 @@
         <x:v>DB integration</x:v>
       </x:c>
       <x:c r="E26" s="141" t="str">
-        <x:v>Route sweep partial</x:v>
+        <x:v>Seeded DB integration: every supported car/bike/part sort over three pages; exact IDs, totals, page counts and no duplicates.</x:v>
       </x:c>
       <x:c r="F26" s="141" t="str">
-        <x:v>Pending automation</x:v>
+        <x:v>Local pass; production-scale/load acceptance pending.</x:v>
       </x:c>
       <x:c r="G26" s="141" t="str">
         <x:v>More than 50 deterministic rows</x:v>
@@ -13531,10 +13534,10 @@
         <x:v>SEO unit + E2E</x:v>
       </x:c>
       <x:c r="E27" s="141" t="str">
-        <x:v>SEO checks plus Playwright unknown facet 404</x:v>
+        <x:v>Desktop/mobile browser: reordered city/facet URLs redirect 308 to canonical car/bike/part paths with query preserved; unknown facets 404.</x:v>
       </x:c>
       <x:c r="F27" s="141" t="str">
-        <x:v>Partial pass: unknown 404; reordered URL browser check pending</x:v>
+        <x:v>Local pass; production HTTPS/canonical acceptance pending.</x:v>
       </x:c>
       <x:c r="G27" s="141" t="str">
         <x:v>Facet cases</x:v>
@@ -13557,10 +13560,10 @@
         <x:v>E2E</x:v>
       </x:c>
       <x:c r="E28" s="141" t="str">
-        <x:v>Route sweep partial</x:v>
+        <x:v>Desktop/mobile browser: car, bike and part detail title, heading, canonical, specifications, lazy-loaded WebP and authorized media response.</x:v>
       </x:c>
       <x:c r="F28" s="141" t="str">
-        <x:v>Pending deep checks</x:v>
+        <x:v>Local pass; live image provider and real-device acceptance pending.</x:v>
       </x:c>
       <x:c r="G28" s="141" t="str">
         <x:v>Representative listing each vertical</x:v>
@@ -13739,10 +13742,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E35" s="141" t="str">
-        <x:v>Playwright desktop/mobile dealer registration</x:v>
+        <x:v>Desktop/mobile browser: two distinct sellers register identical dealer names; unique permanent slugs, dealer user types and no duplicate on revisit.</x:v>
       </x:c>
       <x:c r="F35" s="141" t="str">
-        <x:v>Partial pass: new dealer dashboard and pending badge; duplicate slug case pending</x:v>
+        <x:v>Local pass; live operational acceptance pending.</x:v>
       </x:c>
       <x:c r="G35" s="141" t="str">
         <x:v>Authenticated individual</x:v>
@@ -13843,10 +13846,10 @@
         <x:v>Security + E2E</x:v>
       </x:c>
       <x:c r="E39" s="141" t="str">
-        <x:v>Desktop/mobile creation/customer history plus direct administration replay by owner, foreign seller and anonymous visitor; admin positive control and unchanged DB/audit checks</x:v>
+        <x:v>Desktop/mobile browser: every inspection intermediate transition through completion; DB status, append-only admin audit, customer history and private-note exclusion. Existing negative/authz checks retained.</x:v>
       </x:c>
       <x:c r="F39" s="141" t="str">
-        <x:v>Local pass for covered paths: unauthorized writes, invalid status jump, missing customer message and terminal-state reopening rejected; valid admin update audited; customer isolation/private-note exclusion pass. Remaining intermediate transitions/live acceptance open.</x:v>
+        <x:v>Local lifecycle pass; live service operations acceptance pending.</x:v>
       </x:c>
       <x:c r="G39" s="141" t="str">
         <x:v>Inspection admin complete</x:v>
@@ -13869,10 +13872,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E40" s="141" t="str">
-        <x:v>Desktop/mobile creation/customer history plus direct administration replay by owner, foreign seller and anonymous visitor; admin positive control and unchanged DB/audit checks</x:v>
+        <x:v>Desktop/mobile browser: every assistance intermediate transition through sold, including follow-up back to ad_live; DB status, append-only admin audit, customer history and private-note exclusion. Existing negative/authz checks retained.</x:v>
       </x:c>
       <x:c r="F40" s="141" t="str">
-        <x:v>Local pass for covered paths: unauthorized writes, invalid status jump, missing customer message and terminal-state reopening rejected; valid admin update audited; customer isolation/private-note exclusion pass. Remaining intermediate transitions/live acceptance open.</x:v>
+        <x:v>Local lifecycle pass; live service operations acceptance pending.</x:v>
       </x:c>
       <x:c r="G40" s="141" t="str">
         <x:v>Public/admin flows complete</x:v>
@@ -14434,7 +14437,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5846b1f59b3d47bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc970f257875142b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14660,7 +14663,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83c92cb47079446c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e96f71a344043d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs: link local acceptance tracker to PR 7
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd4f27787aefa4591"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R07f997ed19184bb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R4a3584fc8c244911"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R6ba96df6d4dc49d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R2fbce3abf6154475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Re66142b2618147a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R83370b6e705648c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0a6bf461c5ae46c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rebfd268bc7de4e72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R7b3a8d60cac54124"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Ra165c7b533214445"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R5479a0cd8b6d44e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rac96213912bb4f44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Ra13ba09686374416"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R436e060765b649ee"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4efe73f2387a48b3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1253,7 +1253,7 @@
         <x:v>Current branch</x:v>
       </x:c>
       <x:c r="H5" s="93" t="str">
-        <x:v>codex/local-acceptance-backlog; PR pending</x:v>
+        <x:v>codex/local-acceptance-backlog; PR #7</x:v>
       </x:c>
       <x:c r="I5" s="93"/>
       <x:c r="J5" s="94"/>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #6 merged after independent review. New local package CI/review pending.</x:v>
+        <x:v>PR #7 open at 0c45b68; CI/review pending. PR #6 merged.</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28c24a69da76441a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbedf5ae3da54d05"/>
 </x:worksheet>
 </file>
 
@@ -1870,7 +1870,7 @@
         <x:v>Current branch</x:v>
       </x:c>
       <x:c r="B8" s="127" t="str">
-        <x:v>codex/local-acceptance-backlog (local package; CI/review pending)</x:v>
+        <x:v>codex/local-acceptance-backlog (pushed; PR #7 open)</x:v>
       </x:c>
       <x:c r="C8" s="127"/>
       <x:c r="D8" s="127"/>
@@ -2269,7 +2269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="133" t="str">
-        <x:v>10 October 2026: PR #6 merged at 117ef9b after independent review. Stage 6.2 local test backlog covered by 22 isolated DB cases, desktop/mobile browser journeys (166 pass, 1 planned skip), 101-route sweep, check/lint/build. New branch CI/review and staging/live provider, infrastructure, load and real-device gates remain open.</x:v>
+        <x:v>10 October 2026: PR #6 merged at 117ef9b after independent review. PR #7 opens the Stage 6.2 local test backlog package: 22 isolated DB cases, 166 desktop/mobile/WebKit/recovery browser passes and 1 planned skip, 101-route sweep, check/lint/build. PR #7 CI/review and staging/live provider, infrastructure, load and real-device gates remain open.</x:v>
       </x:c>
       <x:c r="B2" s="133"/>
       <x:c r="C2" s="133"/>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2360629eb7024562"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f700ab5ab8e4680"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12869,7 +12869,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0b436774a914404"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbca17b14ec784f37"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14437,7 +14437,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc970f257875142b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6864d1af704a4299"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14663,7 +14663,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e96f71a344043d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ff80b3304f248fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Fix PR7 dealer race and local acceptance regressions
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0a6bf461c5ae46c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rebfd268bc7de4e72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R7b3a8d60cac54124"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="Ra165c7b533214445"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R5479a0cd8b6d44e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rac96213912bb4f44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Ra13ba09686374416"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3854babc910945d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R198f168069eb4622"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R7483c7ded5194485"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R701eae0f50ef4685"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R77705a82c16248ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R9c0ab968cd7d4e34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R7f6cce22414a431b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4efe73f2387a48b3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5d231a9b7c3142e1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #7 open at 0c45b68; CI/review pending. PR #6 merged.</x:v>
+        <x:v>PR #7 review: three findings fixed locally; new CI/re-review pending.</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Local: 22 DB, 101 routes, 166 browser pass/1 planned skip; checks/build pass. CI pending.</x:v>
+        <x:v>Local: 22 DB, 101 routes, 168 browser pass/1 planned skip; checks/build pass. New CI pending.</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>10 October: PR #6 merged after independent re-review. Local acceptance backlog T-004, T-019/020, T-022/023/024, T-031 and T-035/036 now has deterministic DB and desktop/mobile browser evidence. Stage 6.2 still needs staging/live provider, production infrastructure, real-device and load acceptance.</x:v>
+        <x:v>10 October: PR #7 review findings addressed. Dealer slug claims now serialize through the unique index; forced overlapping registrations pass. Owned detail fixtures pass in two repeated 2-worker desktop/mobile runs. Contrasting search fixtures reject disabled car assembly and bike fuel predicates. Stage 6.2 still needs PR re-review and deployment/provider/device/load acceptance.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbedf5ae3da54d05"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17900221fb934dbe"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>10 October: PR #6 merged at 117ef9b following independent re-review with no new actionable finding. Local backlog package adds exact seeded car/bike facet and multi-page sort assertions plus desktop/mobile session, URL canonicalization, detail/photo, dealer slug and complete service-transition checks. 22 DB and 166 browser cases pass with one planned skip; route sweep, check, lint and build pass. New branch CI/review and live deployment/provider/device gates remain open.</x:v>
+        <x:v>10 October PR #7 re-review found concurrent dealer slug 23505, shared-photo test race and non-discriminating assembly/fuel fixtures. Atomic slug insert and suffix retry preserve dealer/user transaction. Forced authenticated overlap desktop/mobile passes; isolated detail fixtures pass twice with 2 workers; both filter-removal mutations fail the intended DB cases. Fresh full local suite: 22 DB, 168 browser pass/1 planned skip, 101 routes, check/lint/build. New exact-head CI/re-review and live deployment/provider/device gates remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2269,7 +2269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="133" t="str">
-        <x:v>10 October 2026: PR #6 merged at 117ef9b after independent review. PR #7 opens the Stage 6.2 local test backlog package: 22 isolated DB cases, 166 desktop/mobile/WebKit/recovery browser passes and 1 planned skip, 101-route sweep, check/lint/build. PR #7 CI/review and staging/live provider, infrastructure, load and real-device gates remain open.</x:v>
+        <x:v>10 October 2026: PR #7 review findings addressed on feature branch. Forced dealer registration overlap, owned parallel photo fixtures and discriminating assembly/fuel search tests pass locally. Full acceptance: 22 isolated DB, 168 browser pass/1 planned skip, 101-route sweep, check/lint/build. New head CI/re-review and staging/live provider, infrastructure, load and real-device gates remain open.</x:v>
       </x:c>
       <x:c r="B2" s="133"/>
       <x:c r="C2" s="133"/>
@@ -2720,7 +2720,7 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>PR #6 latest-head CI #63 green and independently re-reviewed with no new actionable findings, then merged at 117ef9b. Local acceptance branch adds 3 seeded search DB cases and 12 desktop/mobile browser cases; local 22 DB, 166 browser passes, 1 planned skip, check/lint/build and 101-route sweep pass. New branch CI pending.</x:v>
+        <x:v>PR #7 prior head CI #66 green. Review fixes add atomic concurrent dealer slug claim, owned parallel photo fixtures and contrasting search filters. Fresh local 22 DB, 168 browser pass/1 planned skip, check/lint/build, 101-route sweep pass; updated-head CI pending.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
         <x:v>Require green new-head CI and independent review; confirm branch protection. Persistent staging and live acceptance remain open.</x:v>
@@ -2955,7 +2955,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Local desktop/mobile automation now covers logout, expired/tampered sessions, canonical/unknown facets, three-vertical detail/photo delivery, duplicate dealer slugs and every inspection/assistance intermediate transition with audit/customer privacy. Full local suite: 166 pass, 1 planned skip; 22 DB cases pass.</x:v>
+        <x:v>Local desktop/mobile suite now includes forced simultaneous same-name dealer registration, owned listing/photo details with two 2-worker repeats, and every service intermediate transition. Full browser suite 168 pass/1 planned skip; 22 DB cases pass. New head review pending.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>New branch CI and maintainer review; live provider, staging and real-device acceptance remain separately tracked.</x:v>
@@ -10663,7 +10663,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>10 Oct local candidate: full desktop/mobile Chromium plus WebKit smoke and recovery suite 166 pass, 1 planned skip; 22 isolated DB cases, 101 routes, check/lint/build pass. New branch CI/review and live provider/device acceptance remain.</x:v>
+        <x:v>10 Oct review fixes: full desktop/mobile Chromium, two WebKit smoke and recovery suite 168 pass/1 planned skip; 22 isolated DB, 101 routes, check/lint/build pass. New exact-head CI/re-review and live provider/device acceptance remain.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Latest-head CI and independent review; staging, live provider and real-device acceptance remain.</x:v>
@@ -10898,7 +10898,7 @@
         <x:v>Checklist review; defect retest</x:v>
       </x:c>
       <x:c r="N186" s="136" t="str">
-        <x:v>Test Matrix now records deterministic local evidence for nine previously open rows. Clean candidate: 22 DB, 166 browser pass/1 planned skip, 101 routes, check/lint/build. No live-provider or real-device sign-off claimed.</x:v>
+        <x:v>Test Matrix records revised local evidence for concurrent dealer registration, isolated detail photos and discriminating assembly/fuel search. Candidate 22 DB, 168 browser pass/1 planned skip, 101 routes, check/lint/build. Live-provider/real-device sign-off remains open.</x:v>
       </x:c>
       <x:c r="O186" s="136" t="str">
         <x:v>Obtain branch review and record candidate-specific staging, live provider, real-device, production infrastructure and load evidence before launch sign-off.</x:v>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f700ab5ab8e4680"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e4f8bd997304144"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12869,7 +12869,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbca17b14ec784f37"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc18b8b44bcec4f9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13430,10 +13430,10 @@
         <x:v>DB integration</x:v>
       </x:c>
       <x:c r="E23" s="141" t="str">
-        <x:v>Seeded DB integration: 15 car facet/combination cases compare exact IDs and totals with independent SQL, including two-feature intersection and empty result.</x:v>
+        <x:v>Seeded SQL oracle plus owned local/imported contrast pair; exact car IDs/counts and combinations. Disabling assembly predicate makes car acceptance fail.</x:v>
       </x:c>
       <x:c r="F23" s="141" t="str">
-        <x:v>Local pass; live inventory/search acceptance pending.</x:v>
+        <x:v>Local pass with contrasting assembly fixture and mutation challenge; live inventory/search acceptance pending.</x:v>
       </x:c>
       <x:c r="G23" s="141" t="str">
         <x:v>Seeded deterministic listings</x:v>
@@ -13456,10 +13456,10 @@
         <x:v>DB integration</x:v>
       </x:c>
       <x:c r="E24" s="141" t="str">
-        <x:v>Seeded DB integration: 10 bike facet/combination cases compare exact IDs and totals with independent SQL.</x:v>
+        <x:v>Seeded SQL oracle plus owned petrol/electric contrast pair; exact bike IDs/counts and combinations. Disabling fuel predicate makes bike acceptance fail.</x:v>
       </x:c>
       <x:c r="F24" s="141" t="str">
-        <x:v>Local pass; live inventory/search acceptance pending.</x:v>
+        <x:v>Local pass with contrasting fuel fixture and mutation challenge; live inventory/search acceptance pending.</x:v>
       </x:c>
       <x:c r="G24" s="141" t="str">
         <x:v>Seeded bike listings</x:v>
@@ -13560,10 +13560,10 @@
         <x:v>E2E</x:v>
       </x:c>
       <x:c r="E28" s="141" t="str">
-        <x:v>Desktop/mobile browser: car, bike and part detail title, heading, canonical, specifications, lazy-loaded WebP and authorized media response.</x:v>
+        <x:v>Desktop/mobile browser: each project owns seller, listing, vertical detail and WebP. Title, canonical, actual spec value and decoded media pass twice with 2 workers.</x:v>
       </x:c>
       <x:c r="F28" s="141" t="str">
-        <x:v>Local pass; live image provider and real-device acceptance pending.</x:v>
+        <x:v>Local pass with parallel-safe owned fixtures; live image provider and real-device acceptance pending.</x:v>
       </x:c>
       <x:c r="G28" s="141" t="str">
         <x:v>Representative listing each vertical</x:v>
@@ -13742,10 +13742,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E35" s="141" t="str">
-        <x:v>Desktop/mobile browser: two distinct sellers register identical dealer names; unique permanent slugs, dealer user types and no duplicate on revisit.</x:v>
+        <x:v>Desktop/mobile authenticated registration: sequential duplicate and forced overlapping same-name submits both create one dealer each, root/root-2 permanent slugs, no server error or duplicate on revisit.</x:v>
       </x:c>
       <x:c r="F35" s="141" t="str">
-        <x:v>Local pass; live operational acceptance pending.</x:v>
+        <x:v>Local pass including forced concurrency; live operational acceptance pending.</x:v>
       </x:c>
       <x:c r="G35" s="141" t="str">
         <x:v>Authenticated individual</x:v>
@@ -14437,7 +14437,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6864d1af704a4299"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83187b6e2b2d47e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14663,7 +14663,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ff80b3304f248fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02775159df4746b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Serialize dealer registration per account and tighten review tests
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3854babc910945d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R198f168069eb4622"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R7483c7ded5194485"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R701eae0f50ef4685"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R77705a82c16248ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R9c0ab968cd7d4e34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R7f6cce22414a431b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdbeddc949b284974"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rd7360ac85a4a4532"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R37aedbd0a99741b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R35550f6874e74f07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rd362bf76ed2f4498"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rd2fcb34825ee4910"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R555ebf80ce7c478f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5d231a9b7c3142e1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb26e38f36a114c54"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #7 review: three findings fixed locally; new CI/re-review pending.</x:v>
+        <x:v>PR #7 second re-review P2/P3 fixed locally; new exact-head CI and independent re-review pending.</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Local: 22 DB, 101 routes, 168 browser pass/1 planned skip; checks/build pass. New CI pending.</x:v>
+        <x:v>Local: 22 DB, 101 routes, 172 browser pass/1 planned skip; check/lint/build pass. WebKit navigation uses reduced motion; default-motion local run timed out.</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1415,7 +1415,7 @@
         <x:v>Final QA blocker</x:v>
       </x:c>
       <x:c r="H11" s="103" t="str">
-        <x:v>Latest-head CI/review plus deployment, provider, device and load acceptance</x:v>
+        <x:v>New exact-head CI/re-review plus deployment, provider, device and load acceptance</x:v>
       </x:c>
       <x:c r="I11" s="103"/>
       <x:c r="J11" s="104"/>
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>10 October: PR #7 review findings addressed. Dealer slug claims now serialize through the unique index; forced overlapping registrations pass. Owned detail fixtures pass in two repeated 2-worker desktop/mobile runs. Contrasting search fixtures reject disabled car assembly and bike fuel predicates. Stage 6.2 still needs PR re-review and deployment/provider/device/load acceptance.</x:v>
+        <x:v>11 October: PR #7 second review findings addressed. Dealer registration locks owner before dealer and rechecks profile in the same transaction; same-account same/different-name and different-owner forced schedules pass desktop/mobile. Overlap test now requires B to wait on this test's A backend, not a global blocked INSERT count. Expired dashboard badge contrast corrected. Clean local acceptance: 22 DB, 101 routes, 172 browser pass/1 planned skip, including two local WebKit smokes (navigation under reduced motion) and three recovery cases. Default-motion local WebKit navigation timed out; CI and real-device gates remain separate. New-head CI/re-review and deployment/provider/device/load acceptance remain open.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17900221fb934dbe"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e7b27d604fc4beb"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>10 October PR #7 re-review found concurrent dealer slug 23505, shared-photo test race and non-discriminating assembly/fuel fixtures. Atomic slug insert and suffix retry preserve dealer/user transaction. Forced authenticated overlap desktop/mobile passes; isolated detail fixtures pass twice with 2 workers; both filter-removal mutations fail the intended DB cases. Fresh full local suite: 22 DB, 168 browser pass/1 planned skip, 101 routes, check/lint/build. New exact-head CI/re-review and live deployment/provider/device gates remain open.</x:v>
+        <x:v>11 October PR #7 second re-review found same-account dealer 23505 and a false-positive overlap test. Owner-first transactional lock and in-transaction dealer recheck make duplicate requests idempotent; exact B-to-A database wait replaces global blocked-INSERT count. Forced desktop/mobile same/different-name tests pass. Full clean local run: 22 DB, 101 routes, 172 browser pass/1 planned skip, check/lint/build. Dashboard expired badge contrast and local WebKit reduced-motion smoke stability were also addressed; default-motion local navigation timed out. New exact-head CI/re-review and staging/live-provider/device/load gates remain open.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2269,7 +2269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="133" t="str">
-        <x:v>10 October 2026: PR #7 review findings addressed on feature branch. Forced dealer registration overlap, owned parallel photo fixtures and discriminating assembly/fuel search tests pass locally. Full acceptance: 22 isolated DB, 168 browser pass/1 planned skip, 101-route sweep, check/lint/build. New head CI/re-review and staging/live provider, infrastructure, load and real-device gates remain open.</x:v>
+        <x:v>11 October 2026: PR #7 second review P2/P3 fixed on feature branch. Same-account dealer registration serialized with owner-first lock; exact backend wait proves different-owner slug contention. Clean local acceptance: 22 isolated DB, 101 routes, 172 browser pass/1 planned skip; check/lint/build pass. New-head CI/re-review and staging/live-provider, infrastructure, load and real-device gates remain open.</x:v>
       </x:c>
       <x:c r="B2" s="133"/>
       <x:c r="C2" s="133"/>
@@ -2720,7 +2720,7 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>PR #7 prior head CI #66 green. Review fixes add atomic concurrent dealer slug claim, owned parallel photo fixtures and contrasting search filters. Fresh local 22 DB, 168 browser pass/1 planned skip, check/lint/build, 101-route sweep pass; updated-head CI pending.</x:v>
+        <x:v>PR #7 prior-head CI #67 green. Second review fixes same-account duplicate registration and forced-overlap test proof; final local 22 DB, 101 routes, 172 browser pass/1 skip, check/lint/build pass. New exact-head CI pending.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
         <x:v>Require green new-head CI and independent review; confirm branch protection. Persistent staging and live acceptance remain open.</x:v>
@@ -2955,7 +2955,7 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Local desktop/mobile suite now includes forced simultaneous same-name dealer registration, owned listing/photo details with two 2-worker repeats, and every service intermediate transition. Full browser suite 168 pass/1 planned skip; 22 DB cases pass. New head review pending.</x:v>
+        <x:v>Desktop/mobile forced dealer registration covers different owners plus same account with same or different names; test observes exact B-to-A backend blocking relation. Owned photo/details, search contrasts and service transitions remain covered. Clean browser 172 pass/1 planned skip; DB 22 pass. New-head review pending.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
         <x:v>New branch CI and maintainer review; live provider, staging and real-device acceptance remain separately tracked.</x:v>
@@ -8454,10 +8454,10 @@
         <x:v>Happy path; duplicate user; duplicate slug; invalid data</x:v>
       </x:c>
       <x:c r="N134" s="136" t="str">
-        <x:v>Dealer registration and owner settings/logo are implemented. Desktop/mobile acceptance creates a dealer/dashboard and verifies account/dealer write limits. Duplicate-slug edge acceptance remains in T-031.</x:v>
+        <x:v>Dealer registration and owner settings/logo implemented. Concurrent same-account duplicate submissions serialize on the owner row and retain exactly one original profile; different-owner slug claims resolve root/root-2. Desktop/mobile forced HTTP acceptance passes; live provider acceptance remains.</x:v>
       </x:c>
       <x:c r="O134" s="136" t="str">
-        <x:v>Complete remaining registration edge cases and live provider acceptance.</x:v>
+        <x:v>Obtain new-head independent review and live operational/provider acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
@@ -10663,7 +10663,7 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>10 Oct review fixes: full desktop/mobile Chromium, two WebKit smoke and recovery suite 168 pass/1 planned skip; 22 isolated DB, 101 routes, check/lint/build pass. New exact-head CI/re-review and live provider/device acceptance remain.</x:v>
+        <x:v>11 Oct clean local acceptance: desktop/mobile Chromium, two local WebKit smoke (navigation in reduced motion) and three recovery cases total 172 browser pass/1 planned skip; 22 DB, 101 routes, check/lint/build pass. Default-motion local WebKit navigation timed out; new exact-head CI/re-review and live provider/device acceptance remain.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
         <x:v>Latest-head CI and independent review; staging, live provider and real-device acceptance remain.</x:v>
@@ -10898,7 +10898,7 @@
         <x:v>Checklist review; defect retest</x:v>
       </x:c>
       <x:c r="N186" s="136" t="str">
-        <x:v>Test Matrix records revised local evidence for concurrent dealer registration, isolated detail photos and discriminating assembly/fuel search. Candidate 22 DB, 168 browser pass/1 planned skip, 101 routes, check/lint/build. Live-provider/real-device sign-off remains open.</x:v>
+        <x:v>Test Matrix T-031 now covers different-owner exact B-to-A slug contention and same-account same/different-name forced registration; owned detail photos and discriminatory assembly/fuel filters remain covered. Clean local 22 DB, 101 routes, 172 browser pass/1 skip. Live-provider/real-device sign-off open.</x:v>
       </x:c>
       <x:c r="O186" s="136" t="str">
         <x:v>Obtain branch review and record candidate-specific staging, live provider, real-device, production infrastructure and load evidence before launch sign-off.</x:v>
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e4f8bd997304144"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd98b671e79d74a80"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12869,7 +12869,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc18b8b44bcec4f9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15491b54efe64e17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13742,10 +13742,10 @@
         <x:v>Integration + E2E</x:v>
       </x:c>
       <x:c r="E35" s="141" t="str">
-        <x:v>Desktop/mobile authenticated registration: sequential duplicate and forced overlapping same-name submits both create one dealer each, root/root-2 permanent slugs, no server error or duplicate on revisit.</x:v>
+        <x:v>Authenticated desktop/mobile registration: different owners contend on same slug with exact B-to-A PostgreSQL wait; same account submits same/different names concurrently behind owner lock. Both responses handled, first permanent profile preserved, exactly one profile per account, no duplicate on revisit.</x:v>
       </x:c>
       <x:c r="F35" s="141" t="str">
-        <x:v>Local pass including forced concurrency; live operational acceptance pending.</x:v>
+        <x:v>Local pass on forced exact lock schedules; new-head independent review and live operational acceptance pending.</x:v>
       </x:c>
       <x:c r="G35" s="141" t="str">
         <x:v>Authenticated individual</x:v>
@@ -14437,7 +14437,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83187b6e2b2d47e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e37bc25434a4e9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14663,7 +14663,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02775159df4746b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R918ce2a9692a49c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Harden prelaunch upload and reporting paths with local acceptance
</commit_message>
<xml_diff>
--- a/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
+++ b/docs/JaniWheels_Complete_Feature_Development_Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdbeddc949b284974"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="Rd7360ac85a4a4532"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R37aedbd0a99741b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R35550f6874e74f07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="Rd362bf76ed2f4498"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="Rd2fcb34825ee4910"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="R555ebf80ce7c478f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R76026efacb3346c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance &amp; Usage" sheetId="2" r:id="R635bce7103724939"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Tracker" sheetId="3" r:id="R63ee9aa259d04bbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Roadmap" sheetId="4" r:id="R3b2c451ca8174c50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Matrix" sheetId="5" r:id="R53054a4093bb47ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope Guardrails" sheetId="6" r:id="R483febfead3f4b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" r:id="Rdc67905e6d2140c7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -890,7 +890,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb26e38f36a114c54"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Raa062310f29a4d61"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1175,7 +1175,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="86" t="str">
-        <x:v>JaniWheels V1 Development Control Sheet - 10 October 2026</x:v>
+        <x:v>JaniWheels V1 Development Control Sheet - 13 October 2026</x:v>
       </x:c>
       <x:c r="B1" s="86"/>
       <x:c r="C1" s="86"/>
@@ -1253,7 +1253,7 @@
         <x:v>Current branch</x:v>
       </x:c>
       <x:c r="H5" s="93" t="str">
-        <x:v>codex/local-acceptance-backlog; PR #7</x:v>
+        <x:v>codex/prelaunch-security-qa; review pending</x:v>
       </x:c>
       <x:c r="I5" s="93"/>
       <x:c r="J5" s="94"/>
@@ -1264,7 +1264,7 @@
       </x:c>
       <x:c r="B6" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>157</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="C6" s="88"/>
       <x:c r="D6" s="97" t="str">
@@ -1280,7 +1280,7 @@
         <x:v>Current stage</x:v>
       </x:c>
       <x:c r="H6" s="98" t="str">
-        <x:v>PR #6 merged; Stage 6.2 local test backlog verified on feature branch</x:v>
+        <x:v>PR #7 merged; prehosting local security and QA verified</x:v>
       </x:c>
       <x:c r="I6" s="98"/>
       <x:c r="J6" s="99"/>
@@ -1291,7 +1291,7 @@
       </x:c>
       <x:c r="B7" s="96" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Complete on Feature Branch - Awaiting Review")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="88"/>
       <x:c r="D7" s="97" t="str">
@@ -1307,7 +1307,7 @@
         <x:v>Current PR / CI</x:v>
       </x:c>
       <x:c r="H7" s="98" t="str">
-        <x:v>PR #7 second re-review P2/P3 fixed locally; new exact-head CI and independent re-review pending.</x:v>
+        <x:v>New candidate CI and independent exact-head review pending.</x:v>
       </x:c>
       <x:c r="I7" s="98"/>
       <x:c r="J7" s="99"/>
@@ -1328,7 +1328,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="F8" s="99" t="str">
-        <x:v>Review-fix build passed; max JS 128 KB</x:v>
+        <x:v>Prehosting production build passed; maximum JS 128 KB</x:v>
       </x:c>
       <x:c r="G8" s="97" t="str">
         <x:v>Next functionality</x:v>
@@ -1361,7 +1361,7 @@
         <x:v>Browser QA</x:v>
       </x:c>
       <x:c r="H9" s="98" t="str">
-        <x:v>Local: 22 DB, 101 routes, 172 browser pass/1 planned skip; check/lint/build pass. WebKit navigation uses reduced motion; default-motion local run timed out.</x:v>
+        <x:v>Local: 22 DB, 101 routes, 179 browser pass/1 planned skip, including 3 WebKit and recovery cases.</x:v>
       </x:c>
       <x:c r="I9" s="98"/>
       <x:c r="J9" s="99"/>
@@ -1409,13 +1409,13 @@
         <x:v>Partial pass</x:v>
       </x:c>
       <x:c r="F11" s="104" t="str">
-        <x:v>Two P2 fixes locally verified; independent re-review pending</x:v>
+        <x:v>Local checks passed; deployed security/load assessment open</x:v>
       </x:c>
       <x:c r="G11" s="102" t="str">
         <x:v>Final QA blocker</x:v>
       </x:c>
       <x:c r="H11" s="103" t="str">
-        <x:v>New exact-head CI/re-review plus deployment, provider, device and load acceptance</x:v>
+        <x:v>New-head CI/review; deployed provider, proxy, device, backup and load acceptance</x:v>
       </x:c>
       <x:c r="I11" s="103"/>
       <x:c r="J11" s="104"/>
@@ -1468,7 +1468,7 @@
       </x:c>
       <x:c r="B15" s="106" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Completed")</x:f>
-        <x:v>157</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="C15" s="107" t="str">
         <x:v>Implemented and available in current code; does not mean production launch approval</x:v>
@@ -1487,7 +1487,7 @@
       </x:c>
       <x:c r="B16" s="109" t="n">
         <x:f>COUNTIF('Feature Tracker'!$F$5:$F$215,"Complete on Feature Branch - Awaiting Review")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C16" s="110" t="str">
         <x:v>Implementation verified on feature branch; PR review/merge outstanding</x:v>
@@ -1640,7 +1640,7 @@
         <x:v>Stage 6.2 CI and acceptance - in progress</x:v>
       </x:c>
       <x:c r="C25" s="110" t="str">
-        <x:v>11 October: PR #7 second review findings addressed. Dealer registration locks owner before dealer and rechecks profile in the same transaction; same-account same/different-name and different-owner forced schedules pass desktop/mobile. Overlap test now requires B to wait on this test's A backend, not a global blocked INSERT count. Expired dashboard badge contrast corrected. Clean local acceptance: 22 DB, 101 routes, 172 browser pass/1 planned skip, including two local WebKit smokes (navigation under reduced motion) and three recovery cases. Default-motion local WebKit navigation timed out; CI and real-device gates remain separate. New-head CI/re-review and deployment/provider/device/load acceptance remain open.</x:v>
+        <x:v>13 October: PR #7 merged. Prehosting branch hardens upload body limits, proxy IP trust, anonymous report identity and retention ledger clock. Fresh local check/lint/build, 22 DB, 101 routes, 179 browser pass/1 planned skip; local WebKit default-motion navigation passes. Local 100-request read smoke has zero errors; 20,000-listing query sample rolled back. Production audit zero; ten dev-tool advisories. Candidate CI/review and deployed provider, proxy, device, backup and 500-user load gates remain open. See docs/PREHOSTING_ACCEPTANCE.md.</x:v>
       </x:c>
       <x:c r="D25" s="88"/>
       <x:c r="E25" s="88"/>
@@ -1775,7 +1775,7 @@
     <x:mergeCell ref="A23:C23"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e7b27d604fc4beb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d2cc5c586e54cc3"/>
 </x:worksheet>
 </file>
 
@@ -1882,7 +1882,7 @@
         <x:v>Current checkpoint</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
-        <x:v>11 October PR #7 second re-review found same-account dealer 23505 and a false-positive overlap test. Owner-first transactional lock and in-transaction dealer recheck make duplicate requests idempotent; exact B-to-A database wait replaces global blocked-INSERT count. Forced desktop/mobile same/different-name tests pass. Full clean local run: 22 DB, 101 routes, 172 browser pass/1 planned skip, check/lint/build. Dashboard expired badge contrast and local WebKit reduced-motion smoke stability were also addressed; default-motion local navigation timed out. New exact-head CI/re-review and staging/live-provider/device/load gates remain open.</x:v>
+        <x:v>13 October prehosting candidate: PR #7 merged; local upload/proxy/report/retention hardening verified. Fresh 22 DB, 101 routes, 179 browser pass/1 skip, check/lint/build, local read smoke and 20,000-listing query sample. Production npm audit zero; ten dev-tool advisories. Independent new-head review and all deployment/provider/real-device/capacity gates remain open. See docs/PREHOSTING_ACCEPTANCE.md.</x:v>
       </x:c>
       <x:c r="C9" s="130"/>
       <x:c r="D9" s="130"/>
@@ -2269,7 +2269,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="133" t="str">
-        <x:v>11 October 2026: PR #7 second review P2/P3 fixed on feature branch. Same-account dealer registration serialized with owner-first lock; exact backend wait proves different-owner slug contention. Clean local acceptance: 22 isolated DB, 101 routes, 172 browser pass/1 planned skip; check/lint/build pass. New-head CI/re-review and staging/live-provider, infrastructure, load and real-device gates remain open.</x:v>
+        <x:v>13 October 2026: PR #7 merged. Prehosting security/QA branch passes check/lint/build, 22 isolated DB, 101 routes and 179 browser cases/1 planned skip; local load and 20,000-listing samples recorded. Candidate CI/review, hosting, live providers, real devices, backups and 500-user capacity remain open.</x:v>
       </x:c>
       <x:c r="B2" s="133"/>
       <x:c r="C2" s="133"/>
@@ -2720,10 +2720,10 @@
         <x:v>Deliberately failing test; protected-branch verification</x:v>
       </x:c>
       <x:c r="N12" s="136" t="str">
-        <x:v>PR #7 prior-head CI #67 green. Second review fixes same-account duplicate registration and forced-overlap test proof; final local 22 DB, 101 routes, 172 browser pass/1 skip, check/lint/build pass. New exact-head CI pending.</x:v>
+        <x:v>PR #7 merged after independent exact-head review. Current prehosting branch passes fresh local check/lint/build, 22 DB, 101 routes and 179 browser cases/1 planned skip; candidate CI and protected-branch enforcement still require verification.</x:v>
       </x:c>
       <x:c r="O12" s="136" t="str">
-        <x:v>Require green new-head CI and independent review; confirm branch protection. Persistent staging and live acceptance remain open.</x:v>
+        <x:v>Obtain green exact-head CI and independent review for prehosting PR; verify required checks and branch protection. Staging and live acceptance remain open.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2931,7 +2931,7 @@
         <x:v>Technical Foundation</x:v>
       </x:c>
       <x:c r="F17" s="136" t="str">
-        <x:v>Complete on Feature Branch - Awaiting Review</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="G17" s="137" t="n">
         <x:v>1</x:v>
@@ -2955,10 +2955,10 @@
         <x:v>E2E happy path; negative path; accessibility</x:v>
       </x:c>
       <x:c r="N17" s="136" t="str">
-        <x:v>Desktop/mobile forced dealer registration covers different owners plus same account with same or different names; test observes exact B-to-A backend blocking relation. Owned photo/details, search contrasts and service transitions remain covered. Clean browser 172 pass/1 planned skip; DB 22 pass. New-head review pending.</x:v>
+        <x:v>PR #7 merged after independent review. Fresh prehosting local run: 22 DB, 101 routes, 179 browser pass/1 planned skip across desktop/mobile Chromium, three local WebKit smokes and recovery; negative upload/report/registration cases added.</x:v>
       </x:c>
       <x:c r="O17" s="136" t="str">
-        <x:v>New branch CI and maintainer review; live provider, staging and real-device acceptance remain separately tracked.</x:v>
+        <x:v>Maintain candidate CI/review; run live-provider, staging and real-device acceptance under separate launch gates.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -10146,10 +10146,10 @@
         <x:v>IDOR; direct action calls; cross-user access</x:v>
       </x:c>
       <x:c r="N170" s="136" t="str">
-        <x:v>New direct-action cases cover shared write limits, foreign Origin, invalid admin enums/IDs/reason length, triple concurrent identical removal with one audit, stale seller action, private deleted media and complaint-hold edit preserving fields/photos. Row locks and conditional status updates protect concurrent transitions; prior auth/provider/mock acceptance retained.</x:v>
+        <x:v>Direct authorization and cross-user regressions pass in fresh local suite. New trusted-proxy IP parsing and anonymous-report source tests add tamper coverage; deployment proxy/storage assessment remains open.</x:v>
       </x:c>
       <x:c r="O170" s="136" t="str">
-        <x:v>Independent final PR security review and live provider/proxy/storage acceptance; actual devices remain separate.</x:v>
+        <x:v>Independent candidate security review, then validate configured proxy and live private storage on HTTPS staging.</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -10193,10 +10193,10 @@
         <x:v>Tampered forms; oversized text; invalid IDs</x:v>
       </x:c>
       <x:c r="N171" s="136" t="str">
-        <x:v>Runtime moderation/listing/user/dealer decision checks added beyond TypeScript types. Direct browser action invalid enum/negative ID/oversize reason cases preserve DB state; complaint-hold edit returns clear error without changing evidence.</x:v>
+        <x:v>Fresh direct malformed registration email, forged report reason/listing ID/oversized comment, vehicle taxonomy and upload size/type/body-cap cases pass. Deployment integrations remain unverified.</x:v>
       </x:c>
       <x:c r="O171" s="136" t="str">
-        <x:v>Retain local negative regression; verify final live integrations/configuration before sign-off.</x:v>
+        <x:v>Keep negative regression in CI; verify live provider/configuration behavior before launch sign-off.</x:v>
       </x:c>
     </x:row>
     <x:row r="172">
@@ -10240,10 +10240,10 @@
         <x:v>Per-IP/user; proxy spoof; reset; fail-open/closed</x:v>
       </x:c>
       <x:c r="N172" s="136" t="str">
-        <x:v>Shared seller/admin write quotas cover edits, sold/delete/reactivation/resubmission, moderation, bans, dealer verification, manual services, retention holds and avatar/logo removal. Exhaustion preserves state/audit, next-window recovery DB check passes; quota notices displayed.</x:v>
+        <x:v>Local atomic quotas and source-header tests pass. Only a configured proxy-overwritten singleton IP is accepted; cookie clearing no longer changes anonymous report identity in proxy mode. Actual proxy thresholds and alerts unverified.</x:v>
       </x:c>
       <x:c r="O172" s="136" t="str">
-        <x:v>Validate trusted proxy IP handling, production thresholds and operational alerts on staging.</x:v>
+        <x:v>On HTTPS staging, block direct Node access, overwrite the selected IP header and test forged headers, request limits and operational alerts.</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -10381,10 +10381,10 @@
         <x:v>Retention job; account deletion; backup implications</x:v>
       </x:c>
       <x:c r="N175" s="136" t="str">
-        <x:v>8 Oct reviews #1/#2/#4: atomic seller-delete receipts, receipt-aware idempotent replay, later moderator rejection preserved, cancelled alerts suppressed. Approved A windows/holds unchanged. Production backup/restore drill remains.</x:v>
+        <x:v>Retention replay now exports and validates ledger times on the database clock; future-ledger regression and existing 22 DB acceptance pass. Live backups, protected ledger export and restore drill remain open.</x:v>
       </x:c>
       <x:c r="O175" s="136" t="str">
-        <x:v>Independent review of repaired replay; deployment owner must export protected current ledger and rehearse restore before clearing maintenance.</x:v>
+        <x:v>Independently review replay change; deployment owner must configure 30-day backups, independent ledger export and restore rehearsal.</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
@@ -10428,10 +10428,10 @@
         <x:v>OWASP review; dependency; auth; IDOR; upload; headers</x:v>
       </x:c>
       <x:c r="N176" s="136" t="str">
-        <x:v>Local application review addressed stale state writes, moderation duplicate audit races, tampered runtime decisions, complaint-evidence edits, upload Origin spoofing, deleted-photo privacy and write-limit gaps. Targeted DB/browser evidence recorded; independent review and infrastructure/provider review still open.</x:v>
+        <x:v>Local security pass covers ownership/origin/rate limits, bounded image uploads, trusted proxy IP parsing, cookie-clearing report abuse, retention clock and production dependency audit (zero). CSP inline-script allowance and deployed infrastructure require separate review.</x:v>
       </x:c>
       <x:c r="O176" s="136" t="str">
-        <x:v>Independent PR review and staging provider/proxy/log/storage security assessment; close any high/critical launch finding.</x:v>
+        <x:v>Independent candidate review; assess actual HTTPS proxy, Cloudflare private media, logging/secrets and provider paths on staging; close any high/critical finding.</x:v>
       </x:c>
     </x:row>
     <x:row r="177">
@@ -10663,10 +10663,10 @@
         <x:v>Happy/negative/authz/mobile</x:v>
       </x:c>
       <x:c r="N181" s="136" t="str">
-        <x:v>11 Oct clean local acceptance: desktop/mobile Chromium, two local WebKit smoke (navigation in reduced motion) and three recovery cases total 172 browser pass/1 planned skip; 22 DB, 101 routes, check/lint/build pass. Default-motion local WebKit navigation timed out; new exact-head CI/re-review and live provider/device acceptance remain.</x:v>
+        <x:v>Fresh local acceptance: 22 DB, 101 URLs, 179 browser pass/1 planned skip; desktop/mobile Chromium, three local WebKit smokes including default-motion tap, and recovery. Candidate CI/review and live acceptance open.</x:v>
       </x:c>
       <x:c r="O181" s="136" t="str">
-        <x:v>Latest-head CI and independent review; staging, live provider and real-device acceptance remain.</x:v>
+        <x:v>Obtain exact-head CI/review; complete deployed provider, device and staging E2E acceptance.</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -10710,10 +10710,10 @@
         <x:v>Real/simulated devices; slow network</x:v>
       </x:c>
       <x:c r="N182" s="136" t="str">
-        <x:v>Full Linux CI run 49 passes mobile Chromium and WebKit navigation/photo upload. Windows local WebKit photo upload passes; navigation timed out waiting for stable Auto Parts tab while local suites ran concurrently. Actual iPhone Safari/Android Chrome HTTPS, camera, keyboard, slow-network and assistive acceptance remain required; no real-device sign-off claimed.</x:v>
+        <x:v>Local mobile Chromium core flows and three WebKit smokes pass, including default-motion tap/navigation and photo upload. WebKit uses local HTTP test cookie injection; actual iPhone/Android unverified.</x:v>
       </x:c>
       <x:c r="O182" s="136" t="str">
-        <x:v>Run real iPhone Safari and Android Chrome on HTTPS staging, including keyboard, camera/file picker, slow network and full posting/contact journeys; local WebKit smoke is not a real-device sign-off.</x:v>
+        <x:v>Run real iPhone Safari and Android Chrome on HTTPS staging with camera, keyboard, slow network and full journeys.</x:v>
       </x:c>
     </x:row>
     <x:row r="183">
@@ -10804,10 +10804,10 @@
         <x:v>Bundle report; Lighthouse; 4G profile</x:v>
       </x:c>
       <x:c r="N184" s="136" t="str">
-        <x:v>Production build remains under the 150 KB JS budget (maximum 128 KB). Local 100-request concurrency-five smoke: zero failures, p50 253 ms, p95 517 ms, max 839 ms. 10,000-row query sample verifies the newest-first index. Reports clearly distinguish local samples from production acceptance.</x:v>
+        <x:v>Prehosting production build maximum First Load JS 128 KB (&lt;150 KB). Local 100-request concurrency-five read smoke: zero failures, p50 250 ms, p95 585 ms, max 811 ms. Real media/Web Vitals remain open.</x:v>
       </x:c>
       <x:c r="O184" s="136" t="str">
-        <x:v>Measure real media/Web Vitals and representative staging capacity before launch.</x:v>
+        <x:v>Measure representative media, mobile Web Vitals and production-like host capacity on staging.</x:v>
       </x:c>
     </x:row>
     <x:row r="185">
@@ -10851,10 +10851,10 @@
         <x:v>Ramp/soak/spike; query plans; pool limits</x:v>
       </x:c>
       <x:c r="N185" s="136" t="str">
-        <x:v>Added repeatable loopback-only 100-request concurrency-five HTTP load smoke; zero failures. Synthetic 10,000-row query fixtures roll back. These are local baselines, not the required 500-user ramp/soak.</x:v>
+        <x:v>Local 100-request concurrency-five smoke passed with zero failures. 20,000 synthetic listings plus demo inventory query-plan sample rolled back; optimized first-page car lookup 0.566 ms, offset-5000 20.535 ms. This is not 500-user capacity.</x:v>
       </x:c>
       <x:c r="O185" s="136" t="str">
-        <x:v>Run representative 500-user ramp/soak with monitoring on the selected staging infrastructure.</x:v>
+        <x:v>Run monitored 500-user ramp/soak and write-path load on selected staging host with realistic data/media.</x:v>
       </x:c>
     </x:row>
     <x:row r="186">
@@ -10898,10 +10898,10 @@
         <x:v>Checklist review; defect retest</x:v>
       </x:c>
       <x:c r="N186" s="136" t="str">
-        <x:v>Test Matrix T-031 now covers different-owner exact B-to-A slug contention and same-account same/different-name forced registration; owned detail photos and discriminatory assembly/fuel filters remain covered. Clean local 22 DB, 101 routes, 172 browser pass/1 skip. Live-provider/real-device sign-off open.</x:v>
+        <x:v>Master matrix updated for fresh 179 browser/22 DB/101-route local evidence, security and performance checks; one planned browser skip. Candidate review and deployed sign-off remain open.</x:v>
       </x:c>
       <x:c r="O186" s="136" t="str">
-        <x:v>Obtain branch review and record candidate-specific staging, live provider, real-device, production infrastructure and load evidence before launch sign-off.</x:v>
+        <x:v>Record exact-head CI/review and deployment/provider/device/load evidence against each open Test Matrix case.</x:v>
       </x:c>
     </x:row>
     <x:row r="187">
@@ -12311,7 +12311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd98b671e79d74a80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1730576df6704d04"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -12869,7 +12869,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15491b54efe64e17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8dfeb112f554f78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12988,10 +12988,10 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E6" s="141" t="str">
-        <x:v>Desktop/mobile Chromium duplicate email, malformed name/password and DB user-count assertions</x:v>
+        <x:v>Desktop/mobile Chromium duplicate and malformed account cases, including direct malformed-email action and DB no-user assertion</x:v>
       </x:c>
       <x:c r="F6" s="141" t="str">
-        <x:v>Partial pass: duplicate, short name and short password rejected without new users; malformed email/phone and direct-action cases remain</x:v>
+        <x:v>Local pass for duplicate, short name/password and direct malformed email; malformed phone/provider acceptance still open</x:v>
       </x:c>
       <x:c r="G6" s="141" t="str">
         <x:v>Existing account and malformed inputs</x:v>
@@ -13144,10 +13144,10 @@
         <x:v>Unit + Integration</x:v>
       </x:c>
       <x:c r="E12" s="141" t="str">
-        <x:v>Automated seller schema boundary checks plus desktop/mobile Chromium car publication and DB verification</x:v>
+        <x:v>Seller schema boundaries plus direct forged/inactive car and bike taxonomy edits in desktop/mobile Chromium</x:v>
       </x:c>
       <x:c r="F12" s="141" t="str">
-        <x:v>Partial pass: price/year/photo limits and registration/auction conflicts; invalid IDs and direct action tampering still open</x:v>
+        <x:v>Local boundary and taxonomy tampering pass; broader live input/provider matrix remains open</x:v>
       </x:c>
       <x:c r="G12" s="141" t="str">
         <x:v>Invalid IDs, price, year, mileage, images</x:v>
@@ -13352,10 +13352,10 @@
         <x:v>Integration</x:v>
       </x:c>
       <x:c r="E20" s="141" t="str">
-        <x:v>Desktop/mobile upload WebP, owner-only pending GET/HEAD, foreign-Origin 403 and request-bucket 429; source size/count/quota guards</x:v>
+        <x:v>Desktop/mobile six-photo upload in two bounded batches; direct six-file HTTP rejection; local ten-MiB and stream body-cap checks</x:v>
       </x:c>
       <x:c r="F20" s="141" t="str">
-        <x:v>Partial pass: valid image and request limit enforced; individual size/count boundaries remain open</x:v>
+        <x:v>Local pass: six valid images stored; &gt;5/request and &gt;10 MiB/file rejected, body cap enforced without Content-Length. Live provider/edge limits open</x:v>
       </x:c>
       <x:c r="G20" s="141" t="str">
         <x:v>Representative image fixtures</x:v>
@@ -13378,10 +13378,10 @@
         <x:v>Security</x:v>
       </x:c>
       <x:c r="E21" s="141" t="str">
-        <x:v>Automated check:uploads decodes/re-encodes valid images, rejects magic-byte-only fake and unsafe keys, preserves safe legacy conversion</x:v>
+        <x:v>Local upload checks reject fake JPEG, disguised SVG, oversized file and unsafe key; re-encode strips trailing script bytes</x:v>
       </x:c>
       <x:c r="F21" s="141" t="str">
-        <x:v>Partial pass: fake image/key rejection and WebP conversion verified; comprehensive oversized, SVG/executable/polyglot HTTP matrix remains</x:v>
+        <x:v>Local pass for covered malicious fixtures; live Cloudflare lifecycle and broader adversarial matrix open</x:v>
       </x:c>
       <x:c r="G21" s="141" t="str">
         <x:v>SVG/executable/polyglot fixtures</x:v>
@@ -13898,10 +13898,10 @@
         <x:v>Integration + Security</x:v>
       </x:c>
       <x:c r="E41" s="141" t="str">
-        <x:v>Desktop/mobile Chromium anonymous/auth reports, duplicate cookie/account checks, rate-limit denial and DB assertions</x:v>
+        <x:v>Desktop/mobile duplicate reports and direct forged reason/ID/oversize rejection; source-HMAC cookie-clearing regression</x:v>
       </x:c>
       <x:c r="F41" s="141" t="str">
-        <x:v>Partial pass: duplicates and excess report writes suppressed; invalid-reason/direct-request cases remain</x:v>
+        <x:v>Local pass for covered report writes; actual trusted proxy source behavior and shared-IP policy need staging validation</x:v>
       </x:c>
       <x:c r="G41" s="141" t="str">
         <x:v>Same listing/user/cookie</x:v>
@@ -14158,10 +14158,10 @@
         <x:v>Security/load</x:v>
       </x:c>
       <x:c r="E51" s="141" t="str">
-        <x:v>Atomic PostgreSQL bucket check plus desktop/mobile sign-in, upload, contact, report, inspection, assistance, car publication and account/dealer settings denial</x:v>
+        <x:v>Atomic PostgreSQL quotas, browser denial/recovery and configured singleton proxy-header parsing tests</x:v>
       </x:c>
       <x:c r="F51" s="141" t="str">
-        <x:v>Partial pass: covered limits block excess writes; denied account/dealer profile, password and image changes preserve database state. Staging proxy, expiry and remaining actions open.</x:v>
+        <x:v>Local pass for covered limits and spoofed/unconfigured header rejection; actual edge proxy, thresholds and alerts open</x:v>
       </x:c>
       <x:c r="G51" s="141" t="str">
         <x:v>Rate limits complete</x:v>
@@ -14184,10 +14184,10 @@
         <x:v>Security review</x:v>
       </x:c>
       <x:c r="E52" s="141" t="str">
-        <x:v>Local authorization replay, upload/content/origin/rate-limit/private-read regressions and CI dependency audit</x:v>
+        <x:v>Local ownership/origin/upload/retention regression, production npm audit, and prehosting security review</x:v>
       </x:c>
       <x:c r="F52" s="141" t="str">
-        <x:v>Partial pass locally; formal infrastructure review, remaining action negatives and Cloudflare private delivery open</x:v>
+        <x:v>Partial local pass: production audit zero, no new confirmed local critical/high; independent candidate and deployed proxy/storage/CSP review open</x:v>
       </x:c>
       <x:c r="G52" s="141" t="str">
         <x:v>Feature-complete staging</x:v>
@@ -14210,10 +14210,10 @@
         <x:v>Database performance</x:v>
       </x:c>
       <x:c r="E53" s="141" t="str">
-        <x:v>Not run</x:v>
+        <x:v>20,000 synthetic listing EXPLAIN ANALYZE sample in isolated PostgreSQL; fixture rollback; core and full browse joins</x:v>
       </x:c>
       <x:c r="F53" s="141" t="str">
-        <x:v>Pre-launch</x:v>
+        <x:v>Local query-plan sample passed; optimized first-page cars 0.566 ms and offset-5000 cars 20.535 ms. Representative staging P95 open</x:v>
       </x:c>
       <x:c r="G53" s="141" t="str">
         <x:v>Production-like DB</x:v>
@@ -14236,10 +14236,10 @@
         <x:v>Load</x:v>
       </x:c>
       <x:c r="E54" s="141" t="str">
-        <x:v>Local bounded smoke and rollback-only query-plan fixtures implemented; 500-user staging ramp/soak not run</x:v>
+        <x:v>Local 100-request concurrency-five HTTP smoke plus 20,000-listing query sample; staging 500-user ramp/soak not run</x:v>
       </x:c>
       <x:c r="F54" s="141" t="str">
-        <x:v>Partial: 100 requests at concurrency five, zero failures; staging 500-user capacity remains open</x:v>
+        <x:v>Partial: local read smoke zero failures, p95 585 ms; production-like 500-user capacity open</x:v>
       </x:c>
       <x:c r="G54" s="141" t="str">
         <x:v>Production-like staging</x:v>
@@ -14437,7 +14437,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e37bc25434a4e9b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R500fa6b9ed87427c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14663,7 +14663,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R918ce2a9692a49c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d0ab4a8450f49e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>